<commit_message>
Dados atualizados em 14/09/2026 09:01
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70A61421-B196-4898-A71A-18AFB2A1BCBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B8B9601-2B09-477B-8901-55D657538979}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -2494,11 +2494,11 @@
       <sheetName val="BASE PYTHON"/>
     </sheetNames>
     <sheetDataSet>
-      <sheetData sheetId="0" refreshError="1"/>
-      <sheetData sheetId="1" refreshError="1"/>
-      <sheetData sheetId="2" refreshError="1"/>
-      <sheetData sheetId="3" refreshError="1"/>
-      <sheetData sheetId="4" refreshError="1"/>
+      <sheetData sheetId="0"/>
+      <sheetData sheetId="1"/>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3"/>
+      <sheetData sheetId="4"/>
       <sheetData sheetId="5">
         <row r="1">
           <cell r="E1" t="str">
@@ -2514,7 +2514,7 @@
             <v>4</v>
           </cell>
           <cell r="M1">
-            <v>512</v>
+            <v>570</v>
           </cell>
         </row>
         <row r="2">
@@ -2573,13 +2573,13 @@
             <v>CAMPINAS</v>
           </cell>
           <cell r="F5">
-            <v>22410.980000000007</v>
+            <v>23194.480000000007</v>
           </cell>
           <cell r="H5" t="str">
             <v>CAMPINAS</v>
           </cell>
           <cell r="I5">
-            <v>3627.7000000000003</v>
+            <v>3806.4000000000005</v>
           </cell>
         </row>
         <row r="6">
@@ -2587,13 +2587,13 @@
             <v>CENTRO</v>
           </cell>
           <cell r="F6">
-            <v>126711.73999999987</v>
+            <v>139883.35999999984</v>
           </cell>
           <cell r="H6" t="str">
             <v>CENTRO</v>
           </cell>
           <cell r="I6">
-            <v>12496.849999999999</v>
+            <v>13827.15</v>
           </cell>
           <cell r="K6" t="str">
             <v>Contagem Distinta de COD_CLIENTE</v>
@@ -2604,16 +2604,16 @@
         </row>
         <row r="7">
           <cell r="E7" t="str">
-            <v>IATAGAM JUNIOR</v>
+            <v>ECOMMERCE</v>
           </cell>
           <cell r="F7">
-            <v>55.04</v>
+            <v>144.9</v>
           </cell>
           <cell r="H7" t="str">
-            <v>INDAIATUBA</v>
+            <v>ECOMMERCE</v>
           </cell>
           <cell r="I7">
-            <v>1693.7899999999997</v>
+            <v>144.9</v>
           </cell>
           <cell r="K7" t="str">
             <v>Rótulos de Linha</v>
@@ -2630,143 +2630,134 @@
         </row>
         <row r="8">
           <cell r="E8" t="str">
+            <v>IATAGAM JUNIOR</v>
+          </cell>
+          <cell r="F8">
+            <v>55.04</v>
+          </cell>
+          <cell r="H8" t="str">
             <v>INDAIATUBA</v>
           </cell>
-          <cell r="F8">
-            <v>29203.570000000014</v>
-          </cell>
-          <cell r="H8" t="str">
-            <v>INTERLAGOS</v>
-          </cell>
           <cell r="I8">
-            <v>17551.800000000003</v>
+            <v>1693.7899999999997</v>
           </cell>
           <cell r="K8" t="str">
             <v>CAMPINAS</v>
           </cell>
           <cell r="L8">
-            <v>11</v>
+            <v>12</v>
           </cell>
           <cell r="N8">
-            <v>11</v>
+            <v>12</v>
           </cell>
         </row>
         <row r="9">
           <cell r="E9" t="str">
+            <v>INDAIATUBA</v>
+          </cell>
+          <cell r="F9">
+            <v>31196.295000000016</v>
+          </cell>
+          <cell r="H9" t="str">
             <v>INTERLAGOS</v>
           </cell>
-          <cell r="F9">
-            <v>84919.079999999973</v>
-          </cell>
-          <cell r="H9" t="str">
-            <v>JUNDIAI</v>
-          </cell>
           <cell r="I9">
-            <v>2974.46</v>
+            <v>17551.800000000003</v>
           </cell>
           <cell r="K9" t="str">
             <v>CENTRO</v>
           </cell>
           <cell r="L9">
-            <v>9</v>
-          </cell>
-          <cell r="M9">
-            <v>1</v>
+            <v>13</v>
           </cell>
           <cell r="N9">
-            <v>10</v>
+            <v>13</v>
           </cell>
         </row>
         <row r="10">
           <cell r="E10" t="str">
+            <v>INTERLAGOS</v>
+          </cell>
+          <cell r="F10">
+            <v>100281.57999999986</v>
+          </cell>
+          <cell r="H10" t="str">
             <v>JUNDIAI</v>
           </cell>
-          <cell r="F10">
-            <v>27341.650000000023</v>
-          </cell>
-          <cell r="H10" t="str">
-            <v>KEY CASA</v>
-          </cell>
           <cell r="I10">
-            <v>739.98</v>
+            <v>2974.4600000000005</v>
           </cell>
           <cell r="K10" t="str">
             <v>INDAIATUBA</v>
           </cell>
           <cell r="L10">
-            <v>8</v>
-          </cell>
-          <cell r="M10">
-            <v>1</v>
+            <v>10</v>
           </cell>
           <cell r="N10">
-            <v>9</v>
+            <v>10</v>
           </cell>
         </row>
         <row r="11">
           <cell r="E11" t="str">
+            <v>JUNDIAI</v>
+          </cell>
+          <cell r="F11">
+            <v>29316.740000000023</v>
+          </cell>
+          <cell r="H11" t="str">
             <v>KEY ABC</v>
           </cell>
-          <cell r="F11">
-            <v>69204.900000000023</v>
-          </cell>
-          <cell r="H11" t="str">
-            <v>KEY INTERIOR</v>
-          </cell>
           <cell r="I11">
-            <v>69258.200000000012</v>
+            <v>18677.400000000001</v>
           </cell>
           <cell r="K11" t="str">
             <v>INTERLAGOS</v>
           </cell>
           <cell r="L11">
-            <v>22</v>
+            <v>28</v>
           </cell>
           <cell r="M11">
-            <v>3</v>
+            <v>1</v>
           </cell>
           <cell r="N11">
-            <v>25</v>
+            <v>29</v>
           </cell>
         </row>
         <row r="12">
           <cell r="E12" t="str">
+            <v>KEY ABC</v>
+          </cell>
+          <cell r="F12">
+            <v>98323.800000000017</v>
+          </cell>
+          <cell r="H12" t="str">
             <v>KEY CASA</v>
           </cell>
-          <cell r="F12">
-            <v>152309.58000000007</v>
-          </cell>
-          <cell r="H12" t="str">
-            <v>KEY SJC</v>
-          </cell>
           <cell r="I12">
-            <v>2978.2</v>
+            <v>54275.380000000005</v>
           </cell>
           <cell r="K12" t="str">
             <v>JUNDIAI</v>
           </cell>
           <cell r="L12">
-            <v>8</v>
-          </cell>
-          <cell r="M12">
-            <v>2</v>
+            <v>11</v>
           </cell>
           <cell r="N12">
-            <v>10</v>
+            <v>11</v>
           </cell>
         </row>
         <row r="13">
           <cell r="E13" t="str">
+            <v>KEY CASA</v>
+          </cell>
+          <cell r="F13">
+            <v>205409.18000000031</v>
+          </cell>
+          <cell r="H13" t="str">
             <v>KEY INTERIOR</v>
           </cell>
-          <cell r="F13">
-            <v>347954.79999999987</v>
-          </cell>
-          <cell r="H13" t="str">
-            <v>KEY SP</v>
-          </cell>
           <cell r="I13">
-            <v>11327.7</v>
+            <v>69258.200000000012</v>
           </cell>
           <cell r="K13" t="str">
             <v>LESTE</v>
@@ -2780,25 +2771,22 @@
         </row>
         <row r="14">
           <cell r="E14" t="str">
+            <v>KEY INTERIOR</v>
+          </cell>
+          <cell r="F14">
+            <v>347954.79999999987</v>
+          </cell>
+          <cell r="H14" t="str">
             <v>KEY SJC</v>
           </cell>
-          <cell r="F14">
-            <v>15180.599999999999</v>
-          </cell>
-          <cell r="H14" t="str">
-            <v>KEY ZL</v>
-          </cell>
           <cell r="I14">
-            <v>264.39999999999998</v>
+            <v>7440.4</v>
           </cell>
           <cell r="K14" t="str">
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="L14">
-            <v>17</v>
-          </cell>
-          <cell r="M14">
-            <v>1</v>
+            <v>18</v>
           </cell>
           <cell r="N14">
             <v>18</v>
@@ -2806,42 +2794,39 @@
         </row>
         <row r="15">
           <cell r="E15" t="str">
+            <v>KEY SJC</v>
+          </cell>
+          <cell r="F15">
+            <v>19642.8</v>
+          </cell>
+          <cell r="H15" t="str">
             <v>KEY SP</v>
           </cell>
-          <cell r="F15">
-            <v>136688.40000000002</v>
-          </cell>
-          <cell r="H15" t="str">
-            <v>LESTE</v>
-          </cell>
           <cell r="I15">
-            <v>5136.3499999999995</v>
+            <v>11327.7</v>
           </cell>
           <cell r="K15" t="str">
             <v>LESTE PENHA</v>
           </cell>
           <cell r="L15">
-            <v>12</v>
-          </cell>
-          <cell r="M15">
-            <v>2</v>
+            <v>15</v>
           </cell>
           <cell r="N15">
-            <v>14</v>
+            <v>15</v>
           </cell>
         </row>
         <row r="16">
           <cell r="E16" t="str">
+            <v>KEY SP</v>
+          </cell>
+          <cell r="F16">
+            <v>145346.00000000003</v>
+          </cell>
+          <cell r="H16" t="str">
             <v>KEY ZL</v>
           </cell>
-          <cell r="F16">
-            <v>67342.790000000008</v>
-          </cell>
-          <cell r="H16" t="str">
-            <v>LESTE MOOCA</v>
-          </cell>
           <cell r="I16">
-            <v>12558.199999999995</v>
+            <v>264.39999999999998</v>
           </cell>
           <cell r="K16" t="str">
             <v>LESTE TATUAPE</v>
@@ -2855,198 +2840,186 @@
         </row>
         <row r="17">
           <cell r="E17" t="str">
+            <v>KEY ZL</v>
+          </cell>
+          <cell r="F17">
+            <v>78739.81</v>
+          </cell>
+          <cell r="H17" t="str">
             <v>LESTE</v>
           </cell>
-          <cell r="F17">
-            <v>29186.920000000009</v>
-          </cell>
-          <cell r="H17" t="str">
-            <v>LESTE PENHA</v>
-          </cell>
           <cell r="I17">
-            <v>4013.4600000000009</v>
+            <v>5556.9499999999989</v>
           </cell>
           <cell r="K17" t="str">
             <v>MOGI</v>
           </cell>
           <cell r="L17">
-            <v>4</v>
+            <v>7</v>
           </cell>
           <cell r="N17">
-            <v>4</v>
+            <v>7</v>
           </cell>
         </row>
         <row r="18">
           <cell r="E18" t="str">
+            <v>LESTE</v>
+          </cell>
+          <cell r="F18">
+            <v>31050.670000000006</v>
+          </cell>
+          <cell r="H18" t="str">
             <v>LESTE MOOCA</v>
           </cell>
-          <cell r="F18">
-            <v>79750.23500000003</v>
-          </cell>
-          <cell r="H18" t="str">
-            <v>LESTE TATUAPE</v>
-          </cell>
           <cell r="I18">
-            <v>1218.4000000000001</v>
+            <v>14553.599999999995</v>
           </cell>
           <cell r="K18" t="str">
             <v>NORTE</v>
           </cell>
           <cell r="L18">
-            <v>20</v>
+            <v>23</v>
           </cell>
           <cell r="N18">
-            <v>20</v>
+            <v>23</v>
           </cell>
         </row>
         <row r="19">
           <cell r="E19" t="str">
+            <v>LESTE MOOCA</v>
+          </cell>
+          <cell r="F19">
+            <v>84326.634999999995</v>
+          </cell>
+          <cell r="H19" t="str">
             <v>LESTE PENHA</v>
           </cell>
-          <cell r="F19">
-            <v>39576.76</v>
-          </cell>
-          <cell r="H19" t="str">
-            <v>MOGI</v>
-          </cell>
           <cell r="I19">
-            <v>3536.8200000000006</v>
+            <v>4013.4600000000009</v>
           </cell>
           <cell r="K19" t="str">
             <v>OSASCO</v>
           </cell>
           <cell r="L19">
-            <v>17</v>
-          </cell>
-          <cell r="M19">
-            <v>2</v>
+            <v>22</v>
           </cell>
           <cell r="N19">
-            <v>19</v>
+            <v>22</v>
           </cell>
         </row>
         <row r="20">
           <cell r="E20" t="str">
+            <v>LESTE PENHA</v>
+          </cell>
+          <cell r="F20">
+            <v>43855.759999999995</v>
+          </cell>
+          <cell r="H20" t="str">
             <v>LESTE TATUAPE</v>
           </cell>
-          <cell r="F20">
-            <v>43899.820000000036</v>
-          </cell>
-          <cell r="H20" t="str">
-            <v>NORTE</v>
-          </cell>
           <cell r="I20">
-            <v>10790.599999999999</v>
+            <v>1218.4000000000001</v>
           </cell>
           <cell r="K20" t="str">
             <v>PIRITUBA</v>
           </cell>
           <cell r="L20">
-            <v>8</v>
+            <v>9</v>
           </cell>
           <cell r="N20">
-            <v>8</v>
+            <v>9</v>
           </cell>
         </row>
         <row r="21">
           <cell r="E21" t="str">
+            <v>LESTE TATUAPE</v>
+          </cell>
+          <cell r="F21">
+            <v>45658.210000000028</v>
+          </cell>
+          <cell r="H21" t="str">
             <v>MOGI</v>
           </cell>
-          <cell r="F21">
-            <v>25440.569999999996</v>
-          </cell>
-          <cell r="H21" t="str">
-            <v>OSASCO</v>
-          </cell>
           <cell r="I21">
-            <v>14911.204999999994</v>
+            <v>4735.8200000000006</v>
           </cell>
           <cell r="K21" t="str">
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="L21">
-            <v>10</v>
-          </cell>
-          <cell r="M21">
-            <v>2</v>
+            <v>13</v>
           </cell>
           <cell r="N21">
-            <v>12</v>
+            <v>13</v>
           </cell>
         </row>
         <row r="22">
           <cell r="E22" t="str">
+            <v>MOGI</v>
+          </cell>
+          <cell r="F22">
+            <v>29544.7</v>
+          </cell>
+          <cell r="H22" t="str">
             <v>NORTE</v>
           </cell>
-          <cell r="F22">
-            <v>85823.090000000084</v>
-          </cell>
-          <cell r="H22" t="str">
-            <v>PIRITUBA</v>
-          </cell>
           <cell r="I22">
-            <v>3034.7000000000003</v>
+            <v>10940.499999999998</v>
           </cell>
           <cell r="K22" t="str">
             <v>SBC</v>
           </cell>
           <cell r="L22">
-            <v>16</v>
-          </cell>
-          <cell r="M22">
-            <v>3</v>
+            <v>20</v>
           </cell>
           <cell r="N22">
-            <v>18</v>
+            <v>20</v>
           </cell>
         </row>
         <row r="23">
           <cell r="E23" t="str">
+            <v>NORTE</v>
+          </cell>
+          <cell r="F23">
+            <v>96164.2</v>
+          </cell>
+          <cell r="H23" t="str">
             <v>OSASCO</v>
           </cell>
-          <cell r="F23">
-            <v>114328.69500000012</v>
-          </cell>
-          <cell r="H23" t="str">
-            <v>SANTO ANDRE</v>
-          </cell>
           <cell r="I23">
-            <v>6302.9400000000005</v>
+            <v>14911.204999999994</v>
           </cell>
           <cell r="K23" t="str">
             <v>SJC</v>
           </cell>
           <cell r="L23">
-            <v>7</v>
+            <v>8</v>
           </cell>
           <cell r="M23">
             <v>1</v>
           </cell>
           <cell r="N23">
-            <v>8</v>
+            <v>9</v>
           </cell>
         </row>
         <row r="24">
           <cell r="E24" t="str">
+            <v>OSASCO</v>
+          </cell>
+          <cell r="F24">
+            <v>125560.12500000007</v>
+          </cell>
+          <cell r="H24" t="str">
             <v>PIRITUBA</v>
           </cell>
-          <cell r="F24">
-            <v>36811.270000000026</v>
-          </cell>
-          <cell r="H24" t="str">
-            <v>SBC</v>
-          </cell>
           <cell r="I24">
-            <v>11125.239999999993</v>
+            <v>3254.9500000000003</v>
           </cell>
           <cell r="K24" t="str">
             <v>SJC/VALE</v>
           </cell>
           <cell r="L24">
-            <v>10</v>
-          </cell>
-          <cell r="M24">
-            <v>1</v>
+            <v>11</v>
           </cell>
           <cell r="N24">
             <v>11</v>
@@ -3054,70 +3027,70 @@
         </row>
         <row r="25">
           <cell r="E25" t="str">
+            <v>PIRITUBA</v>
+          </cell>
+          <cell r="F25">
+            <v>40663.720000000038</v>
+          </cell>
+          <cell r="H25" t="str">
             <v>SANTO ANDRE</v>
           </cell>
-          <cell r="F25">
-            <v>66351.140000000014</v>
-          </cell>
-          <cell r="H25" t="str">
-            <v>SJC</v>
-          </cell>
           <cell r="I25">
-            <v>1518.5800000000002</v>
+            <v>6734.5400000000009</v>
           </cell>
           <cell r="K25" t="str">
             <v>Total Geral</v>
           </cell>
           <cell r="L25">
-            <v>193</v>
+            <v>234</v>
           </cell>
           <cell r="M25">
-            <v>19</v>
+            <v>2</v>
           </cell>
           <cell r="N25">
-            <v>211</v>
+            <v>236</v>
           </cell>
         </row>
         <row r="26">
           <cell r="E26" t="str">
+            <v>SANTO ANDRE</v>
+          </cell>
+          <cell r="F26">
+            <v>68771.89</v>
+          </cell>
+          <cell r="H26" t="str">
             <v>SBC</v>
           </cell>
-          <cell r="F26">
-            <v>95578.979999999952</v>
-          </cell>
-          <cell r="H26" t="str">
-            <v>SJC/VALE</v>
-          </cell>
           <cell r="I26">
-            <v>844.31999999999994</v>
+            <v>11125.239999999993</v>
           </cell>
         </row>
         <row r="27">
           <cell r="E27" t="str">
+            <v>SBC</v>
+          </cell>
+          <cell r="F27">
+            <v>100639.89999999994</v>
+          </cell>
+          <cell r="H27" t="str">
             <v>SJC</v>
           </cell>
-          <cell r="F27">
-            <v>25035.579999999998</v>
-          </cell>
-          <cell r="H27" t="str">
-            <v>VENDEDOR INTERNO 1</v>
-          </cell>
           <cell r="I27">
-            <v>675</v>
+            <v>1518.5800000000002</v>
           </cell>
         </row>
         <row r="28">
           <cell r="E28" t="str">
+            <v>SJC</v>
+          </cell>
+          <cell r="F28">
+            <v>27935.73000000001</v>
+          </cell>
+          <cell r="H28" t="str">
             <v>SJC/VALE</v>
           </cell>
-          <cell r="F28">
-            <v>18754.78</v>
-          </cell>
-          <cell r="H28" t="str">
-            <v>Total Geral</v>
-          </cell>
           <cell r="I28">
-            <v>198578.89499999984</v>
+            <v>1399.22</v>
           </cell>
           <cell r="K28" t="str">
             <v>POSITIVAÇÃO GERAL</v>
@@ -3125,10 +3098,16 @@
         </row>
         <row r="29">
           <cell r="E29" t="str">
+            <v>SJC/VALE</v>
+          </cell>
+          <cell r="F29">
+            <v>21675.470000000005</v>
+          </cell>
+          <cell r="H29" t="str">
             <v>VENDEDOR INTERNO 1</v>
           </cell>
-          <cell r="F29">
-            <v>19519.940000000002</v>
+          <cell r="I29">
+            <v>3039</v>
           </cell>
           <cell r="K29" t="str">
             <v>DATA</v>
@@ -3139,16 +3118,30 @@
         </row>
         <row r="30">
           <cell r="E30" t="str">
+            <v>VENDEDOR INTERNO 1</v>
+          </cell>
+          <cell r="F30">
+            <v>28037.200000000004</v>
+          </cell>
+          <cell r="H30" t="str">
             <v>Total Geral</v>
           </cell>
-          <cell r="F30">
-            <v>1759380.9100000095</v>
+          <cell r="I30">
+            <v>284243.44499999977</v>
           </cell>
           <cell r="K30" t="str">
             <v>DES_TIPO_OPERACAO</v>
           </cell>
           <cell r="L30" t="str" vm="3">
             <v>(Vários itens)</v>
+          </cell>
+        </row>
+        <row r="31">
+          <cell r="E31" t="str">
+            <v>Total Geral</v>
+          </cell>
+          <cell r="F31">
+            <v>1963372.9950000106</v>
           </cell>
         </row>
         <row r="32">
@@ -3181,13 +3174,13 @@
             <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="L34">
-            <v>43</v>
+            <v>47</v>
           </cell>
           <cell r="M34">
-            <v>3</v>
+            <v>9</v>
           </cell>
           <cell r="N34">
-            <v>45</v>
+            <v>49</v>
           </cell>
         </row>
         <row r="35">
@@ -3195,13 +3188,13 @@
             <v>Total Geral</v>
           </cell>
           <cell r="L35">
-            <v>43</v>
+            <v>47</v>
           </cell>
           <cell r="M35">
-            <v>3</v>
+            <v>9</v>
           </cell>
           <cell r="N35">
-            <v>45</v>
+            <v>49</v>
           </cell>
         </row>
         <row r="47">
@@ -3358,52 +3351,36 @@
             <v>SEMANA 5</v>
           </cell>
         </row>
-        <row r="87">
-          <cell r="E87">
-            <v>96500</v>
-          </cell>
-          <cell r="F87">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="88">
-          <cell r="E88">
-            <v>103500</v>
-          </cell>
-          <cell r="F88">
-            <v>145500</v>
-          </cell>
-        </row>
-        <row r="89">
-          <cell r="E89">
-            <v>372000</v>
-          </cell>
-          <cell r="F89">
-            <v>132000</v>
-          </cell>
-        </row>
         <row r="90">
           <cell r="E90">
-            <v>129000</v>
+            <v>372000</v>
           </cell>
           <cell r="F90">
-            <v>253000</v>
+            <v>132000</v>
           </cell>
         </row>
         <row r="91">
           <cell r="E91">
-            <v>37000</v>
+            <v>129000</v>
           </cell>
           <cell r="F91">
-            <v>75000</v>
+            <v>253000</v>
           </cell>
         </row>
         <row r="92">
           <cell r="E92">
-            <v>160500</v>
+            <v>37000</v>
           </cell>
           <cell r="F92">
-            <v>45500</v>
+            <v>75000</v>
+          </cell>
+        </row>
+        <row r="93">
+          <cell r="E93">
+            <v>87000</v>
+          </cell>
+          <cell r="F93">
+            <v>89000</v>
           </cell>
         </row>
         <row r="135">
@@ -3425,13 +3402,13 @@
             <v>9</v>
           </cell>
           <cell r="F136">
-            <v>8</v>
+            <v>9</v>
           </cell>
           <cell r="H136" t="str">
-            <v>D</v>
+            <v>C</v>
           </cell>
           <cell r="I136">
-            <v>1</v>
+            <v>5</v>
           </cell>
         </row>
         <row r="137">
@@ -3439,13 +3416,13 @@
             <v>36</v>
           </cell>
           <cell r="F137">
-            <v>45</v>
+            <v>49</v>
           </cell>
           <cell r="H137" t="str">
             <v>C</v>
           </cell>
           <cell r="I137">
-            <v>11</v>
+            <v>7</v>
           </cell>
         </row>
         <row r="138">
@@ -3453,13 +3430,13 @@
             <v>9</v>
           </cell>
           <cell r="F138">
-            <v>10</v>
+            <v>13</v>
           </cell>
           <cell r="H138" t="str">
             <v>C</v>
           </cell>
           <cell r="I138">
-            <v>4</v>
+            <v>1</v>
           </cell>
         </row>
         <row r="139">
@@ -3467,13 +3444,13 @@
             <v>9</v>
           </cell>
           <cell r="F139">
-            <v>19</v>
+            <v>22</v>
           </cell>
           <cell r="H139" t="str">
-            <v>A</v>
+            <v>OBJETIVO ALCANÇADO</v>
           </cell>
           <cell r="I139">
-            <v>1</v>
+            <v>0</v>
           </cell>
         </row>
         <row r="140">
@@ -3481,7 +3458,7 @@
             <v>9</v>
           </cell>
           <cell r="F140">
-            <v>25</v>
+            <v>29</v>
           </cell>
           <cell r="H140" t="str">
             <v>OBJETIVO ALCANÇADO</v>
@@ -3509,13 +3486,13 @@
             <v>9</v>
           </cell>
           <cell r="F142">
-            <v>12</v>
+            <v>13</v>
           </cell>
           <cell r="H142" t="str">
             <v>C</v>
           </cell>
           <cell r="I142">
-            <v>2</v>
+            <v>1</v>
           </cell>
         </row>
         <row r="143">
@@ -3523,7 +3500,7 @@
             <v>9</v>
           </cell>
           <cell r="F143">
-            <v>20</v>
+            <v>23</v>
           </cell>
           <cell r="H143" t="str">
             <v>OBJETIVO ALCANÇADO</v>
@@ -3565,13 +3542,13 @@
             <v>9</v>
           </cell>
           <cell r="F146">
-            <v>9</v>
+            <v>10</v>
           </cell>
           <cell r="H146" t="str">
             <v>C</v>
           </cell>
           <cell r="I146">
-            <v>5</v>
+            <v>4</v>
           </cell>
         </row>
         <row r="147">
@@ -3579,13 +3556,13 @@
             <v>9</v>
           </cell>
           <cell r="F147">
-            <v>11</v>
+            <v>12</v>
           </cell>
           <cell r="H147" t="str">
             <v>C</v>
           </cell>
           <cell r="I147">
-            <v>3</v>
+            <v>2</v>
           </cell>
         </row>
         <row r="148">
@@ -3593,13 +3570,13 @@
             <v>9</v>
           </cell>
           <cell r="F148">
-            <v>10</v>
+            <v>11</v>
           </cell>
           <cell r="H148" t="str">
             <v>C</v>
           </cell>
           <cell r="I148">
-            <v>4</v>
+            <v>3</v>
           </cell>
         </row>
         <row r="149">
@@ -3607,13 +3584,13 @@
             <v>9</v>
           </cell>
           <cell r="F149">
-            <v>8</v>
+            <v>9</v>
           </cell>
           <cell r="H149" t="str">
-            <v>D</v>
+            <v>C</v>
           </cell>
           <cell r="I149">
-            <v>1</v>
+            <v>5</v>
           </cell>
         </row>
         <row r="150">
@@ -3621,13 +3598,13 @@
             <v>9</v>
           </cell>
           <cell r="F150">
-            <v>14</v>
+            <v>15</v>
           </cell>
           <cell r="H150" t="str">
             <v>B</v>
           </cell>
           <cell r="I150">
-            <v>3</v>
+            <v>2</v>
           </cell>
         </row>
         <row r="151">
@@ -3635,13 +3612,13 @@
             <v>9</v>
           </cell>
           <cell r="F151">
-            <v>18</v>
+            <v>20</v>
           </cell>
           <cell r="H151" t="str">
-            <v>A</v>
+            <v>OBJETIVO ALCANÇADO</v>
           </cell>
           <cell r="I151">
-            <v>2</v>
+            <v>0</v>
           </cell>
         </row>
         <row r="152">
@@ -3649,13 +3626,13 @@
             <v>9</v>
           </cell>
           <cell r="F152">
-            <v>4</v>
+            <v>7</v>
           </cell>
           <cell r="H152" t="str">
             <v>D</v>
           </cell>
           <cell r="I152">
-            <v>5</v>
+            <v>2</v>
           </cell>
         </row>
         <row r="153">
@@ -3677,10 +3654,10 @@
             <v>189</v>
           </cell>
           <cell r="F154">
-            <v>256</v>
+            <v>285</v>
           </cell>
           <cell r="I154">
-            <v>51</v>
+            <v>41</v>
           </cell>
         </row>
         <row r="158">
@@ -3702,13 +3679,13 @@
             <v>38250</v>
           </cell>
           <cell r="F159">
-            <v>25035.579999999998</v>
+            <v>27935.73000000001</v>
           </cell>
           <cell r="H159" t="str">
             <v>D</v>
           </cell>
           <cell r="I159">
-            <v>13214.420000000002</v>
+            <v>10314.26999999999</v>
           </cell>
         </row>
         <row r="160">
@@ -3716,13 +3693,13 @@
             <v>34425</v>
           </cell>
           <cell r="F160">
-            <v>19519.940000000002</v>
+            <v>28037.200000000004</v>
           </cell>
           <cell r="H160" t="str">
             <v>D</v>
           </cell>
           <cell r="I160">
-            <v>14905.059999999998</v>
+            <v>6387.7999999999956</v>
           </cell>
         </row>
         <row r="161">
@@ -3730,13 +3707,13 @@
             <v>153000</v>
           </cell>
           <cell r="F161">
-            <v>126711.73999999987</v>
+            <v>139883.35999999984</v>
           </cell>
           <cell r="H161" t="str">
             <v>D</v>
           </cell>
           <cell r="I161">
-            <v>26288.260000000126</v>
+            <v>13116.640000000159</v>
           </cell>
         </row>
         <row r="162">
@@ -3744,13 +3721,13 @@
             <v>146925</v>
           </cell>
           <cell r="F162">
-            <v>114328.69500000012</v>
+            <v>125560.12500000007</v>
           </cell>
           <cell r="H162" t="str">
             <v>D</v>
           </cell>
           <cell r="I162">
-            <v>32596.304999999877</v>
+            <v>21364.874999999927</v>
           </cell>
         </row>
         <row r="163">
@@ -3758,13 +3735,13 @@
             <v>124200</v>
           </cell>
           <cell r="F163">
-            <v>84919.079999999973</v>
+            <v>100281.57999999986</v>
           </cell>
           <cell r="H163" t="str">
             <v>D</v>
           </cell>
           <cell r="I163">
-            <v>39280.920000000027</v>
+            <v>23918.420000000144</v>
           </cell>
         </row>
         <row r="164">
@@ -3772,13 +3749,13 @@
             <v>91350</v>
           </cell>
           <cell r="F164">
-            <v>79750.23500000003</v>
+            <v>84326.634999999995</v>
           </cell>
           <cell r="H164" t="str">
             <v>D</v>
           </cell>
           <cell r="I164">
-            <v>11599.76499999997</v>
+            <v>7023.3650000000052</v>
           </cell>
         </row>
         <row r="165">
@@ -3786,13 +3763,13 @@
             <v>76500</v>
           </cell>
           <cell r="F165">
-            <v>66351.140000000014</v>
+            <v>68771.89</v>
           </cell>
           <cell r="H165" t="str">
             <v>D</v>
           </cell>
           <cell r="I165">
-            <v>10148.859999999986</v>
+            <v>7728.1100000000006</v>
           </cell>
         </row>
         <row r="166">
@@ -3800,13 +3777,13 @@
             <v>110250</v>
           </cell>
           <cell r="F166">
-            <v>85823.090000000084</v>
+            <v>96164.2</v>
           </cell>
           <cell r="H166" t="str">
             <v>D</v>
           </cell>
           <cell r="I166">
-            <v>24426.909999999916</v>
+            <v>14085.800000000003</v>
           </cell>
         </row>
         <row r="167">
@@ -3814,13 +3791,13 @@
             <v>54900</v>
           </cell>
           <cell r="F167">
-            <v>29186.920000000009</v>
+            <v>31050.670000000006</v>
           </cell>
           <cell r="H167" t="str">
             <v>D</v>
           </cell>
           <cell r="I167">
-            <v>25713.079999999991</v>
+            <v>23849.329999999994</v>
           </cell>
         </row>
         <row r="168">
@@ -3828,13 +3805,13 @@
             <v>24750</v>
           </cell>
           <cell r="F168">
-            <v>18754.78</v>
+            <v>21675.470000000005</v>
           </cell>
           <cell r="H168" t="str">
             <v>D</v>
           </cell>
           <cell r="I168">
-            <v>5995.2200000000012</v>
+            <v>3074.5299999999952</v>
           </cell>
         </row>
         <row r="169">
@@ -3842,13 +3819,13 @@
             <v>41850</v>
           </cell>
           <cell r="F169">
-            <v>29203.570000000014</v>
+            <v>31196.295000000016</v>
           </cell>
           <cell r="H169" t="str">
             <v>D</v>
           </cell>
           <cell r="I169">
-            <v>12646.429999999986</v>
+            <v>10653.704999999984</v>
           </cell>
         </row>
         <row r="170">
@@ -3856,13 +3833,13 @@
             <v>30375</v>
           </cell>
           <cell r="F170">
-            <v>22410.980000000007</v>
+            <v>23194.480000000007</v>
           </cell>
           <cell r="H170" t="str">
             <v>D</v>
           </cell>
           <cell r="I170">
-            <v>7964.0199999999932</v>
+            <v>7180.5199999999932</v>
           </cell>
         </row>
         <row r="171">
@@ -3870,13 +3847,13 @@
             <v>36450</v>
           </cell>
           <cell r="F171">
-            <v>27341.650000000023</v>
+            <v>29316.740000000023</v>
           </cell>
           <cell r="H171" t="str">
             <v>D</v>
           </cell>
           <cell r="I171">
-            <v>9108.3499999999767</v>
+            <v>7133.2599999999766</v>
           </cell>
         </row>
         <row r="172">
@@ -3884,13 +3861,13 @@
             <v>63900</v>
           </cell>
           <cell r="F172">
-            <v>36811.270000000026</v>
+            <v>40663.720000000038</v>
           </cell>
           <cell r="H172" t="str">
             <v>D</v>
           </cell>
           <cell r="I172">
-            <v>27088.729999999974</v>
+            <v>23236.279999999962</v>
           </cell>
         </row>
         <row r="173">
@@ -3898,13 +3875,13 @@
             <v>65250</v>
           </cell>
           <cell r="F173">
-            <v>39576.76</v>
+            <v>43855.759999999995</v>
           </cell>
           <cell r="H173" t="str">
             <v>D</v>
           </cell>
           <cell r="I173">
-            <v>25673.239999999998</v>
+            <v>21394.240000000005</v>
           </cell>
         </row>
         <row r="174">
@@ -3912,13 +3889,13 @@
             <v>119250</v>
           </cell>
           <cell r="F174">
-            <v>95578.979999999952</v>
+            <v>100639.89999999994</v>
           </cell>
           <cell r="H174" t="str">
             <v>D</v>
           </cell>
           <cell r="I174">
-            <v>23671.020000000048</v>
+            <v>18610.100000000064</v>
           </cell>
         </row>
         <row r="175">
@@ -3926,13 +3903,13 @@
             <v>36000</v>
           </cell>
           <cell r="F175">
-            <v>25440.569999999996</v>
+            <v>29544.7</v>
           </cell>
           <cell r="H175" t="str">
             <v>D</v>
           </cell>
           <cell r="I175">
-            <v>10559.430000000004</v>
+            <v>6455.2999999999993</v>
           </cell>
         </row>
         <row r="176">
@@ -3940,13 +3917,13 @@
             <v>66150</v>
           </cell>
           <cell r="F176">
-            <v>43899.820000000036</v>
+            <v>45658.210000000028</v>
           </cell>
           <cell r="H176" t="str">
             <v>D</v>
           </cell>
           <cell r="I176">
-            <v>22250.179999999964</v>
+            <v>20491.789999999972</v>
           </cell>
         </row>
         <row r="177">
@@ -3954,10 +3931,10 @@
             <v>1313775</v>
           </cell>
           <cell r="F177">
-            <v>970644.80000000028</v>
+            <v>1067756.6649999998</v>
           </cell>
           <cell r="I177">
-            <v>343130.19999999984</v>
+            <v>246018.33500000017</v>
           </cell>
         </row>
       </sheetData>
@@ -4802,19 +4779,19 @@
       </c>
       <c r="AD3" s="29">
         <f>IFERROR(_xlfn.XLOOKUP(Y3,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0),0)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AE3" s="29" t="str" cm="1">
         <f t="array" ref="AE3">_xlfn.IFS(AD3&gt;=Z3,"A",AD3&gt;=AA3,"B",AD3&gt;=AB3,"C",AD3&gt;=AC3,"D",TRUE,"NÃO ATINGIDO")</f>
-        <v>NÃO ATINGIDO</v>
+        <v>D</v>
       </c>
       <c r="AF3" s="29" t="str" cm="1">
         <f t="array" ref="AF3">_xlfn.IFS(AE3="NÃO ATINGIDO","D",AE3="D","C",AE3="C","B",AE3="B","A",AE3="A","OBJETIVO ALCANÇADO")</f>
-        <v>D</v>
+        <v>C</v>
       </c>
       <c r="AG3" s="29" cm="1">
         <f t="array" ref="AG3">_xlfn.IFS(AF3="D",MAX(AC3-AD3,0),AF3="C",MAX(AB3-AD3,0),AF3="B",MAX(AA3-AD3,0),AF3="A",MAX(Z3-AD3,0),AF3="OBJETIVO ALCANÇADO",0)</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AI3" t="s">
         <v>22</v>
@@ -4837,7 +4814,7 @@
       </c>
       <c r="AN3" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI3,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>25035.579999999998</v>
+        <v>27935.73000000001</v>
       </c>
       <c r="AO3" s="26" t="str" cm="1">
         <f t="array" ref="AO3">_xlfn.IFS(AN3&gt;=AJ3,"A",AN3&gt;=AK3,"B",AN3&gt;=AL3,"C",AN3&gt;=AM3,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -4849,7 +4826,7 @@
       </c>
       <c r="AQ3" s="25" cm="1">
         <f t="array" ref="AQ3">_xlfn.IFS(AP3="D",MAX(AM3-AN3,0),AP3="C",MAX(AL3-AN3,0),AP3="B",MAX(AK3-AN3,0),AP3="A",MAX(AJ3-AN3,0),AP3="OBJETIVO ALCANÇADO",0)</f>
-        <v>13214.420000000002</v>
+        <v>10314.26999999999</v>
       </c>
     </row>
     <row r="4" spans="1:43" x14ac:dyDescent="0.25">
@@ -4870,7 +4847,7 @@
       </c>
       <c r="I4" s="7">
         <f>SUM(I10:I27)</f>
-        <v>150140</v>
+        <v>300630</v>
       </c>
       <c r="J4" s="4"/>
       <c r="K4" s="4"/>
@@ -4881,7 +4858,7 @@
       </c>
       <c r="O4" s="7">
         <f>SUM(O11:O17)</f>
-        <v>661000</v>
+        <v>391000</v>
       </c>
       <c r="P4" s="4"/>
       <c r="Q4" s="4"/>
@@ -4917,7 +4894,7 @@
       </c>
       <c r="AD4" s="31">
         <f>IFERROR(_xlfn.XLOOKUP(Y4,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$M:$M,0),0)</f>
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="AE4" s="31" t="str" cm="1">
         <f t="array" ref="AE4">_xlfn.IFS(AD4&gt;=Z4,"A",AD4&gt;=AA4,"B",AD4&gt;=AB4,"C",AD4&gt;=AC4,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -4929,7 +4906,7 @@
       </c>
       <c r="AG4" s="31" cm="1">
         <f t="array" ref="AG4">_xlfn.IFS(AF4="D",MAX(AC4-AD4,0),AF4="C",MAX(AB4-AD4,0),AF4="B",MAX(AA4-AD4,0),AF4="A",MAX(Z4-AD4,0),AF4="OBJETIVO ALCANÇADO",0)</f>
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="AI4" t="s">
         <v>24</v>
@@ -4952,7 +4929,7 @@
       </c>
       <c r="AN4" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI4,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>19519.940000000002</v>
+        <v>28037.200000000004</v>
       </c>
       <c r="AO4" s="26" t="str" cm="1">
         <f t="array" ref="AO4">_xlfn.IFS(AN4&gt;=AJ4,"A",AN4&gt;=AK4,"B",AN4&gt;=AL4,"C",AN4&gt;=AM4,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -4964,7 +4941,7 @@
       </c>
       <c r="AQ4" s="25" cm="1">
         <f t="array" ref="AQ4">_xlfn.IFS(AP4="D",MAX(AM4-AN4,0),AP4="C",MAX(AL4-AN4,0),AP4="B",MAX(AK4-AN4,0),AP4="A",MAX(AJ4-AN4,0),AP4="OBJETIVO ALCANÇADO",0)</f>
-        <v>14905.059999999998</v>
+        <v>6387.7999999999956</v>
       </c>
     </row>
     <row r="5" spans="1:43" x14ac:dyDescent="0.25">
@@ -4974,7 +4951,7 @@
       </c>
       <c r="C5" s="2">
         <f>SUM(D10:D36)</f>
-        <v>1759380.9100000004</v>
+        <v>1963372.9949999994</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -4985,7 +4962,7 @@
       </c>
       <c r="I5" s="7">
         <f>SUM(J10:J27)</f>
-        <v>114010.41500000001</v>
+        <v>122855.06499999999</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -4996,7 +4973,7 @@
       </c>
       <c r="O5" s="7">
         <f>SUM(P11:P17)</f>
-        <v>619826.15999999992</v>
+        <v>6348.4</v>
       </c>
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
@@ -5006,8 +4983,8 @@
         <v>1</v>
       </c>
       <c r="U5" s="4">
-        <f>SUM(V10:V26)</f>
-        <v>211</v>
+        <f ca="1">SUM(V10:V26)</f>
+        <v>236</v>
       </c>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -5032,7 +5009,7 @@
       </c>
       <c r="AD5" s="29">
         <f>IFERROR(_xlfn.XLOOKUP(Y5,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0),0)</f>
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="AE5" s="29" t="str" cm="1">
         <f t="array" ref="AE5">_xlfn.IFS(AD5&gt;=Z5,"A",AD5&gt;=AA5,"B",AD5&gt;=AB5,"C",AD5&gt;=AC5,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -5044,7 +5021,7 @@
       </c>
       <c r="AG5" s="29" cm="1">
         <f t="array" ref="AG5">_xlfn.IFS(AF5="D",MAX(AC5-AD5,0),AF5="C",MAX(AB5-AD5,0),AF5="B",MAX(AA5-AD5,0),AF5="A",MAX(Z5-AD5,0),AF5="OBJETIVO ALCANÇADO",0)</f>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AI5" t="s">
         <v>8</v>
@@ -5067,7 +5044,7 @@
       </c>
       <c r="AN5" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI5,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>126711.73999999987</v>
+        <v>139883.35999999984</v>
       </c>
       <c r="AO5" s="26" t="str" cm="1">
         <f t="array" ref="AO5">_xlfn.IFS(AN5&gt;=AJ5,"A",AN5&gt;=AK5,"B",AN5&gt;=AL5,"C",AN5&gt;=AM5,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -5079,7 +5056,7 @@
       </c>
       <c r="AQ5" s="25" cm="1">
         <f t="array" ref="AQ5">_xlfn.IFS(AP5="D",MAX(AM5-AN5,0),AP5="C",MAX(AL5-AN5,0),AP5="B",MAX(AK5-AN5,0),AP5="A",MAX(AJ5-AN5,0),AP5="OBJETIVO ALCANÇADO",0)</f>
-        <v>26288.260000000126</v>
+        <v>13116.640000000159</v>
       </c>
     </row>
     <row r="6" spans="1:43" x14ac:dyDescent="0.25">
@@ -5089,7 +5066,7 @@
       </c>
       <c r="C6" s="2">
         <f>C4-C5</f>
-        <v>4143119.09</v>
+        <v>3939127.0050000008</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="4"/>
@@ -5100,7 +5077,7 @@
       </c>
       <c r="I6" s="7">
         <f>I4-I5</f>
-        <v>36129.584999999992</v>
+        <v>177774.935</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -5111,7 +5088,7 @@
       </c>
       <c r="O6" s="7">
         <f>O4-O5</f>
-        <v>41173.840000000084</v>
+        <v>384651.6</v>
       </c>
       <c r="P6" s="4"/>
       <c r="Q6" s="4"/>
@@ -5121,8 +5098,8 @@
         <v>2</v>
       </c>
       <c r="U6" s="4">
-        <f>U4-U5</f>
-        <v>129</v>
+        <f ca="1">U4-U5</f>
+        <v>104</v>
       </c>
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
@@ -5147,19 +5124,19 @@
       </c>
       <c r="AD6" s="31">
         <f>IFERROR(_xlfn.XLOOKUP(Y6,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0),0)</f>
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="AE6" s="31" t="str" cm="1">
         <f t="array" ref="AE6">_xlfn.IFS(AD6&gt;=Z6,"A",AD6&gt;=AA6,"B",AD6&gt;=AB6,"C",AD6&gt;=AC6,"D",TRUE,"NÃO ATINGIDO")</f>
-        <v>B</v>
+        <v>A</v>
       </c>
       <c r="AF6" s="31" t="str" cm="1">
         <f t="array" ref="AF6">_xlfn.IFS(AE6="NÃO ATINGIDO","D",AE6="D","C",AE6="C","B",AE6="B","A",AE6="A","OBJETIVO ALCANÇADO")</f>
-        <v>A</v>
+        <v>OBJETIVO ALCANÇADO</v>
       </c>
       <c r="AG6" s="31" cm="1">
         <f t="array" ref="AG6">_xlfn.IFS(AF6="D",MAX(AC6-AD6,0),AF6="C",MAX(AB6-AD6,0),AF6="B",MAX(AA6-AD6,0),AF6="A",MAX(Z6-AD6,0),AF6="OBJETIVO ALCANÇADO",0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AI6" t="s">
         <v>18</v>
@@ -5182,7 +5159,7 @@
       </c>
       <c r="AN6" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI6,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>114328.69500000012</v>
+        <v>125560.12500000007</v>
       </c>
       <c r="AO6" s="26" t="str" cm="1">
         <f t="array" ref="AO6">_xlfn.IFS(AN6&gt;=AJ6,"A",AN6&gt;=AK6,"B",AN6&gt;=AL6,"C",AN6&gt;=AM6,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -5194,7 +5171,7 @@
       </c>
       <c r="AQ6" s="25" cm="1">
         <f t="array" ref="AQ6">_xlfn.IFS(AP6="D",MAX(AM6-AN6,0),AP6="C",MAX(AL6-AN6,0),AP6="B",MAX(AK6-AN6,0),AP6="A",MAX(AJ6-AN6,0),AP6="OBJETIVO ALCANÇADO",0)</f>
-        <v>32596.304999999877</v>
+        <v>21364.874999999927</v>
       </c>
     </row>
     <row r="7" spans="1:43" x14ac:dyDescent="0.25">
@@ -5204,7 +5181,7 @@
       </c>
       <c r="C7" s="3">
         <f>1-(C6/C4)</f>
-        <v>0.29807385175772982</v>
+        <v>0.33263413722998714</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="4"/>
@@ -5215,7 +5192,7 @@
       </c>
       <c r="I7" s="3">
         <f>1-(I6/I4)</f>
-        <v>0.7593606966830958</v>
+        <v>0.4086587000632006</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -5226,7 +5203,7 @@
       </c>
       <c r="O7" s="3">
         <f>1-(O6/O4)</f>
-        <v>0.93770977307110426</v>
+        <v>1.623631713554996E-2</v>
       </c>
       <c r="P7" s="4"/>
       <c r="Q7" s="4"/>
@@ -5236,8 +5213,8 @@
         <v>3</v>
       </c>
       <c r="U7" s="3">
-        <f>1-(U6/U4)</f>
-        <v>0.62058823529411766</v>
+        <f ca="1">1-(U6/U4)</f>
+        <v>0.69411764705882351</v>
       </c>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
@@ -5262,7 +5239,7 @@
       </c>
       <c r="AD7" s="29">
         <f>IFERROR(_xlfn.XLOOKUP(Y7,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0),0)</f>
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="AE7" s="29" t="str" cm="1">
         <f t="array" ref="AE7">_xlfn.IFS(AD7&gt;=Z7,"A",AD7&gt;=AA7,"B",AD7&gt;=AB7,"C",AD7&gt;=AC7,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -5297,7 +5274,7 @@
       </c>
       <c r="AN7" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI7,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>84919.079999999973</v>
+        <v>100281.57999999986</v>
       </c>
       <c r="AO7" s="26" t="str" cm="1">
         <f t="array" ref="AO7">_xlfn.IFS(AN7&gt;=AJ7,"A",AN7&gt;=AK7,"B",AN7&gt;=AL7,"C",AN7&gt;=AM7,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -5309,7 +5286,7 @@
       </c>
       <c r="AQ7" s="25" cm="1">
         <f t="array" ref="AQ7">_xlfn.IFS(AP7="D",MAX(AM7-AN7,0),AP7="C",MAX(AL7-AN7,0),AP7="B",MAX(AK7-AN7,0),AP7="A",MAX(AJ7-AN7,0),AP7="OBJETIVO ALCANÇADO",0)</f>
-        <v>39280.920000000027</v>
+        <v>23918.420000000144</v>
       </c>
     </row>
     <row r="8" spans="1:43" x14ac:dyDescent="0.25">
@@ -5391,7 +5368,7 @@
       </c>
       <c r="AN8" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI8,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>79750.23500000003</v>
+        <v>84326.634999999995</v>
       </c>
       <c r="AO8" s="26" t="str" cm="1">
         <f t="array" ref="AO8">_xlfn.IFS(AN8&gt;=AJ8,"A",AN8&gt;=AK8,"B",AN8&gt;=AL8,"C",AN8&gt;=AM8,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -5403,7 +5380,7 @@
       </c>
       <c r="AQ8" s="25" cm="1">
         <f t="array" ref="AQ8">_xlfn.IFS(AP8="D",MAX(AM8-AN8,0),AP8="C",MAX(AL8-AN8,0),AP8="B",MAX(AK8-AN8,0),AP8="A",MAX(AJ8-AN8,0),AP8="OBJETIVO ALCANÇADO",0)</f>
-        <v>11599.76499999997</v>
+        <v>7023.3650000000052</v>
       </c>
     </row>
     <row r="9" spans="1:43" x14ac:dyDescent="0.25">
@@ -5442,7 +5419,7 @@
       <c r="M9" s="4"/>
       <c r="N9" s="4"/>
       <c r="O9" s="8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="P9" s="4"/>
       <c r="Q9" s="4"/>
@@ -5483,7 +5460,7 @@
       </c>
       <c r="AD9" s="29">
         <f>IFERROR(_xlfn.XLOOKUP(Y9,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0),0)</f>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="AE9" s="29" t="str" cm="1">
         <f t="array" ref="AE9">_xlfn.IFS(AD9&gt;=Z9,"A",AD9&gt;=AA9,"B",AD9&gt;=AB9,"C",AD9&gt;=AC9,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -5495,7 +5472,7 @@
       </c>
       <c r="AG9" s="29" cm="1">
         <f t="array" ref="AG9">_xlfn.IFS(AF9="D",MAX(AC9-AD9,0),AF9="C",MAX(AB9-AD9,0),AF9="B",MAX(AA9-AD9,0),AF9="A",MAX(Z9-AD9,0),AF9="OBJETIVO ALCANÇADO",0)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AI9" t="s">
         <v>20</v>
@@ -5518,7 +5495,7 @@
       </c>
       <c r="AN9" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI9,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>66351.140000000014</v>
+        <v>68771.89</v>
       </c>
       <c r="AO9" s="26" t="str" cm="1">
         <f t="array" ref="AO9">_xlfn.IFS(AN9&gt;=AJ9,"A",AN9&gt;=AK9,"B",AN9&gt;=AL9,"C",AN9&gt;=AM9,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -5530,7 +5507,7 @@
       </c>
       <c r="AQ9" s="25" cm="1">
         <f t="array" ref="AQ9">_xlfn.IFS(AP9="D",MAX(AM9-AN9,0),AP9="C",MAX(AL9-AN9,0),AP9="B",MAX(AK9-AN9,0),AP9="A",MAX(AJ9-AN9,0),AP9="OBJETIVO ALCANÇADO",0)</f>
-        <v>10148.859999999986</v>
+        <v>7728.1100000000006</v>
       </c>
     </row>
     <row r="10" spans="1:43" x14ac:dyDescent="0.25">
@@ -5546,11 +5523,11 @@
       </c>
       <c r="D10" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>22410.980000000007</v>
+        <v>23194.480000000007</v>
       </c>
       <c r="E10" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>45089.01999999999</v>
+        <v>44305.51999999999</v>
       </c>
       <c r="F10" s="4"/>
       <c r="G10" s="18" t="s">
@@ -5561,7 +5538,7 @@
       </c>
       <c r="I10" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>17000</v>
+        <v>30650</v>
       </c>
       <c r="J10" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
@@ -5569,7 +5546,7 @@
       </c>
       <c r="K10" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>2088.7950000000055</v>
+        <v>15738.795000000006</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4" t="s">
@@ -5599,12 +5576,12 @@
         <v>20</v>
       </c>
       <c r="V10" s="17">
-        <f>VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
-        <v>11</v>
+        <f ca="1">VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
+        <v>12</v>
       </c>
       <c r="W10" s="17">
-        <f>U10-V10</f>
-        <v>9</v>
+        <f ca="1">U10-V10</f>
+        <v>8</v>
       </c>
       <c r="Y10" s="33" t="s">
         <v>17</v>
@@ -5627,7 +5604,7 @@
       </c>
       <c r="AD10" s="31">
         <f>IFERROR(_xlfn.XLOOKUP(Y10,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0),0)</f>
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="AE10" s="31" t="str" cm="1">
         <f t="array" ref="AE10">_xlfn.IFS(AD10&gt;=Z10,"A",AD10&gt;=AA10,"B",AD10&gt;=AB10,"C",AD10&gt;=AC10,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -5662,7 +5639,7 @@
       </c>
       <c r="AN10" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI10,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>85823.090000000084</v>
+        <v>96164.2</v>
       </c>
       <c r="AO10" s="26" t="str" cm="1">
         <f t="array" ref="AO10">_xlfn.IFS(AN10&gt;=AJ10,"A",AN10&gt;=AK10,"B",AN10&gt;=AL10,"C",AN10&gt;=AM10,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -5674,7 +5651,7 @@
       </c>
       <c r="AQ10" s="25" cm="1">
         <f t="array" ref="AQ10">_xlfn.IFS(AP10="D",MAX(AM10-AN10,0),AP10="C",MAX(AL10-AN10,0),AP10="B",MAX(AK10-AN10,0),AP10="A",MAX(AJ10-AN10,0),AP10="OBJETIVO ALCANÇADO",0)</f>
-        <v>24426.909999999916</v>
+        <v>14085.800000000003</v>
       </c>
     </row>
     <row r="11" spans="1:43" x14ac:dyDescent="0.25">
@@ -5690,11 +5667,11 @@
       </c>
       <c r="D11" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>126711.73999999987</v>
+        <v>139883.35999999984</v>
       </c>
       <c r="E11" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>213288.26000000013</v>
+        <v>200116.64000000016</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="18" t="s">
@@ -5705,15 +5682,15 @@
       </c>
       <c r="I11" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>14780</v>
+        <v>27160</v>
       </c>
       <c r="J11" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>10790.599999999999</v>
+        <v>10940.499999999998</v>
       </c>
       <c r="K11" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3989.4000000000015</v>
+        <v>16219.500000000002</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4" t="s">
@@ -5724,15 +5701,15 @@
       </c>
       <c r="O11" s="2" cm="1">
         <f t="array" ref="O11">IFERROR(_xlfn.XLOOKUP(M11,[1]!Tabela3[[#All],[VENDEDOR]],INDEX([1]!Tabela3[#All],0,MATCH($O$9,[1]!Tabela3[#Headers],0))),0)</f>
-        <v>69500</v>
+        <v>0</v>
       </c>
       <c r="P11" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[REGIAO]","[Intervalo 2].[REGIAO].&amp;["&amp;N11&amp;"]","[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;["&amp;RIGHT($O$9,1)&amp;"]"),0)</f>
-        <v>48058.600000000013</v>
+        <v>0</v>
       </c>
       <c r="Q11" s="2">
         <f>Tabela8[[#This Row],[COMPROMISSO]]-Tabela8[[#This Row],[ATINGIDO]]</f>
-        <v>21441.399999999987</v>
+        <v>0</v>
       </c>
       <c r="R11" s="2"/>
       <c r="S11" s="17" t="s">
@@ -5746,12 +5723,12 @@
         <v>20</v>
       </c>
       <c r="V11" s="17">
-        <f>VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
-        <v>10</v>
+        <f ca="1">VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
+        <v>13</v>
       </c>
       <c r="W11" s="17">
-        <f t="shared" ref="W11:W20" si="0">U11-V11</f>
-        <v>10</v>
+        <f t="shared" ref="W11:W20" ca="1" si="0">U11-V11</f>
+        <v>7</v>
       </c>
       <c r="Y11" s="32" t="s">
         <v>12</v>
@@ -5809,7 +5786,7 @@
       </c>
       <c r="AN11" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI11,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>29186.920000000009</v>
+        <v>31050.670000000006</v>
       </c>
       <c r="AO11" s="26" t="str" cm="1">
         <f t="array" ref="AO11">_xlfn.IFS(AN11&gt;=AJ11,"A",AN11&gt;=AK11,"B",AN11&gt;=AL11,"C",AN11&gt;=AM11,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -5821,7 +5798,7 @@
       </c>
       <c r="AQ11" s="25" cm="1">
         <f t="array" ref="AQ11">_xlfn.IFS(AP11="D",MAX(AM11-AN11,0),AP11="C",MAX(AL11-AN11,0),AP11="B",MAX(AK11-AN11,0),AP11="A",MAX(AJ11-AN11,0),AP11="OBJETIVO ALCANÇADO",0)</f>
-        <v>25713.079999999991</v>
+        <v>23849.329999999994</v>
       </c>
     </row>
     <row r="12" spans="1:43" x14ac:dyDescent="0.25">
@@ -5852,15 +5829,15 @@
       </c>
       <c r="I12" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>8680</v>
+        <v>15600</v>
       </c>
       <c r="J12" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>3034.7000000000003</v>
+        <v>3254.9500000000003</v>
       </c>
       <c r="K12" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>5645.2999999999993</v>
+        <v>12345.05</v>
       </c>
       <c r="L12" s="4"/>
       <c r="M12" s="4" t="s">
@@ -5893,12 +5870,12 @@
         <v>20</v>
       </c>
       <c r="V12" s="17">
-        <f>VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
-        <v>9</v>
+        <f ca="1">VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
+        <v>10</v>
       </c>
       <c r="W12" s="17">
-        <f t="shared" si="0"/>
-        <v>11</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>10</v>
       </c>
       <c r="Y12" s="33" t="s">
         <v>23</v>
@@ -5956,7 +5933,7 @@
       </c>
       <c r="AN12" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI12,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>18754.78</v>
+        <v>21675.470000000005</v>
       </c>
       <c r="AO12" s="26" t="str" cm="1">
         <f t="array" ref="AO12">_xlfn.IFS(AN12&gt;=AJ12,"A",AN12&gt;=AK12,"B",AN12&gt;=AL12,"C",AN12&gt;=AM12,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -5968,7 +5945,7 @@
       </c>
       <c r="AQ12" s="25" cm="1">
         <f t="array" ref="AQ12">_xlfn.IFS(AP12="D",MAX(AM12-AN12,0),AP12="C",MAX(AL12-AN12,0),AP12="B",MAX(AK12-AN12,0),AP12="A",MAX(AJ12-AN12,0),AP12="OBJETIVO ALCANÇADO",0)</f>
-        <v>5995.2200000000012</v>
+        <v>3074.5299999999952</v>
       </c>
     </row>
     <row r="13" spans="1:43" x14ac:dyDescent="0.25">
@@ -5984,11 +5961,11 @@
       </c>
       <c r="D13" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>29203.570000000014</v>
+        <v>31196.295000000016</v>
       </c>
       <c r="E13" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>63796.429999999986</v>
+        <v>61803.704999999987</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="18" t="s">
@@ -5999,7 +5976,7 @@
       </c>
       <c r="I13" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>11560</v>
+        <v>23440</v>
       </c>
       <c r="J13" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
@@ -6007,7 +5984,7 @@
       </c>
       <c r="K13" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>434.76000000000749</v>
+        <v>12314.760000000007</v>
       </c>
       <c r="L13" s="4"/>
       <c r="M13" s="4" t="s">
@@ -6018,15 +5995,15 @@
       </c>
       <c r="O13" s="2" cm="1">
         <f t="array" ref="O13">IFERROR(_xlfn.XLOOKUP(M13,[1]!Tabela3[[#All],[VENDEDOR]],INDEX([1]!Tabela3[#All],0,MATCH($O$9,[1]!Tabela3[#Headers],0))),0)</f>
-        <v>81000</v>
+        <v>0</v>
       </c>
       <c r="P13" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[REGIAO]","[Intervalo 2].[REGIAO].&amp;["&amp;N13&amp;"]","[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;["&amp;RIGHT($O$9,1)&amp;"]"),0)</f>
-        <v>53921.19000000001</v>
+        <v>0</v>
       </c>
       <c r="Q13" s="2">
         <f>Tabela8[[#This Row],[COMPROMISSO]]-Tabela8[[#This Row],[ATINGIDO]]</f>
-        <v>27078.80999999999</v>
+        <v>0</v>
       </c>
       <c r="R13" s="2"/>
       <c r="S13" s="17" t="s">
@@ -6040,12 +6017,12 @@
         <v>20</v>
       </c>
       <c r="V13" s="17">
-        <f>VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
-        <v>25</v>
+        <f ca="1">VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
+        <v>29</v>
       </c>
       <c r="W13" s="17">
-        <f t="shared" si="0"/>
-        <v>-5</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>-9</v>
       </c>
       <c r="Y13" s="32" t="s">
         <v>9</v>
@@ -6068,7 +6045,7 @@
       </c>
       <c r="AD13" s="29">
         <f>IFERROR(_xlfn.XLOOKUP(Y13,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0),0)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AE13" s="29" t="str" cm="1">
         <f t="array" ref="AE13">_xlfn.IFS(AD13&gt;=Z13,"A",AD13&gt;=AA13,"B",AD13&gt;=AB13,"C",AD13&gt;=AC13,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -6080,7 +6057,7 @@
       </c>
       <c r="AG13" s="29" cm="1">
         <f t="array" ref="AG13">_xlfn.IFS(AF13="D",MAX(AC13-AD13,0),AF13="C",MAX(AB13-AD13,0),AF13="B",MAX(AA13-AD13,0),AF13="A",MAX(Z13-AD13,0),AF13="OBJETIVO ALCANÇADO",0)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AI13" t="s">
         <v>9</v>
@@ -6103,7 +6080,7 @@
       </c>
       <c r="AN13" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI13,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>29203.570000000014</v>
+        <v>31196.295000000016</v>
       </c>
       <c r="AO13" s="26" t="str" cm="1">
         <f t="array" ref="AO13">_xlfn.IFS(AN13&gt;=AJ13,"A",AN13&gt;=AK13,"B",AN13&gt;=AL13,"C",AN13&gt;=AM13,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -6115,7 +6092,7 @@
       </c>
       <c r="AQ13" s="25" cm="1">
         <f t="array" ref="AQ13">_xlfn.IFS(AP13="D",MAX(AM13-AN13,0),AP13="C",MAX(AL13-AN13,0),AP13="B",MAX(AK13-AN13,0),AP13="A",MAX(AJ13-AN13,0),AP13="OBJETIVO ALCANÇADO",0)</f>
-        <v>12646.429999999986</v>
+        <v>10653.704999999984</v>
       </c>
     </row>
     <row r="14" spans="1:43" x14ac:dyDescent="0.25">
@@ -6131,11 +6108,11 @@
       </c>
       <c r="D14" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>84919.079999999973</v>
+        <v>100281.57999999986</v>
       </c>
       <c r="E14" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>191080.92000000004</v>
+        <v>175718.42000000016</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="18" t="s">
@@ -6146,7 +6123,7 @@
       </c>
       <c r="I14" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>5350</v>
+        <v>16770</v>
       </c>
       <c r="J14" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
@@ -6154,7 +6131,7 @@
       </c>
       <c r="K14" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>4131.6000000000004</v>
+        <v>15551.6</v>
       </c>
       <c r="L14" s="4"/>
       <c r="M14" s="4" t="s">
@@ -6165,15 +6142,15 @@
       </c>
       <c r="O14" s="2" cm="1">
         <f t="array" ref="O14">IFERROR(_xlfn.XLOOKUP(M14,[1]!Tabela3[[#All],[VENDEDOR]],INDEX([1]!Tabela3[#All],0,MATCH($O$9,[1]!Tabela3[#Headers],0))),0)</f>
-        <v>360000</v>
+        <v>73000</v>
       </c>
       <c r="P14" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[REGIAO]","[Intervalo 2].[REGIAO].&amp;["&amp;N14&amp;"]","[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;["&amp;RIGHT($O$9,1)&amp;"]"),0)</f>
-        <v>345599.59999999992</v>
+        <v>0</v>
       </c>
       <c r="Q14" s="2">
         <f>Tabela8[[#This Row],[COMPROMISSO]]-Tabela8[[#This Row],[ATINGIDO]]</f>
-        <v>14400.400000000081</v>
+        <v>73000</v>
       </c>
       <c r="R14" s="2"/>
       <c r="S14" s="17" t="s">
@@ -6187,12 +6164,12 @@
         <v>20</v>
       </c>
       <c r="V14" s="17">
-        <f>VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
-        <v>10</v>
+        <f ca="1">VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
+        <v>11</v>
       </c>
       <c r="W14" s="17">
-        <f t="shared" si="0"/>
-        <v>10</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>9</v>
       </c>
       <c r="Y14" s="33" t="s">
         <v>7</v>
@@ -6215,7 +6192,7 @@
       </c>
       <c r="AD14" s="31">
         <f>IFERROR(_xlfn.XLOOKUP(Y14,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0),0)</f>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AE14" s="31" t="str" cm="1">
         <f t="array" ref="AE14">_xlfn.IFS(AD14&gt;=Z14,"A",AD14&gt;=AA14,"B",AD14&gt;=AB14,"C",AD14&gt;=AC14,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -6227,7 +6204,7 @@
       </c>
       <c r="AG14" s="31" cm="1">
         <f t="array" ref="AG14">_xlfn.IFS(AF14="D",MAX(AC14-AD14,0),AF14="C",MAX(AB14-AD14,0),AF14="B",MAX(AA14-AD14,0),AF14="A",MAX(Z14-AD14,0),AF14="OBJETIVO ALCANÇADO",0)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AI14" t="s">
         <v>7</v>
@@ -6250,7 +6227,7 @@
       </c>
       <c r="AN14" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI14,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>22410.980000000007</v>
+        <v>23194.480000000007</v>
       </c>
       <c r="AO14" s="26" t="str" cm="1">
         <f t="array" ref="AO14">_xlfn.IFS(AN14&gt;=AJ14,"A",AN14&gt;=AK14,"B",AN14&gt;=AL14,"C",AN14&gt;=AM14,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -6262,7 +6239,7 @@
       </c>
       <c r="AQ14" s="25" cm="1">
         <f t="array" ref="AQ14">_xlfn.IFS(AP14="D",MAX(AM14-AN14,0),AP14="C",MAX(AL14-AN14,0),AP14="B",MAX(AK14-AN14,0),AP14="A",MAX(AJ14-AN14,0),AP14="OBJETIVO ALCANÇADO",0)</f>
-        <v>7964.0199999999932</v>
+        <v>7180.5199999999932</v>
       </c>
     </row>
     <row r="15" spans="1:43" x14ac:dyDescent="0.25">
@@ -6278,11 +6255,11 @@
       </c>
       <c r="D15" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>27341.650000000023</v>
+        <v>29316.740000000023</v>
       </c>
       <c r="E15" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>53658.349999999977</v>
+        <v>51683.25999999998</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="18" t="s">
@@ -6293,15 +6270,15 @@
       </c>
       <c r="I15" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>20090</v>
+        <v>38000</v>
       </c>
       <c r="J15" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>12496.849999999999</v>
+        <v>13827.15</v>
       </c>
       <c r="K15" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>7593.1500000000015</v>
+        <v>24172.85</v>
       </c>
       <c r="L15" s="4"/>
       <c r="M15" s="4" t="s">
@@ -6312,15 +6289,15 @@
       </c>
       <c r="O15" s="2" cm="1">
         <f t="array" ref="O15">IFERROR(_xlfn.XLOOKUP(M15,[1]!Tabela3[[#All],[VENDEDOR]],INDEX([1]!Tabela3[#All],0,MATCH($O$9,[1]!Tabela3[#Headers],0))),0)</f>
-        <v>68000</v>
+        <v>112000</v>
       </c>
       <c r="P15" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[REGIAO]","[Intervalo 2].[REGIAO].&amp;["&amp;N15&amp;"]","[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;["&amp;RIGHT($O$9,1)&amp;"]"),0)</f>
-        <v>66628.390000000014</v>
+        <v>6348.4</v>
       </c>
       <c r="Q15" s="2">
         <f>Tabela8[[#This Row],[COMPROMISSO]]-Tabela8[[#This Row],[ATINGIDO]]</f>
-        <v>1371.609999999986</v>
+        <v>105651.6</v>
       </c>
       <c r="R15" s="2"/>
       <c r="S15" s="17" t="s">
@@ -6334,11 +6311,11 @@
         <v>20</v>
       </c>
       <c r="V15" s="17">
-        <f>VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
+        <f ca="1">VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
         <v>8</v>
       </c>
       <c r="W15" s="17">
-        <f>U15-V15</f>
+        <f ca="1">U15-V15</f>
         <v>12</v>
       </c>
       <c r="Y15" s="32" t="s">
@@ -6362,7 +6339,7 @@
       </c>
       <c r="AD15" s="29">
         <f>IFERROR(_xlfn.XLOOKUP(Y15,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0),0)</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AE15" s="29" t="str" cm="1">
         <f t="array" ref="AE15">_xlfn.IFS(AD15&gt;=Z15,"A",AD15&gt;=AA15,"B",AD15&gt;=AB15,"C",AD15&gt;=AC15,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -6374,7 +6351,7 @@
       </c>
       <c r="AG15" s="29" cm="1">
         <f t="array" ref="AG15">_xlfn.IFS(AF15="D",MAX(AC15-AD15,0),AF15="C",MAX(AB15-AD15,0),AF15="B",MAX(AA15-AD15,0),AF15="A",MAX(Z15-AD15,0),AF15="OBJETIVO ALCANÇADO",0)</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AI15" t="s">
         <v>11</v>
@@ -6397,7 +6374,7 @@
       </c>
       <c r="AN15" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI15,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>27341.650000000023</v>
+        <v>29316.740000000023</v>
       </c>
       <c r="AO15" s="26" t="str" cm="1">
         <f t="array" ref="AO15">_xlfn.IFS(AN15&gt;=AJ15,"A",AN15&gt;=AK15,"B",AN15&gt;=AL15,"C",AN15&gt;=AM15,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -6409,7 +6386,7 @@
       </c>
       <c r="AQ15" s="25" cm="1">
         <f t="array" ref="AQ15">_xlfn.IFS(AP15="D",MAX(AM15-AN15,0),AP15="C",MAX(AL15-AN15,0),AP15="B",MAX(AK15-AN15,0),AP15="A",MAX(AJ15-AN15,0),AP15="OBJETIVO ALCANÇADO",0)</f>
-        <v>9108.3499999999767</v>
+        <v>7133.2599999999766</v>
       </c>
     </row>
     <row r="16" spans="1:43" x14ac:dyDescent="0.25">
@@ -6425,11 +6402,11 @@
       </c>
       <c r="D16" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>69204.900000000023</v>
+        <v>98323.800000000017</v>
       </c>
       <c r="E16" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>280795.09999999998</v>
+        <v>251676.19999999998</v>
       </c>
       <c r="F16" s="4"/>
       <c r="G16" s="18" t="s">
@@ -6440,15 +6417,15 @@
       </c>
       <c r="I16" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>7290</v>
+        <v>19560</v>
       </c>
       <c r="J16" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>6302.9400000000005</v>
+        <v>6734.5400000000009</v>
       </c>
       <c r="K16" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>987.05999999999949</v>
+        <v>12825.46</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4" t="s">
@@ -6463,11 +6440,11 @@
       </c>
       <c r="P16" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[REGIAO]","[Intervalo 2].[REGIAO].&amp;["&amp;N16&amp;"]","[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;["&amp;RIGHT($O$9,1)&amp;"]"),0)</f>
-        <v>8811.2000000000007</v>
+        <v>0</v>
       </c>
       <c r="Q16" s="2">
         <f>Tabela8[[#This Row],[COMPROMISSO]]-Tabela8[[#This Row],[ATINGIDO]]</f>
-        <v>14188.8</v>
+        <v>23000</v>
       </c>
       <c r="R16" s="2"/>
       <c r="S16" s="17" t="s">
@@ -6481,12 +6458,12 @@
         <v>20</v>
       </c>
       <c r="V16" s="17">
-        <f>VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
-        <v>4</v>
+        <f ca="1">VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
+        <v>7</v>
       </c>
       <c r="W16" s="17">
-        <f t="shared" si="0"/>
-        <v>16</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>13</v>
       </c>
       <c r="Y16" s="33" t="s">
         <v>19</v>
@@ -6509,19 +6486,19 @@
       </c>
       <c r="AD16" s="31">
         <f>IFERROR(_xlfn.XLOOKUP(Y16,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0),0)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AE16" s="31" t="str" cm="1">
         <f t="array" ref="AE16">_xlfn.IFS(AD16&gt;=Z16,"A",AD16&gt;=AA16,"B",AD16&gt;=AB16,"C",AD16&gt;=AC16,"D",TRUE,"NÃO ATINGIDO")</f>
-        <v>NÃO ATINGIDO</v>
+        <v>D</v>
       </c>
       <c r="AF16" s="31" t="str" cm="1">
         <f t="array" ref="AF16">_xlfn.IFS(AE16="NÃO ATINGIDO","D",AE16="D","C",AE16="C","B",AE16="B","A",AE16="A","OBJETIVO ALCANÇADO")</f>
-        <v>D</v>
+        <v>C</v>
       </c>
       <c r="AG16" s="31" cm="1">
         <f t="array" ref="AG16">_xlfn.IFS(AF16="D",MAX(AC16-AD16,0),AF16="C",MAX(AB16-AD16,0),AF16="B",MAX(AA16-AD16,0),AF16="A",MAX(Z16-AD16,0),AF16="OBJETIVO ALCANÇADO",0)</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AI16" t="s">
         <v>19</v>
@@ -6544,7 +6521,7 @@
       </c>
       <c r="AN16" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI16,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>36811.270000000026</v>
+        <v>40663.720000000038</v>
       </c>
       <c r="AO16" s="26" t="str" cm="1">
         <f t="array" ref="AO16">_xlfn.IFS(AN16&gt;=AJ16,"A",AN16&gt;=AK16,"B",AN16&gt;=AL16,"C",AN16&gt;=AM16,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -6556,7 +6533,7 @@
       </c>
       <c r="AQ16" s="25" cm="1">
         <f t="array" ref="AQ16">_xlfn.IFS(AP16="D",MAX(AM16-AN16,0),AP16="C",MAX(AL16-AN16,0),AP16="B",MAX(AK16-AN16,0),AP16="A",MAX(AJ16-AN16,0),AP16="OBJETIVO ALCANÇADO",0)</f>
-        <v>27088.729999999974</v>
+        <v>23236.279999999962</v>
       </c>
     </row>
     <row r="17" spans="1:43" x14ac:dyDescent="0.25">
@@ -6572,11 +6549,11 @@
       </c>
       <c r="D17" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>152309.58000000007</v>
+        <v>205409.18000000031</v>
       </c>
       <c r="E17" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>297690.41999999993</v>
+        <v>244590.81999999969</v>
       </c>
       <c r="F17" s="4"/>
       <c r="G17" s="18" t="s">
@@ -6587,15 +6564,15 @@
       </c>
       <c r="I17" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>5290</v>
+        <v>2760</v>
       </c>
       <c r="J17" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>3536.8200000000006</v>
+        <v>4735.8200000000006</v>
       </c>
       <c r="K17" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>1753.1799999999994</v>
+        <v>-1975.8200000000006</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="4" t="s">
@@ -6606,15 +6583,15 @@
       </c>
       <c r="O17" s="2" cm="1">
         <f t="array" ref="O17">IFERROR(_xlfn.XLOOKUP(M17,[1]!Tabela3[[#All],[VENDEDOR]],INDEX([1]!Tabela3[#All],0,MATCH($O$9,[1]!Tabela3[#Headers],0))),0)</f>
-        <v>59500</v>
+        <v>183000</v>
       </c>
       <c r="P17" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[REGIAO]","[Intervalo 2].[REGIAO].&amp;["&amp;N17&amp;"]","[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;["&amp;RIGHT($O$9,1)&amp;"]"),0)</f>
-        <v>96807.179999999949</v>
+        <v>0</v>
       </c>
       <c r="Q17" s="2">
         <f>Tabela8[[#This Row],[COMPROMISSO]]-Tabela8[[#This Row],[ATINGIDO]]</f>
-        <v>-37307.179999999949</v>
+        <v>183000</v>
       </c>
       <c r="R17" s="2"/>
       <c r="S17" s="17" t="s">
@@ -6628,11 +6605,11 @@
         <v>20</v>
       </c>
       <c r="V17" s="17">
-        <f>VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
+        <f ca="1">VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
         <v>18</v>
       </c>
       <c r="W17" s="17">
-        <f t="shared" si="0"/>
+        <f t="shared" ca="1" si="0"/>
         <v>2</v>
       </c>
       <c r="Y17" s="32" t="s">
@@ -6656,7 +6633,7 @@
       </c>
       <c r="AD17" s="29">
         <f>IFERROR(_xlfn.XLOOKUP(Y17,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0),0)</f>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="AE17" s="29" t="str" cm="1">
         <f t="array" ref="AE17">_xlfn.IFS(AD17&gt;=Z17,"A",AD17&gt;=AA17,"B",AD17&gt;=AB17,"C",AD17&gt;=AC17,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -6668,7 +6645,7 @@
       </c>
       <c r="AG17" s="29" cm="1">
         <f t="array" ref="AG17">_xlfn.IFS(AF17="D",MAX(AC17-AD17,0),AF17="C",MAX(AB17-AD17,0),AF17="B",MAX(AA17-AD17,0),AF17="A",MAX(Z17-AD17,0),AF17="OBJETIVO ALCANÇADO",0)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AI17" t="s">
         <v>14</v>
@@ -6691,7 +6668,7 @@
       </c>
       <c r="AN17" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI17,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>39576.76</v>
+        <v>43855.759999999995</v>
       </c>
       <c r="AO17" s="26" t="str" cm="1">
         <f t="array" ref="AO17">_xlfn.IFS(AN17&gt;=AJ17,"A",AN17&gt;=AK17,"B",AN17&gt;=AL17,"C",AN17&gt;=AM17,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -6703,7 +6680,7 @@
       </c>
       <c r="AQ17" s="25" cm="1">
         <f t="array" ref="AQ17">_xlfn.IFS(AP17="D",MAX(AM17-AN17,0),AP17="C",MAX(AL17-AN17,0),AP17="B",MAX(AK17-AN17,0),AP17="A",MAX(AJ17-AN17,0),AP17="OBJETIVO ALCANÇADO",0)</f>
-        <v>25673.239999999998</v>
+        <v>21394.240000000005</v>
       </c>
     </row>
     <row r="18" spans="1:43" x14ac:dyDescent="0.25">
@@ -6734,15 +6711,15 @@
       </c>
       <c r="I18" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>4600</v>
+        <v>13450</v>
       </c>
       <c r="J18" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>5136.3499999999995</v>
+        <v>5556.9499999999989</v>
       </c>
       <c r="K18" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>-536.34999999999945</v>
+        <v>7893.0500000000011</v>
       </c>
       <c r="L18" s="4"/>
       <c r="M18" s="15"/>
@@ -6762,12 +6739,12 @@
         <v>20</v>
       </c>
       <c r="V18" s="17">
-        <f>VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
-        <v>20</v>
+        <f ca="1">VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
+        <v>23</v>
       </c>
       <c r="W18" s="17">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>-3</v>
       </c>
       <c r="Y18" s="33" t="s">
         <v>21</v>
@@ -6790,19 +6767,19 @@
       </c>
       <c r="AD18" s="31">
         <f>IFERROR(_xlfn.XLOOKUP(Y18,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0),0)</f>
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="AE18" s="31" t="str" cm="1">
         <f t="array" ref="AE18">_xlfn.IFS(AD18&gt;=Z18,"A",AD18&gt;=AA18,"B",AD18&gt;=AB18,"C",AD18&gt;=AC18,"D",TRUE,"NÃO ATINGIDO")</f>
-        <v>B</v>
+        <v>A</v>
       </c>
       <c r="AF18" s="31" t="str" cm="1">
         <f t="array" ref="AF18">_xlfn.IFS(AE18="NÃO ATINGIDO","D",AE18="D","C",AE18="C","B",AE18="B","A",AE18="A","OBJETIVO ALCANÇADO")</f>
-        <v>A</v>
+        <v>OBJETIVO ALCANÇADO</v>
       </c>
       <c r="AG18" s="31" cm="1">
         <f t="array" ref="AG18">_xlfn.IFS(AF18="D",MAX(AC18-AD18,0),AF18="C",MAX(AB18-AD18,0),AF18="B",MAX(AA18-AD18,0),AF18="A",MAX(Z18-AD18,0),AF18="OBJETIVO ALCANÇADO",0)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AI18" t="s">
         <v>21</v>
@@ -6825,7 +6802,7 @@
       </c>
       <c r="AN18" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI18,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>95578.979999999952</v>
+        <v>100639.89999999994</v>
       </c>
       <c r="AO18" s="26" t="str" cm="1">
         <f t="array" ref="AO18">_xlfn.IFS(AN18&gt;=AJ18,"A",AN18&gt;=AK18,"B",AN18&gt;=AL18,"C",AN18&gt;=AM18,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -6837,7 +6814,7 @@
       </c>
       <c r="AQ18" s="25" cm="1">
         <f t="array" ref="AQ18">_xlfn.IFS(AP18="D",MAX(AM18-AN18,0),AP18="C",MAX(AL18-AN18,0),AP18="B",MAX(AK18-AN18,0),AP18="A",MAX(AJ18-AN18,0),AP18="OBJETIVO ALCANÇADO",0)</f>
-        <v>23671.020000000048</v>
+        <v>18610.100000000064</v>
       </c>
     </row>
     <row r="19" spans="1:43" x14ac:dyDescent="0.25">
@@ -6853,11 +6830,11 @@
       </c>
       <c r="D19" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>15180.599999999999</v>
+        <v>19642.8</v>
       </c>
       <c r="E19" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>126819.4</v>
+        <v>122357.2</v>
       </c>
       <c r="F19" s="4"/>
       <c r="G19" s="18" t="s">
@@ -6868,15 +6845,15 @@
       </c>
       <c r="I19" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>6700</v>
+        <v>16550</v>
       </c>
       <c r="J19" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>12558.199999999995</v>
+        <v>14553.599999999995</v>
       </c>
       <c r="K19" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>-5858.1999999999953</v>
+        <v>1996.4000000000051</v>
       </c>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
@@ -6892,12 +6869,12 @@
         <v>20</v>
       </c>
       <c r="V19" s="17">
-        <f>VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
-        <v>19</v>
+        <f ca="1">VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
+        <v>22</v>
       </c>
       <c r="W19" s="17">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>-2</v>
       </c>
       <c r="Y19" s="32" t="s">
         <v>16</v>
@@ -6920,7 +6897,7 @@
       </c>
       <c r="AD19" s="29">
         <f>IFERROR(_xlfn.XLOOKUP(Y19,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0),0)</f>
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="AE19" s="29" t="str" cm="1">
         <f t="array" ref="AE19">_xlfn.IFS(AD19&gt;=Z19,"A",AD19&gt;=AA19,"B",AD19&gt;=AB19,"C",AD19&gt;=AC19,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -6932,7 +6909,7 @@
       </c>
       <c r="AG19" s="29" cm="1">
         <f t="array" ref="AG19">_xlfn.IFS(AF19="D",MAX(AC19-AD19,0),AF19="C",MAX(AB19-AD19,0),AF19="B",MAX(AA19-AD19,0),AF19="A",MAX(Z19-AD19,0),AF19="OBJETIVO ALCANÇADO",0)</f>
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AI19" t="s">
         <v>16</v>
@@ -6955,7 +6932,7 @@
       </c>
       <c r="AN19" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI19,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>25440.569999999996</v>
+        <v>29544.7</v>
       </c>
       <c r="AO19" s="26" t="str" cm="1">
         <f t="array" ref="AO19">_xlfn.IFS(AN19&gt;=AJ19,"A",AN19&gt;=AK19,"B",AN19&gt;=AL19,"C",AN19&gt;=AM19,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -6967,7 +6944,7 @@
       </c>
       <c r="AQ19" s="25" cm="1">
         <f t="array" ref="AQ19">_xlfn.IFS(AP19="D",MAX(AM19-AN19,0),AP19="C",MAX(AL19-AN19,0),AP19="B",MAX(AK19-AN19,0),AP19="A",MAX(AJ19-AN19,0),AP19="OBJETIVO ALCANÇADO",0)</f>
-        <v>10559.430000000004</v>
+        <v>6455.2999999999993</v>
       </c>
     </row>
     <row r="20" spans="1:43" x14ac:dyDescent="0.25">
@@ -6983,11 +6960,11 @@
       </c>
       <c r="D20" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>136688.40000000002</v>
+        <v>145346.00000000003</v>
       </c>
       <c r="E20" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>443311.6</v>
+        <v>434654</v>
       </c>
       <c r="F20" s="4"/>
       <c r="G20" s="18" t="s">
@@ -6998,7 +6975,7 @@
       </c>
       <c r="I20" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>19310</v>
+        <v>27640</v>
       </c>
       <c r="J20" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
@@ -7006,7 +6983,7 @@
       </c>
       <c r="K20" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>1758.1999999999971</v>
+        <v>10088.199999999997</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
@@ -7034,12 +7011,12 @@
         <v>20</v>
       </c>
       <c r="V20" s="17">
-        <f>VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
-        <v>14</v>
+        <f ca="1">VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
+        <v>15</v>
       </c>
       <c r="W20" s="17">
-        <f t="shared" si="0"/>
-        <v>6</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>5</v>
       </c>
       <c r="Y20" s="33" t="s">
         <v>15</v>
@@ -7097,7 +7074,7 @@
       </c>
       <c r="AN20" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI20,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>43899.820000000036</v>
+        <v>45658.210000000028</v>
       </c>
       <c r="AO20" s="26" t="str" cm="1">
         <f t="array" ref="AO20">_xlfn.IFS(AN20&gt;=AJ20,"A",AN20&gt;=AK20,"B",AN20&gt;=AL20,"C",AN20&gt;=AM20,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -7109,7 +7086,7 @@
       </c>
       <c r="AQ20" s="25" cm="1">
         <f t="array" ref="AQ20">_xlfn.IFS(AP20="D",MAX(AM20-AN20,0),AP20="C",MAX(AL20-AN20,0),AP20="B",MAX(AK20-AN20,0),AP20="A",MAX(AJ20-AN20,0),AP20="OBJETIVO ALCANÇADO",0)</f>
-        <v>22250.179999999964</v>
+        <v>20491.789999999972</v>
       </c>
     </row>
     <row r="21" spans="1:43" x14ac:dyDescent="0.25">
@@ -7125,11 +7102,11 @@
       </c>
       <c r="D21" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>67342.790000000008</v>
+        <v>78739.81</v>
       </c>
       <c r="E21" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>412657.20999999996</v>
+        <v>401260.19</v>
       </c>
       <c r="F21" s="4"/>
       <c r="G21" s="18" t="s">
@@ -7140,15 +7117,15 @@
       </c>
       <c r="I21" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>2800</v>
+        <v>4550</v>
       </c>
       <c r="J21" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2974.46</v>
+        <v>2974.4600000000005</v>
       </c>
       <c r="K21" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>-174.46000000000004</v>
+        <v>1575.5399999999995</v>
       </c>
       <c r="L21" s="4"/>
       <c r="M21" s="4"/>
@@ -7179,12 +7156,12 @@
         <v>20</v>
       </c>
       <c r="V21" s="17">
-        <f>VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
-        <v>8</v>
+        <f ca="1">VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
+        <v>9</v>
       </c>
       <c r="W21" s="17">
-        <f t="shared" ref="W21:W26" si="1">U21-V21</f>
-        <v>12</v>
+        <f t="shared" ref="W21:W26" ca="1" si="1">U21-V21</f>
+        <v>11</v>
       </c>
       <c r="Y21" s="36" t="s">
         <v>60</v>
@@ -7207,13 +7184,13 @@
       </c>
       <c r="AD21" s="37">
         <f>SUBTOTAL(109,Planilha1!$AD$3:$AD$20)</f>
-        <v>214</v>
+        <v>245</v>
       </c>
       <c r="AE21" s="37"/>
       <c r="AF21" s="37"/>
       <c r="AG21" s="38">
         <f>SUBTOTAL(109,Planilha1!$AG$3:$AG$20)</f>
-        <v>73</v>
+        <v>61</v>
       </c>
       <c r="AI21" t="s">
         <v>60</v>
@@ -7236,13 +7213,13 @@
       </c>
       <c r="AN21" s="26">
         <f>SUBTOTAL(109,Tabela817[ATINGIDO])</f>
-        <v>970644.80000000028</v>
+        <v>1067756.6649999998</v>
       </c>
       <c r="AO21" s="4"/>
       <c r="AP21" s="4"/>
       <c r="AQ21" s="27">
         <f>SUBTOTAL(109,Tabela817[FALTA])</f>
-        <v>343130.19999999984</v>
+        <v>246018.33500000017</v>
       </c>
     </row>
     <row r="22" spans="1:43" x14ac:dyDescent="0.25">
@@ -7258,11 +7235,11 @@
       </c>
       <c r="D22" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>29186.920000000009</v>
+        <v>31050.670000000006</v>
       </c>
       <c r="E22" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>92813.079999999987</v>
+        <v>90949.329999999987</v>
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="18" t="s">
@@ -7273,7 +7250,7 @@
       </c>
       <c r="I22" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>6430</v>
+        <v>16180</v>
       </c>
       <c r="J22" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
@@ -7281,7 +7258,7 @@
       </c>
       <c r="K22" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>2416.5399999999991</v>
+        <v>12166.539999999999</v>
       </c>
       <c r="L22" s="4"/>
       <c r="M22" s="4"/>
@@ -7294,11 +7271,11 @@
       </c>
       <c r="P22" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>619826.16000000061</v>
+        <v>720213.08000000042</v>
       </c>
       <c r="Q22" s="7">
         <f>O22-P22</f>
-        <v>-51826.160000000615</v>
+        <v>-152213.08000000042</v>
       </c>
       <c r="R22" s="4"/>
       <c r="S22" s="17" t="s">
@@ -7312,12 +7289,12 @@
         <v>20</v>
       </c>
       <c r="V22" s="17">
-        <f>VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
-        <v>12</v>
+        <f ca="1">VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
+        <v>13</v>
       </c>
       <c r="W22" s="17">
-        <f t="shared" si="1"/>
-        <v>8</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>7</v>
       </c>
     </row>
     <row r="23" spans="1:43" x14ac:dyDescent="0.25">
@@ -7333,11 +7310,11 @@
       </c>
       <c r="D23" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>79750.23500000003</v>
+        <v>84326.634999999995</v>
       </c>
       <c r="E23" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>123249.76499999997</v>
+        <v>118673.36500000001</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="18" t="s">
@@ -7348,7 +7325,7 @@
       </c>
       <c r="I23" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>3370</v>
+        <v>13170</v>
       </c>
       <c r="J23" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
@@ -7356,7 +7333,7 @@
       </c>
       <c r="K23" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>1676.2100000000003</v>
+        <v>11476.210000000001</v>
       </c>
       <c r="L23" s="4"/>
       <c r="M23" s="4"/>
@@ -7369,11 +7346,11 @@
       </c>
       <c r="P23" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>0</v>
+        <v>6348.4</v>
       </c>
       <c r="Q23" s="7">
         <f>O23-P23</f>
-        <v>710000</v>
+        <v>703651.6</v>
       </c>
       <c r="R23" s="4"/>
       <c r="S23" s="17" t="s">
@@ -7387,12 +7364,12 @@
         <v>20</v>
       </c>
       <c r="V23" s="17">
-        <f>VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
-        <v>18</v>
+        <f ca="1">VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
+        <v>20</v>
       </c>
       <c r="W23" s="17">
-        <f t="shared" si="1"/>
-        <v>2</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:43" x14ac:dyDescent="0.25">
@@ -7408,11 +7385,11 @@
       </c>
       <c r="D24" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>39576.76</v>
+        <v>43855.759999999995</v>
       </c>
       <c r="E24" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>105423.23999999999</v>
+        <v>101144.24</v>
       </c>
       <c r="F24" s="4"/>
       <c r="G24" s="18" t="s">
@@ -7423,15 +7400,15 @@
       </c>
       <c r="I24" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>4430</v>
+        <v>10460</v>
       </c>
       <c r="J24" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>675</v>
+        <v>3039</v>
       </c>
       <c r="K24" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3755</v>
+        <v>7421</v>
       </c>
       <c r="L24" s="4"/>
       <c r="M24" s="4"/>
@@ -7462,12 +7439,12 @@
         <v>20</v>
       </c>
       <c r="V24" s="17">
-        <f>VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
-        <v>8</v>
+        <f ca="1">VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
+        <v>9</v>
       </c>
       <c r="W24" s="17">
-        <f t="shared" si="1"/>
-        <v>12</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>11</v>
       </c>
     </row>
     <row r="25" spans="1:43" x14ac:dyDescent="0.25">
@@ -7483,11 +7460,11 @@
       </c>
       <c r="D25" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>43899.820000000036</v>
+        <v>45658.210000000028</v>
       </c>
       <c r="E25" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>103100.17999999996</v>
+        <v>101341.78999999998</v>
       </c>
       <c r="F25" s="4"/>
       <c r="G25" s="18" t="s">
@@ -7498,7 +7475,7 @@
       </c>
       <c r="I25" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>3250</v>
+        <v>13350</v>
       </c>
       <c r="J25" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
@@ -7506,7 +7483,7 @@
       </c>
       <c r="K25" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>1731.4199999999998</v>
+        <v>11831.42</v>
       </c>
       <c r="L25" s="4"/>
       <c r="M25" s="4"/>
@@ -7537,11 +7514,11 @@
         <v>20</v>
       </c>
       <c r="V25" s="17">
-        <f>VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
+        <f ca="1">VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
         <v>6</v>
       </c>
       <c r="W25" s="17">
-        <f t="shared" si="1"/>
+        <f t="shared" ca="1" si="1"/>
         <v>14</v>
       </c>
     </row>
@@ -7558,11 +7535,11 @@
       </c>
       <c r="D26" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>25440.569999999996</v>
+        <v>29544.7</v>
       </c>
       <c r="E26" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>54559.430000000008</v>
+        <v>50455.3</v>
       </c>
       <c r="F26" s="4"/>
       <c r="G26" s="18" t="s">
@@ -7573,15 +7550,15 @@
       </c>
       <c r="I26" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>3820</v>
+        <v>6100</v>
       </c>
       <c r="J26" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>844.31999999999994</v>
+        <v>1399.22</v>
       </c>
       <c r="K26" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>2975.6800000000003</v>
+        <v>4700.78</v>
       </c>
       <c r="L26" s="4"/>
       <c r="M26" s="4"/>
@@ -7601,11 +7578,11 @@
         <v>20</v>
       </c>
       <c r="V26" s="17">
-        <f>VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
+        <f ca="1">VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
         <v>11</v>
       </c>
       <c r="W26" s="17">
-        <f t="shared" si="1"/>
+        <f t="shared" ca="1" si="1"/>
         <v>9</v>
       </c>
     </row>
@@ -7622,11 +7599,11 @@
       </c>
       <c r="D27" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>85823.090000000084</v>
+        <v>96164.2</v>
       </c>
       <c r="E27" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>159176.90999999992</v>
+        <v>148835.79999999999</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="18" t="s">
@@ -7637,15 +7614,15 @@
       </c>
       <c r="I27" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>5390</v>
+        <v>5240</v>
       </c>
       <c r="J27" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>3627.7000000000003</v>
+        <v>3806.4000000000005</v>
       </c>
       <c r="K27" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>1762.2999999999997</v>
+        <v>1433.5999999999995</v>
       </c>
       <c r="L27" s="4"/>
       <c r="M27" s="4"/>
@@ -7668,11 +7645,11 @@
       </c>
       <c r="D28" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>114328.69500000012</v>
+        <v>125560.12500000007</v>
       </c>
       <c r="E28" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>212171.30499999988</v>
+        <v>200939.87499999994</v>
       </c>
       <c r="F28" s="4"/>
       <c r="L28" s="4"/>
@@ -7747,11 +7724,11 @@
       </c>
       <c r="D30" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>36811.270000000026</v>
+        <v>40663.720000000038</v>
       </c>
       <c r="E30" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>105188.72999999998</v>
+        <v>101336.27999999997</v>
       </c>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
@@ -7784,11 +7761,11 @@
       </c>
       <c r="V30" s="5">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE 2]",'[1]BASE PYTHON'!$P$83,"[Intervalo 3].[SEMANAL]","[Intervalo 3].[SEMANAL].&amp;[1]"),0)</f>
-        <v>153</v>
+        <v>160</v>
       </c>
       <c r="W30" s="6">
         <f>U30-V30</f>
-        <v>-88.238095238095241</v>
+        <v>-95.238095238095241</v>
       </c>
     </row>
     <row r="31" spans="1:43" x14ac:dyDescent="0.25">
@@ -7804,11 +7781,11 @@
       </c>
       <c r="D31" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>66351.140000000014</v>
+        <v>68771.89</v>
       </c>
       <c r="E31" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>103648.85999999999</v>
+        <v>101228.11</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
@@ -7821,11 +7798,11 @@
       </c>
       <c r="J31" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[1]"),0)</f>
-        <v>415668.52000000159</v>
+        <v>415588.02000000159</v>
       </c>
       <c r="K31" s="7">
         <f>I31-J31</f>
-        <v>140426.71809523652</v>
+        <v>140507.21809523652</v>
       </c>
       <c r="L31" s="4"/>
       <c r="M31" s="4"/>
@@ -7844,11 +7821,11 @@
       </c>
       <c r="V31" s="5">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE 2]",'[1]BASE PYTHON'!$P$83,"[Intervalo 3].[SEMANAL]","[Intervalo 3].[SEMANAL].&amp;[2]"),0)</f>
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="W31" s="6">
         <f t="shared" ref="W31:W33" si="2">U31-V31</f>
-        <v>6.7619047619047592</v>
+        <v>-11.238095238095241</v>
       </c>
     </row>
     <row r="32" spans="1:43" x14ac:dyDescent="0.25">
@@ -7864,11 +7841,11 @@
       </c>
       <c r="D32" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>95578.979999999952</v>
+        <v>100639.89999999994</v>
       </c>
       <c r="E32" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>169421.02000000005</v>
+        <v>164360.10000000006</v>
       </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
@@ -7881,11 +7858,11 @@
       </c>
       <c r="J32" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>475226.04500000185</v>
+        <v>546956.19000000309</v>
       </c>
       <c r="K32" s="7">
         <f t="shared" ref="K32:K34" si="3">I32-J32</f>
-        <v>80869.19309523626</v>
+        <v>9139.048095235019</v>
       </c>
       <c r="L32" s="4"/>
       <c r="M32" s="4"/>
@@ -7924,11 +7901,11 @@
       </c>
       <c r="D33" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>25035.579999999998</v>
+        <v>27935.73000000001</v>
       </c>
       <c r="E33" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>59964.42</v>
+        <v>57064.26999999999</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -7941,11 +7918,11 @@
       </c>
       <c r="J33" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>0</v>
+        <v>20885.819999999996</v>
       </c>
       <c r="K33" s="7">
         <f t="shared" si="3"/>
-        <v>695119.04761904757</v>
+        <v>674233.22761904763</v>
       </c>
       <c r="L33" s="4"/>
       <c r="M33" s="4"/>
@@ -7984,11 +7961,11 @@
       </c>
       <c r="D34" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>18754.78</v>
+        <v>21675.470000000005</v>
       </c>
       <c r="E34" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>36245.22</v>
+        <v>33324.53</v>
       </c>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
@@ -8044,11 +8021,11 @@
       </c>
       <c r="D35" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>19519.940000000002</v>
+        <v>28037.200000000004</v>
       </c>
       <c r="E35" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>56980.06</v>
+        <v>48462.799999999996</v>
       </c>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
@@ -8093,11 +8070,11 @@
       </c>
       <c r="D36" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>0</v>
+        <v>144.9</v>
       </c>
       <c r="E36" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>1000</v>
+        <v>855.1</v>
       </c>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
@@ -8204,11 +8181,11 @@
       </c>
       <c r="D40" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[1]"),0)</f>
-        <v>617118.84000000393</v>
+        <v>617038.34000000393</v>
       </c>
       <c r="E40" s="7">
         <f>C40-D40</f>
-        <v>507166.87428571039</v>
+        <v>507247.37428571039</v>
       </c>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
@@ -8240,11 +8217,11 @@
       </c>
       <c r="D41" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>1142262.0700000015</v>
+        <v>1319100.4349999954</v>
       </c>
       <c r="E41" s="7">
         <f t="shared" ref="E41:E43" si="4">C41-D41</f>
-        <v>-17976.355714287143</v>
+        <v>-194814.72071428108</v>
       </c>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
@@ -8276,11 +8253,11 @@
       </c>
       <c r="D42" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>0</v>
+        <v>27234.22</v>
       </c>
       <c r="E42" s="7">
         <f t="shared" si="4"/>
-        <v>1405357.142857143</v>
+        <v>1378122.922857143</v>
       </c>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>

</xml_diff>

<commit_message>
Dados atualizados em 29/09/2026 07:34
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B8B9601-2B09-477B-8901-55D657538979}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE2CCDBF-01D2-4965-9F58-BCC42C66C6E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -45,9 +45,9 @@
   <metadataStrings count="5">
     <s v="ThisWorkbookDataModel"/>
     <s v="{[Intervalo 2].[DATA].[All]}"/>
-    <s v="{[Intervalo 2].[DATA].&amp;[2026-09-10T00:00:00]}"/>
     <s v="{[Intervalo 2].[DES_TIPO_OPERACAO].&amp;[VENDA],[Intervalo 2].[DES_TIPO_OPERACAO].&amp;[VENDA SAT]}"/>
-    <s v="{[Intervalo 2].[PRODUTO].&amp;[MIST PAO DA FAZENDA 20KG CAIXA],[Intervalo 2].[PRODUTO].&amp;[MIST PAO DA FAZENDA VIAPANE 10KG],[Intervalo 2].[PRODUTO].&amp;[MIST PAO DA FAZENDA COM ETIQUETA VIAPANE 10KG],[Intervalo 2].[PRODUTO].&amp;[MIST PAO DA FAZENDA ETIQUETA VIAPANE 20KG CAIXA]}"/>
+    <s v="{[Intervalo 2].[PRODUTO].&amp;[MIST PAO DA FAZENDA 20KG CAIXA],[Intervalo 2].[PRODUTO].&amp;[MIST PAO DA FAZENDA VIAPANE 10KG]}"/>
+    <s v="{[Intervalo 2].[DATA].&amp;[2026-09-28T00:00:00]}"/>
   </metadataStrings>
   <mdxMetadata count="4">
     <mdx n="0" f="s">
@@ -2494,11 +2494,11 @@
       <sheetName val="BASE PYTHON"/>
     </sheetNames>
     <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
+      <sheetData sheetId="0" refreshError="1"/>
+      <sheetData sheetId="1" refreshError="1"/>
+      <sheetData sheetId="2" refreshError="1"/>
+      <sheetData sheetId="3" refreshError="1"/>
+      <sheetData sheetId="4" refreshError="1"/>
       <sheetData sheetId="5">
         <row r="1">
           <cell r="E1" t="str">
@@ -2511,10 +2511,10 @@
             <v>POSITIVACAO PAO DA FAZENDA</v>
           </cell>
           <cell r="L1">
-            <v>4</v>
+            <v>3</v>
           </cell>
           <cell r="M1">
-            <v>570</v>
+            <v>0</v>
           </cell>
         </row>
         <row r="2">
@@ -2527,8 +2527,8 @@
           <cell r="H2" t="str">
             <v>DATA</v>
           </cell>
-          <cell r="I2" t="str" vm="2">
-            <v>10/09/2026</v>
+          <cell r="I2" t="str" vm="4">
+            <v>28/09/2026</v>
           </cell>
           <cell r="K2" t="str">
             <v>DATA</v>
@@ -2541,7 +2541,7 @@
           <cell r="K3" t="str">
             <v>DES_TIPO_OPERACAO</v>
           </cell>
-          <cell r="L3" t="str" vm="3">
+          <cell r="L3" t="str" vm="2">
             <v>(Vários itens)</v>
           </cell>
         </row>
@@ -2561,7 +2561,7 @@
           <cell r="K4" t="str">
             <v>PRODUTO</v>
           </cell>
-          <cell r="L4" t="str" vm="4">
+          <cell r="L4" t="str" vm="3">
             <v>(Vários itens)</v>
           </cell>
           <cell r="P4" t="str">
@@ -2573,13 +2573,13 @@
             <v>CAMPINAS</v>
           </cell>
           <cell r="F5">
-            <v>23194.480000000007</v>
+            <v>62470.590000000004</v>
           </cell>
           <cell r="H5" t="str">
             <v>CAMPINAS</v>
           </cell>
           <cell r="I5">
-            <v>3806.4000000000005</v>
+            <v>4561.2000000000007</v>
           </cell>
         </row>
         <row r="6">
@@ -2587,13 +2587,13 @@
             <v>CENTRO</v>
           </cell>
           <cell r="F6">
-            <v>139883.35999999984</v>
+            <v>320791.82000000047</v>
           </cell>
           <cell r="H6" t="str">
             <v>CENTRO</v>
           </cell>
           <cell r="I6">
-            <v>13827.15</v>
+            <v>26804.570000000011</v>
           </cell>
           <cell r="K6" t="str">
             <v>Contagem Distinta de COD_CLIENTE</v>
@@ -2607,13 +2607,13 @@
             <v>ECOMMERCE</v>
           </cell>
           <cell r="F7">
-            <v>144.9</v>
+            <v>1003.86</v>
           </cell>
           <cell r="H7" t="str">
-            <v>ECOMMERCE</v>
+            <v>INDAIATUBA</v>
           </cell>
           <cell r="I7">
-            <v>144.9</v>
+            <v>10844.970000000001</v>
           </cell>
           <cell r="K7" t="str">
             <v>Rótulos de Linha</v>
@@ -2622,9 +2622,6 @@
             <v>ACUMULADO</v>
           </cell>
           <cell r="M7" t="str">
-            <v>DIA</v>
-          </cell>
-          <cell r="N7" t="str">
             <v>Total Geral</v>
           </cell>
         </row>
@@ -2633,22 +2630,22 @@
             <v>IATAGAM JUNIOR</v>
           </cell>
           <cell r="F8">
-            <v>55.04</v>
+            <v>102</v>
           </cell>
           <cell r="H8" t="str">
-            <v>INDAIATUBA</v>
+            <v>INTERLAGOS</v>
           </cell>
           <cell r="I8">
-            <v>1693.7899999999997</v>
+            <v>17482.909999999996</v>
           </cell>
           <cell r="K8" t="str">
             <v>CAMPINAS</v>
           </cell>
           <cell r="L8">
-            <v>12</v>
-          </cell>
-          <cell r="N8">
-            <v>12</v>
+            <v>20</v>
+          </cell>
+          <cell r="M8">
+            <v>20</v>
           </cell>
         </row>
         <row r="9">
@@ -2656,22 +2653,22 @@
             <v>INDAIATUBA</v>
           </cell>
           <cell r="F9">
-            <v>31196.295000000016</v>
+            <v>86297.000000000015</v>
           </cell>
           <cell r="H9" t="str">
-            <v>INTERLAGOS</v>
+            <v>JUNDIAI</v>
           </cell>
           <cell r="I9">
-            <v>17551.800000000003</v>
+            <v>8545.5799999999981</v>
           </cell>
           <cell r="K9" t="str">
             <v>CENTRO</v>
           </cell>
           <cell r="L9">
-            <v>13</v>
-          </cell>
-          <cell r="N9">
-            <v>13</v>
+            <v>22</v>
+          </cell>
+          <cell r="M9">
+            <v>22</v>
           </cell>
         </row>
         <row r="10">
@@ -2679,22 +2676,22 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="F10">
-            <v>100281.57999999986</v>
+            <v>251396.75999999963</v>
           </cell>
           <cell r="H10" t="str">
-            <v>JUNDIAI</v>
+            <v>KEY ABC</v>
           </cell>
           <cell r="I10">
-            <v>2974.4600000000005</v>
+            <v>3361</v>
           </cell>
           <cell r="K10" t="str">
             <v>INDAIATUBA</v>
           </cell>
           <cell r="L10">
-            <v>10</v>
-          </cell>
-          <cell r="N10">
-            <v>10</v>
+            <v>19</v>
+          </cell>
+          <cell r="M10">
+            <v>19</v>
           </cell>
         </row>
         <row r="11">
@@ -2702,25 +2699,22 @@
             <v>JUNDIAI</v>
           </cell>
           <cell r="F11">
-            <v>29316.740000000023</v>
+            <v>77850.589999999909</v>
           </cell>
           <cell r="H11" t="str">
-            <v>KEY ABC</v>
+            <v>KEY CASA</v>
           </cell>
           <cell r="I11">
-            <v>18677.400000000001</v>
+            <v>33644.200000000004</v>
           </cell>
           <cell r="K11" t="str">
             <v>INTERLAGOS</v>
           </cell>
           <cell r="L11">
-            <v>28</v>
+            <v>54</v>
           </cell>
           <cell r="M11">
-            <v>1</v>
-          </cell>
-          <cell r="N11">
-            <v>29</v>
+            <v>54</v>
           </cell>
         </row>
         <row r="12">
@@ -2728,22 +2722,22 @@
             <v>KEY ABC</v>
           </cell>
           <cell r="F12">
-            <v>98323.800000000017</v>
+            <v>261108.89999999991</v>
           </cell>
           <cell r="H12" t="str">
-            <v>KEY CASA</v>
+            <v>KEY INTERIOR</v>
           </cell>
           <cell r="I12">
-            <v>54275.380000000005</v>
+            <v>2300.4</v>
           </cell>
           <cell r="K12" t="str">
             <v>JUNDIAI</v>
           </cell>
           <cell r="L12">
-            <v>11</v>
-          </cell>
-          <cell r="N12">
-            <v>11</v>
+            <v>26</v>
+          </cell>
+          <cell r="M12">
+            <v>26</v>
           </cell>
         </row>
         <row r="13">
@@ -2751,22 +2745,22 @@
             <v>KEY CASA</v>
           </cell>
           <cell r="F13">
-            <v>205409.18000000031</v>
+            <v>645986.02999999968</v>
           </cell>
           <cell r="H13" t="str">
-            <v>KEY INTERIOR</v>
+            <v>KEY SJC</v>
           </cell>
           <cell r="I13">
-            <v>69258.200000000012</v>
+            <v>483.95</v>
           </cell>
           <cell r="K13" t="str">
             <v>LESTE</v>
           </cell>
           <cell r="L13">
-            <v>8</v>
-          </cell>
-          <cell r="N13">
-            <v>8</v>
+            <v>21</v>
+          </cell>
+          <cell r="M13">
+            <v>21</v>
           </cell>
         </row>
         <row r="14">
@@ -2774,22 +2768,22 @@
             <v>KEY INTERIOR</v>
           </cell>
           <cell r="F14">
-            <v>347954.79999999987</v>
+            <v>816833.8</v>
           </cell>
           <cell r="H14" t="str">
-            <v>KEY SJC</v>
+            <v>KEY SP</v>
           </cell>
           <cell r="I14">
-            <v>7440.4</v>
+            <v>17609.66</v>
           </cell>
           <cell r="K14" t="str">
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="L14">
-            <v>18</v>
-          </cell>
-          <cell r="N14">
-            <v>18</v>
+            <v>25</v>
+          </cell>
+          <cell r="M14">
+            <v>25</v>
           </cell>
         </row>
         <row r="15">
@@ -2797,22 +2791,22 @@
             <v>KEY SJC</v>
           </cell>
           <cell r="F15">
-            <v>19642.8</v>
+            <v>55652.650000000009</v>
           </cell>
           <cell r="H15" t="str">
-            <v>KEY SP</v>
+            <v>KEY ZL</v>
           </cell>
           <cell r="I15">
-            <v>11327.7</v>
+            <v>30069.5</v>
           </cell>
           <cell r="K15" t="str">
             <v>LESTE PENHA</v>
           </cell>
           <cell r="L15">
-            <v>15</v>
-          </cell>
-          <cell r="N15">
-            <v>15</v>
+            <v>20</v>
+          </cell>
+          <cell r="M15">
+            <v>20</v>
           </cell>
         </row>
         <row r="16">
@@ -2820,22 +2814,22 @@
             <v>KEY SP</v>
           </cell>
           <cell r="F16">
-            <v>145346.00000000003</v>
+            <v>316150.64000000007</v>
           </cell>
           <cell r="H16" t="str">
-            <v>KEY ZL</v>
+            <v>LESTE</v>
           </cell>
           <cell r="I16">
-            <v>264.39999999999998</v>
+            <v>11939.229999999998</v>
           </cell>
           <cell r="K16" t="str">
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="L16">
-            <v>6</v>
-          </cell>
-          <cell r="N16">
-            <v>6</v>
+            <v>20</v>
+          </cell>
+          <cell r="M16">
+            <v>20</v>
           </cell>
         </row>
         <row r="17">
@@ -2843,22 +2837,22 @@
             <v>KEY ZL</v>
           </cell>
           <cell r="F17">
-            <v>78739.81</v>
+            <v>293729.78999999986</v>
           </cell>
           <cell r="H17" t="str">
-            <v>LESTE</v>
+            <v>LESTE MOOCA</v>
           </cell>
           <cell r="I17">
-            <v>5556.9499999999989</v>
+            <v>11443.519999999995</v>
           </cell>
           <cell r="K17" t="str">
             <v>MOGI</v>
           </cell>
           <cell r="L17">
-            <v>7</v>
-          </cell>
-          <cell r="N17">
-            <v>7</v>
+            <v>21</v>
+          </cell>
+          <cell r="M17">
+            <v>21</v>
           </cell>
         </row>
         <row r="18">
@@ -2866,22 +2860,22 @@
             <v>LESTE</v>
           </cell>
           <cell r="F18">
-            <v>31050.670000000006</v>
+            <v>93024.129999999917</v>
           </cell>
           <cell r="H18" t="str">
-            <v>LESTE MOOCA</v>
+            <v>LESTE PENHA</v>
           </cell>
           <cell r="I18">
-            <v>14553.599999999995</v>
+            <v>15529.049999999997</v>
           </cell>
           <cell r="K18" t="str">
             <v>NORTE</v>
           </cell>
           <cell r="L18">
-            <v>23</v>
-          </cell>
-          <cell r="N18">
-            <v>23</v>
+            <v>44</v>
+          </cell>
+          <cell r="M18">
+            <v>44</v>
           </cell>
         </row>
         <row r="19">
@@ -2889,22 +2883,22 @@
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="F19">
-            <v>84326.634999999995</v>
+            <v>190895.0149999992</v>
           </cell>
           <cell r="H19" t="str">
-            <v>LESTE PENHA</v>
+            <v>LESTE TATUAPE</v>
           </cell>
           <cell r="I19">
-            <v>4013.4600000000009</v>
+            <v>13741.719999999994</v>
           </cell>
           <cell r="K19" t="str">
             <v>OSASCO</v>
           </cell>
           <cell r="L19">
-            <v>22</v>
-          </cell>
-          <cell r="N19">
-            <v>22</v>
+            <v>35</v>
+          </cell>
+          <cell r="M19">
+            <v>35</v>
           </cell>
         </row>
         <row r="20">
@@ -2912,22 +2906,22 @@
             <v>LESTE PENHA</v>
           </cell>
           <cell r="F20">
-            <v>43855.759999999995</v>
+            <v>126001.7799999999</v>
           </cell>
           <cell r="H20" t="str">
-            <v>LESTE TATUAPE</v>
+            <v>MOGI</v>
           </cell>
           <cell r="I20">
-            <v>1218.4000000000001</v>
+            <v>5865.7599999999993</v>
           </cell>
           <cell r="K20" t="str">
             <v>PIRITUBA</v>
           </cell>
           <cell r="L20">
-            <v>9</v>
-          </cell>
-          <cell r="N20">
-            <v>9</v>
+            <v>20</v>
+          </cell>
+          <cell r="M20">
+            <v>20</v>
           </cell>
         </row>
         <row r="21">
@@ -2935,22 +2929,22 @@
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="F21">
-            <v>45658.210000000028</v>
+            <v>140208.75999999949</v>
           </cell>
           <cell r="H21" t="str">
-            <v>MOGI</v>
+            <v>NORTE</v>
           </cell>
           <cell r="I21">
-            <v>4735.8200000000006</v>
+            <v>23232.1</v>
           </cell>
           <cell r="K21" t="str">
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="L21">
-            <v>13</v>
-          </cell>
-          <cell r="N21">
-            <v>13</v>
+            <v>32</v>
+          </cell>
+          <cell r="M21">
+            <v>32</v>
           </cell>
         </row>
         <row r="22">
@@ -2958,22 +2952,22 @@
             <v>MOGI</v>
           </cell>
           <cell r="F22">
-            <v>29544.7</v>
+            <v>67490.080000000045</v>
           </cell>
           <cell r="H22" t="str">
-            <v>NORTE</v>
+            <v>OSASCO</v>
           </cell>
           <cell r="I22">
-            <v>10940.499999999998</v>
+            <v>19803.94999999999</v>
           </cell>
           <cell r="K22" t="str">
             <v>SBC</v>
           </cell>
           <cell r="L22">
-            <v>20</v>
-          </cell>
-          <cell r="N22">
-            <v>20</v>
+            <v>28</v>
+          </cell>
+          <cell r="M22">
+            <v>28</v>
           </cell>
         </row>
         <row r="23">
@@ -2981,25 +2975,22 @@
             <v>NORTE</v>
           </cell>
           <cell r="F23">
-            <v>96164.2</v>
+            <v>233973.21999999901</v>
           </cell>
           <cell r="H23" t="str">
-            <v>OSASCO</v>
+            <v>PIRITUBA</v>
           </cell>
           <cell r="I23">
-            <v>14911.204999999994</v>
+            <v>9069.65</v>
           </cell>
           <cell r="K23" t="str">
             <v>SJC</v>
           </cell>
           <cell r="L23">
-            <v>8</v>
+            <v>20</v>
           </cell>
           <cell r="M23">
-            <v>1</v>
-          </cell>
-          <cell r="N23">
-            <v>9</v>
+            <v>20</v>
           </cell>
         </row>
         <row r="24">
@@ -3007,22 +2998,22 @@
             <v>OSASCO</v>
           </cell>
           <cell r="F24">
-            <v>125560.12500000007</v>
+            <v>304475.37500000017</v>
           </cell>
           <cell r="H24" t="str">
-            <v>PIRITUBA</v>
+            <v>SANTO ANDRE</v>
           </cell>
           <cell r="I24">
-            <v>3254.9500000000003</v>
+            <v>16650.419999999998</v>
           </cell>
           <cell r="K24" t="str">
             <v>SJC/VALE</v>
           </cell>
           <cell r="L24">
-            <v>11</v>
-          </cell>
-          <cell r="N24">
-            <v>11</v>
+            <v>28</v>
+          </cell>
+          <cell r="M24">
+            <v>28</v>
           </cell>
         </row>
         <row r="25">
@@ -3030,25 +3021,22 @@
             <v>PIRITUBA</v>
           </cell>
           <cell r="F25">
-            <v>40663.720000000038</v>
+            <v>112939.21999999965</v>
           </cell>
           <cell r="H25" t="str">
-            <v>SANTO ANDRE</v>
+            <v>SBC</v>
           </cell>
           <cell r="I25">
-            <v>6734.5400000000009</v>
+            <v>18462.34</v>
           </cell>
           <cell r="K25" t="str">
             <v>Total Geral</v>
           </cell>
           <cell r="L25">
-            <v>234</v>
+            <v>455</v>
           </cell>
           <cell r="M25">
-            <v>2</v>
-          </cell>
-          <cell r="N25">
-            <v>236</v>
+            <v>455</v>
           </cell>
         </row>
         <row r="26">
@@ -3056,13 +3044,13 @@
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="F26">
-            <v>68771.89</v>
+            <v>173369.35999999978</v>
           </cell>
           <cell r="H26" t="str">
-            <v>SBC</v>
+            <v>SJC</v>
           </cell>
           <cell r="I26">
-            <v>11125.239999999993</v>
+            <v>8027.9999999999991</v>
           </cell>
         </row>
         <row r="27">
@@ -3070,13 +3058,13 @@
             <v>SBC</v>
           </cell>
           <cell r="F27">
-            <v>100639.89999999994</v>
+            <v>244477.96999999936</v>
           </cell>
           <cell r="H27" t="str">
-            <v>SJC</v>
+            <v>SJC/VALE</v>
           </cell>
           <cell r="I27">
-            <v>1518.5800000000002</v>
+            <v>7277.4499999999989</v>
           </cell>
         </row>
         <row r="28">
@@ -3084,13 +3072,13 @@
             <v>SJC</v>
           </cell>
           <cell r="F28">
-            <v>27935.73000000001</v>
+            <v>75978.280000000057</v>
           </cell>
           <cell r="H28" t="str">
-            <v>SJC/VALE</v>
+            <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="I28">
-            <v>1399.22</v>
+            <v>6480.75</v>
           </cell>
           <cell r="K28" t="str">
             <v>POSITIVAÇÃO GERAL</v>
@@ -3101,13 +3089,13 @@
             <v>SJC/VALE</v>
           </cell>
           <cell r="F29">
-            <v>21675.470000000005</v>
+            <v>56813.940000000111</v>
           </cell>
           <cell r="H29" t="str">
-            <v>VENDEDOR INTERNO 1</v>
+            <v>Total Geral</v>
           </cell>
           <cell r="I29">
-            <v>3039</v>
+            <v>323231.87999999977</v>
           </cell>
           <cell r="K29" t="str">
             <v>DATA</v>
@@ -3121,18 +3109,12 @@
             <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="F30">
-            <v>28037.200000000004</v>
-          </cell>
-          <cell r="H30" t="str">
-            <v>Total Geral</v>
-          </cell>
-          <cell r="I30">
-            <v>284243.44499999977</v>
+            <v>65317.66</v>
           </cell>
           <cell r="K30" t="str">
             <v>DES_TIPO_OPERACAO</v>
           </cell>
-          <cell r="L30" t="str" vm="3">
+          <cell r="L30" t="str" vm="2">
             <v>(Vários itens)</v>
           </cell>
         </row>
@@ -3141,7 +3123,7 @@
             <v>Total Geral</v>
           </cell>
           <cell r="F31">
-            <v>1963372.9950000106</v>
+            <v>5074339.2199998768</v>
           </cell>
         </row>
         <row r="32">
@@ -3163,9 +3145,6 @@
             <v>ACUMULADO</v>
           </cell>
           <cell r="M33" t="str">
-            <v>DIA</v>
-          </cell>
-          <cell r="N33" t="str">
             <v>Total Geral</v>
           </cell>
         </row>
@@ -3174,13 +3153,10 @@
             <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="L34">
-            <v>47</v>
+            <v>65</v>
           </cell>
           <cell r="M34">
-            <v>9</v>
-          </cell>
-          <cell r="N34">
-            <v>49</v>
+            <v>65</v>
           </cell>
         </row>
         <row r="35">
@@ -3188,13 +3164,10 @@
             <v>Total Geral</v>
           </cell>
           <cell r="L35">
-            <v>47</v>
+            <v>65</v>
           </cell>
           <cell r="M35">
-            <v>9</v>
-          </cell>
-          <cell r="N35">
-            <v>49</v>
+            <v>65</v>
           </cell>
         </row>
         <row r="47">
@@ -3402,13 +3375,13 @@
             <v>9</v>
           </cell>
           <cell r="F136">
-            <v>9</v>
+            <v>20</v>
           </cell>
           <cell r="H136" t="str">
-            <v>C</v>
+            <v>OBJETIVO ALCANÇADO</v>
           </cell>
           <cell r="I136">
-            <v>5</v>
+            <v>0</v>
           </cell>
         </row>
         <row r="137">
@@ -3416,13 +3389,13 @@
             <v>36</v>
           </cell>
           <cell r="F137">
-            <v>49</v>
+            <v>65</v>
           </cell>
           <cell r="H137" t="str">
-            <v>C</v>
+            <v>B</v>
           </cell>
           <cell r="I137">
-            <v>7</v>
+            <v>3</v>
           </cell>
         </row>
         <row r="138">
@@ -3430,13 +3403,13 @@
             <v>9</v>
           </cell>
           <cell r="F138">
-            <v>13</v>
+            <v>22</v>
           </cell>
           <cell r="H138" t="str">
-            <v>C</v>
+            <v>OBJETIVO ALCANÇADO</v>
           </cell>
           <cell r="I138">
-            <v>1</v>
+            <v>0</v>
           </cell>
         </row>
         <row r="139">
@@ -3444,7 +3417,7 @@
             <v>9</v>
           </cell>
           <cell r="F139">
-            <v>22</v>
+            <v>35</v>
           </cell>
           <cell r="H139" t="str">
             <v>OBJETIVO ALCANÇADO</v>
@@ -3458,7 +3431,7 @@
             <v>9</v>
           </cell>
           <cell r="F140">
-            <v>29</v>
+            <v>54</v>
           </cell>
           <cell r="H140" t="str">
             <v>OBJETIVO ALCANÇADO</v>
@@ -3472,13 +3445,13 @@
             <v>9</v>
           </cell>
           <cell r="F141">
-            <v>18</v>
+            <v>25</v>
           </cell>
           <cell r="H141" t="str">
-            <v>A</v>
+            <v>OBJETIVO ALCANÇADO</v>
           </cell>
           <cell r="I141">
-            <v>2</v>
+            <v>0</v>
           </cell>
         </row>
         <row r="142">
@@ -3486,13 +3459,13 @@
             <v>9</v>
           </cell>
           <cell r="F142">
-            <v>13</v>
+            <v>32</v>
           </cell>
           <cell r="H142" t="str">
-            <v>C</v>
+            <v>OBJETIVO ALCANÇADO</v>
           </cell>
           <cell r="I142">
-            <v>1</v>
+            <v>0</v>
           </cell>
         </row>
         <row r="143">
@@ -3500,7 +3473,7 @@
             <v>9</v>
           </cell>
           <cell r="F143">
-            <v>23</v>
+            <v>44</v>
           </cell>
           <cell r="H143" t="str">
             <v>OBJETIVO ALCANÇADO</v>
@@ -3514,13 +3487,13 @@
             <v>9</v>
           </cell>
           <cell r="F144">
-            <v>8</v>
+            <v>21</v>
           </cell>
           <cell r="H144" t="str">
-            <v>D</v>
+            <v>OBJETIVO ALCANÇADO</v>
           </cell>
           <cell r="I144">
-            <v>1</v>
+            <v>0</v>
           </cell>
         </row>
         <row r="145">
@@ -3528,13 +3501,13 @@
             <v>9</v>
           </cell>
           <cell r="F145">
-            <v>11</v>
+            <v>28</v>
           </cell>
           <cell r="H145" t="str">
-            <v>C</v>
+            <v>OBJETIVO ALCANÇADO</v>
           </cell>
           <cell r="I145">
-            <v>3</v>
+            <v>0</v>
           </cell>
         </row>
         <row r="146">
@@ -3542,13 +3515,13 @@
             <v>9</v>
           </cell>
           <cell r="F146">
-            <v>10</v>
+            <v>19</v>
           </cell>
           <cell r="H146" t="str">
-            <v>C</v>
+            <v>A</v>
           </cell>
           <cell r="I146">
-            <v>4</v>
+            <v>1</v>
           </cell>
         </row>
         <row r="147">
@@ -3556,13 +3529,13 @@
             <v>9</v>
           </cell>
           <cell r="F147">
-            <v>12</v>
+            <v>20</v>
           </cell>
           <cell r="H147" t="str">
-            <v>C</v>
+            <v>OBJETIVO ALCANÇADO</v>
           </cell>
           <cell r="I147">
-            <v>2</v>
+            <v>0</v>
           </cell>
         </row>
         <row r="148">
@@ -3570,13 +3543,13 @@
             <v>9</v>
           </cell>
           <cell r="F148">
-            <v>11</v>
+            <v>26</v>
           </cell>
           <cell r="H148" t="str">
-            <v>C</v>
+            <v>OBJETIVO ALCANÇADO</v>
           </cell>
           <cell r="I148">
-            <v>3</v>
+            <v>0</v>
           </cell>
         </row>
         <row r="149">
@@ -3584,13 +3557,13 @@
             <v>9</v>
           </cell>
           <cell r="F149">
-            <v>9</v>
+            <v>20</v>
           </cell>
           <cell r="H149" t="str">
-            <v>C</v>
+            <v>OBJETIVO ALCANÇADO</v>
           </cell>
           <cell r="I149">
-            <v>5</v>
+            <v>0</v>
           </cell>
         </row>
         <row r="150">
@@ -3598,13 +3571,13 @@
             <v>9</v>
           </cell>
           <cell r="F150">
-            <v>15</v>
+            <v>20</v>
           </cell>
           <cell r="H150" t="str">
-            <v>B</v>
+            <v>OBJETIVO ALCANÇADO</v>
           </cell>
           <cell r="I150">
-            <v>2</v>
+            <v>0</v>
           </cell>
         </row>
         <row r="151">
@@ -3612,7 +3585,7 @@
             <v>9</v>
           </cell>
           <cell r="F151">
-            <v>20</v>
+            <v>28</v>
           </cell>
           <cell r="H151" t="str">
             <v>OBJETIVO ALCANÇADO</v>
@@ -3626,13 +3599,13 @@
             <v>9</v>
           </cell>
           <cell r="F152">
-            <v>7</v>
+            <v>21</v>
           </cell>
           <cell r="H152" t="str">
-            <v>D</v>
+            <v>OBJETIVO ALCANÇADO</v>
           </cell>
           <cell r="I152">
-            <v>2</v>
+            <v>0</v>
           </cell>
         </row>
         <row r="153">
@@ -3640,13 +3613,13 @@
             <v>9</v>
           </cell>
           <cell r="F153">
-            <v>6</v>
+            <v>20</v>
           </cell>
           <cell r="H153" t="str">
-            <v>D</v>
+            <v>OBJETIVO ALCANÇADO</v>
           </cell>
           <cell r="I153">
-            <v>3</v>
+            <v>0</v>
           </cell>
         </row>
         <row r="154">
@@ -3654,10 +3627,10 @@
             <v>189</v>
           </cell>
           <cell r="F154">
-            <v>285</v>
+            <v>520</v>
           </cell>
           <cell r="I154">
-            <v>41</v>
+            <v>4</v>
           </cell>
         </row>
         <row r="158">
@@ -3679,13 +3652,13 @@
             <v>38250</v>
           </cell>
           <cell r="F159">
-            <v>27935.73000000001</v>
+            <v>75978.280000000057</v>
           </cell>
           <cell r="H159" t="str">
-            <v>D</v>
+            <v>A</v>
           </cell>
           <cell r="I159">
-            <v>10314.26999999999</v>
+            <v>9021.719999999943</v>
           </cell>
         </row>
         <row r="160">
@@ -3693,13 +3666,13 @@
             <v>34425</v>
           </cell>
           <cell r="F160">
-            <v>28037.200000000004</v>
+            <v>65317.66</v>
           </cell>
           <cell r="H160" t="str">
-            <v>D</v>
+            <v>A</v>
           </cell>
           <cell r="I160">
-            <v>6387.7999999999956</v>
+            <v>11182.339999999997</v>
           </cell>
         </row>
         <row r="161">
@@ -3707,13 +3680,13 @@
             <v>153000</v>
           </cell>
           <cell r="F161">
-            <v>139883.35999999984</v>
+            <v>320791.82000000047</v>
           </cell>
           <cell r="H161" t="str">
-            <v>D</v>
+            <v>A</v>
           </cell>
           <cell r="I161">
-            <v>13116.640000000159</v>
+            <v>19208.179999999527</v>
           </cell>
         </row>
         <row r="162">
@@ -3721,13 +3694,13 @@
             <v>146925</v>
           </cell>
           <cell r="F162">
-            <v>125560.12500000007</v>
+            <v>304475.37500000017</v>
           </cell>
           <cell r="H162" t="str">
-            <v>D</v>
+            <v>A</v>
           </cell>
           <cell r="I162">
-            <v>21364.874999999927</v>
+            <v>22024.624999999825</v>
           </cell>
         </row>
         <row r="163">
@@ -3735,13 +3708,13 @@
             <v>124200</v>
           </cell>
           <cell r="F163">
-            <v>100281.57999999986</v>
+            <v>251396.75999999963</v>
           </cell>
           <cell r="H163" t="str">
-            <v>D</v>
+            <v>A</v>
           </cell>
           <cell r="I163">
-            <v>23918.420000000144</v>
+            <v>24603.240000000369</v>
           </cell>
         </row>
         <row r="164">
@@ -3749,13 +3722,13 @@
             <v>91350</v>
           </cell>
           <cell r="F164">
-            <v>84326.634999999995</v>
+            <v>190895.0149999992</v>
           </cell>
           <cell r="H164" t="str">
-            <v>D</v>
+            <v>A</v>
           </cell>
           <cell r="I164">
-            <v>7023.3650000000052</v>
+            <v>12104.985000000801</v>
           </cell>
         </row>
         <row r="165">
@@ -3763,13 +3736,13 @@
             <v>76500</v>
           </cell>
           <cell r="F165">
-            <v>68771.89</v>
+            <v>173369.35999999978</v>
           </cell>
           <cell r="H165" t="str">
-            <v>D</v>
+            <v>OBJETIVO ALCANÇADO</v>
           </cell>
           <cell r="I165">
-            <v>7728.1100000000006</v>
+            <v>0</v>
           </cell>
         </row>
         <row r="166">
@@ -3777,13 +3750,13 @@
             <v>110250</v>
           </cell>
           <cell r="F166">
-            <v>96164.2</v>
+            <v>233973.21999999901</v>
           </cell>
           <cell r="H166" t="str">
-            <v>D</v>
+            <v>A</v>
           </cell>
           <cell r="I166">
-            <v>14085.800000000003</v>
+            <v>11026.780000000988</v>
           </cell>
         </row>
         <row r="167">
@@ -3791,13 +3764,13 @@
             <v>54900</v>
           </cell>
           <cell r="F167">
-            <v>31050.670000000006</v>
+            <v>93024.129999999917</v>
           </cell>
           <cell r="H167" t="str">
-            <v>D</v>
+            <v>B</v>
           </cell>
           <cell r="I167">
-            <v>23849.329999999994</v>
+            <v>10675.870000000083</v>
           </cell>
         </row>
         <row r="168">
@@ -3805,13 +3778,13 @@
             <v>24750</v>
           </cell>
           <cell r="F168">
-            <v>21675.470000000005</v>
+            <v>56813.940000000111</v>
           </cell>
           <cell r="H168" t="str">
-            <v>D</v>
+            <v>OBJETIVO ALCANÇADO</v>
           </cell>
           <cell r="I168">
-            <v>3074.5299999999952</v>
+            <v>0</v>
           </cell>
         </row>
         <row r="169">
@@ -3819,13 +3792,13 @@
             <v>41850</v>
           </cell>
           <cell r="F169">
-            <v>31196.295000000016</v>
+            <v>86297.000000000015</v>
           </cell>
           <cell r="H169" t="str">
-            <v>D</v>
+            <v>A</v>
           </cell>
           <cell r="I169">
-            <v>10653.704999999984</v>
+            <v>6702.9999999999854</v>
           </cell>
         </row>
         <row r="170">
@@ -3833,13 +3806,13 @@
             <v>30375</v>
           </cell>
           <cell r="F170">
-            <v>23194.480000000007</v>
+            <v>62470.590000000004</v>
           </cell>
           <cell r="H170" t="str">
-            <v>D</v>
+            <v>A</v>
           </cell>
           <cell r="I170">
-            <v>7180.5199999999932</v>
+            <v>5029.4099999999962</v>
           </cell>
         </row>
         <row r="171">
@@ -3847,13 +3820,13 @@
             <v>36450</v>
           </cell>
           <cell r="F171">
-            <v>29316.740000000023</v>
+            <v>77850.589999999909</v>
           </cell>
           <cell r="H171" t="str">
-            <v>D</v>
+            <v>A</v>
           </cell>
           <cell r="I171">
-            <v>7133.2599999999766</v>
+            <v>3149.4100000000908</v>
           </cell>
         </row>
         <row r="172">
@@ -3861,13 +3834,13 @@
             <v>63900</v>
           </cell>
           <cell r="F172">
-            <v>40663.720000000038</v>
+            <v>112939.21999999965</v>
           </cell>
           <cell r="H172" t="str">
-            <v>D</v>
+            <v>B</v>
           </cell>
           <cell r="I172">
-            <v>23236.279999999962</v>
+            <v>7760.7800000003481</v>
           </cell>
         </row>
         <row r="173">
@@ -3875,13 +3848,13 @@
             <v>65250</v>
           </cell>
           <cell r="F173">
-            <v>43855.759999999995</v>
+            <v>126001.7799999999</v>
           </cell>
           <cell r="H173" t="str">
-            <v>D</v>
+            <v>A</v>
           </cell>
           <cell r="I173">
-            <v>21394.240000000005</v>
+            <v>18998.220000000103</v>
           </cell>
         </row>
         <row r="174">
@@ -3889,13 +3862,13 @@
             <v>119250</v>
           </cell>
           <cell r="F174">
-            <v>100639.89999999994</v>
+            <v>244477.96999999936</v>
           </cell>
           <cell r="H174" t="str">
-            <v>D</v>
+            <v>A</v>
           </cell>
           <cell r="I174">
-            <v>18610.100000000064</v>
+            <v>20522.030000000639</v>
           </cell>
         </row>
         <row r="175">
@@ -3903,13 +3876,13 @@
             <v>36000</v>
           </cell>
           <cell r="F175">
-            <v>29544.7</v>
+            <v>67490.080000000045</v>
           </cell>
           <cell r="H175" t="str">
-            <v>D</v>
+            <v>B</v>
           </cell>
           <cell r="I175">
-            <v>6455.2999999999993</v>
+            <v>509.9199999999546</v>
           </cell>
         </row>
         <row r="176">
@@ -3917,13 +3890,13 @@
             <v>66150</v>
           </cell>
           <cell r="F176">
-            <v>45658.210000000028</v>
+            <v>140208.75999999949</v>
           </cell>
           <cell r="H176" t="str">
-            <v>D</v>
+            <v>A</v>
           </cell>
           <cell r="I176">
-            <v>20491.789999999972</v>
+            <v>6791.2400000005146</v>
           </cell>
         </row>
         <row r="177">
@@ -3931,10 +3904,10 @@
             <v>1313775</v>
           </cell>
           <cell r="F177">
-            <v>1067756.6649999998</v>
+            <v>2683771.5499999966</v>
           </cell>
           <cell r="I177">
-            <v>246018.33500000017</v>
+            <v>189311.75000000314</v>
           </cell>
         </row>
       </sheetData>
@@ -4779,19 +4752,19 @@
       </c>
       <c r="AD3" s="29">
         <f>IFERROR(_xlfn.XLOOKUP(Y3,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0),0)</f>
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="AE3" s="29" t="str" cm="1">
         <f t="array" ref="AE3">_xlfn.IFS(AD3&gt;=Z3,"A",AD3&gt;=AA3,"B",AD3&gt;=AB3,"C",AD3&gt;=AC3,"D",TRUE,"NÃO ATINGIDO")</f>
-        <v>D</v>
+        <v>NÃO ATINGIDO</v>
       </c>
       <c r="AF3" s="29" t="str" cm="1">
         <f t="array" ref="AF3">_xlfn.IFS(AE3="NÃO ATINGIDO","D",AE3="D","C",AE3="C","B",AE3="B","A",AE3="A","OBJETIVO ALCANÇADO")</f>
-        <v>C</v>
+        <v>D</v>
       </c>
       <c r="AG3" s="29" cm="1">
         <f t="array" ref="AG3">_xlfn.IFS(AF3="D",MAX(AC3-AD3,0),AF3="C",MAX(AB3-AD3,0),AF3="B",MAX(AA3-AD3,0),AF3="A",MAX(Z3-AD3,0),AF3="OBJETIVO ALCANÇADO",0)</f>
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="AI3" t="s">
         <v>22</v>
@@ -4814,19 +4787,19 @@
       </c>
       <c r="AN3" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI3,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>27935.73000000001</v>
+        <v>75978.280000000057</v>
       </c>
       <c r="AO3" s="26" t="str" cm="1">
         <f t="array" ref="AO3">_xlfn.IFS(AN3&gt;=AJ3,"A",AN3&gt;=AK3,"B",AN3&gt;=AL3,"C",AN3&gt;=AM3,"D",TRUE,"NÃO ATINGIDO")</f>
-        <v>NÃO ATINGIDO</v>
+        <v>B</v>
       </c>
       <c r="AP3" s="26" t="str" cm="1">
         <f t="array" ref="AP3">_xlfn.IFS(AO3="NÃO ATINGIDO","D",AO3="D","C",AO3="C","B",AO3="B","A",AO3="A","OBJETIVO ALCANÇADO")</f>
-        <v>D</v>
+        <v>A</v>
       </c>
       <c r="AQ3" s="25" cm="1">
         <f t="array" ref="AQ3">_xlfn.IFS(AP3="D",MAX(AM3-AN3,0),AP3="C",MAX(AL3-AN3,0),AP3="B",MAX(AK3-AN3,0),AP3="A",MAX(AJ3-AN3,0),AP3="OBJETIVO ALCANÇADO",0)</f>
-        <v>10314.26999999999</v>
+        <v>9021.719999999943</v>
       </c>
     </row>
     <row r="4" spans="1:43" x14ac:dyDescent="0.25">
@@ -4847,7 +4820,7 @@
       </c>
       <c r="I4" s="7">
         <f>SUM(I10:I27)</f>
-        <v>300630</v>
+        <v>200230</v>
       </c>
       <c r="J4" s="4"/>
       <c r="K4" s="4"/>
@@ -4858,7 +4831,7 @@
       </c>
       <c r="O4" s="7">
         <f>SUM(O11:O17)</f>
-        <v>391000</v>
+        <v>549000</v>
       </c>
       <c r="P4" s="4"/>
       <c r="Q4" s="4"/>
@@ -4894,19 +4867,19 @@
       </c>
       <c r="AD4" s="31">
         <f>IFERROR(_xlfn.XLOOKUP(Y4,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$M:$M,0),0)</f>
-        <v>9</v>
+        <v>65</v>
       </c>
       <c r="AE4" s="31" t="str" cm="1">
         <f t="array" ref="AE4">_xlfn.IFS(AD4&gt;=Z4,"A",AD4&gt;=AA4,"B",AD4&gt;=AB4,"C",AD4&gt;=AC4,"D",TRUE,"NÃO ATINGIDO")</f>
-        <v>NÃO ATINGIDO</v>
+        <v>C</v>
       </c>
       <c r="AF4" s="31" t="str" cm="1">
         <f t="array" ref="AF4">_xlfn.IFS(AE4="NÃO ATINGIDO","D",AE4="D","C",AE4="C","B",AE4="B","A",AE4="A","OBJETIVO ALCANÇADO")</f>
-        <v>D</v>
+        <v>B</v>
       </c>
       <c r="AG4" s="31" cm="1">
         <f t="array" ref="AG4">_xlfn.IFS(AF4="D",MAX(AC4-AD4,0),AF4="C",MAX(AB4-AD4,0),AF4="B",MAX(AA4-AD4,0),AF4="A",MAX(Z4-AD4,0),AF4="OBJETIVO ALCANÇADO",0)</f>
-        <v>27</v>
+        <v>3</v>
       </c>
       <c r="AI4" t="s">
         <v>24</v>
@@ -4929,19 +4902,19 @@
       </c>
       <c r="AN4" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI4,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>28037.200000000004</v>
+        <v>65317.66</v>
       </c>
       <c r="AO4" s="26" t="str" cm="1">
         <f t="array" ref="AO4">_xlfn.IFS(AN4&gt;=AJ4,"A",AN4&gt;=AK4,"B",AN4&gt;=AL4,"C",AN4&gt;=AM4,"D",TRUE,"NÃO ATINGIDO")</f>
-        <v>NÃO ATINGIDO</v>
+        <v>B</v>
       </c>
       <c r="AP4" s="26" t="str" cm="1">
         <f t="array" ref="AP4">_xlfn.IFS(AO4="NÃO ATINGIDO","D",AO4="D","C",AO4="C","B",AO4="B","A",AO4="A","OBJETIVO ALCANÇADO")</f>
-        <v>D</v>
+        <v>A</v>
       </c>
       <c r="AQ4" s="25" cm="1">
         <f t="array" ref="AQ4">_xlfn.IFS(AP4="D",MAX(AM4-AN4,0),AP4="C",MAX(AL4-AN4,0),AP4="B",MAX(AK4-AN4,0),AP4="A",MAX(AJ4-AN4,0),AP4="OBJETIVO ALCANÇADO",0)</f>
-        <v>6387.7999999999956</v>
+        <v>11182.339999999997</v>
       </c>
     </row>
     <row r="5" spans="1:43" x14ac:dyDescent="0.25">
@@ -4951,7 +4924,7 @@
       </c>
       <c r="C5" s="2">
         <f>SUM(D10:D36)</f>
-        <v>1963372.9949999994</v>
+        <v>5074339.2199999969</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -4962,7 +4935,7 @@
       </c>
       <c r="I5" s="7">
         <f>SUM(J10:J27)</f>
-        <v>122855.06499999999</v>
+        <v>235763.16999999998</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -4973,7 +4946,7 @@
       </c>
       <c r="O5" s="7">
         <f>SUM(P11:P17)</f>
-        <v>6348.4</v>
+        <v>87468.709999999992</v>
       </c>
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
@@ -4983,8 +4956,8 @@
         <v>1</v>
       </c>
       <c r="U5" s="4">
-        <f ca="1">SUM(V10:V26)</f>
-        <v>236</v>
+        <f>SUM(V10:V26)</f>
+        <v>455</v>
       </c>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -5009,19 +4982,19 @@
       </c>
       <c r="AD5" s="29">
         <f>IFERROR(_xlfn.XLOOKUP(Y5,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0),0)</f>
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="AE5" s="29" t="str" cm="1">
         <f t="array" ref="AE5">_xlfn.IFS(AD5&gt;=Z5,"A",AD5&gt;=AA5,"B",AD5&gt;=AB5,"C",AD5&gt;=AC5,"D",TRUE,"NÃO ATINGIDO")</f>
-        <v>D</v>
+        <v>NÃO ATINGIDO</v>
       </c>
       <c r="AF5" s="29" t="str" cm="1">
         <f t="array" ref="AF5">_xlfn.IFS(AE5="NÃO ATINGIDO","D",AE5="D","C",AE5="C","B",AE5="B","A",AE5="A","OBJETIVO ALCANÇADO")</f>
-        <v>C</v>
+        <v>D</v>
       </c>
       <c r="AG5" s="29" cm="1">
         <f t="array" ref="AG5">_xlfn.IFS(AF5="D",MAX(AC5-AD5,0),AF5="C",MAX(AB5-AD5,0),AF5="B",MAX(AA5-AD5,0),AF5="A",MAX(Z5-AD5,0),AF5="OBJETIVO ALCANÇADO",0)</f>
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="AI5" t="s">
         <v>8</v>
@@ -5044,19 +5017,19 @@
       </c>
       <c r="AN5" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI5,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>139883.35999999984</v>
+        <v>320791.82000000047</v>
       </c>
       <c r="AO5" s="26" t="str" cm="1">
         <f t="array" ref="AO5">_xlfn.IFS(AN5&gt;=AJ5,"A",AN5&gt;=AK5,"B",AN5&gt;=AL5,"C",AN5&gt;=AM5,"D",TRUE,"NÃO ATINGIDO")</f>
-        <v>NÃO ATINGIDO</v>
+        <v>B</v>
       </c>
       <c r="AP5" s="26" t="str" cm="1">
         <f t="array" ref="AP5">_xlfn.IFS(AO5="NÃO ATINGIDO","D",AO5="D","C",AO5="C","B",AO5="B","A",AO5="A","OBJETIVO ALCANÇADO")</f>
-        <v>D</v>
+        <v>A</v>
       </c>
       <c r="AQ5" s="25" cm="1">
         <f t="array" ref="AQ5">_xlfn.IFS(AP5="D",MAX(AM5-AN5,0),AP5="C",MAX(AL5-AN5,0),AP5="B",MAX(AK5-AN5,0),AP5="A",MAX(AJ5-AN5,0),AP5="OBJETIVO ALCANÇADO",0)</f>
-        <v>13116.640000000159</v>
+        <v>19208.179999999527</v>
       </c>
     </row>
     <row r="6" spans="1:43" x14ac:dyDescent="0.25">
@@ -5066,7 +5039,7 @@
       </c>
       <c r="C6" s="2">
         <f>C4-C5</f>
-        <v>3939127.0050000008</v>
+        <v>828160.78000000305</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="4"/>
@@ -5077,7 +5050,7 @@
       </c>
       <c r="I6" s="7">
         <f>I4-I5</f>
-        <v>177774.935</v>
+        <v>-35533.169999999984</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -5088,7 +5061,7 @@
       </c>
       <c r="O6" s="7">
         <f>O4-O5</f>
-        <v>384651.6</v>
+        <v>461531.29000000004</v>
       </c>
       <c r="P6" s="4"/>
       <c r="Q6" s="4"/>
@@ -5098,8 +5071,8 @@
         <v>2</v>
       </c>
       <c r="U6" s="4">
-        <f ca="1">U4-U5</f>
-        <v>104</v>
+        <f>U4-U5</f>
+        <v>-115</v>
       </c>
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
@@ -5124,19 +5097,19 @@
       </c>
       <c r="AD6" s="31">
         <f>IFERROR(_xlfn.XLOOKUP(Y6,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0),0)</f>
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="AE6" s="31" t="str" cm="1">
         <f t="array" ref="AE6">_xlfn.IFS(AD6&gt;=Z6,"A",AD6&gt;=AA6,"B",AD6&gt;=AB6,"C",AD6&gt;=AC6,"D",TRUE,"NÃO ATINGIDO")</f>
-        <v>A</v>
+        <v>NÃO ATINGIDO</v>
       </c>
       <c r="AF6" s="31" t="str" cm="1">
         <f t="array" ref="AF6">_xlfn.IFS(AE6="NÃO ATINGIDO","D",AE6="D","C",AE6="C","B",AE6="B","A",AE6="A","OBJETIVO ALCANÇADO")</f>
-        <v>OBJETIVO ALCANÇADO</v>
+        <v>D</v>
       </c>
       <c r="AG6" s="31" cm="1">
         <f t="array" ref="AG6">_xlfn.IFS(AF6="D",MAX(AC6-AD6,0),AF6="C",MAX(AB6-AD6,0),AF6="B",MAX(AA6-AD6,0),AF6="A",MAX(Z6-AD6,0),AF6="OBJETIVO ALCANÇADO",0)</f>
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="AI6" t="s">
         <v>18</v>
@@ -5159,19 +5132,19 @@
       </c>
       <c r="AN6" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI6,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>125560.12500000007</v>
+        <v>304475.37500000017</v>
       </c>
       <c r="AO6" s="26" t="str" cm="1">
         <f t="array" ref="AO6">_xlfn.IFS(AN6&gt;=AJ6,"A",AN6&gt;=AK6,"B",AN6&gt;=AL6,"C",AN6&gt;=AM6,"D",TRUE,"NÃO ATINGIDO")</f>
-        <v>NÃO ATINGIDO</v>
+        <v>B</v>
       </c>
       <c r="AP6" s="26" t="str" cm="1">
         <f t="array" ref="AP6">_xlfn.IFS(AO6="NÃO ATINGIDO","D",AO6="D","C",AO6="C","B",AO6="B","A",AO6="A","OBJETIVO ALCANÇADO")</f>
-        <v>D</v>
+        <v>A</v>
       </c>
       <c r="AQ6" s="25" cm="1">
         <f t="array" ref="AQ6">_xlfn.IFS(AP6="D",MAX(AM6-AN6,0),AP6="C",MAX(AL6-AN6,0),AP6="B",MAX(AK6-AN6,0),AP6="A",MAX(AJ6-AN6,0),AP6="OBJETIVO ALCANÇADO",0)</f>
-        <v>21364.874999999927</v>
+        <v>22024.624999999825</v>
       </c>
     </row>
     <row r="7" spans="1:43" x14ac:dyDescent="0.25">
@@ -5181,7 +5154,7 @@
       </c>
       <c r="C7" s="3">
         <f>1-(C6/C4)</f>
-        <v>0.33263413722998714</v>
+        <v>0.85969321812791133</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="4"/>
@@ -5192,7 +5165,7 @@
       </c>
       <c r="I7" s="3">
         <f>1-(I6/I4)</f>
-        <v>0.4086587000632006</v>
+        <v>1.1774617689656894</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -5203,7 +5176,7 @@
       </c>
       <c r="O7" s="3">
         <f>1-(O6/O4)</f>
-        <v>1.623631713554996E-2</v>
+        <v>0.15932369763205823</v>
       </c>
       <c r="P7" s="4"/>
       <c r="Q7" s="4"/>
@@ -5213,8 +5186,8 @@
         <v>3</v>
       </c>
       <c r="U7" s="3">
-        <f ca="1">1-(U6/U4)</f>
-        <v>0.69411764705882351</v>
+        <f>1-(U6/U4)</f>
+        <v>1.3382352941176472</v>
       </c>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
@@ -5239,19 +5212,19 @@
       </c>
       <c r="AD7" s="29">
         <f>IFERROR(_xlfn.XLOOKUP(Y7,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0),0)</f>
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="AE7" s="29" t="str" cm="1">
         <f t="array" ref="AE7">_xlfn.IFS(AD7&gt;=Z7,"A",AD7&gt;=AA7,"B",AD7&gt;=AB7,"C",AD7&gt;=AC7,"D",TRUE,"NÃO ATINGIDO")</f>
-        <v>A</v>
+        <v>NÃO ATINGIDO</v>
       </c>
       <c r="AF7" s="29" t="str" cm="1">
         <f t="array" ref="AF7">_xlfn.IFS(AE7="NÃO ATINGIDO","D",AE7="D","C",AE7="C","B",AE7="B","A",AE7="A","OBJETIVO ALCANÇADO")</f>
-        <v>OBJETIVO ALCANÇADO</v>
+        <v>D</v>
       </c>
       <c r="AG7" s="29" cm="1">
         <f t="array" ref="AG7">_xlfn.IFS(AF7="D",MAX(AC7-AD7,0),AF7="C",MAX(AB7-AD7,0),AF7="B",MAX(AA7-AD7,0),AF7="A",MAX(Z7-AD7,0),AF7="OBJETIVO ALCANÇADO",0)</f>
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="AI7" t="s">
         <v>10</v>
@@ -5274,19 +5247,19 @@
       </c>
       <c r="AN7" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI7,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>100281.57999999986</v>
+        <v>251396.75999999963</v>
       </c>
       <c r="AO7" s="26" t="str" cm="1">
         <f t="array" ref="AO7">_xlfn.IFS(AN7&gt;=AJ7,"A",AN7&gt;=AK7,"B",AN7&gt;=AL7,"C",AN7&gt;=AM7,"D",TRUE,"NÃO ATINGIDO")</f>
-        <v>NÃO ATINGIDO</v>
+        <v>B</v>
       </c>
       <c r="AP7" s="26" t="str" cm="1">
         <f t="array" ref="AP7">_xlfn.IFS(AO7="NÃO ATINGIDO","D",AO7="D","C",AO7="C","B",AO7="B","A",AO7="A","OBJETIVO ALCANÇADO")</f>
-        <v>D</v>
+        <v>A</v>
       </c>
       <c r="AQ7" s="25" cm="1">
         <f t="array" ref="AQ7">_xlfn.IFS(AP7="D",MAX(AM7-AN7,0),AP7="C",MAX(AL7-AN7,0),AP7="B",MAX(AK7-AN7,0),AP7="A",MAX(AJ7-AN7,0),AP7="OBJETIVO ALCANÇADO",0)</f>
-        <v>23918.420000000144</v>
+        <v>24603.240000000369</v>
       </c>
     </row>
     <row r="8" spans="1:43" x14ac:dyDescent="0.25">
@@ -5333,19 +5306,19 @@
       </c>
       <c r="AD8" s="31">
         <f>IFERROR(_xlfn.XLOOKUP(Y8,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0),0)</f>
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="AE8" s="31" t="str" cm="1">
         <f t="array" ref="AE8">_xlfn.IFS(AD8&gt;=Z8,"A",AD8&gt;=AA8,"B",AD8&gt;=AB8,"C",AD8&gt;=AC8,"D",TRUE,"NÃO ATINGIDO")</f>
-        <v>B</v>
+        <v>NÃO ATINGIDO</v>
       </c>
       <c r="AF8" s="31" t="str" cm="1">
         <f t="array" ref="AF8">_xlfn.IFS(AE8="NÃO ATINGIDO","D",AE8="D","C",AE8="C","B",AE8="B","A",AE8="A","OBJETIVO ALCANÇADO")</f>
-        <v>A</v>
+        <v>D</v>
       </c>
       <c r="AG8" s="31" cm="1">
         <f t="array" ref="AG8">_xlfn.IFS(AF8="D",MAX(AC8-AD8,0),AF8="C",MAX(AB8-AD8,0),AF8="B",MAX(AA8-AD8,0),AF8="A",MAX(Z8-AD8,0),AF8="OBJETIVO ALCANÇADO",0)</f>
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="AI8" t="s">
         <v>13</v>
@@ -5368,19 +5341,19 @@
       </c>
       <c r="AN8" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI8,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>84326.634999999995</v>
+        <v>190895.0149999992</v>
       </c>
       <c r="AO8" s="26" t="str" cm="1">
         <f t="array" ref="AO8">_xlfn.IFS(AN8&gt;=AJ8,"A",AN8&gt;=AK8,"B",AN8&gt;=AL8,"C",AN8&gt;=AM8,"D",TRUE,"NÃO ATINGIDO")</f>
-        <v>NÃO ATINGIDO</v>
+        <v>B</v>
       </c>
       <c r="AP8" s="26" t="str" cm="1">
         <f t="array" ref="AP8">_xlfn.IFS(AO8="NÃO ATINGIDO","D",AO8="D","C",AO8="C","B",AO8="B","A",AO8="A","OBJETIVO ALCANÇADO")</f>
-        <v>D</v>
+        <v>A</v>
       </c>
       <c r="AQ8" s="25" cm="1">
         <f t="array" ref="AQ8">_xlfn.IFS(AP8="D",MAX(AM8-AN8,0),AP8="C",MAX(AL8-AN8,0),AP8="B",MAX(AK8-AN8,0),AP8="A",MAX(AJ8-AN8,0),AP8="OBJETIVO ALCANÇADO",0)</f>
-        <v>7023.3650000000052</v>
+        <v>12104.985000000801</v>
       </c>
     </row>
     <row r="9" spans="1:43" x14ac:dyDescent="0.25">
@@ -5419,7 +5392,7 @@
       <c r="M9" s="4"/>
       <c r="N9" s="4"/>
       <c r="O9" s="8" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="P9" s="4"/>
       <c r="Q9" s="4"/>
@@ -5460,19 +5433,19 @@
       </c>
       <c r="AD9" s="29">
         <f>IFERROR(_xlfn.XLOOKUP(Y9,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0),0)</f>
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="AE9" s="29" t="str" cm="1">
         <f t="array" ref="AE9">_xlfn.IFS(AD9&gt;=Z9,"A",AD9&gt;=AA9,"B",AD9&gt;=AB9,"C",AD9&gt;=AC9,"D",TRUE,"NÃO ATINGIDO")</f>
-        <v>D</v>
+        <v>NÃO ATINGIDO</v>
       </c>
       <c r="AF9" s="29" t="str" cm="1">
         <f t="array" ref="AF9">_xlfn.IFS(AE9="NÃO ATINGIDO","D",AE9="D","C",AE9="C","B",AE9="B","A",AE9="A","OBJETIVO ALCANÇADO")</f>
-        <v>C</v>
+        <v>D</v>
       </c>
       <c r="AG9" s="29" cm="1">
         <f t="array" ref="AG9">_xlfn.IFS(AF9="D",MAX(AC9-AD9,0),AF9="C",MAX(AB9-AD9,0),AF9="B",MAX(AA9-AD9,0),AF9="A",MAX(Z9-AD9,0),AF9="OBJETIVO ALCANÇADO",0)</f>
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="AI9" t="s">
         <v>20</v>
@@ -5495,19 +5468,19 @@
       </c>
       <c r="AN9" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI9,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>68771.89</v>
+        <v>173369.35999999978</v>
       </c>
       <c r="AO9" s="26" t="str" cm="1">
         <f t="array" ref="AO9">_xlfn.IFS(AN9&gt;=AJ9,"A",AN9&gt;=AK9,"B",AN9&gt;=AL9,"C",AN9&gt;=AM9,"D",TRUE,"NÃO ATINGIDO")</f>
-        <v>NÃO ATINGIDO</v>
+        <v>A</v>
       </c>
       <c r="AP9" s="26" t="str" cm="1">
         <f t="array" ref="AP9">_xlfn.IFS(AO9="NÃO ATINGIDO","D",AO9="D","C",AO9="C","B",AO9="B","A",AO9="A","OBJETIVO ALCANÇADO")</f>
-        <v>D</v>
+        <v>OBJETIVO ALCANÇADO</v>
       </c>
       <c r="AQ9" s="25" cm="1">
         <f t="array" ref="AQ9">_xlfn.IFS(AP9="D",MAX(AM9-AN9,0),AP9="C",MAX(AL9-AN9,0),AP9="B",MAX(AK9-AN9,0),AP9="A",MAX(AJ9-AN9,0),AP9="OBJETIVO ALCANÇADO",0)</f>
-        <v>7728.1100000000006</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:43" x14ac:dyDescent="0.25">
@@ -5523,11 +5496,11 @@
       </c>
       <c r="D10" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>23194.480000000007</v>
+        <v>62470.590000000004</v>
       </c>
       <c r="E10" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>44305.51999999999</v>
+        <v>5029.4099999999962</v>
       </c>
       <c r="F10" s="4"/>
       <c r="G10" s="18" t="s">
@@ -5538,15 +5511,15 @@
       </c>
       <c r="I10" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>30650</v>
+        <v>20000</v>
       </c>
       <c r="J10" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>14911.204999999994</v>
+        <v>19803.94999999999</v>
       </c>
       <c r="K10" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>15738.795000000006</v>
+        <v>196.05000000001019</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4" t="s">
@@ -5576,12 +5549,12 @@
         <v>20</v>
       </c>
       <c r="V10" s="17">
-        <f ca="1">VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
-        <v>12</v>
+        <f>VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
+        <v>20</v>
       </c>
       <c r="W10" s="17">
-        <f ca="1">U10-V10</f>
-        <v>8</v>
+        <f>U10-V10</f>
+        <v>0</v>
       </c>
       <c r="Y10" s="33" t="s">
         <v>17</v>
@@ -5604,19 +5577,19 @@
       </c>
       <c r="AD10" s="31">
         <f>IFERROR(_xlfn.XLOOKUP(Y10,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0),0)</f>
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="AE10" s="31" t="str" cm="1">
         <f t="array" ref="AE10">_xlfn.IFS(AD10&gt;=Z10,"A",AD10&gt;=AA10,"B",AD10&gt;=AB10,"C",AD10&gt;=AC10,"D",TRUE,"NÃO ATINGIDO")</f>
-        <v>A</v>
+        <v>NÃO ATINGIDO</v>
       </c>
       <c r="AF10" s="31" t="str" cm="1">
         <f t="array" ref="AF10">_xlfn.IFS(AE10="NÃO ATINGIDO","D",AE10="D","C",AE10="C","B",AE10="B","A",AE10="A","OBJETIVO ALCANÇADO")</f>
-        <v>OBJETIVO ALCANÇADO</v>
+        <v>D</v>
       </c>
       <c r="AG10" s="31" cm="1">
         <f t="array" ref="AG10">_xlfn.IFS(AF10="D",MAX(AC10-AD10,0),AF10="C",MAX(AB10-AD10,0),AF10="B",MAX(AA10-AD10,0),AF10="A",MAX(Z10-AD10,0),AF10="OBJETIVO ALCANÇADO",0)</f>
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="AI10" t="s">
         <v>17</v>
@@ -5639,19 +5612,19 @@
       </c>
       <c r="AN10" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI10,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>96164.2</v>
+        <v>233973.21999999901</v>
       </c>
       <c r="AO10" s="26" t="str" cm="1">
         <f t="array" ref="AO10">_xlfn.IFS(AN10&gt;=AJ10,"A",AN10&gt;=AK10,"B",AN10&gt;=AL10,"C",AN10&gt;=AM10,"D",TRUE,"NÃO ATINGIDO")</f>
-        <v>NÃO ATINGIDO</v>
+        <v>B</v>
       </c>
       <c r="AP10" s="26" t="str" cm="1">
         <f t="array" ref="AP10">_xlfn.IFS(AO10="NÃO ATINGIDO","D",AO10="D","C",AO10="C","B",AO10="B","A",AO10="A","OBJETIVO ALCANÇADO")</f>
-        <v>D</v>
+        <v>A</v>
       </c>
       <c r="AQ10" s="25" cm="1">
         <f t="array" ref="AQ10">_xlfn.IFS(AP10="D",MAX(AM10-AN10,0),AP10="C",MAX(AL10-AN10,0),AP10="B",MAX(AK10-AN10,0),AP10="A",MAX(AJ10-AN10,0),AP10="OBJETIVO ALCANÇADO",0)</f>
-        <v>14085.800000000003</v>
+        <v>11026.780000000988</v>
       </c>
     </row>
     <row r="11" spans="1:43" x14ac:dyDescent="0.25">
@@ -5667,11 +5640,11 @@
       </c>
       <c r="D11" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>139883.35999999984</v>
+        <v>320791.82000000047</v>
       </c>
       <c r="E11" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>200116.64000000016</v>
+        <v>19208.179999999527</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="18" t="s">
@@ -5682,15 +5655,15 @@
       </c>
       <c r="I11" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>27160</v>
+        <v>16540</v>
       </c>
       <c r="J11" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>10940.499999999998</v>
+        <v>23232.1</v>
       </c>
       <c r="K11" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>16219.500000000002</v>
+        <v>-6692.0999999999985</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4" t="s">
@@ -5705,11 +5678,11 @@
       </c>
       <c r="P11" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[REGIAO]","[Intervalo 2].[REGIAO].&amp;["&amp;N11&amp;"]","[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;["&amp;RIGHT($O$9,1)&amp;"]"),0)</f>
-        <v>0</v>
+        <v>3361</v>
       </c>
       <c r="Q11" s="2">
         <f>Tabela8[[#This Row],[COMPROMISSO]]-Tabela8[[#This Row],[ATINGIDO]]</f>
-        <v>0</v>
+        <v>-3361</v>
       </c>
       <c r="R11" s="2"/>
       <c r="S11" s="17" t="s">
@@ -5723,12 +5696,12 @@
         <v>20</v>
       </c>
       <c r="V11" s="17">
-        <f ca="1">VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
-        <v>13</v>
+        <f>VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
+        <v>22</v>
       </c>
       <c r="W11" s="17">
-        <f t="shared" ref="W11:W20" ca="1" si="0">U11-V11</f>
-        <v>7</v>
+        <f t="shared" ref="W11:W20" si="0">U11-V11</f>
+        <v>-2</v>
       </c>
       <c r="Y11" s="32" t="s">
         <v>12</v>
@@ -5751,7 +5724,7 @@
       </c>
       <c r="AD11" s="29">
         <f>IFERROR(_xlfn.XLOOKUP(Y11,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0),0)</f>
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="AE11" s="29" t="str" cm="1">
         <f t="array" ref="AE11">_xlfn.IFS(AD11&gt;=Z11,"A",AD11&gt;=AA11,"B",AD11&gt;=AB11,"C",AD11&gt;=AC11,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -5763,7 +5736,7 @@
       </c>
       <c r="AG11" s="29" cm="1">
         <f t="array" ref="AG11">_xlfn.IFS(AF11="D",MAX(AC11-AD11,0),AF11="C",MAX(AB11-AD11,0),AF11="B",MAX(AA11-AD11,0),AF11="A",MAX(Z11-AD11,0),AF11="OBJETIVO ALCANÇADO",0)</f>
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="AI11" t="s">
         <v>12</v>
@@ -5786,19 +5759,19 @@
       </c>
       <c r="AN11" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI11,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>31050.670000000006</v>
+        <v>93024.129999999917</v>
       </c>
       <c r="AO11" s="26" t="str" cm="1">
         <f t="array" ref="AO11">_xlfn.IFS(AN11&gt;=AJ11,"A",AN11&gt;=AK11,"B",AN11&gt;=AL11,"C",AN11&gt;=AM11,"D",TRUE,"NÃO ATINGIDO")</f>
-        <v>NÃO ATINGIDO</v>
+        <v>C</v>
       </c>
       <c r="AP11" s="26" t="str" cm="1">
         <f t="array" ref="AP11">_xlfn.IFS(AO11="NÃO ATINGIDO","D",AO11="D","C",AO11="C","B",AO11="B","A",AO11="A","OBJETIVO ALCANÇADO")</f>
-        <v>D</v>
+        <v>B</v>
       </c>
       <c r="AQ11" s="25" cm="1">
         <f t="array" ref="AQ11">_xlfn.IFS(AP11="D",MAX(AM11-AN11,0),AP11="C",MAX(AL11-AN11,0),AP11="B",MAX(AK11-AN11,0),AP11="A",MAX(AJ11-AN11,0),AP11="OBJETIVO ALCANÇADO",0)</f>
-        <v>23849.329999999994</v>
+        <v>10675.870000000083</v>
       </c>
     </row>
     <row r="12" spans="1:43" x14ac:dyDescent="0.25">
@@ -5814,11 +5787,11 @@
       </c>
       <c r="D12" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>55.04</v>
+        <v>102</v>
       </c>
       <c r="E12" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>-55.04</v>
+        <v>-102</v>
       </c>
       <c r="F12" s="4"/>
       <c r="G12" s="18" t="s">
@@ -5829,15 +5802,15 @@
       </c>
       <c r="I12" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>15600</v>
+        <v>10430</v>
       </c>
       <c r="J12" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>3254.9500000000003</v>
+        <v>9069.65</v>
       </c>
       <c r="K12" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>12345.05</v>
+        <v>1360.3500000000004</v>
       </c>
       <c r="L12" s="4"/>
       <c r="M12" s="4" t="s">
@@ -5870,12 +5843,12 @@
         <v>20</v>
       </c>
       <c r="V12" s="17">
-        <f ca="1">VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
-        <v>10</v>
+        <f>VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
+        <v>19</v>
       </c>
       <c r="W12" s="17">
-        <f t="shared" ca="1" si="0"/>
-        <v>10</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="Y12" s="33" t="s">
         <v>23</v>
@@ -5898,19 +5871,19 @@
       </c>
       <c r="AD12" s="31">
         <f>IFERROR(_xlfn.XLOOKUP(Y12,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0),0)</f>
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="AE12" s="31" t="str" cm="1">
         <f t="array" ref="AE12">_xlfn.IFS(AD12&gt;=Z12,"A",AD12&gt;=AA12,"B",AD12&gt;=AB12,"C",AD12&gt;=AC12,"D",TRUE,"NÃO ATINGIDO")</f>
-        <v>D</v>
+        <v>NÃO ATINGIDO</v>
       </c>
       <c r="AF12" s="31" t="str" cm="1">
         <f t="array" ref="AF12">_xlfn.IFS(AE12="NÃO ATINGIDO","D",AE12="D","C",AE12="C","B",AE12="B","A",AE12="A","OBJETIVO ALCANÇADO")</f>
-        <v>C</v>
+        <v>D</v>
       </c>
       <c r="AG12" s="31" cm="1">
         <f t="array" ref="AG12">_xlfn.IFS(AF12="D",MAX(AC12-AD12,0),AF12="C",MAX(AB12-AD12,0),AF12="B",MAX(AA12-AD12,0),AF12="A",MAX(Z12-AD12,0),AF12="OBJETIVO ALCANÇADO",0)</f>
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="AI12" t="s">
         <v>23</v>
@@ -5933,19 +5906,19 @@
       </c>
       <c r="AN12" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI12,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>21675.470000000005</v>
+        <v>56813.940000000111</v>
       </c>
       <c r="AO12" s="26" t="str" cm="1">
         <f t="array" ref="AO12">_xlfn.IFS(AN12&gt;=AJ12,"A",AN12&gt;=AK12,"B",AN12&gt;=AL12,"C",AN12&gt;=AM12,"D",TRUE,"NÃO ATINGIDO")</f>
-        <v>NÃO ATINGIDO</v>
+        <v>A</v>
       </c>
       <c r="AP12" s="26" t="str" cm="1">
         <f t="array" ref="AP12">_xlfn.IFS(AO12="NÃO ATINGIDO","D",AO12="D","C",AO12="C","B",AO12="B","A",AO12="A","OBJETIVO ALCANÇADO")</f>
-        <v>D</v>
+        <v>OBJETIVO ALCANÇADO</v>
       </c>
       <c r="AQ12" s="25" cm="1">
         <f t="array" ref="AQ12">_xlfn.IFS(AP12="D",MAX(AM12-AN12,0),AP12="C",MAX(AL12-AN12,0),AP12="B",MAX(AK12-AN12,0),AP12="A",MAX(AJ12-AN12,0),AP12="OBJETIVO ALCANÇADO",0)</f>
-        <v>3074.5299999999952</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:43" x14ac:dyDescent="0.25">
@@ -5961,11 +5934,11 @@
       </c>
       <c r="D13" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>31196.295000000016</v>
+        <v>86297.000000000015</v>
       </c>
       <c r="E13" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>61803.704999999987</v>
+        <v>6702.9999999999854</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="18" t="s">
@@ -5976,15 +5949,15 @@
       </c>
       <c r="I13" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>23440</v>
+        <v>20690</v>
       </c>
       <c r="J13" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>11125.239999999993</v>
+        <v>18462.34</v>
       </c>
       <c r="K13" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>12314.760000000007</v>
+        <v>2227.66</v>
       </c>
       <c r="L13" s="4"/>
       <c r="M13" s="4" t="s">
@@ -5999,11 +5972,11 @@
       </c>
       <c r="P13" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[REGIAO]","[Intervalo 2].[REGIAO].&amp;["&amp;N13&amp;"]","[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;["&amp;RIGHT($O$9,1)&amp;"]"),0)</f>
-        <v>0</v>
+        <v>30069.5</v>
       </c>
       <c r="Q13" s="2">
         <f>Tabela8[[#This Row],[COMPROMISSO]]-Tabela8[[#This Row],[ATINGIDO]]</f>
-        <v>0</v>
+        <v>-30069.5</v>
       </c>
       <c r="R13" s="2"/>
       <c r="S13" s="17" t="s">
@@ -6017,12 +5990,12 @@
         <v>20</v>
       </c>
       <c r="V13" s="17">
-        <f ca="1">VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
-        <v>29</v>
+        <f>VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
+        <v>54</v>
       </c>
       <c r="W13" s="17">
-        <f t="shared" ca="1" si="0"/>
-        <v>-9</v>
+        <f t="shared" si="0"/>
+        <v>-34</v>
       </c>
       <c r="Y13" s="32" t="s">
         <v>9</v>
@@ -6045,19 +6018,19 @@
       </c>
       <c r="AD13" s="29">
         <f>IFERROR(_xlfn.XLOOKUP(Y13,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0),0)</f>
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="AE13" s="29" t="str" cm="1">
         <f t="array" ref="AE13">_xlfn.IFS(AD13&gt;=Z13,"A",AD13&gt;=AA13,"B",AD13&gt;=AB13,"C",AD13&gt;=AC13,"D",TRUE,"NÃO ATINGIDO")</f>
-        <v>D</v>
+        <v>NÃO ATINGIDO</v>
       </c>
       <c r="AF13" s="29" t="str" cm="1">
         <f t="array" ref="AF13">_xlfn.IFS(AE13="NÃO ATINGIDO","D",AE13="D","C",AE13="C","B",AE13="B","A",AE13="A","OBJETIVO ALCANÇADO")</f>
-        <v>C</v>
+        <v>D</v>
       </c>
       <c r="AG13" s="29" cm="1">
         <f t="array" ref="AG13">_xlfn.IFS(AF13="D",MAX(AC13-AD13,0),AF13="C",MAX(AB13-AD13,0),AF13="B",MAX(AA13-AD13,0),AF13="A",MAX(Z13-AD13,0),AF13="OBJETIVO ALCANÇADO",0)</f>
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="AI13" t="s">
         <v>9</v>
@@ -6080,19 +6053,19 @@
       </c>
       <c r="AN13" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI13,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>31196.295000000016</v>
+        <v>86297.000000000015</v>
       </c>
       <c r="AO13" s="26" t="str" cm="1">
         <f t="array" ref="AO13">_xlfn.IFS(AN13&gt;=AJ13,"A",AN13&gt;=AK13,"B",AN13&gt;=AL13,"C",AN13&gt;=AM13,"D",TRUE,"NÃO ATINGIDO")</f>
-        <v>NÃO ATINGIDO</v>
+        <v>B</v>
       </c>
       <c r="AP13" s="26" t="str" cm="1">
         <f t="array" ref="AP13">_xlfn.IFS(AO13="NÃO ATINGIDO","D",AO13="D","C",AO13="C","B",AO13="B","A",AO13="A","OBJETIVO ALCANÇADO")</f>
-        <v>D</v>
+        <v>A</v>
       </c>
       <c r="AQ13" s="25" cm="1">
         <f t="array" ref="AQ13">_xlfn.IFS(AP13="D",MAX(AM13-AN13,0),AP13="C",MAX(AL13-AN13,0),AP13="B",MAX(AK13-AN13,0),AP13="A",MAX(AJ13-AN13,0),AP13="OBJETIVO ALCANÇADO",0)</f>
-        <v>10653.704999999984</v>
+        <v>6702.9999999999854</v>
       </c>
     </row>
     <row r="14" spans="1:43" x14ac:dyDescent="0.25">
@@ -6108,11 +6081,11 @@
       </c>
       <c r="D14" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>100281.57999999986</v>
+        <v>251396.75999999963</v>
       </c>
       <c r="E14" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>175718.42000000016</v>
+        <v>24603.240000000369</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="18" t="s">
@@ -6123,15 +6096,15 @@
       </c>
       <c r="I14" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>16770</v>
+        <v>8920</v>
       </c>
       <c r="J14" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1218.4000000000001</v>
+        <v>13741.719999999994</v>
       </c>
       <c r="K14" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>15551.6</v>
+        <v>-4821.7199999999939</v>
       </c>
       <c r="L14" s="4"/>
       <c r="M14" s="4" t="s">
@@ -6142,15 +6115,15 @@
       </c>
       <c r="O14" s="2" cm="1">
         <f t="array" ref="O14">IFERROR(_xlfn.XLOOKUP(M14,[1]!Tabela3[[#All],[VENDEDOR]],INDEX([1]!Tabela3[#All],0,MATCH($O$9,[1]!Tabela3[#Headers],0))),0)</f>
-        <v>73000</v>
+        <v>132000</v>
       </c>
       <c r="P14" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[REGIAO]","[Intervalo 2].[REGIAO].&amp;["&amp;N14&amp;"]","[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;["&amp;RIGHT($O$9,1)&amp;"]"),0)</f>
-        <v>0</v>
+        <v>2300.4</v>
       </c>
       <c r="Q14" s="2">
         <f>Tabela8[[#This Row],[COMPROMISSO]]-Tabela8[[#This Row],[ATINGIDO]]</f>
-        <v>73000</v>
+        <v>129699.6</v>
       </c>
       <c r="R14" s="2"/>
       <c r="S14" s="17" t="s">
@@ -6164,12 +6137,12 @@
         <v>20</v>
       </c>
       <c r="V14" s="17">
-        <f ca="1">VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
-        <v>11</v>
+        <f>VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
+        <v>26</v>
       </c>
       <c r="W14" s="17">
-        <f t="shared" ca="1" si="0"/>
-        <v>9</v>
+        <f t="shared" si="0"/>
+        <v>-6</v>
       </c>
       <c r="Y14" s="33" t="s">
         <v>7</v>
@@ -6192,19 +6165,19 @@
       </c>
       <c r="AD14" s="31">
         <f>IFERROR(_xlfn.XLOOKUP(Y14,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0),0)</f>
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="AE14" s="31" t="str" cm="1">
         <f t="array" ref="AE14">_xlfn.IFS(AD14&gt;=Z14,"A",AD14&gt;=AA14,"B",AD14&gt;=AB14,"C",AD14&gt;=AC14,"D",TRUE,"NÃO ATINGIDO")</f>
-        <v>D</v>
+        <v>NÃO ATINGIDO</v>
       </c>
       <c r="AF14" s="31" t="str" cm="1">
         <f t="array" ref="AF14">_xlfn.IFS(AE14="NÃO ATINGIDO","D",AE14="D","C",AE14="C","B",AE14="B","A",AE14="A","OBJETIVO ALCANÇADO")</f>
-        <v>C</v>
+        <v>D</v>
       </c>
       <c r="AG14" s="31" cm="1">
         <f t="array" ref="AG14">_xlfn.IFS(AF14="D",MAX(AC14-AD14,0),AF14="C",MAX(AB14-AD14,0),AF14="B",MAX(AA14-AD14,0),AF14="A",MAX(Z14-AD14,0),AF14="OBJETIVO ALCANÇADO",0)</f>
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="AI14" t="s">
         <v>7</v>
@@ -6227,19 +6200,19 @@
       </c>
       <c r="AN14" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI14,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>23194.480000000007</v>
+        <v>62470.590000000004</v>
       </c>
       <c r="AO14" s="26" t="str" cm="1">
         <f t="array" ref="AO14">_xlfn.IFS(AN14&gt;=AJ14,"A",AN14&gt;=AK14,"B",AN14&gt;=AL14,"C",AN14&gt;=AM14,"D",TRUE,"NÃO ATINGIDO")</f>
-        <v>NÃO ATINGIDO</v>
+        <v>B</v>
       </c>
       <c r="AP14" s="26" t="str" cm="1">
         <f t="array" ref="AP14">_xlfn.IFS(AO14="NÃO ATINGIDO","D",AO14="D","C",AO14="C","B",AO14="B","A",AO14="A","OBJETIVO ALCANÇADO")</f>
-        <v>D</v>
+        <v>A</v>
       </c>
       <c r="AQ14" s="25" cm="1">
         <f t="array" ref="AQ14">_xlfn.IFS(AP14="D",MAX(AM14-AN14,0),AP14="C",MAX(AL14-AN14,0),AP14="B",MAX(AK14-AN14,0),AP14="A",MAX(AJ14-AN14,0),AP14="OBJETIVO ALCANÇADO",0)</f>
-        <v>7180.5199999999932</v>
+        <v>5029.4099999999962</v>
       </c>
     </row>
     <row r="15" spans="1:43" x14ac:dyDescent="0.25">
@@ -6255,11 +6228,11 @@
       </c>
       <c r="D15" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>29316.740000000023</v>
+        <v>77850.589999999909</v>
       </c>
       <c r="E15" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>51683.25999999998</v>
+        <v>3149.4100000000908</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="18" t="s">
@@ -6270,15 +6243,15 @@
       </c>
       <c r="I15" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>38000</v>
+        <v>22510</v>
       </c>
       <c r="J15" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>13827.15</v>
+        <v>26804.570000000011</v>
       </c>
       <c r="K15" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>24172.85</v>
+        <v>-4294.5700000000106</v>
       </c>
       <c r="L15" s="4"/>
       <c r="M15" s="4" t="s">
@@ -6289,15 +6262,15 @@
       </c>
       <c r="O15" s="2" cm="1">
         <f t="array" ref="O15">IFERROR(_xlfn.XLOOKUP(M15,[1]!Tabela3[[#All],[VENDEDOR]],INDEX([1]!Tabela3[#All],0,MATCH($O$9,[1]!Tabela3[#Headers],0))),0)</f>
-        <v>112000</v>
+        <v>253000</v>
       </c>
       <c r="P15" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[REGIAO]","[Intervalo 2].[REGIAO].&amp;["&amp;N15&amp;"]","[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;["&amp;RIGHT($O$9,1)&amp;"]"),0)</f>
-        <v>6348.4</v>
+        <v>17609.66</v>
       </c>
       <c r="Q15" s="2">
         <f>Tabela8[[#This Row],[COMPROMISSO]]-Tabela8[[#This Row],[ATINGIDO]]</f>
-        <v>105651.6</v>
+        <v>235390.34</v>
       </c>
       <c r="R15" s="2"/>
       <c r="S15" s="17" t="s">
@@ -6311,12 +6284,12 @@
         <v>20</v>
       </c>
       <c r="V15" s="17">
-        <f ca="1">VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
-        <v>8</v>
+        <f>VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
+        <v>21</v>
       </c>
       <c r="W15" s="17">
-        <f ca="1">U15-V15</f>
-        <v>12</v>
+        <f>U15-V15</f>
+        <v>-1</v>
       </c>
       <c r="Y15" s="32" t="s">
         <v>11</v>
@@ -6339,19 +6312,19 @@
       </c>
       <c r="AD15" s="29">
         <f>IFERROR(_xlfn.XLOOKUP(Y15,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0),0)</f>
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="AE15" s="29" t="str" cm="1">
         <f t="array" ref="AE15">_xlfn.IFS(AD15&gt;=Z15,"A",AD15&gt;=AA15,"B",AD15&gt;=AB15,"C",AD15&gt;=AC15,"D",TRUE,"NÃO ATINGIDO")</f>
-        <v>D</v>
+        <v>NÃO ATINGIDO</v>
       </c>
       <c r="AF15" s="29" t="str" cm="1">
         <f t="array" ref="AF15">_xlfn.IFS(AE15="NÃO ATINGIDO","D",AE15="D","C",AE15="C","B",AE15="B","A",AE15="A","OBJETIVO ALCANÇADO")</f>
-        <v>C</v>
+        <v>D</v>
       </c>
       <c r="AG15" s="29" cm="1">
         <f t="array" ref="AG15">_xlfn.IFS(AF15="D",MAX(AC15-AD15,0),AF15="C",MAX(AB15-AD15,0),AF15="B",MAX(AA15-AD15,0),AF15="A",MAX(Z15-AD15,0),AF15="OBJETIVO ALCANÇADO",0)</f>
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="AI15" t="s">
         <v>11</v>
@@ -6374,19 +6347,19 @@
       </c>
       <c r="AN15" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI15,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>29316.740000000023</v>
+        <v>77850.589999999909</v>
       </c>
       <c r="AO15" s="26" t="str" cm="1">
         <f t="array" ref="AO15">_xlfn.IFS(AN15&gt;=AJ15,"A",AN15&gt;=AK15,"B",AN15&gt;=AL15,"C",AN15&gt;=AM15,"D",TRUE,"NÃO ATINGIDO")</f>
-        <v>NÃO ATINGIDO</v>
+        <v>B</v>
       </c>
       <c r="AP15" s="26" t="str" cm="1">
         <f t="array" ref="AP15">_xlfn.IFS(AO15="NÃO ATINGIDO","D",AO15="D","C",AO15="C","B",AO15="B","A",AO15="A","OBJETIVO ALCANÇADO")</f>
-        <v>D</v>
+        <v>A</v>
       </c>
       <c r="AQ15" s="25" cm="1">
         <f t="array" ref="AQ15">_xlfn.IFS(AP15="D",MAX(AM15-AN15,0),AP15="C",MAX(AL15-AN15,0),AP15="B",MAX(AK15-AN15,0),AP15="A",MAX(AJ15-AN15,0),AP15="OBJETIVO ALCANÇADO",0)</f>
-        <v>7133.2599999999766</v>
+        <v>3149.4100000000908</v>
       </c>
     </row>
     <row r="16" spans="1:43" x14ac:dyDescent="0.25">
@@ -6402,11 +6375,11 @@
       </c>
       <c r="D16" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>98323.800000000017</v>
+        <v>261108.89999999991</v>
       </c>
       <c r="E16" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>251676.19999999998</v>
+        <v>88891.100000000093</v>
       </c>
       <c r="F16" s="4"/>
       <c r="G16" s="18" t="s">
@@ -6417,15 +6390,15 @@
       </c>
       <c r="I16" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>19560</v>
+        <v>11710</v>
       </c>
       <c r="J16" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>6734.5400000000009</v>
+        <v>16650.419999999998</v>
       </c>
       <c r="K16" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>12825.46</v>
+        <v>-4940.4199999999983</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4" t="s">
@@ -6436,15 +6409,15 @@
       </c>
       <c r="O16" s="2" cm="1">
         <f t="array" ref="O16">IFERROR(_xlfn.XLOOKUP(M16,[1]!Tabela3[[#All],[VENDEDOR]],INDEX([1]!Tabela3[#All],0,MATCH($O$9,[1]!Tabela3[#Headers],0))),0)</f>
-        <v>23000</v>
+        <v>75000</v>
       </c>
       <c r="P16" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[REGIAO]","[Intervalo 2].[REGIAO].&amp;["&amp;N16&amp;"]","[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;["&amp;RIGHT($O$9,1)&amp;"]"),0)</f>
-        <v>0</v>
+        <v>483.95</v>
       </c>
       <c r="Q16" s="2">
         <f>Tabela8[[#This Row],[COMPROMISSO]]-Tabela8[[#This Row],[ATINGIDO]]</f>
-        <v>23000</v>
+        <v>74516.05</v>
       </c>
       <c r="R16" s="2"/>
       <c r="S16" s="17" t="s">
@@ -6458,12 +6431,12 @@
         <v>20</v>
       </c>
       <c r="V16" s="17">
-        <f ca="1">VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
-        <v>7</v>
+        <f>VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
+        <v>21</v>
       </c>
       <c r="W16" s="17">
-        <f t="shared" ca="1" si="0"/>
-        <v>13</v>
+        <f t="shared" si="0"/>
+        <v>-1</v>
       </c>
       <c r="Y16" s="33" t="s">
         <v>19</v>
@@ -6486,19 +6459,19 @@
       </c>
       <c r="AD16" s="31">
         <f>IFERROR(_xlfn.XLOOKUP(Y16,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0),0)</f>
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="AE16" s="31" t="str" cm="1">
         <f t="array" ref="AE16">_xlfn.IFS(AD16&gt;=Z16,"A",AD16&gt;=AA16,"B",AD16&gt;=AB16,"C",AD16&gt;=AC16,"D",TRUE,"NÃO ATINGIDO")</f>
-        <v>D</v>
+        <v>NÃO ATINGIDO</v>
       </c>
       <c r="AF16" s="31" t="str" cm="1">
         <f t="array" ref="AF16">_xlfn.IFS(AE16="NÃO ATINGIDO","D",AE16="D","C",AE16="C","B",AE16="B","A",AE16="A","OBJETIVO ALCANÇADO")</f>
-        <v>C</v>
+        <v>D</v>
       </c>
       <c r="AG16" s="31" cm="1">
         <f t="array" ref="AG16">_xlfn.IFS(AF16="D",MAX(AC16-AD16,0),AF16="C",MAX(AB16-AD16,0),AF16="B",MAX(AA16-AD16,0),AF16="A",MAX(Z16-AD16,0),AF16="OBJETIVO ALCANÇADO",0)</f>
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="AI16" t="s">
         <v>19</v>
@@ -6521,19 +6494,19 @@
       </c>
       <c r="AN16" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI16,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>40663.720000000038</v>
+        <v>112939.21999999965</v>
       </c>
       <c r="AO16" s="26" t="str" cm="1">
         <f t="array" ref="AO16">_xlfn.IFS(AN16&gt;=AJ16,"A",AN16&gt;=AK16,"B",AN16&gt;=AL16,"C",AN16&gt;=AM16,"D",TRUE,"NÃO ATINGIDO")</f>
-        <v>NÃO ATINGIDO</v>
+        <v>C</v>
       </c>
       <c r="AP16" s="26" t="str" cm="1">
         <f t="array" ref="AP16">_xlfn.IFS(AO16="NÃO ATINGIDO","D",AO16="D","C",AO16="C","B",AO16="B","A",AO16="A","OBJETIVO ALCANÇADO")</f>
-        <v>D</v>
+        <v>B</v>
       </c>
       <c r="AQ16" s="25" cm="1">
         <f t="array" ref="AQ16">_xlfn.IFS(AP16="D",MAX(AM16-AN16,0),AP16="C",MAX(AL16-AN16,0),AP16="B",MAX(AK16-AN16,0),AP16="A",MAX(AJ16-AN16,0),AP16="OBJETIVO ALCANÇADO",0)</f>
-        <v>23236.279999999962</v>
+        <v>7760.7800000003481</v>
       </c>
     </row>
     <row r="17" spans="1:43" x14ac:dyDescent="0.25">
@@ -6549,11 +6522,11 @@
       </c>
       <c r="D17" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>205409.18000000031</v>
+        <v>645986.02999999968</v>
       </c>
       <c r="E17" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>244590.81999999969</v>
+        <v>-195986.02999999968</v>
       </c>
       <c r="F17" s="4"/>
       <c r="G17" s="18" t="s">
@@ -6564,15 +6537,15 @@
       </c>
       <c r="I17" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>2760</v>
+        <v>4830</v>
       </c>
       <c r="J17" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>4735.8200000000006</v>
+        <v>5865.7599999999993</v>
       </c>
       <c r="K17" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>-1975.8200000000006</v>
+        <v>-1035.7599999999993</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="4" t="s">
@@ -6583,15 +6556,15 @@
       </c>
       <c r="O17" s="2" cm="1">
         <f t="array" ref="O17">IFERROR(_xlfn.XLOOKUP(M17,[1]!Tabela3[[#All],[VENDEDOR]],INDEX([1]!Tabela3[#All],0,MATCH($O$9,[1]!Tabela3[#Headers],0))),0)</f>
-        <v>183000</v>
+        <v>89000</v>
       </c>
       <c r="P17" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[REGIAO]","[Intervalo 2].[REGIAO].&amp;["&amp;N17&amp;"]","[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;["&amp;RIGHT($O$9,1)&amp;"]"),0)</f>
-        <v>0</v>
+        <v>33644.19999999999</v>
       </c>
       <c r="Q17" s="2">
         <f>Tabela8[[#This Row],[COMPROMISSO]]-Tabela8[[#This Row],[ATINGIDO]]</f>
-        <v>183000</v>
+        <v>55355.80000000001</v>
       </c>
       <c r="R17" s="2"/>
       <c r="S17" s="17" t="s">
@@ -6605,12 +6578,12 @@
         <v>20</v>
       </c>
       <c r="V17" s="17">
-        <f ca="1">VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
-        <v>18</v>
+        <f>VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
+        <v>25</v>
       </c>
       <c r="W17" s="17">
-        <f t="shared" ca="1" si="0"/>
-        <v>2</v>
+        <f t="shared" si="0"/>
+        <v>-5</v>
       </c>
       <c r="Y17" s="32" t="s">
         <v>14</v>
@@ -6633,19 +6606,19 @@
       </c>
       <c r="AD17" s="29">
         <f>IFERROR(_xlfn.XLOOKUP(Y17,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0),0)</f>
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="AE17" s="29" t="str" cm="1">
         <f t="array" ref="AE17">_xlfn.IFS(AD17&gt;=Z17,"A",AD17&gt;=AA17,"B",AD17&gt;=AB17,"C",AD17&gt;=AC17,"D",TRUE,"NÃO ATINGIDO")</f>
-        <v>C</v>
+        <v>NÃO ATINGIDO</v>
       </c>
       <c r="AF17" s="29" t="str" cm="1">
         <f t="array" ref="AF17">_xlfn.IFS(AE17="NÃO ATINGIDO","D",AE17="D","C",AE17="C","B",AE17="B","A",AE17="A","OBJETIVO ALCANÇADO")</f>
-        <v>B</v>
+        <v>D</v>
       </c>
       <c r="AG17" s="29" cm="1">
         <f t="array" ref="AG17">_xlfn.IFS(AF17="D",MAX(AC17-AD17,0),AF17="C",MAX(AB17-AD17,0),AF17="B",MAX(AA17-AD17,0),AF17="A",MAX(Z17-AD17,0),AF17="OBJETIVO ALCANÇADO",0)</f>
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="AI17" t="s">
         <v>14</v>
@@ -6668,19 +6641,19 @@
       </c>
       <c r="AN17" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI17,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>43855.759999999995</v>
+        <v>126001.7799999999</v>
       </c>
       <c r="AO17" s="26" t="str" cm="1">
         <f t="array" ref="AO17">_xlfn.IFS(AN17&gt;=AJ17,"A",AN17&gt;=AK17,"B",AN17&gt;=AL17,"C",AN17&gt;=AM17,"D",TRUE,"NÃO ATINGIDO")</f>
-        <v>NÃO ATINGIDO</v>
+        <v>B</v>
       </c>
       <c r="AP17" s="26" t="str" cm="1">
         <f t="array" ref="AP17">_xlfn.IFS(AO17="NÃO ATINGIDO","D",AO17="D","C",AO17="C","B",AO17="B","A",AO17="A","OBJETIVO ALCANÇADO")</f>
-        <v>D</v>
+        <v>A</v>
       </c>
       <c r="AQ17" s="25" cm="1">
         <f t="array" ref="AQ17">_xlfn.IFS(AP17="D",MAX(AM17-AN17,0),AP17="C",MAX(AL17-AN17,0),AP17="B",MAX(AK17-AN17,0),AP17="A",MAX(AJ17-AN17,0),AP17="OBJETIVO ALCANÇADO",0)</f>
-        <v>21394.240000000005</v>
+        <v>18998.220000000103</v>
       </c>
     </row>
     <row r="18" spans="1:43" x14ac:dyDescent="0.25">
@@ -6696,11 +6669,11 @@
       </c>
       <c r="D18" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>347954.79999999987</v>
+        <v>816833.8</v>
       </c>
       <c r="E18" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>632045.20000000019</v>
+        <v>163166.19999999995</v>
       </c>
       <c r="F18" s="4"/>
       <c r="G18" s="18" t="s">
@@ -6711,15 +6684,15 @@
       </c>
       <c r="I18" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>13450</v>
+        <v>10020</v>
       </c>
       <c r="J18" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>5556.9499999999989</v>
+        <v>11939.229999999998</v>
       </c>
       <c r="K18" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>7893.0500000000011</v>
+        <v>-1919.2299999999977</v>
       </c>
       <c r="L18" s="4"/>
       <c r="M18" s="15"/>
@@ -6739,12 +6712,12 @@
         <v>20</v>
       </c>
       <c r="V18" s="17">
-        <f ca="1">VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
-        <v>23</v>
+        <f>VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
+        <v>44</v>
       </c>
       <c r="W18" s="17">
-        <f t="shared" ca="1" si="0"/>
-        <v>-3</v>
+        <f t="shared" si="0"/>
+        <v>-24</v>
       </c>
       <c r="Y18" s="33" t="s">
         <v>21</v>
@@ -6767,19 +6740,19 @@
       </c>
       <c r="AD18" s="31">
         <f>IFERROR(_xlfn.XLOOKUP(Y18,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0),0)</f>
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="AE18" s="31" t="str" cm="1">
         <f t="array" ref="AE18">_xlfn.IFS(AD18&gt;=Z18,"A",AD18&gt;=AA18,"B",AD18&gt;=AB18,"C",AD18&gt;=AC18,"D",TRUE,"NÃO ATINGIDO")</f>
-        <v>A</v>
+        <v>NÃO ATINGIDO</v>
       </c>
       <c r="AF18" s="31" t="str" cm="1">
         <f t="array" ref="AF18">_xlfn.IFS(AE18="NÃO ATINGIDO","D",AE18="D","C",AE18="C","B",AE18="B","A",AE18="A","OBJETIVO ALCANÇADO")</f>
-        <v>OBJETIVO ALCANÇADO</v>
+        <v>D</v>
       </c>
       <c r="AG18" s="31" cm="1">
         <f t="array" ref="AG18">_xlfn.IFS(AF18="D",MAX(AC18-AD18,0),AF18="C",MAX(AB18-AD18,0),AF18="B",MAX(AA18-AD18,0),AF18="A",MAX(Z18-AD18,0),AF18="OBJETIVO ALCANÇADO",0)</f>
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="AI18" t="s">
         <v>21</v>
@@ -6802,19 +6775,19 @@
       </c>
       <c r="AN18" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI18,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>100639.89999999994</v>
+        <v>244477.96999999936</v>
       </c>
       <c r="AO18" s="26" t="str" cm="1">
         <f t="array" ref="AO18">_xlfn.IFS(AN18&gt;=AJ18,"A",AN18&gt;=AK18,"B",AN18&gt;=AL18,"C",AN18&gt;=AM18,"D",TRUE,"NÃO ATINGIDO")</f>
-        <v>NÃO ATINGIDO</v>
+        <v>B</v>
       </c>
       <c r="AP18" s="26" t="str" cm="1">
         <f t="array" ref="AP18">_xlfn.IFS(AO18="NÃO ATINGIDO","D",AO18="D","C",AO18="C","B",AO18="B","A",AO18="A","OBJETIVO ALCANÇADO")</f>
-        <v>D</v>
+        <v>A</v>
       </c>
       <c r="AQ18" s="25" cm="1">
         <f t="array" ref="AQ18">_xlfn.IFS(AP18="D",MAX(AM18-AN18,0),AP18="C",MAX(AL18-AN18,0),AP18="B",MAX(AK18-AN18,0),AP18="A",MAX(AJ18-AN18,0),AP18="OBJETIVO ALCANÇADO",0)</f>
-        <v>18610.100000000064</v>
+        <v>20522.030000000639</v>
       </c>
     </row>
     <row r="19" spans="1:43" x14ac:dyDescent="0.25">
@@ -6830,11 +6803,11 @@
       </c>
       <c r="D19" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>19642.8</v>
+        <v>55652.650000000009</v>
       </c>
       <c r="E19" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>122357.2</v>
+        <v>86347.349999999991</v>
       </c>
       <c r="F19" s="4"/>
       <c r="G19" s="18" t="s">
@@ -6845,15 +6818,15 @@
       </c>
       <c r="I19" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>16550</v>
+        <v>20000</v>
       </c>
       <c r="J19" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>14553.599999999995</v>
+        <v>11443.519999999995</v>
       </c>
       <c r="K19" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>1996.4000000000051</v>
+        <v>8556.480000000005</v>
       </c>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
@@ -6869,12 +6842,12 @@
         <v>20</v>
       </c>
       <c r="V19" s="17">
-        <f ca="1">VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
-        <v>22</v>
+        <f>VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
+        <v>35</v>
       </c>
       <c r="W19" s="17">
-        <f t="shared" ca="1" si="0"/>
-        <v>-2</v>
+        <f t="shared" si="0"/>
+        <v>-15</v>
       </c>
       <c r="Y19" s="32" t="s">
         <v>16</v>
@@ -6897,7 +6870,7 @@
       </c>
       <c r="AD19" s="29">
         <f>IFERROR(_xlfn.XLOOKUP(Y19,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0),0)</f>
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="AE19" s="29" t="str" cm="1">
         <f t="array" ref="AE19">_xlfn.IFS(AD19&gt;=Z19,"A",AD19&gt;=AA19,"B",AD19&gt;=AB19,"C",AD19&gt;=AC19,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -6909,7 +6882,7 @@
       </c>
       <c r="AG19" s="29" cm="1">
         <f t="array" ref="AG19">_xlfn.IFS(AF19="D",MAX(AC19-AD19,0),AF19="C",MAX(AB19-AD19,0),AF19="B",MAX(AA19-AD19,0),AF19="A",MAX(Z19-AD19,0),AF19="OBJETIVO ALCANÇADO",0)</f>
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="AI19" t="s">
         <v>16</v>
@@ -6932,19 +6905,19 @@
       </c>
       <c r="AN19" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI19,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>29544.7</v>
+        <v>67490.080000000045</v>
       </c>
       <c r="AO19" s="26" t="str" cm="1">
         <f t="array" ref="AO19">_xlfn.IFS(AN19&gt;=AJ19,"A",AN19&gt;=AK19,"B",AN19&gt;=AL19,"C",AN19&gt;=AM19,"D",TRUE,"NÃO ATINGIDO")</f>
-        <v>NÃO ATINGIDO</v>
+        <v>C</v>
       </c>
       <c r="AP19" s="26" t="str" cm="1">
         <f t="array" ref="AP19">_xlfn.IFS(AO19="NÃO ATINGIDO","D",AO19="D","C",AO19="C","B",AO19="B","A",AO19="A","OBJETIVO ALCANÇADO")</f>
-        <v>D</v>
+        <v>B</v>
       </c>
       <c r="AQ19" s="25" cm="1">
         <f t="array" ref="AQ19">_xlfn.IFS(AP19="D",MAX(AM19-AN19,0),AP19="C",MAX(AL19-AN19,0),AP19="B",MAX(AK19-AN19,0),AP19="A",MAX(AJ19-AN19,0),AP19="OBJETIVO ALCANÇADO",0)</f>
-        <v>6455.2999999999993</v>
+        <v>509.9199999999546</v>
       </c>
     </row>
     <row r="20" spans="1:43" x14ac:dyDescent="0.25">
@@ -6960,11 +6933,11 @@
       </c>
       <c r="D20" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>145346.00000000003</v>
+        <v>316150.64000000007</v>
       </c>
       <c r="E20" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>434654</v>
+        <v>263849.35999999993</v>
       </c>
       <c r="F20" s="4"/>
       <c r="G20" s="18" t="s">
@@ -6975,15 +6948,15 @@
       </c>
       <c r="I20" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>27640</v>
+        <v>12140</v>
       </c>
       <c r="J20" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>17551.800000000003</v>
+        <v>17482.909999999996</v>
       </c>
       <c r="K20" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>10088.199999999997</v>
+        <v>-5342.9099999999962</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
@@ -7011,12 +6984,12 @@
         <v>20</v>
       </c>
       <c r="V20" s="17">
-        <f ca="1">VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
-        <v>15</v>
+        <f>VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
+        <v>20</v>
       </c>
       <c r="W20" s="17">
-        <f t="shared" ca="1" si="0"/>
-        <v>5</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="Y20" s="33" t="s">
         <v>15</v>
@@ -7039,7 +7012,7 @@
       </c>
       <c r="AD20" s="31">
         <f>IFERROR(_xlfn.XLOOKUP(Y20,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0),0)</f>
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AE20" s="31" t="str" cm="1">
         <f t="array" ref="AE20">_xlfn.IFS(AD20&gt;=Z20,"A",AD20&gt;=AA20,"B",AD20&gt;=AB20,"C",AD20&gt;=AC20,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -7051,7 +7024,7 @@
       </c>
       <c r="AG20" s="31" cm="1">
         <f t="array" ref="AG20">_xlfn.IFS(AF20="D",MAX(AC20-AD20,0),AF20="C",MAX(AB20-AD20,0),AF20="B",MAX(AA20-AD20,0),AF20="A",MAX(Z20-AD20,0),AF20="OBJETIVO ALCANÇADO",0)</f>
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="AI20" t="s">
         <v>15</v>
@@ -7074,19 +7047,19 @@
       </c>
       <c r="AN20" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI20,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>45658.210000000028</v>
+        <v>140208.75999999949</v>
       </c>
       <c r="AO20" s="26" t="str" cm="1">
         <f t="array" ref="AO20">_xlfn.IFS(AN20&gt;=AJ20,"A",AN20&gt;=AK20,"B",AN20&gt;=AL20,"C",AN20&gt;=AM20,"D",TRUE,"NÃO ATINGIDO")</f>
-        <v>NÃO ATINGIDO</v>
+        <v>B</v>
       </c>
       <c r="AP20" s="26" t="str" cm="1">
         <f t="array" ref="AP20">_xlfn.IFS(AO20="NÃO ATINGIDO","D",AO20="D","C",AO20="C","B",AO20="B","A",AO20="A","OBJETIVO ALCANÇADO")</f>
-        <v>D</v>
+        <v>A</v>
       </c>
       <c r="AQ20" s="25" cm="1">
         <f t="array" ref="AQ20">_xlfn.IFS(AP20="D",MAX(AM20-AN20,0),AP20="C",MAX(AL20-AN20,0),AP20="B",MAX(AK20-AN20,0),AP20="A",MAX(AJ20-AN20,0),AP20="OBJETIVO ALCANÇADO",0)</f>
-        <v>20491.789999999972</v>
+        <v>6791.2400000005146</v>
       </c>
     </row>
     <row r="21" spans="1:43" x14ac:dyDescent="0.25">
@@ -7102,11 +7075,11 @@
       </c>
       <c r="D21" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>78739.81</v>
+        <v>293729.78999999986</v>
       </c>
       <c r="E21" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>401260.19</v>
+        <v>186270.21000000014</v>
       </c>
       <c r="F21" s="4"/>
       <c r="G21" s="18" t="s">
@@ -7117,15 +7090,15 @@
       </c>
       <c r="I21" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>4550</v>
+        <v>8900</v>
       </c>
       <c r="J21" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2974.4600000000005</v>
+        <v>8545.5799999999981</v>
       </c>
       <c r="K21" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>1575.5399999999995</v>
+        <v>354.42000000000189</v>
       </c>
       <c r="L21" s="4"/>
       <c r="M21" s="4"/>
@@ -7156,12 +7129,12 @@
         <v>20</v>
       </c>
       <c r="V21" s="17">
-        <f ca="1">VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
-        <v>9</v>
+        <f>VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
+        <v>20</v>
       </c>
       <c r="W21" s="17">
-        <f t="shared" ref="W21:W26" ca="1" si="1">U21-V21</f>
-        <v>11</v>
+        <f t="shared" ref="W21:W26" si="1">U21-V21</f>
+        <v>0</v>
       </c>
       <c r="Y21" s="36" t="s">
         <v>60</v>
@@ -7184,13 +7157,13 @@
       </c>
       <c r="AD21" s="37">
         <f>SUBTOTAL(109,Planilha1!$AD$3:$AD$20)</f>
-        <v>245</v>
+        <v>65</v>
       </c>
       <c r="AE21" s="37"/>
       <c r="AF21" s="37"/>
       <c r="AG21" s="38">
         <f>SUBTOTAL(109,Planilha1!$AG$3:$AG$20)</f>
-        <v>61</v>
+        <v>156</v>
       </c>
       <c r="AI21" t="s">
         <v>60</v>
@@ -7213,13 +7186,13 @@
       </c>
       <c r="AN21" s="26">
         <f>SUBTOTAL(109,Tabela817[ATINGIDO])</f>
-        <v>1067756.6649999998</v>
+        <v>2683771.5499999966</v>
       </c>
       <c r="AO21" s="4"/>
       <c r="AP21" s="4"/>
       <c r="AQ21" s="27">
         <f>SUBTOTAL(109,Tabela817[FALTA])</f>
-        <v>246018.33500000017</v>
+        <v>189311.75000000314</v>
       </c>
     </row>
     <row r="22" spans="1:43" x14ac:dyDescent="0.25">
@@ -7235,11 +7208,11 @@
       </c>
       <c r="D22" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>31050.670000000006</v>
+        <v>93024.129999999917</v>
       </c>
       <c r="E22" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>90949.329999999987</v>
+        <v>28975.870000000083</v>
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="18" t="s">
@@ -7250,15 +7223,15 @@
       </c>
       <c r="I22" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>16180</v>
+        <v>6600</v>
       </c>
       <c r="J22" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>4013.4600000000009</v>
+        <v>15529.049999999997</v>
       </c>
       <c r="K22" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>12166.539999999999</v>
+        <v>-8929.0499999999975</v>
       </c>
       <c r="L22" s="4"/>
       <c r="M22" s="4"/>
@@ -7271,11 +7244,11 @@
       </c>
       <c r="P22" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>720213.08000000042</v>
+        <v>695196.28000000026</v>
       </c>
       <c r="Q22" s="7">
         <f>O22-P22</f>
-        <v>-152213.08000000042</v>
+        <v>-127196.28000000026</v>
       </c>
       <c r="R22" s="4"/>
       <c r="S22" s="17" t="s">
@@ -7289,12 +7262,12 @@
         <v>20</v>
       </c>
       <c r="V22" s="17">
-        <f ca="1">VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
-        <v>13</v>
+        <f>VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
+        <v>32</v>
       </c>
       <c r="W22" s="17">
-        <f t="shared" ca="1" si="1"/>
-        <v>7</v>
+        <f t="shared" si="1"/>
+        <v>-12</v>
       </c>
     </row>
     <row r="23" spans="1:43" x14ac:dyDescent="0.25">
@@ -7310,11 +7283,11 @@
       </c>
       <c r="D23" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>84326.634999999995</v>
+        <v>190895.0149999992</v>
       </c>
       <c r="E23" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>118673.36500000001</v>
+        <v>12104.985000000801</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="18" t="s">
@@ -7325,15 +7298,15 @@
       </c>
       <c r="I23" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>13170</v>
+        <v>6690</v>
       </c>
       <c r="J23" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1693.7899999999997</v>
+        <v>10844.970000000001</v>
       </c>
       <c r="K23" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>11476.210000000001</v>
+        <v>-4154.9700000000012</v>
       </c>
       <c r="L23" s="4"/>
       <c r="M23" s="4"/>
@@ -7346,11 +7319,11 @@
       </c>
       <c r="P23" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>6348.4</v>
+        <v>641093.54999999923</v>
       </c>
       <c r="Q23" s="7">
         <f>O23-P23</f>
-        <v>703651.6</v>
+        <v>68906.450000000768</v>
       </c>
       <c r="R23" s="4"/>
       <c r="S23" s="17" t="s">
@@ -7364,12 +7337,12 @@
         <v>20</v>
       </c>
       <c r="V23" s="17">
-        <f ca="1">VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
-        <v>20</v>
+        <f>VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
+        <v>28</v>
       </c>
       <c r="W23" s="17">
-        <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <f t="shared" si="1"/>
+        <v>-8</v>
       </c>
     </row>
     <row r="24" spans="1:43" x14ac:dyDescent="0.25">
@@ -7385,11 +7358,11 @@
       </c>
       <c r="D24" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>43855.759999999995</v>
+        <v>126001.7799999999</v>
       </c>
       <c r="E24" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>101144.24</v>
+        <v>18998.220000000103</v>
       </c>
       <c r="F24" s="4"/>
       <c r="G24" s="18" t="s">
@@ -7400,15 +7373,15 @@
       </c>
       <c r="I24" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>10460</v>
+        <v>4310</v>
       </c>
       <c r="J24" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>3039</v>
+        <v>6480.75</v>
       </c>
       <c r="K24" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>7421</v>
+        <v>-2170.75</v>
       </c>
       <c r="L24" s="4"/>
       <c r="M24" s="4"/>
@@ -7421,11 +7394,11 @@
       </c>
       <c r="P24" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>0</v>
+        <v>796848.35999999952</v>
       </c>
       <c r="Q24" s="7">
         <f>O24-P24</f>
-        <v>710000</v>
+        <v>-86848.35999999952</v>
       </c>
       <c r="R24" s="4"/>
       <c r="S24" s="17" t="s">
@@ -7439,12 +7412,12 @@
         <v>20</v>
       </c>
       <c r="V24" s="17">
-        <f ca="1">VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
-        <v>9</v>
+        <f>VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
+        <v>20</v>
       </c>
       <c r="W24" s="17">
-        <f t="shared" ca="1" si="1"/>
-        <v>11</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:43" x14ac:dyDescent="0.25">
@@ -7460,11 +7433,11 @@
       </c>
       <c r="D25" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>45658.210000000028</v>
+        <v>140208.75999999949</v>
       </c>
       <c r="E25" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>101341.78999999998</v>
+        <v>6791.2400000005146</v>
       </c>
       <c r="F25" s="4"/>
       <c r="G25" s="18" t="s">
@@ -7475,15 +7448,15 @@
       </c>
       <c r="I25" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>13350</v>
+        <v>5620</v>
       </c>
       <c r="J25" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1518.5800000000002</v>
+        <v>8027.9999999999991</v>
       </c>
       <c r="K25" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>11831.42</v>
+        <v>-2407.9999999999991</v>
       </c>
       <c r="L25" s="4"/>
       <c r="M25" s="4"/>
@@ -7496,11 +7469,11 @@
       </c>
       <c r="P25" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>0</v>
+        <v>87468.710000000021</v>
       </c>
       <c r="Q25" s="7">
         <f>O25-P25</f>
-        <v>426000</v>
+        <v>338531.29</v>
       </c>
       <c r="R25" s="4"/>
       <c r="S25" s="17" t="s">
@@ -7514,12 +7487,12 @@
         <v>20</v>
       </c>
       <c r="V25" s="17">
-        <f ca="1">VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
-        <v>6</v>
+        <f>VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
+        <v>20</v>
       </c>
       <c r="W25" s="17">
-        <f t="shared" ca="1" si="1"/>
-        <v>14</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:43" x14ac:dyDescent="0.25">
@@ -7535,11 +7508,11 @@
       </c>
       <c r="D26" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>29544.7</v>
+        <v>67490.080000000045</v>
       </c>
       <c r="E26" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>50455.3</v>
+        <v>12509.919999999955</v>
       </c>
       <c r="F26" s="4"/>
       <c r="G26" s="18" t="s">
@@ -7550,15 +7523,15 @@
       </c>
       <c r="I26" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>6100</v>
+        <v>3650</v>
       </c>
       <c r="J26" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1399.22</v>
+        <v>7277.4499999999989</v>
       </c>
       <c r="K26" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>4700.78</v>
+        <v>-3627.4499999999989</v>
       </c>
       <c r="L26" s="4"/>
       <c r="M26" s="4"/>
@@ -7578,12 +7551,12 @@
         <v>20</v>
       </c>
       <c r="V26" s="17">
-        <f ca="1">VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
-        <v>11</v>
+        <f>VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0)</f>
+        <v>28</v>
       </c>
       <c r="W26" s="17">
-        <f t="shared" ca="1" si="1"/>
-        <v>9</v>
+        <f t="shared" si="1"/>
+        <v>-8</v>
       </c>
     </row>
     <row r="27" spans="1:43" x14ac:dyDescent="0.25">
@@ -7599,11 +7572,11 @@
       </c>
       <c r="D27" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>96164.2</v>
+        <v>233973.21999999901</v>
       </c>
       <c r="E27" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>148835.79999999999</v>
+        <v>11026.780000000988</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="18" t="s">
@@ -7614,15 +7587,15 @@
       </c>
       <c r="I27" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],[1]!Tabela1[VENDEDOR],[1]!Tabela1[VALOR])</f>
-        <v>5240</v>
+        <v>6670</v>
       </c>
       <c r="J27" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>3806.4000000000005</v>
+        <v>4561.2000000000007</v>
       </c>
       <c r="K27" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>1433.5999999999995</v>
+        <v>2108.7999999999993</v>
       </c>
       <c r="L27" s="4"/>
       <c r="M27" s="4"/>
@@ -7645,11 +7618,11 @@
       </c>
       <c r="D28" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>125560.12500000007</v>
+        <v>304475.37500000017</v>
       </c>
       <c r="E28" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>200939.87499999994</v>
+        <v>22024.624999999825</v>
       </c>
       <c r="F28" s="4"/>
       <c r="L28" s="4"/>
@@ -7724,11 +7697,11 @@
       </c>
       <c r="D30" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>40663.720000000038</v>
+        <v>112939.21999999965</v>
       </c>
       <c r="E30" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>101336.27999999997</v>
+        <v>29060.780000000348</v>
       </c>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
@@ -7761,11 +7734,11 @@
       </c>
       <c r="V30" s="5">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE 2]",'[1]BASE PYTHON'!$P$83,"[Intervalo 3].[SEMANAL]","[Intervalo 3].[SEMANAL].&amp;[1]"),0)</f>
-        <v>160</v>
+        <v>209</v>
       </c>
       <c r="W30" s="6">
         <f>U30-V30</f>
-        <v>-95.238095238095241</v>
+        <v>-144.23809523809524</v>
       </c>
     </row>
     <row r="31" spans="1:43" x14ac:dyDescent="0.25">
@@ -7781,11 +7754,11 @@
       </c>
       <c r="D31" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>68771.89</v>
+        <v>173369.35999999978</v>
       </c>
       <c r="E31" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>101228.11</v>
+        <v>-3369.3599999997823</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
@@ -7798,11 +7771,11 @@
       </c>
       <c r="J31" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[1]"),0)</f>
-        <v>415588.02000000159</v>
+        <v>415312.13000000152</v>
       </c>
       <c r="K31" s="7">
         <f>I31-J31</f>
-        <v>140507.21809523652</v>
+        <v>140783.10809523659</v>
       </c>
       <c r="L31" s="4"/>
       <c r="M31" s="4"/>
@@ -7821,11 +7794,11 @@
       </c>
       <c r="V31" s="5">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE 2]",'[1]BASE PYTHON'!$P$83,"[Intervalo 3].[SEMANAL]","[Intervalo 3].[SEMANAL].&amp;[2]"),0)</f>
-        <v>76</v>
+        <v>132</v>
       </c>
       <c r="W31" s="6">
         <f t="shared" ref="W31:W33" si="2">U31-V31</f>
-        <v>-11.238095238095241</v>
+        <v>-67.238095238095241</v>
       </c>
     </row>
     <row r="32" spans="1:43" x14ac:dyDescent="0.25">
@@ -7841,11 +7814,11 @@
       </c>
       <c r="D32" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>100639.89999999994</v>
+        <v>244477.96999999936</v>
       </c>
       <c r="E32" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>164360.10000000006</v>
+        <v>20522.030000000639</v>
       </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
@@ -7858,11 +7831,11 @@
       </c>
       <c r="J32" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>546956.19000000309</v>
+        <v>545254.94000000297</v>
       </c>
       <c r="K32" s="7">
         <f t="shared" ref="K32:K34" si="3">I32-J32</f>
-        <v>9139.048095235019</v>
+        <v>10840.298095235135</v>
       </c>
       <c r="L32" s="4"/>
       <c r="M32" s="4"/>
@@ -7881,11 +7854,11 @@
       </c>
       <c r="V32" s="5">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE 2]",'[1]BASE PYTHON'!$P$83,"[Intervalo 3].[SEMANAL]","[Intervalo 3].[SEMANAL].&amp;[3]"),0)</f>
-        <v>0</v>
+        <v>86</v>
       </c>
       <c r="W32" s="6">
         <f t="shared" si="2"/>
-        <v>80.952380952380949</v>
+        <v>-5.047619047619051</v>
       </c>
     </row>
     <row r="33" spans="1:23" x14ac:dyDescent="0.25">
@@ -7901,11 +7874,11 @@
       </c>
       <c r="D33" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>27935.73000000001</v>
+        <v>75978.280000000057</v>
       </c>
       <c r="E33" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>57064.26999999999</v>
+        <v>9021.719999999943</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -7918,11 +7891,11 @@
       </c>
       <c r="J33" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>20885.819999999996</v>
+        <v>648237.12000000419</v>
       </c>
       <c r="K33" s="7">
         <f t="shared" si="3"/>
-        <v>674233.22761904763</v>
+        <v>46881.927619043388</v>
       </c>
       <c r="L33" s="4"/>
       <c r="M33" s="4"/>
@@ -7941,11 +7914,11 @@
       </c>
       <c r="V33" s="5">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE 2]",'[1]BASE PYTHON'!$P$83,"[Intervalo 3].[SEMANAL]","[Intervalo 3].[SEMANAL].&amp;[4]"),0)</f>
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="W33" s="6">
         <f t="shared" si="2"/>
-        <v>80.952380952380949</v>
+        <v>54.952380952380949</v>
       </c>
     </row>
     <row r="34" spans="1:23" x14ac:dyDescent="0.25">
@@ -7961,11 +7934,11 @@
       </c>
       <c r="D34" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>21675.470000000005</v>
+        <v>56813.940000000111</v>
       </c>
       <c r="E34" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>33324.53</v>
+        <v>-1813.9400000001115</v>
       </c>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
@@ -7978,11 +7951,11 @@
       </c>
       <c r="J34" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>0</v>
+        <v>659752.69500000682</v>
       </c>
       <c r="K34" s="7">
         <f t="shared" si="3"/>
-        <v>695119.04761904757</v>
+        <v>35366.352619040757</v>
       </c>
       <c r="L34" s="4"/>
       <c r="M34" s="4"/>
@@ -8001,11 +7974,11 @@
       </c>
       <c r="V34" s="5">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE 2]",'[1]BASE PYTHON'!$P$83,"[Intervalo 3].[SEMANAL]","[Intervalo 3].[SEMANAL].&amp;[5]"),0)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="W34" s="6">
         <f>U34-V34</f>
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="35" spans="1:23" x14ac:dyDescent="0.25">
@@ -8021,11 +7994,11 @@
       </c>
       <c r="D35" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>28037.200000000004</v>
+        <v>65317.66</v>
       </c>
       <c r="E35" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>48462.799999999996</v>
+        <v>11182.339999999997</v>
       </c>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
@@ -8038,11 +8011,11 @@
       </c>
       <c r="J35" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>0</v>
+        <v>224319.64999999956</v>
       </c>
       <c r="K35" s="7">
         <f>I35-J35</f>
-        <v>417071.42857142858</v>
+        <v>192751.77857142902</v>
       </c>
       <c r="L35" s="4"/>
       <c r="M35" s="4"/>
@@ -8070,11 +8043,11 @@
       </c>
       <c r="D36" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>144.9</v>
+        <v>1003.86</v>
       </c>
       <c r="E36" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>855.1</v>
+        <v>-3.8600000000000136</v>
       </c>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
@@ -8181,11 +8154,11 @@
       </c>
       <c r="D40" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[1]"),0)</f>
-        <v>617038.34000000393</v>
+        <v>616762.45000000391</v>
       </c>
       <c r="E40" s="7">
         <f>C40-D40</f>
-        <v>507247.37428571039</v>
+        <v>507523.26428571041</v>
       </c>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
@@ -8217,11 +8190,11 @@
       </c>
       <c r="D41" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>1319100.4349999954</v>
+        <v>1291382.8849999958</v>
       </c>
       <c r="E41" s="7">
         <f t="shared" ref="E41:E43" si="4">C41-D41</f>
-        <v>-194814.72071428108</v>
+        <v>-167097.1707142815</v>
       </c>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
@@ -8253,11 +8226,11 @@
       </c>
       <c r="D42" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
-        <v>27234.22</v>
+        <v>1327217.3399999917</v>
       </c>
       <c r="E42" s="7">
         <f t="shared" si="4"/>
-        <v>1378122.922857143</v>
+        <v>78139.802857151255</v>
       </c>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>
@@ -8289,11 +8262,11 @@
       </c>
       <c r="D43" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
-        <v>0</v>
+        <v>1515744.6649999928</v>
       </c>
       <c r="E43" s="7">
         <f t="shared" si="4"/>
-        <v>1405357.142857143</v>
+        <v>-110387.52214284986</v>
       </c>
     </row>
     <row r="44" spans="1:23" x14ac:dyDescent="0.25">
@@ -8307,11 +8280,11 @@
       </c>
       <c r="D44" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
-        <v>0</v>
+        <v>323231.88000000117</v>
       </c>
       <c r="E44" s="7">
         <f t="shared" ref="E44" si="5">C44-D44</f>
-        <v>843214.28571428568</v>
+        <v>519982.40571428451</v>
       </c>
     </row>
     <row r="45" spans="1:23" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Dados atualizados em 06/10/2026 11:42
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E88B4DB-0F4F-464A-8DB8-CE7A878F491F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48D2EF07-B315-48A9-9137-09EAAA0D77E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -705,40 +705,6 @@
   <dxfs count="118">
     <dxf>
       <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="7" tint="0.39997558519241921"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -1914,6 +1880,40 @@
       </fill>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="7" tint="0.39997558519241921"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
         <left/>
         <right/>
         <top style="thin">
@@ -2511,10 +2511,10 @@
             <v>POSITIVACAO PAO DA FAZENDA</v>
           </cell>
           <cell r="L1">
-            <v>4</v>
+            <v>3</v>
           </cell>
           <cell r="M1">
-            <v>118</v>
+            <v>0</v>
           </cell>
         </row>
         <row r="2">
@@ -2573,13 +2573,13 @@
             <v>CAMPINAS</v>
           </cell>
           <cell r="F5">
-            <v>4765.8999999999996</v>
+            <v>4765.8499999999995</v>
           </cell>
           <cell r="H5" t="str">
             <v>CAMPINAS</v>
           </cell>
           <cell r="I5">
-            <v>3066.15</v>
+            <v>3066.1000000000004</v>
           </cell>
         </row>
         <row r="6">
@@ -2587,7 +2587,7 @@
             <v>CENTRO</v>
           </cell>
           <cell r="F6">
-            <v>59621.760000000031</v>
+            <v>59621.690000000039</v>
           </cell>
           <cell r="H6" t="str">
             <v>CENTRO</v>
@@ -2604,16 +2604,16 @@
         </row>
         <row r="7">
           <cell r="E7" t="str">
-            <v>IATAGAM JUNIOR</v>
+            <v>INDAIATUBA</v>
           </cell>
           <cell r="F7">
-            <v>0.1</v>
+            <v>10293.539999999999</v>
           </cell>
           <cell r="H7" t="str">
-            <v>IATAGAM JUNIOR</v>
+            <v>INDAIATUBA</v>
           </cell>
           <cell r="I7">
-            <v>0.1</v>
+            <v>8426.4</v>
           </cell>
           <cell r="K7" t="str">
             <v>Rótulos de Linha</v>
@@ -2622,50 +2622,44 @@
             <v>ACUMULADO</v>
           </cell>
           <cell r="M7" t="str">
-            <v>DIA</v>
-          </cell>
-          <cell r="N7" t="str">
             <v>Total Geral</v>
           </cell>
         </row>
         <row r="8">
           <cell r="E8" t="str">
-            <v>INDAIATUBA</v>
+            <v>INTERLAGOS</v>
           </cell>
           <cell r="F8">
-            <v>10293.6</v>
+            <v>32988.290000000023</v>
           </cell>
           <cell r="H8" t="str">
-            <v>INDAIATUBA</v>
+            <v>INTERLAGOS</v>
           </cell>
           <cell r="I8">
-            <v>8426.4499999999989</v>
+            <v>19596.890000000007</v>
           </cell>
           <cell r="K8" t="str">
             <v>INTERLAGOS</v>
           </cell>
           <cell r="L8">
-            <v>2</v>
+            <v>7</v>
           </cell>
           <cell r="M8">
-            <v>3</v>
-          </cell>
-          <cell r="N8">
-            <v>5</v>
+            <v>7</v>
           </cell>
         </row>
         <row r="9">
           <cell r="E9" t="str">
-            <v>INTERLAGOS</v>
+            <v>JUNDIAI</v>
           </cell>
           <cell r="F9">
-            <v>31839.209999999995</v>
+            <v>12263.809999999998</v>
           </cell>
           <cell r="H9" t="str">
-            <v>INTERLAGOS</v>
+            <v>JUNDIAI</v>
           </cell>
           <cell r="I9">
-            <v>18447.749999999985</v>
+            <v>4585.25</v>
           </cell>
           <cell r="K9" t="str">
             <v>JUNDIAI</v>
@@ -2673,367 +2667,343 @@
           <cell r="L9">
             <v>1</v>
           </cell>
-          <cell r="N9">
+          <cell r="M9">
             <v>1</v>
           </cell>
         </row>
         <row r="10">
           <cell r="E10" t="str">
-            <v>JUNDIAI</v>
+            <v>KEY ABC</v>
           </cell>
           <cell r="F10">
-            <v>11111.86</v>
+            <v>2016.6</v>
           </cell>
           <cell r="H10" t="str">
-            <v>JUNDIAI</v>
+            <v>KEY ABC</v>
           </cell>
           <cell r="I10">
-            <v>3433.25</v>
+            <v>0</v>
           </cell>
           <cell r="K10" t="str">
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="L10">
-            <v>2</v>
+            <v>4</v>
           </cell>
           <cell r="M10">
-            <v>2</v>
-          </cell>
-          <cell r="N10">
             <v>4</v>
           </cell>
         </row>
         <row r="11">
           <cell r="E11" t="str">
-            <v>KEY ABC</v>
+            <v>KEY CASA</v>
           </cell>
           <cell r="F11">
-            <v>2017.1999999999998</v>
+            <v>63215.649999999965</v>
           </cell>
           <cell r="H11" t="str">
-            <v>KEY ABC</v>
+            <v>KEY CASA</v>
           </cell>
           <cell r="I11">
-            <v>0.6</v>
+            <v>59732.449999999968</v>
           </cell>
           <cell r="K11" t="str">
             <v>OSASCO</v>
           </cell>
           <cell r="L11">
-            <v>5</v>
+            <v>11</v>
           </cell>
           <cell r="M11">
-            <v>6</v>
-          </cell>
-          <cell r="N11">
             <v>11</v>
           </cell>
         </row>
         <row r="12">
           <cell r="E12" t="str">
-            <v>KEY CASA</v>
+            <v>KEY INTERIOR</v>
           </cell>
           <cell r="F12">
-            <v>12150</v>
+            <v>94941.200000000012</v>
           </cell>
           <cell r="H12" t="str">
-            <v>KEY CASA</v>
+            <v>KEY INTERIOR</v>
           </cell>
           <cell r="I12">
-            <v>8666.7999999999993</v>
+            <v>87269.200000000012</v>
           </cell>
           <cell r="K12" t="str">
             <v>PIRITUBA</v>
           </cell>
+          <cell r="L12">
+            <v>2</v>
+          </cell>
           <cell r="M12">
-            <v>1</v>
-          </cell>
-          <cell r="N12">
-            <v>1</v>
+            <v>2</v>
           </cell>
         </row>
         <row r="13">
           <cell r="E13" t="str">
-            <v>KEY INTERIOR</v>
+            <v>KEY SJC</v>
           </cell>
           <cell r="F13">
-            <v>7672</v>
+            <v>4315.6000000000004</v>
           </cell>
           <cell r="H13" t="str">
-            <v>KEY INTERIOR</v>
+            <v>KEY SJC</v>
           </cell>
           <cell r="I13">
-            <v>0</v>
+            <v>4315.6000000000004</v>
           </cell>
           <cell r="K13" t="str">
             <v>SANTO ANDRE</v>
           </cell>
+          <cell r="L13">
+            <v>2</v>
+          </cell>
           <cell r="M13">
             <v>2</v>
           </cell>
-          <cell r="N13">
-            <v>2</v>
-          </cell>
         </row>
         <row r="14">
           <cell r="E14" t="str">
-            <v>KEY SJC</v>
+            <v>KEY SP</v>
           </cell>
           <cell r="F14">
-            <v>4315.6000000000004</v>
+            <v>15188.2</v>
           </cell>
           <cell r="H14" t="str">
-            <v>KEY SJC</v>
+            <v>KEY SP</v>
           </cell>
           <cell r="I14">
-            <v>4315.6000000000004</v>
+            <v>13814.5</v>
           </cell>
           <cell r="K14" t="str">
             <v>SBC</v>
           </cell>
           <cell r="L14">
-            <v>2</v>
+            <v>4</v>
           </cell>
           <cell r="M14">
-            <v>2</v>
-          </cell>
-          <cell r="N14">
             <v>4</v>
           </cell>
         </row>
         <row r="15">
           <cell r="E15" t="str">
-            <v>KEY SP</v>
+            <v>KEY ZL</v>
           </cell>
           <cell r="F15">
-            <v>15188.2</v>
+            <v>40356.879999999961</v>
           </cell>
           <cell r="H15" t="str">
-            <v>KEY SP</v>
+            <v>KEY ZL</v>
           </cell>
           <cell r="I15">
-            <v>13814.5</v>
+            <v>34294.479999999967</v>
           </cell>
           <cell r="K15" t="str">
             <v>SJC</v>
           </cell>
+          <cell r="L15">
+            <v>1</v>
+          </cell>
           <cell r="M15">
             <v>1</v>
           </cell>
-          <cell r="N15">
-            <v>1</v>
-          </cell>
         </row>
         <row r="16">
           <cell r="E16" t="str">
-            <v>KEY ZL</v>
+            <v>LESTE MOOCA</v>
           </cell>
           <cell r="F16">
-            <v>40356.879999999961</v>
+            <v>20123.86</v>
           </cell>
           <cell r="H16" t="str">
-            <v>KEY ZL</v>
+            <v>LESTE MOOCA</v>
           </cell>
           <cell r="I16">
-            <v>34294.479999999967</v>
+            <v>13425.409999999993</v>
           </cell>
           <cell r="K16" t="str">
             <v>Total Geral</v>
           </cell>
           <cell r="L16">
-            <v>12</v>
+            <v>32</v>
           </cell>
           <cell r="M16">
-            <v>17</v>
-          </cell>
-          <cell r="N16">
-            <v>29</v>
+            <v>32</v>
           </cell>
         </row>
         <row r="17">
           <cell r="E17" t="str">
-            <v>LESTE MOOCA</v>
+            <v>LESTE PENHA</v>
           </cell>
           <cell r="F17">
-            <v>20124.039999999997</v>
+            <v>24013.079999999998</v>
           </cell>
           <cell r="H17" t="str">
-            <v>LESTE MOOCA</v>
+            <v>LESTE PENHA</v>
           </cell>
           <cell r="I17">
-            <v>13425.569999999992</v>
+            <v>14168.76</v>
           </cell>
         </row>
         <row r="18">
           <cell r="E18" t="str">
-            <v>LESTE PENHA</v>
+            <v>LESTE TATUAPE</v>
           </cell>
           <cell r="F18">
-            <v>24013.129999999997</v>
+            <v>14652.809999999996</v>
           </cell>
           <cell r="H18" t="str">
-            <v>LESTE PENHA</v>
+            <v>LESTE TATUAPE</v>
           </cell>
           <cell r="I18">
-            <v>14168.78</v>
+            <v>12159.649999999998</v>
           </cell>
         </row>
         <row r="19">
           <cell r="E19" t="str">
-            <v>LESTE TATUAPE</v>
+            <v>MOGI</v>
           </cell>
           <cell r="F19">
-            <v>12662.729999999998</v>
+            <v>5238.87</v>
           </cell>
           <cell r="H19" t="str">
-            <v>LESTE TATUAPE</v>
+            <v>MOGI</v>
           </cell>
           <cell r="I19">
-            <v>10169.540000000001</v>
+            <v>4213.3100000000004</v>
           </cell>
         </row>
         <row r="20">
           <cell r="E20" t="str">
-            <v>MOGI</v>
+            <v>NORTE</v>
           </cell>
           <cell r="F20">
-            <v>3489.02</v>
+            <v>37419.070000000022</v>
           </cell>
           <cell r="H20" t="str">
-            <v>MOGI</v>
+            <v>NORTE</v>
           </cell>
           <cell r="I20">
-            <v>2463.46</v>
+            <v>23646.760000000002</v>
           </cell>
         </row>
         <row r="21">
           <cell r="E21" t="str">
-            <v>NORTE</v>
+            <v>OSASCO</v>
           </cell>
           <cell r="F21">
-            <v>37419.410000000025</v>
+            <v>52714.41</v>
           </cell>
           <cell r="H21" t="str">
-            <v>NORTE</v>
+            <v>OSASCO</v>
           </cell>
           <cell r="I21">
-            <v>23647.030000000006</v>
+            <v>28873.46000000001</v>
           </cell>
         </row>
         <row r="22">
           <cell r="E22" t="str">
-            <v>OSASCO</v>
+            <v>PIRITUBA</v>
           </cell>
           <cell r="F22">
-            <v>52714.710000000036</v>
+            <v>16296.58</v>
           </cell>
           <cell r="H22" t="str">
-            <v>OSASCO</v>
+            <v>PIRITUBA</v>
           </cell>
           <cell r="I22">
-            <v>28873.699999999993</v>
+            <v>10320.560000000003</v>
           </cell>
         </row>
         <row r="23">
           <cell r="E23" t="str">
-            <v>PIRITUBA</v>
+            <v>SANTO ANDRE</v>
           </cell>
           <cell r="F23">
-            <v>15519.85</v>
+            <v>20419.93</v>
           </cell>
           <cell r="H23" t="str">
-            <v>PIRITUBA</v>
+            <v>SANTO ANDRE</v>
           </cell>
           <cell r="I23">
-            <v>9543.8000000000011</v>
+            <v>16407.95</v>
           </cell>
         </row>
         <row r="24">
           <cell r="E24" t="str">
-            <v>SANTO ANDRE</v>
+            <v>SBC</v>
           </cell>
           <cell r="F24">
-            <v>20117.779999999992</v>
+            <v>32294.379999999983</v>
           </cell>
           <cell r="H24" t="str">
-            <v>SANTO ANDRE</v>
+            <v>SBC</v>
           </cell>
           <cell r="I24">
-            <v>16105.800000000005</v>
+            <v>13145.080000000002</v>
           </cell>
         </row>
         <row r="25">
           <cell r="E25" t="str">
-            <v>SBC</v>
+            <v>SJC</v>
           </cell>
           <cell r="F25">
-            <v>32294.459999999985</v>
+            <v>13559.139999999998</v>
           </cell>
           <cell r="H25" t="str">
-            <v>SBC</v>
+            <v>SJC</v>
           </cell>
           <cell r="I25">
-            <v>13145.130000000003</v>
+            <v>10532.269999999999</v>
           </cell>
         </row>
         <row r="26">
           <cell r="E26" t="str">
-            <v>SJC</v>
+            <v>SJC/VALE</v>
           </cell>
           <cell r="F26">
-            <v>12237.629999999997</v>
+            <v>7270.8299999999963</v>
           </cell>
           <cell r="H26" t="str">
-            <v>SJC</v>
+            <v>SJC/VALE</v>
           </cell>
           <cell r="I26">
-            <v>9210.7599999999984</v>
+            <v>4425.9999999999991</v>
           </cell>
         </row>
         <row r="27">
           <cell r="E27" t="str">
-            <v>SJC/VALE</v>
+            <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="F27">
-            <v>6469.4299999999976</v>
+            <v>9212.1200000000008</v>
           </cell>
           <cell r="H27" t="str">
-            <v>SJC/VALE</v>
+            <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="I27">
-            <v>3624.6000000000004</v>
+            <v>8884.1</v>
           </cell>
         </row>
         <row r="28">
           <cell r="E28" t="str">
-            <v>VENDEDOR INTERNO 1</v>
+            <v>Total Geral</v>
           </cell>
           <cell r="F28">
-            <v>8237.1200000000008</v>
+            <v>593182.38999999885</v>
           </cell>
           <cell r="H28" t="str">
-            <v>VENDEDOR INTERNO 1</v>
+            <v>Total Geral</v>
           </cell>
           <cell r="I28">
-            <v>7909.1</v>
+            <v>429012.9099999998</v>
           </cell>
           <cell r="K28" t="str">
             <v>POSITIVAÇÃO GERAL</v>
           </cell>
         </row>
         <row r="29">
-          <cell r="E29" t="str">
-            <v>Total Geral</v>
-          </cell>
-          <cell r="F29">
-            <v>444631.62000000151</v>
-          </cell>
-          <cell r="H29" t="str">
-            <v>Total Geral</v>
-          </cell>
-          <cell r="I29">
-            <v>280461.68000000069</v>
-          </cell>
           <cell r="K29" t="str">
             <v>DATA</v>
           </cell>
@@ -3068,9 +3038,6 @@
             <v>ACUMULADO</v>
           </cell>
           <cell r="M33" t="str">
-            <v>DIA</v>
-          </cell>
-          <cell r="N33" t="str">
             <v>Total Geral</v>
           </cell>
         </row>
@@ -3079,13 +3046,10 @@
             <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="L34">
-            <v>3</v>
+            <v>33</v>
           </cell>
           <cell r="M34">
-            <v>27</v>
-          </cell>
-          <cell r="N34">
-            <v>30</v>
+            <v>33</v>
           </cell>
         </row>
         <row r="35">
@@ -3093,13 +3057,10 @@
             <v>Total Geral</v>
           </cell>
           <cell r="L35">
-            <v>3</v>
+            <v>33</v>
           </cell>
           <cell r="M35">
-            <v>27</v>
-          </cell>
-          <cell r="N35">
-            <v>30</v>
+            <v>33</v>
           </cell>
         </row>
         <row r="39">
@@ -3107,7 +3068,7 @@
             <v>CAMPINAS</v>
           </cell>
           <cell r="B39">
-            <v>6810</v>
+            <v>4820</v>
           </cell>
         </row>
         <row r="40">
@@ -3115,7 +3076,7 @@
             <v>CENTRO</v>
           </cell>
           <cell r="B40">
-            <v>32180</v>
+            <v>25020</v>
           </cell>
         </row>
         <row r="41">
@@ -3123,7 +3084,7 @@
             <v>INDAIATUBA</v>
           </cell>
           <cell r="B41">
-            <v>15240</v>
+            <v>6580</v>
           </cell>
         </row>
         <row r="42">
@@ -3131,7 +3092,7 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="B42">
-            <v>25860</v>
+            <v>17000</v>
           </cell>
         </row>
         <row r="43">
@@ -3139,7 +3100,7 @@
             <v>JUNDIAI</v>
           </cell>
           <cell r="B43">
-            <v>4890</v>
+            <v>5990</v>
           </cell>
         </row>
         <row r="44">
@@ -3147,7 +3108,7 @@
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="B44">
-            <v>18810</v>
+            <v>18340</v>
           </cell>
         </row>
         <row r="45">
@@ -3155,7 +3116,7 @@
             <v>LESTE PENHA</v>
           </cell>
           <cell r="B45">
-            <v>21810</v>
+            <v>9950</v>
           </cell>
         </row>
         <row r="46">
@@ -3163,7 +3124,7 @@
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="B46">
-            <v>19910</v>
+            <v>16120</v>
           </cell>
         </row>
         <row r="47">
@@ -3171,7 +3132,7 @@
             <v>MOGI</v>
           </cell>
           <cell r="B47">
-            <v>10200</v>
+            <v>4590</v>
           </cell>
           <cell r="P47" t="str">
             <v>Soma de TOTAL</v>
@@ -3182,7 +3143,7 @@
             <v>NORTE</v>
           </cell>
           <cell r="B48">
-            <v>25040</v>
+            <v>13060</v>
           </cell>
         </row>
         <row r="49">
@@ -3190,7 +3151,7 @@
             <v>OSASCO</v>
           </cell>
           <cell r="B49">
-            <v>27520</v>
+            <v>20980</v>
           </cell>
         </row>
         <row r="50">
@@ -3198,7 +3159,7 @@
             <v>PIRITUBA</v>
           </cell>
           <cell r="B50">
-            <v>15210</v>
+            <v>9390</v>
           </cell>
         </row>
         <row r="51">
@@ -3206,7 +3167,7 @@
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="B51">
-            <v>17760</v>
+            <v>13880</v>
           </cell>
         </row>
         <row r="52">
@@ -3214,7 +3175,7 @@
             <v>SBC</v>
           </cell>
           <cell r="B52">
-            <v>23160</v>
+            <v>19350</v>
           </cell>
         </row>
         <row r="53">
@@ -3222,7 +3183,7 @@
             <v>SJC</v>
           </cell>
           <cell r="B53">
-            <v>15120</v>
+            <v>5850</v>
           </cell>
         </row>
         <row r="54">
@@ -3230,7 +3191,7 @@
             <v>SJC/VALE</v>
           </cell>
           <cell r="B54">
-            <v>8690</v>
+            <v>3770</v>
           </cell>
         </row>
         <row r="55">
@@ -3238,7 +3199,7 @@
             <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="B55">
-            <v>12050</v>
+            <v>5530</v>
           </cell>
         </row>
         <row r="63">
@@ -3423,13 +3384,13 @@
             <v>36</v>
           </cell>
           <cell r="F137">
-            <v>30</v>
+            <v>33</v>
           </cell>
           <cell r="H137" t="str">
             <v>D</v>
           </cell>
           <cell r="I137">
-            <v>6</v>
+            <v>3</v>
           </cell>
         </row>
         <row r="138">
@@ -3465,13 +3426,13 @@
             <v>14</v>
           </cell>
           <cell r="F140">
-            <v>5</v>
+            <v>7</v>
           </cell>
           <cell r="H140" t="str">
             <v>D</v>
           </cell>
           <cell r="I140">
-            <v>9</v>
+            <v>7</v>
           </cell>
         </row>
         <row r="141">
@@ -3591,13 +3552,13 @@
             <v>14</v>
           </cell>
           <cell r="F149">
-            <v>1</v>
+            <v>2</v>
           </cell>
           <cell r="H149" t="str">
             <v>D</v>
           </cell>
           <cell r="I149">
-            <v>13</v>
+            <v>12</v>
           </cell>
         </row>
         <row r="150">
@@ -3686,13 +3647,13 @@
             <v>39600</v>
           </cell>
           <cell r="F159">
-            <v>12237.629999999997</v>
+            <v>13559.139999999998</v>
           </cell>
           <cell r="H159" t="str">
             <v>D</v>
           </cell>
           <cell r="I159">
-            <v>27362.370000000003</v>
+            <v>26040.86</v>
           </cell>
         </row>
         <row r="160">
@@ -3700,13 +3661,13 @@
             <v>35550</v>
           </cell>
           <cell r="F160">
-            <v>8237.1200000000008</v>
+            <v>9212.1200000000008</v>
           </cell>
           <cell r="H160" t="str">
             <v>D</v>
           </cell>
           <cell r="I160">
-            <v>27312.879999999997</v>
+            <v>26337.879999999997</v>
           </cell>
         </row>
         <row r="161">
@@ -3714,13 +3675,13 @@
             <v>155250</v>
           </cell>
           <cell r="F161">
-            <v>59621.760000000031</v>
+            <v>59621.690000000039</v>
           </cell>
           <cell r="H161" t="str">
             <v>D</v>
           </cell>
           <cell r="I161">
-            <v>95628.239999999962</v>
+            <v>95628.309999999969</v>
           </cell>
         </row>
         <row r="162">
@@ -3728,13 +3689,13 @@
             <v>149175</v>
           </cell>
           <cell r="F162">
-            <v>52714.710000000036</v>
+            <v>52714.41</v>
           </cell>
           <cell r="H162" t="str">
             <v>D</v>
           </cell>
           <cell r="I162">
-            <v>96460.289999999964</v>
+            <v>96460.59</v>
           </cell>
         </row>
         <row r="163">
@@ -3742,13 +3703,13 @@
             <v>126450</v>
           </cell>
           <cell r="F163">
-            <v>31839.209999999995</v>
+            <v>32988.290000000023</v>
           </cell>
           <cell r="H163" t="str">
             <v>D</v>
           </cell>
           <cell r="I163">
-            <v>94610.790000000008</v>
+            <v>93461.709999999977</v>
           </cell>
         </row>
         <row r="164">
@@ -3756,13 +3717,13 @@
             <v>92700</v>
           </cell>
           <cell r="F164">
-            <v>20124.039999999997</v>
+            <v>20123.86</v>
           </cell>
           <cell r="H164" t="str">
             <v>D</v>
           </cell>
           <cell r="I164">
-            <v>72575.960000000006</v>
+            <v>72576.14</v>
           </cell>
         </row>
         <row r="165">
@@ -3770,13 +3731,13 @@
             <v>78750</v>
           </cell>
           <cell r="F165">
-            <v>20117.779999999992</v>
+            <v>20419.93</v>
           </cell>
           <cell r="H165" t="str">
             <v>D</v>
           </cell>
           <cell r="I165">
-            <v>58632.220000000008</v>
+            <v>58330.07</v>
           </cell>
         </row>
         <row r="166">
@@ -3784,13 +3745,13 @@
             <v>121131</v>
           </cell>
           <cell r="F166">
-            <v>37419.410000000025</v>
+            <v>37419.070000000022</v>
           </cell>
           <cell r="H166" t="str">
             <v>D</v>
           </cell>
           <cell r="I166">
-            <v>83711.589999999967</v>
+            <v>83711.929999999978</v>
           </cell>
         </row>
         <row r="167">
@@ -3812,13 +3773,13 @@
             <v>26100</v>
           </cell>
           <cell r="F168">
-            <v>6469.4299999999976</v>
+            <v>7270.8299999999963</v>
           </cell>
           <cell r="H168" t="str">
             <v>D</v>
           </cell>
           <cell r="I168">
-            <v>19630.570000000003</v>
+            <v>18829.170000000006</v>
           </cell>
         </row>
         <row r="169">
@@ -3826,13 +3787,13 @@
             <v>43200</v>
           </cell>
           <cell r="F169">
-            <v>10293.6</v>
+            <v>10293.539999999999</v>
           </cell>
           <cell r="H169" t="str">
             <v>D</v>
           </cell>
           <cell r="I169">
-            <v>32906.400000000001</v>
+            <v>32906.46</v>
           </cell>
         </row>
         <row r="170">
@@ -3840,13 +3801,13 @@
             <v>31725</v>
           </cell>
           <cell r="F170">
-            <v>4765.8999999999996</v>
+            <v>4765.8499999999995</v>
           </cell>
           <cell r="H170" t="str">
             <v>D</v>
           </cell>
           <cell r="I170">
-            <v>26959.1</v>
+            <v>26959.15</v>
           </cell>
         </row>
         <row r="171">
@@ -3854,13 +3815,13 @@
             <v>37800</v>
           </cell>
           <cell r="F171">
-            <v>11111.86</v>
+            <v>12263.809999999998</v>
           </cell>
           <cell r="H171" t="str">
             <v>D</v>
           </cell>
           <cell r="I171">
-            <v>26688.14</v>
+            <v>25536.190000000002</v>
           </cell>
         </row>
         <row r="172">
@@ -3868,13 +3829,13 @@
             <v>63900</v>
           </cell>
           <cell r="F172">
-            <v>15519.85</v>
+            <v>16296.58</v>
           </cell>
           <cell r="H172" t="str">
             <v>D</v>
           </cell>
           <cell r="I172">
-            <v>48380.15</v>
+            <v>47603.42</v>
           </cell>
         </row>
         <row r="173">
@@ -3882,13 +3843,13 @@
             <v>74970</v>
           </cell>
           <cell r="F173">
-            <v>24013.129999999997</v>
+            <v>24013.079999999998</v>
           </cell>
           <cell r="H173" t="str">
             <v>D</v>
           </cell>
           <cell r="I173">
-            <v>50956.87</v>
+            <v>50956.92</v>
           </cell>
         </row>
         <row r="174">
@@ -3896,13 +3857,13 @@
             <v>121500</v>
           </cell>
           <cell r="F174">
-            <v>32294.459999999985</v>
+            <v>32294.379999999983</v>
           </cell>
           <cell r="H174" t="str">
             <v>D</v>
           </cell>
           <cell r="I174">
-            <v>89205.540000000008</v>
+            <v>89205.620000000024</v>
           </cell>
         </row>
         <row r="175">
@@ -3910,13 +3871,13 @@
             <v>42975</v>
           </cell>
           <cell r="F175">
-            <v>3489.02</v>
+            <v>5238.87</v>
           </cell>
           <cell r="H175" t="str">
             <v>D</v>
           </cell>
           <cell r="I175">
-            <v>39485.980000000003</v>
+            <v>37736.129999999997</v>
           </cell>
         </row>
         <row r="176">
@@ -3924,13 +3885,13 @@
             <v>97875</v>
           </cell>
           <cell r="F176">
-            <v>12662.729999999998</v>
+            <v>14652.809999999996</v>
           </cell>
           <cell r="H176" t="str">
             <v>D</v>
           </cell>
           <cell r="I176">
-            <v>85212.27</v>
+            <v>83222.19</v>
           </cell>
         </row>
         <row r="177">
@@ -3938,10 +3899,10 @@
             <v>1338651</v>
           </cell>
           <cell r="F177">
-            <v>362931.64000000007</v>
+            <v>373148.26000000007</v>
           </cell>
           <cell r="I177">
-            <v>975719.36</v>
+            <v>965502.74</v>
           </cell>
         </row>
       </sheetData>
@@ -3975,18 +3936,18 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{E3745920-1197-4A81-B558-958DBAB19EA3}" name="Tabela5" displayName="Tabela5" ref="G9:K27" totalsRowShown="0" headerRowDxfId="58" dataDxfId="57" tableBorderDxfId="56">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{E3745920-1197-4A81-B558-958DBAB19EA3}" name="Tabela5" displayName="Tabela5" ref="G9:K27" totalsRowShown="0" headerRowDxfId="57" dataDxfId="56" tableBorderDxfId="55">
   <autoFilter ref="G9:K27" xr:uid="{E3745920-1197-4A81-B558-958DBAB19EA3}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{D324C7DB-F877-4A7E-BC26-EF8905C85433}" name="REFERENCIA" dataDxfId="55"/>
-    <tableColumn id="2" xr3:uid="{A71A6478-3B31-4F54-A10C-E6EC00E95E0B}" name="VENDEDOR" dataDxfId="54"/>
-    <tableColumn id="3" xr3:uid="{9F5EDCDD-D442-4FBE-9C74-26084F24EFCB}" name="COMPROMISSO" dataDxfId="53" dataCellStyle="Moeda">
+    <tableColumn id="1" xr3:uid="{D324C7DB-F877-4A7E-BC26-EF8905C85433}" name="REFERENCIA" dataDxfId="54"/>
+    <tableColumn id="2" xr3:uid="{A71A6478-3B31-4F54-A10C-E6EC00E95E0B}" name="VENDEDOR" dataDxfId="53"/>
+    <tableColumn id="3" xr3:uid="{9F5EDCDD-D442-4FBE-9C74-26084F24EFCB}" name="COMPROMISSO" dataDxfId="52" dataCellStyle="Moeda">
       <calculatedColumnFormula>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{2E4F9793-0E4B-42F0-B595-748F8481D0D0}" name="ATINGIDO" dataDxfId="52" dataCellStyle="Moeda">
+    <tableColumn id="4" xr3:uid="{2E4F9793-0E4B-42F0-B595-748F8481D0D0}" name="ATINGIDO" dataDxfId="51" dataCellStyle="Moeda">
       <calculatedColumnFormula>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{3CEFD09C-EF55-4119-A139-BD17682D2B73}" name="FALTA" dataDxfId="51">
+    <tableColumn id="5" xr3:uid="{3CEFD09C-EF55-4119-A139-BD17682D2B73}" name="FALTA" dataDxfId="50">
       <calculatedColumnFormula>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3995,7 +3956,7 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{3A7104A0-4D5E-4CED-9364-119005653576}" name="Tabela13" displayName="Tabela13" ref="A9:E36" headerRowDxfId="50" dataDxfId="49" totalsRowDxfId="47" tableBorderDxfId="48">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{3A7104A0-4D5E-4CED-9364-119005653576}" name="Tabela13" displayName="Tabela13" ref="A9:E36" headerRowDxfId="49" dataDxfId="48" totalsRowDxfId="46" tableBorderDxfId="47">
   <autoFilter ref="A9:E36" xr:uid="{3A7104A0-4D5E-4CED-9364-119005653576}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -4004,15 +3965,15 @@
     <filterColumn colId="4" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{50EE0FE5-ADD7-4A3A-9DF8-D52FFFCF08DA}" name="REFERENCIA" totalsRowLabel="Total" dataDxfId="46" totalsRowDxfId="45"/>
-    <tableColumn id="2" xr3:uid="{4F0BAF4D-D0FC-4B7C-8FF4-8DDD6505FDA1}" name="VENDEDOR" dataDxfId="44" totalsRowDxfId="43"/>
-    <tableColumn id="3" xr3:uid="{CCB341E8-8BC2-4209-AEA0-D6F26BFCB356}" name="META A" dataDxfId="42" totalsRowDxfId="41" dataCellStyle="Moeda">
+    <tableColumn id="1" xr3:uid="{50EE0FE5-ADD7-4A3A-9DF8-D52FFFCF08DA}" name="REFERENCIA" totalsRowLabel="Total" dataDxfId="45" totalsRowDxfId="44"/>
+    <tableColumn id="2" xr3:uid="{4F0BAF4D-D0FC-4B7C-8FF4-8DDD6505FDA1}" name="VENDEDOR" dataDxfId="43" totalsRowDxfId="42"/>
+    <tableColumn id="3" xr3:uid="{CCB341E8-8BC2-4209-AEA0-D6F26BFCB356}" name="META A" dataDxfId="41" totalsRowDxfId="40" dataCellStyle="Moeda">
       <calculatedColumnFormula>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],[1]!Tabela2[VENDEDOR],[1]!Tabela2[META A],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{9AA985E6-33FD-40FD-9473-5AF6B4D03030}" name="ATINGIDO" dataDxfId="40" totalsRowDxfId="39" dataCellStyle="Moeda">
+    <tableColumn id="4" xr3:uid="{9AA985E6-33FD-40FD-9473-5AF6B4D03030}" name="ATINGIDO" dataDxfId="39" totalsRowDxfId="38" dataCellStyle="Moeda">
       <calculatedColumnFormula>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{7B8A46E1-DE6F-44C0-A6C8-83887563A4C0}" name="FALTA" totalsRowFunction="sum" dataDxfId="38" totalsRowDxfId="37">
+    <tableColumn id="5" xr3:uid="{7B8A46E1-DE6F-44C0-A6C8-83887563A4C0}" name="FALTA" totalsRowFunction="sum" dataDxfId="37" totalsRowDxfId="36">
       <calculatedColumnFormula>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4021,32 +3982,32 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="16" xr:uid="{55BE7188-8888-41FA-ABCF-B57822EB82A5}" name="Tabela817" displayName="Tabela817" ref="AI2:AQ21" totalsRowCount="1" dataDxfId="36" dataCellStyle="Moeda">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="16" xr:uid="{55BE7188-8888-41FA-ABCF-B57822EB82A5}" name="Tabela817" displayName="Tabela817" ref="AI2:AQ21" totalsRowCount="1" dataDxfId="35" dataCellStyle="Moeda">
   <autoFilter ref="AI2:AQ20" xr:uid="{55BE7188-8888-41FA-ABCF-B57822EB82A5}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{9DC09787-B029-495D-ADCF-A6C94B8ED537}" name="VENDEDOR" totalsRowLabel="Total"/>
-    <tableColumn id="2" xr3:uid="{94315AF9-FE56-4F51-82DE-7907A99BB7DD}" name="META A" totalsRowFunction="sum" dataDxfId="35" totalsRowDxfId="34" dataCellStyle="Moeda">
+    <tableColumn id="2" xr3:uid="{94315AF9-FE56-4F51-82DE-7907A99BB7DD}" name="META A" totalsRowFunction="sum" dataDxfId="34" totalsRowDxfId="33" dataCellStyle="Moeda">
       <calculatedColumnFormula>_xlfn.XLOOKUP(Tabela817[[#This Row],[VENDEDOR]],[1]!Tabela8[VENDEDOR],[1]!Tabela8[META A])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{715CA431-D204-4F64-9916-9AE4C60EC6B9}" name="META B" totalsRowFunction="sum" dataDxfId="33" totalsRowDxfId="32" dataCellStyle="Moeda">
+    <tableColumn id="3" xr3:uid="{715CA431-D204-4F64-9916-9AE4C60EC6B9}" name="META B" totalsRowFunction="sum" dataDxfId="32" totalsRowDxfId="31" dataCellStyle="Moeda">
       <calculatedColumnFormula>_xlfn.XLOOKUP(Tabela817[[#This Row],[VENDEDOR]],[1]!Tabela8[VENDEDOR],[1]!Tabela8[META B])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{499A8278-63E6-4339-A908-FB77667C4F8A}" name="META C" totalsRowFunction="sum" dataDxfId="31" totalsRowDxfId="30" dataCellStyle="Moeda">
+    <tableColumn id="4" xr3:uid="{499A8278-63E6-4339-A908-FB77667C4F8A}" name="META C" totalsRowFunction="sum" dataDxfId="30" totalsRowDxfId="29" dataCellStyle="Moeda">
       <calculatedColumnFormula>_xlfn.XLOOKUP(Tabela817[[#This Row],[VENDEDOR]],[1]!Tabela8[VENDEDOR],[1]!Tabela8[META C])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{D02E4F6F-A83C-4A30-A474-49B37289EA09}" name="META D" totalsRowFunction="sum" dataDxfId="29" totalsRowDxfId="28" dataCellStyle="Moeda">
+    <tableColumn id="5" xr3:uid="{D02E4F6F-A83C-4A30-A474-49B37289EA09}" name="META D" totalsRowFunction="sum" dataDxfId="28" totalsRowDxfId="27" dataCellStyle="Moeda">
       <calculatedColumnFormula>_xlfn.XLOOKUP(Tabela817[[#This Row],[VENDEDOR]],[1]!Tabela8[VENDEDOR],[1]!Tabela8[META D])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{A6275BB8-634B-41DE-9C0C-38DE46A74438}" name="ATINGIDO" totalsRowFunction="sum" dataDxfId="27" totalsRowDxfId="26" dataCellStyle="Moeda">
+    <tableColumn id="6" xr3:uid="{A6275BB8-634B-41DE-9C0C-38DE46A74438}" name="ATINGIDO" totalsRowFunction="sum" dataDxfId="26" totalsRowDxfId="25" dataCellStyle="Moeda">
       <calculatedColumnFormula>IFERROR(_xlfn.XLOOKUP(AI3,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{7C64A4D6-2D58-41F0-866B-9B1CB6514952}" name="PREMIAÇÃO ATINGIDA" dataDxfId="25" totalsRowDxfId="24">
+    <tableColumn id="7" xr3:uid="{7C64A4D6-2D58-41F0-866B-9B1CB6514952}" name="PREMIAÇÃO ATINGIDA" dataDxfId="24" totalsRowDxfId="23">
       <calculatedColumnFormula array="1">_xlfn.IFS(AN3&gt;=AJ3,"A",AN3&gt;=AK3,"B",AN3&gt;=AL3,"C",AN3&gt;=AM3,"D",TRUE,"NÃO ATINGIDO")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{A4232C53-895F-4F8E-9C8E-0B0BF2C0ED6F}" name="PRÓXIMA META" dataDxfId="23" totalsRowDxfId="22">
+    <tableColumn id="8" xr3:uid="{A4232C53-895F-4F8E-9C8E-0B0BF2C0ED6F}" name="PRÓXIMA META" dataDxfId="22" totalsRowDxfId="21">
       <calculatedColumnFormula array="1">_xlfn.IFS(AO3="NÃO ATINGIDO","D",AO3="D","C",AO3="C","B",AO3="B","A",AO3="A","OBJETIVO ALCANÇADO")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{48707A36-6A09-40D7-A590-A88562D8F521}" name="FALTA" totalsRowFunction="sum" dataDxfId="21" totalsRowDxfId="20" dataCellStyle="Moeda">
+    <tableColumn id="9" xr3:uid="{48707A36-6A09-40D7-A590-A88562D8F521}" name="FALTA" totalsRowFunction="sum" dataDxfId="20" totalsRowDxfId="19" dataCellStyle="Moeda">
       <calculatedColumnFormula array="1">_xlfn.IFS(AP3="D",MAX(AM3-AN3,0),AP3="C",MAX(AL3-AN3,0),AP3="B",MAX(AK3-AN3,0),AP3="A",MAX(AJ3-AN3,0),AP3="OBJETIVO ALCANÇADO",0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4055,7 +4016,7 @@
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{7A100617-BF77-4A79-B506-53CDBC26C911}" name="Tabela17" displayName="Tabela17" ref="Y2:AG20" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18" tableBorderDxfId="17">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{7A100617-BF77-4A79-B506-53CDBC26C911}" name="Tabela17" displayName="Tabela17" ref="Y2:AG20" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17" tableBorderDxfId="16">
   <autoFilter ref="Y2:AG20" xr:uid="{7A100617-BF77-4A79-B506-53CDBC26C911}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -4068,29 +4029,29 @@
     <filterColumn colId="8" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{E374FEB3-F510-4F3F-9C13-58E25924121E}" name="VENDEDOR" dataDxfId="16"/>
-    <tableColumn id="2" xr3:uid="{8DACCDF0-1F48-4D1F-936B-1BD572540814}" name="META A" dataDxfId="15">
+    <tableColumn id="1" xr3:uid="{E374FEB3-F510-4F3F-9C13-58E25924121E}" name="VENDEDOR" dataDxfId="15"/>
+    <tableColumn id="2" xr3:uid="{8DACCDF0-1F48-4D1F-936B-1BD572540814}" name="META A" dataDxfId="14">
       <calculatedColumnFormula>_xlfn.XLOOKUP(Tabela17[[#This Row],[VENDEDOR]],[1]!Tabela4[VENDEDOR],[1]!Tabela4[META A])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{283DD7D7-EAA0-41F2-A03E-A94402C351D8}" name="META B" dataDxfId="14">
+    <tableColumn id="3" xr3:uid="{283DD7D7-EAA0-41F2-A03E-A94402C351D8}" name="META B" dataDxfId="13">
       <calculatedColumnFormula>_xlfn.XLOOKUP(Tabela17[[#This Row],[VENDEDOR]],[1]!Tabela4[VENDEDOR],[1]!Tabela4[META B])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{FA7094C0-E343-4D2F-A021-CE4770011F17}" name="META C" dataDxfId="13">
+    <tableColumn id="4" xr3:uid="{FA7094C0-E343-4D2F-A021-CE4770011F17}" name="META C" dataDxfId="12">
       <calculatedColumnFormula>_xlfn.XLOOKUP(Tabela17[[#This Row],[VENDEDOR]],[1]!Tabela4[VENDEDOR],[1]!Tabela4[META C])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{B6D91B25-84F6-4BBF-AFFE-776A8AB5FD86}" name="META D" dataDxfId="12">
+    <tableColumn id="5" xr3:uid="{B6D91B25-84F6-4BBF-AFFE-776A8AB5FD86}" name="META D" dataDxfId="11">
       <calculatedColumnFormula>_xlfn.XLOOKUP(Tabela17[[#This Row],[VENDEDOR]],[1]!Tabela4[VENDEDOR],[1]!Tabela4[META D])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{DD3D2046-BE2C-43C9-8F6C-13D785756968}" name="ATINGIDO" dataDxfId="11">
+    <tableColumn id="6" xr3:uid="{DD3D2046-BE2C-43C9-8F6C-13D785756968}" name="ATINGIDO" dataDxfId="10">
       <calculatedColumnFormula>IFERROR(_xlfn.XLOOKUP(Y3,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0),0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{FE9C4B8F-98E5-474D-B959-1D70DA5A76FE}" name="PREMIAÇÃO ATINGIDA" dataDxfId="10">
+    <tableColumn id="7" xr3:uid="{FE9C4B8F-98E5-474D-B959-1D70DA5A76FE}" name="PREMIAÇÃO ATINGIDA" dataDxfId="9">
       <calculatedColumnFormula array="1">_xlfn.IFS(AD3&gt;=Z3,"A",AD3&gt;=AA3,"B",AD3&gt;=AB3,"C",AD3&gt;=AC3,"D",TRUE,"NÃO ATINGIDO")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{9A7A5F0B-ED50-4C50-BA8D-CCEF51A55D3B}" name="PRÓXIMA META" dataDxfId="9">
+    <tableColumn id="8" xr3:uid="{9A7A5F0B-ED50-4C50-BA8D-CCEF51A55D3B}" name="PRÓXIMA META" dataDxfId="8">
       <calculatedColumnFormula array="1">_xlfn.IFS(AE3="NÃO ATINGIDO","D",AE3="D","C",AE3="C","B",AE3="B","A",AE3="A","OBJETIVO ALCANÇADO")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{E1C246FF-4D71-4AB4-804E-54960DFC2111}" name="FALTA" dataDxfId="8">
+    <tableColumn id="9" xr3:uid="{E1C246FF-4D71-4AB4-804E-54960DFC2111}" name="FALTA" dataDxfId="7">
       <calculatedColumnFormula array="1">_xlfn.IFS(AF3="D",MAX(AC3-AD3,0),AF3="C",MAX(AB3-AD3,0),AF3="B",MAX(AA3-AD3,0),AF3="A",MAX(Z3-AD3,0),AF3="OBJETIVO ALCANÇADO",0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4099,10 +4060,10 @@
 </file>
 
 <file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2C97E85A-DD10-4825-81C1-53CD3989178B}" name="Tabela1" displayName="Tabela1" ref="B4:C7" headerRowCount="0" totalsRowShown="0" headerRowDxfId="7" dataDxfId="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2C97E85A-DD10-4825-81C1-53CD3989178B}" name="Tabela1" displayName="Tabela1" ref="B4:C7" headerRowCount="0" totalsRowShown="0" headerRowDxfId="6" dataDxfId="5">
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{3308613D-E7FC-469E-B078-C5AC910E183B}" name="Coluna1" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{C994D666-6174-475E-AE71-1F12062A5225}" name="Coluna2" headerRowDxfId="4" dataDxfId="3" dataCellStyle="Moeda"/>
+    <tableColumn id="1" xr3:uid="{3308613D-E7FC-469E-B078-C5AC910E183B}" name="Coluna1" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{C994D666-6174-475E-AE71-1F12062A5225}" name="Coluna2" headerRowDxfId="3" dataDxfId="2" dataCellStyle="Moeda"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4247,10 +4208,10 @@
     <tableColumn id="1" xr3:uid="{96702934-C966-496F-B51E-ADD7BF9BB7D8}" name="REFERENCIA" dataDxfId="62"/>
     <tableColumn id="2" xr3:uid="{E2D85F5C-4525-4FA4-B813-A1322F5C254D}" name="VENDEDOR" dataDxfId="61"/>
     <tableColumn id="3" xr3:uid="{53C55BB3-DDD4-47EF-87D5-552E4D02B5BA}" name="META A" dataDxfId="60"/>
-    <tableColumn id="4" xr3:uid="{018C7BF7-4C79-4668-95B2-CBF2E10B657D}" name="ATINGIDO" dataDxfId="0">
+    <tableColumn id="4" xr3:uid="{018C7BF7-4C79-4668-95B2-CBF2E10B657D}" name="ATINGIDO" dataDxfId="59">
       <calculatedColumnFormula>IFERROR(VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0),0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{37E12533-09AB-4B65-AEC8-6BB07B5CC2B1}" name="FALTA" dataDxfId="59">
+    <tableColumn id="5" xr3:uid="{37E12533-09AB-4B65-AEC8-6BB07B5CC2B1}" name="FALTA" dataDxfId="58">
       <calculatedColumnFormula>U10-V10</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4786,7 +4747,7 @@
       </c>
       <c r="AD3" s="29">
         <f>IFERROR(_xlfn.XLOOKUP(Y3,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0),0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AE3" s="29" t="str" cm="1">
         <f t="array" ref="AE3">_xlfn.IFS(AD3&gt;=Z3,"A",AD3&gt;=AA3,"B",AD3&gt;=AB3,"C",AD3&gt;=AC3,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -4798,7 +4759,7 @@
       </c>
       <c r="AG3" s="29" cm="1">
         <f t="array" ref="AG3">_xlfn.IFS(AF3="D",MAX(AC3-AD3,0),AF3="C",MAX(AB3-AD3,0),AF3="B",MAX(AA3-AD3,0),AF3="A",MAX(Z3-AD3,0),AF3="OBJETIVO ALCANÇADO",0)</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="AI3" t="s">
         <v>22</v>
@@ -4821,7 +4782,7 @@
       </c>
       <c r="AN3" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI3,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>12237.629999999997</v>
+        <v>13559.139999999998</v>
       </c>
       <c r="AO3" s="26" t="str" cm="1">
         <f t="array" ref="AO3">_xlfn.IFS(AN3&gt;=AJ3,"A",AN3&gt;=AK3,"B",AN3&gt;=AL3,"C",AN3&gt;=AM3,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -4833,7 +4794,7 @@
       </c>
       <c r="AQ3" s="25" cm="1">
         <f t="array" ref="AQ3">_xlfn.IFS(AP3="D",MAX(AM3-AN3,0),AP3="C",MAX(AL3-AN3,0),AP3="B",MAX(AK3-AN3,0),AP3="A",MAX(AJ3-AN3,0),AP3="OBJETIVO ALCANÇADO",0)</f>
-        <v>27362.370000000003</v>
+        <v>26040.86</v>
       </c>
     </row>
     <row r="4" spans="1:43" x14ac:dyDescent="0.25">
@@ -4854,7 +4815,7 @@
       </c>
       <c r="I4" s="7">
         <f>SUM(I10:I27)</f>
-        <v>300260</v>
+        <v>200220</v>
       </c>
       <c r="J4" s="4"/>
       <c r="K4" s="4"/>
@@ -4901,7 +4862,7 @@
       </c>
       <c r="AD4" s="31">
         <f>IFERROR(_xlfn.XLOOKUP(Y4,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$M:$M,0),0)</f>
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="AE4" s="31" t="str" cm="1">
         <f t="array" ref="AE4">_xlfn.IFS(AD4&gt;=Z4,"A",AD4&gt;=AA4,"B",AD4&gt;=AB4,"C",AD4&gt;=AC4,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -4913,7 +4874,7 @@
       </c>
       <c r="AG4" s="31" cm="1">
         <f t="array" ref="AG4">_xlfn.IFS(AF4="D",MAX(AC4-AD4,0),AF4="C",MAX(AB4-AD4,0),AF4="B",MAX(AA4-AD4,0),AF4="A",MAX(Z4-AD4,0),AF4="OBJETIVO ALCANÇADO",0)</f>
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="AI4" t="s">
         <v>24</v>
@@ -4936,7 +4897,7 @@
       </c>
       <c r="AN4" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI4,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>8237.1200000000008</v>
+        <v>9212.1200000000008</v>
       </c>
       <c r="AO4" s="26" t="str" cm="1">
         <f t="array" ref="AO4">_xlfn.IFS(AN4&gt;=AJ4,"A",AN4&gt;=AK4,"B",AN4&gt;=AL4,"C",AN4&gt;=AM4,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -4948,7 +4909,7 @@
       </c>
       <c r="AQ4" s="25" cm="1">
         <f t="array" ref="AQ4">_xlfn.IFS(AP4="D",MAX(AM4-AN4,0),AP4="C",MAX(AL4-AN4,0),AP4="B",MAX(AK4-AN4,0),AP4="A",MAX(AJ4-AN4,0),AP4="OBJETIVO ALCANÇADO",0)</f>
-        <v>27312.879999999997</v>
+        <v>26337.879999999997</v>
       </c>
     </row>
     <row r="5" spans="1:43" x14ac:dyDescent="0.25">
@@ -4958,7 +4919,7 @@
       </c>
       <c r="C5" s="2">
         <f>SUM(D10:D36)</f>
-        <v>444631.61999999994</v>
+        <v>593182.3899999999</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -4969,7 +4930,7 @@
       </c>
       <c r="I5" s="7">
         <f ca="1">SUM(J10:J27)</f>
-        <v>219369.60000000003</v>
+        <v>229586.68000000005</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -4980,7 +4941,7 @@
       </c>
       <c r="O5" s="7">
         <f>SUM(P11:P17)</f>
-        <v>8666.7999999999993</v>
+        <v>59732.449999999968</v>
       </c>
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
@@ -4991,7 +4952,7 @@
       </c>
       <c r="U5" s="4">
         <f ca="1">SUM(V10:V26)</f>
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -5051,7 +5012,7 @@
       </c>
       <c r="AN5" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI5,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>59621.760000000031</v>
+        <v>59621.690000000039</v>
       </c>
       <c r="AO5" s="26" t="str" cm="1">
         <f t="array" ref="AO5">_xlfn.IFS(AN5&gt;=AJ5,"A",AN5&gt;=AK5,"B",AN5&gt;=AL5,"C",AN5&gt;=AM5,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -5063,7 +5024,7 @@
       </c>
       <c r="AQ5" s="25" cm="1">
         <f t="array" ref="AQ5">_xlfn.IFS(AP5="D",MAX(AM5-AN5,0),AP5="C",MAX(AL5-AN5,0),AP5="B",MAX(AK5-AN5,0),AP5="A",MAX(AJ5-AN5,0),AP5="OBJETIVO ALCANÇADO",0)</f>
-        <v>95628.239999999962</v>
+        <v>95628.309999999969</v>
       </c>
     </row>
     <row r="6" spans="1:43" x14ac:dyDescent="0.25">
@@ -5073,7 +5034,7 @@
       </c>
       <c r="C6" s="2">
         <f>C4-C5</f>
-        <v>5581145.3799999999</v>
+        <v>5432594.6100000003</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="4"/>
@@ -5084,7 +5045,7 @@
       </c>
       <c r="I6" s="7">
         <f ca="1">I4-I5</f>
-        <v>80890.399999999965</v>
+        <v>-29366.680000000051</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -5095,7 +5056,7 @@
       </c>
       <c r="O6" s="7">
         <f>O4-O5</f>
-        <v>-8666.7999999999993</v>
+        <v>-59732.449999999968</v>
       </c>
       <c r="P6" s="4"/>
       <c r="Q6" s="4"/>
@@ -5106,7 +5067,7 @@
       </c>
       <c r="U6" s="4">
         <f ca="1">U4-U5</f>
-        <v>531</v>
+        <v>528</v>
       </c>
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
@@ -5131,7 +5092,7 @@
       </c>
       <c r="AD6" s="31">
         <f>IFERROR(_xlfn.XLOOKUP(Y6,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0),0)</f>
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="AE6" s="31" t="str" cm="1">
         <f t="array" ref="AE6">_xlfn.IFS(AD6&gt;=Z6,"A",AD6&gt;=AA6,"B",AD6&gt;=AB6,"C",AD6&gt;=AC6,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -5143,7 +5104,7 @@
       </c>
       <c r="AG6" s="31" cm="1">
         <f t="array" ref="AG6">_xlfn.IFS(AF6="D",MAX(AC6-AD6,0),AF6="C",MAX(AB6-AD6,0),AF6="B",MAX(AA6-AD6,0),AF6="A",MAX(Z6-AD6,0),AF6="OBJETIVO ALCANÇADO",0)</f>
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="AI6" t="s">
         <v>18</v>
@@ -5166,7 +5127,7 @@
       </c>
       <c r="AN6" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI6,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>52714.710000000036</v>
+        <v>52714.41</v>
       </c>
       <c r="AO6" s="26" t="str" cm="1">
         <f t="array" ref="AO6">_xlfn.IFS(AN6&gt;=AJ6,"A",AN6&gt;=AK6,"B",AN6&gt;=AL6,"C",AN6&gt;=AM6,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -5178,7 +5139,7 @@
       </c>
       <c r="AQ6" s="25" cm="1">
         <f t="array" ref="AQ6">_xlfn.IFS(AP6="D",MAX(AM6-AN6,0),AP6="C",MAX(AL6-AN6,0),AP6="B",MAX(AK6-AN6,0),AP6="A",MAX(AJ6-AN6,0),AP6="OBJETIVO ALCANÇADO",0)</f>
-        <v>96460.289999999964</v>
+        <v>96460.59</v>
       </c>
     </row>
     <row r="7" spans="1:43" x14ac:dyDescent="0.25">
@@ -5188,7 +5149,7 @@
       </c>
       <c r="C7" s="3">
         <f>1-(C6/C4)</f>
-        <v>7.3788263322721703E-2</v>
+        <v>9.8440813524961146E-2</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="4"/>
@@ -5199,7 +5160,7 @@
       </c>
       <c r="I7" s="3">
         <f ca="1">1-(I6/I4)</f>
-        <v>0.73059881436088736</v>
+        <v>1.1466720607331937</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -5221,7 +5182,7 @@
       </c>
       <c r="U7" s="3">
         <f ca="1">1-(U6/U4)</f>
-        <v>5.1785714285714324E-2</v>
+        <v>5.7142857142857162E-2</v>
       </c>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
@@ -5246,7 +5207,7 @@
       </c>
       <c r="AD7" s="29">
         <f>IFERROR(_xlfn.XLOOKUP(Y7,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0),0)</f>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AE7" s="29" t="str" cm="1">
         <f t="array" ref="AE7">_xlfn.IFS(AD7&gt;=Z7,"A",AD7&gt;=AA7,"B",AD7&gt;=AB7,"C",AD7&gt;=AC7,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -5258,7 +5219,7 @@
       </c>
       <c r="AG7" s="29" cm="1">
         <f t="array" ref="AG7">_xlfn.IFS(AF7="D",MAX(AC7-AD7,0),AF7="C",MAX(AB7-AD7,0),AF7="B",MAX(AA7-AD7,0),AF7="A",MAX(Z7-AD7,0),AF7="OBJETIVO ALCANÇADO",0)</f>
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="AI7" t="s">
         <v>10</v>
@@ -5281,7 +5242,7 @@
       </c>
       <c r="AN7" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI7,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>31839.209999999995</v>
+        <v>32988.290000000023</v>
       </c>
       <c r="AO7" s="26" t="str" cm="1">
         <f t="array" ref="AO7">_xlfn.IFS(AN7&gt;=AJ7,"A",AN7&gt;=AK7,"B",AN7&gt;=AL7,"C",AN7&gt;=AM7,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -5293,7 +5254,7 @@
       </c>
       <c r="AQ7" s="25" cm="1">
         <f t="array" ref="AQ7">_xlfn.IFS(AP7="D",MAX(AM7-AN7,0),AP7="C",MAX(AL7-AN7,0),AP7="B",MAX(AK7-AN7,0),AP7="A",MAX(AJ7-AN7,0),AP7="OBJETIVO ALCANÇADO",0)</f>
-        <v>94610.790000000008</v>
+        <v>93461.709999999977</v>
       </c>
     </row>
     <row r="8" spans="1:43" x14ac:dyDescent="0.25">
@@ -5340,7 +5301,7 @@
       </c>
       <c r="AD8" s="31">
         <f>IFERROR(_xlfn.XLOOKUP(Y8,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0),0)</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="AE8" s="31" t="str" cm="1">
         <f t="array" ref="AE8">_xlfn.IFS(AD8&gt;=Z8,"A",AD8&gt;=AA8,"B",AD8&gt;=AB8,"C",AD8&gt;=AC8,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -5352,7 +5313,7 @@
       </c>
       <c r="AG8" s="31" cm="1">
         <f t="array" ref="AG8">_xlfn.IFS(AF8="D",MAX(AC8-AD8,0),AF8="C",MAX(AB8-AD8,0),AF8="B",MAX(AA8-AD8,0),AF8="A",MAX(Z8-AD8,0),AF8="OBJETIVO ALCANÇADO",0)</f>
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="AI8" t="s">
         <v>13</v>
@@ -5375,7 +5336,7 @@
       </c>
       <c r="AN8" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI8,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>20124.039999999997</v>
+        <v>20123.86</v>
       </c>
       <c r="AO8" s="26" t="str" cm="1">
         <f t="array" ref="AO8">_xlfn.IFS(AN8&gt;=AJ8,"A",AN8&gt;=AK8,"B",AN8&gt;=AL8,"C",AN8&gt;=AM8,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -5387,7 +5348,7 @@
       </c>
       <c r="AQ8" s="25" cm="1">
         <f t="array" ref="AQ8">_xlfn.IFS(AP8="D",MAX(AM8-AN8,0),AP8="C",MAX(AL8-AN8,0),AP8="B",MAX(AK8-AN8,0),AP8="A",MAX(AJ8-AN8,0),AP8="OBJETIVO ALCANÇADO",0)</f>
-        <v>72575.960000000006</v>
+        <v>72576.14</v>
       </c>
     </row>
     <row r="9" spans="1:43" x14ac:dyDescent="0.25">
@@ -5467,7 +5428,7 @@
       </c>
       <c r="AD9" s="29">
         <f>IFERROR(_xlfn.XLOOKUP(Y9,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0),0)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AE9" s="29" t="str" cm="1">
         <f t="array" ref="AE9">_xlfn.IFS(AD9&gt;=Z9,"A",AD9&gt;=AA9,"B",AD9&gt;=AB9,"C",AD9&gt;=AC9,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -5479,7 +5440,7 @@
       </c>
       <c r="AG9" s="29" cm="1">
         <f t="array" ref="AG9">_xlfn.IFS(AF9="D",MAX(AC9-AD9,0),AF9="C",MAX(AB9-AD9,0),AF9="B",MAX(AA9-AD9,0),AF9="A",MAX(Z9-AD9,0),AF9="OBJETIVO ALCANÇADO",0)</f>
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="AI9" t="s">
         <v>20</v>
@@ -5502,7 +5463,7 @@
       </c>
       <c r="AN9" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI9,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>20117.779999999992</v>
+        <v>20419.93</v>
       </c>
       <c r="AO9" s="26" t="str" cm="1">
         <f t="array" ref="AO9">_xlfn.IFS(AN9&gt;=AJ9,"A",AN9&gt;=AK9,"B",AN9&gt;=AL9,"C",AN9&gt;=AM9,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -5514,7 +5475,7 @@
       </c>
       <c r="AQ9" s="25" cm="1">
         <f t="array" ref="AQ9">_xlfn.IFS(AP9="D",MAX(AM9-AN9,0),AP9="C",MAX(AL9-AN9,0),AP9="B",MAX(AK9-AN9,0),AP9="A",MAX(AJ9-AN9,0),AP9="OBJETIVO ALCANÇADO",0)</f>
-        <v>58632.220000000008</v>
+        <v>58330.07</v>
       </c>
     </row>
     <row r="10" spans="1:43" x14ac:dyDescent="0.25">
@@ -5530,11 +5491,11 @@
       </c>
       <c r="D10" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>4765.8999999999996</v>
+        <v>4765.8499999999995</v>
       </c>
       <c r="E10" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>65734.100000000006</v>
+        <v>65734.149999999994</v>
       </c>
       <c r="F10" s="4"/>
       <c r="G10" s="18" t="s">
@@ -5545,15 +5506,15 @@
       </c>
       <c r="I10" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>27520</v>
+        <v>20980</v>
       </c>
       <c r="J10" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>28873.699999999993</v>
+        <v>28873.46000000001</v>
       </c>
       <c r="K10" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>-1353.6999999999935</v>
+        <v>-7893.46000000001</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4" t="s">
@@ -5646,7 +5607,7 @@
       </c>
       <c r="AN10" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI10,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>37419.410000000025</v>
+        <v>37419.070000000022</v>
       </c>
       <c r="AO10" s="26" t="str" cm="1">
         <f t="array" ref="AO10">_xlfn.IFS(AN10&gt;=AJ10,"A",AN10&gt;=AK10,"B",AN10&gt;=AL10,"C",AN10&gt;=AM10,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -5658,7 +5619,7 @@
       </c>
       <c r="AQ10" s="25" cm="1">
         <f t="array" ref="AQ10">_xlfn.IFS(AP10="D",MAX(AM10-AN10,0),AP10="C",MAX(AL10-AN10,0),AP10="B",MAX(AK10-AN10,0),AP10="A",MAX(AJ10-AN10,0),AP10="OBJETIVO ALCANÇADO",0)</f>
-        <v>83711.589999999967</v>
+        <v>83711.929999999978</v>
       </c>
     </row>
     <row r="11" spans="1:43" x14ac:dyDescent="0.25">
@@ -5674,11 +5635,11 @@
       </c>
       <c r="D11" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>59621.760000000031</v>
+        <v>59621.690000000039</v>
       </c>
       <c r="E11" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>285378.24</v>
+        <v>285378.30999999994</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="18" t="s">
@@ -5689,15 +5650,15 @@
       </c>
       <c r="I11" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>25040</v>
+        <v>13060</v>
       </c>
       <c r="J11" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>23647.030000000006</v>
+        <v>23646.760000000002</v>
       </c>
       <c r="K11" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>1392.9699999999939</v>
+        <v>-10586.760000000002</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4" t="s">
@@ -5821,11 +5782,11 @@
       </c>
       <c r="D12" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="E12" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>-0.1</v>
+        <v>0</v>
       </c>
       <c r="F12" s="4"/>
       <c r="G12" s="18" t="s">
@@ -5836,15 +5797,15 @@
       </c>
       <c r="I12" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>15210</v>
+        <v>9390</v>
       </c>
       <c r="J12" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>9543.8000000000011</v>
+        <v>10320.560000000003</v>
       </c>
       <c r="K12" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>5666.1999999999989</v>
+        <v>-930.56000000000313</v>
       </c>
       <c r="L12" s="4"/>
       <c r="M12" s="4" t="s">
@@ -5940,7 +5901,7 @@
       </c>
       <c r="AN12" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI12,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>6469.4299999999976</v>
+        <v>7270.8299999999963</v>
       </c>
       <c r="AO12" s="26" t="str" cm="1">
         <f t="array" ref="AO12">_xlfn.IFS(AN12&gt;=AJ12,"A",AN12&gt;=AK12,"B",AN12&gt;=AL12,"C",AN12&gt;=AM12,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -5952,7 +5913,7 @@
       </c>
       <c r="AQ12" s="25" cm="1">
         <f t="array" ref="AQ12">_xlfn.IFS(AP12="D",MAX(AM12-AN12,0),AP12="C",MAX(AL12-AN12,0),AP12="B",MAX(AK12-AN12,0),AP12="A",MAX(AJ12-AN12,0),AP12="OBJETIVO ALCANÇADO",0)</f>
-        <v>19630.570000000003</v>
+        <v>18829.170000000006</v>
       </c>
     </row>
     <row r="13" spans="1:43" x14ac:dyDescent="0.25">
@@ -5968,11 +5929,11 @@
       </c>
       <c r="D13" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>10293.6</v>
+        <v>10293.539999999999</v>
       </c>
       <c r="E13" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>85706.4</v>
+        <v>85706.46</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="18" t="s">
@@ -5983,15 +5944,15 @@
       </c>
       <c r="I13" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>23160</v>
+        <v>19350</v>
       </c>
       <c r="J13" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>13145.130000000003</v>
+        <v>13145.080000000002</v>
       </c>
       <c r="K13" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>10014.869999999997</v>
+        <v>6204.9199999999983</v>
       </c>
       <c r="L13" s="4"/>
       <c r="M13" s="4" t="s">
@@ -6025,11 +5986,11 @@
       </c>
       <c r="V13" s="17">
         <f ca="1">IFERROR(VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0),0)</f>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="W13" s="17">
         <f t="shared" ca="1" si="0"/>
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="Y13" s="32" t="s">
         <v>9</v>
@@ -6087,7 +6048,7 @@
       </c>
       <c r="AN13" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI13,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>10293.6</v>
+        <v>10293.539999999999</v>
       </c>
       <c r="AO13" s="26" t="str" cm="1">
         <f t="array" ref="AO13">_xlfn.IFS(AN13&gt;=AJ13,"A",AN13&gt;=AK13,"B",AN13&gt;=AL13,"C",AN13&gt;=AM13,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -6099,7 +6060,7 @@
       </c>
       <c r="AQ13" s="25" cm="1">
         <f t="array" ref="AQ13">_xlfn.IFS(AP13="D",MAX(AM13-AN13,0),AP13="C",MAX(AL13-AN13,0),AP13="B",MAX(AK13-AN13,0),AP13="A",MAX(AJ13-AN13,0),AP13="OBJETIVO ALCANÇADO",0)</f>
-        <v>32906.400000000001</v>
+        <v>32906.46</v>
       </c>
     </row>
     <row r="14" spans="1:43" x14ac:dyDescent="0.25">
@@ -6115,11 +6076,11 @@
       </c>
       <c r="D14" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>31839.209999999995</v>
+        <v>32988.290000000023</v>
       </c>
       <c r="E14" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>249160.79</v>
+        <v>248011.70999999996</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="18" t="s">
@@ -6130,15 +6091,15 @@
       </c>
       <c r="I14" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>19910</v>
+        <v>16120</v>
       </c>
       <c r="J14" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>10169.540000000001</v>
+        <v>12159.649999999998</v>
       </c>
       <c r="K14" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>9740.4599999999991</v>
+        <v>3960.3500000000022</v>
       </c>
       <c r="L14" s="4"/>
       <c r="M14" s="4" t="s">
@@ -6234,7 +6195,7 @@
       </c>
       <c r="AN14" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI14,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>4765.8999999999996</v>
+        <v>4765.8499999999995</v>
       </c>
       <c r="AO14" s="26" t="str" cm="1">
         <f t="array" ref="AO14">_xlfn.IFS(AN14&gt;=AJ14,"A",AN14&gt;=AK14,"B",AN14&gt;=AL14,"C",AN14&gt;=AM14,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -6246,7 +6207,7 @@
       </c>
       <c r="AQ14" s="25" cm="1">
         <f t="array" ref="AQ14">_xlfn.IFS(AP14="D",MAX(AM14-AN14,0),AP14="C",MAX(AL14-AN14,0),AP14="B",MAX(AK14-AN14,0),AP14="A",MAX(AJ14-AN14,0),AP14="OBJETIVO ALCANÇADO",0)</f>
-        <v>26959.1</v>
+        <v>26959.15</v>
       </c>
     </row>
     <row r="15" spans="1:43" x14ac:dyDescent="0.25">
@@ -6262,11 +6223,11 @@
       </c>
       <c r="D15" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>11111.86</v>
+        <v>12263.809999999998</v>
       </c>
       <c r="E15" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>72888.14</v>
+        <v>71736.19</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="18" t="s">
@@ -6277,7 +6238,7 @@
       </c>
       <c r="I15" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>32180</v>
+        <v>25020</v>
       </c>
       <c r="J15" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
@@ -6285,7 +6246,7 @@
       </c>
       <c r="K15" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>-1528.7300000000032</v>
+        <v>-8688.7300000000032</v>
       </c>
       <c r="L15" s="4"/>
       <c r="M15" s="4" t="s">
@@ -6346,7 +6307,7 @@
       </c>
       <c r="AD15" s="29">
         <f>IFERROR(_xlfn.XLOOKUP(Y15,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0),0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AE15" s="29" t="str" cm="1">
         <f t="array" ref="AE15">_xlfn.IFS(AD15&gt;=Z15,"A",AD15&gt;=AA15,"B",AD15&gt;=AB15,"C",AD15&gt;=AC15,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -6358,7 +6319,7 @@
       </c>
       <c r="AG15" s="29" cm="1">
         <f t="array" ref="AG15">_xlfn.IFS(AF15="D",MAX(AC15-AD15,0),AF15="C",MAX(AB15-AD15,0),AF15="B",MAX(AA15-AD15,0),AF15="A",MAX(Z15-AD15,0),AF15="OBJETIVO ALCANÇADO",0)</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="AI15" t="s">
         <v>11</v>
@@ -6381,7 +6342,7 @@
       </c>
       <c r="AN15" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI15,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>11111.86</v>
+        <v>12263.809999999998</v>
       </c>
       <c r="AO15" s="26" t="str" cm="1">
         <f t="array" ref="AO15">_xlfn.IFS(AN15&gt;=AJ15,"A",AN15&gt;=AK15,"B",AN15&gt;=AL15,"C",AN15&gt;=AM15,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -6393,7 +6354,7 @@
       </c>
       <c r="AQ15" s="25" cm="1">
         <f t="array" ref="AQ15">_xlfn.IFS(AP15="D",MAX(AM15-AN15,0),AP15="C",MAX(AL15-AN15,0),AP15="B",MAX(AK15-AN15,0),AP15="A",MAX(AJ15-AN15,0),AP15="OBJETIVO ALCANÇADO",0)</f>
-        <v>26688.14</v>
+        <v>25536.190000000002</v>
       </c>
     </row>
     <row r="16" spans="1:43" x14ac:dyDescent="0.25">
@@ -6409,11 +6370,11 @@
       </c>
       <c r="D16" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>2017.1999999999998</v>
+        <v>2016.6</v>
       </c>
       <c r="E16" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>347982.8</v>
+        <v>347983.4</v>
       </c>
       <c r="F16" s="4"/>
       <c r="G16" s="18" t="s">
@@ -6424,15 +6385,15 @@
       </c>
       <c r="I16" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>17760</v>
+        <v>13880</v>
       </c>
       <c r="J16" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>16105.800000000005</v>
+        <v>16407.95</v>
       </c>
       <c r="K16" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>1654.1999999999953</v>
+        <v>-2527.9500000000007</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4" t="s">
@@ -6493,7 +6454,7 @@
       </c>
       <c r="AD16" s="31">
         <f>IFERROR(_xlfn.XLOOKUP(Y16,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0),0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AE16" s="31" t="str" cm="1">
         <f t="array" ref="AE16">_xlfn.IFS(AD16&gt;=Z16,"A",AD16&gt;=AA16,"B",AD16&gt;=AB16,"C",AD16&gt;=AC16,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -6505,7 +6466,7 @@
       </c>
       <c r="AG16" s="31" cm="1">
         <f t="array" ref="AG16">_xlfn.IFS(AF16="D",MAX(AC16-AD16,0),AF16="C",MAX(AB16-AD16,0),AF16="B",MAX(AA16-AD16,0),AF16="A",MAX(Z16-AD16,0),AF16="OBJETIVO ALCANÇADO",0)</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="AI16" t="s">
         <v>19</v>
@@ -6528,7 +6489,7 @@
       </c>
       <c r="AN16" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI16,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>15519.85</v>
+        <v>16296.58</v>
       </c>
       <c r="AO16" s="26" t="str" cm="1">
         <f t="array" ref="AO16">_xlfn.IFS(AN16&gt;=AJ16,"A",AN16&gt;=AK16,"B",AN16&gt;=AL16,"C",AN16&gt;=AM16,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -6540,7 +6501,7 @@
       </c>
       <c r="AQ16" s="25" cm="1">
         <f t="array" ref="AQ16">_xlfn.IFS(AP16="D",MAX(AM16-AN16,0),AP16="C",MAX(AL16-AN16,0),AP16="B",MAX(AK16-AN16,0),AP16="A",MAX(AJ16-AN16,0),AP16="OBJETIVO ALCANÇADO",0)</f>
-        <v>48380.15</v>
+        <v>47603.42</v>
       </c>
     </row>
     <row r="17" spans="1:43" x14ac:dyDescent="0.25">
@@ -6556,11 +6517,11 @@
       </c>
       <c r="D17" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>12150</v>
+        <v>63215.649999999965</v>
       </c>
       <c r="E17" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>487850</v>
+        <v>436784.35000000003</v>
       </c>
       <c r="F17" s="4"/>
       <c r="G17" s="18" t="s">
@@ -6571,15 +6532,15 @@
       </c>
       <c r="I17" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>10200</v>
+        <v>4590</v>
       </c>
       <c r="J17" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2463.46</v>
+        <v>4213.3100000000004</v>
       </c>
       <c r="K17" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>7736.54</v>
+        <v>376.6899999999996</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="4" t="s">
@@ -6594,11 +6555,11 @@
       </c>
       <c r="P17" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[REGIAO]","[Intervalo 2].[REGIAO].&amp;["&amp;N17&amp;"]","[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;["&amp;RIGHT($O$9,1)&amp;"]"),0)</f>
-        <v>8666.7999999999993</v>
+        <v>59732.449999999968</v>
       </c>
       <c r="Q17" s="2">
         <f>Tabela8[[#This Row],[COMPROMISSO]]-Tabela8[[#This Row],[ATINGIDO]]</f>
-        <v>-8666.7999999999993</v>
+        <v>-59732.449999999968</v>
       </c>
       <c r="R17" s="2"/>
       <c r="S17" s="17" t="s">
@@ -6675,7 +6636,7 @@
       </c>
       <c r="AN17" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI17,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>24013.129999999997</v>
+        <v>24013.079999999998</v>
       </c>
       <c r="AO17" s="26" t="str" cm="1">
         <f t="array" ref="AO17">_xlfn.IFS(AN17&gt;=AJ17,"A",AN17&gt;=AK17,"B",AN17&gt;=AL17,"C",AN17&gt;=AM17,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -6687,7 +6648,7 @@
       </c>
       <c r="AQ17" s="25" cm="1">
         <f t="array" ref="AQ17">_xlfn.IFS(AP17="D",MAX(AM17-AN17,0),AP17="C",MAX(AL17-AN17,0),AP17="B",MAX(AK17-AN17,0),AP17="A",MAX(AJ17-AN17,0),AP17="OBJETIVO ALCANÇADO",0)</f>
-        <v>50956.87</v>
+        <v>50956.92</v>
       </c>
     </row>
     <row r="18" spans="1:43" x14ac:dyDescent="0.25">
@@ -6703,11 +6664,11 @@
       </c>
       <c r="D18" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>7672</v>
+        <v>94941.200000000012</v>
       </c>
       <c r="E18" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>972328</v>
+        <v>885058.8</v>
       </c>
       <c r="F18" s="4"/>
       <c r="G18" s="18" t="s">
@@ -6774,7 +6735,7 @@
       </c>
       <c r="AD18" s="31">
         <f>IFERROR(_xlfn.XLOOKUP(Y18,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$N:$N,0),0)</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="AE18" s="31" t="str" cm="1">
         <f t="array" ref="AE18">_xlfn.IFS(AD18&gt;=Z18,"A",AD18&gt;=AA18,"B",AD18&gt;=AB18,"C",AD18&gt;=AC18,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -6786,7 +6747,7 @@
       </c>
       <c r="AG18" s="31" cm="1">
         <f t="array" ref="AG18">_xlfn.IFS(AF18="D",MAX(AC18-AD18,0),AF18="C",MAX(AB18-AD18,0),AF18="B",MAX(AA18-AD18,0),AF18="A",MAX(Z18-AD18,0),AF18="OBJETIVO ALCANÇADO",0)</f>
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="AI18" t="s">
         <v>21</v>
@@ -6809,7 +6770,7 @@
       </c>
       <c r="AN18" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI18,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>32294.459999999985</v>
+        <v>32294.379999999983</v>
       </c>
       <c r="AO18" s="26" t="str" cm="1">
         <f t="array" ref="AO18">_xlfn.IFS(AN18&gt;=AJ18,"A",AN18&gt;=AK18,"B",AN18&gt;=AL18,"C",AN18&gt;=AM18,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -6821,7 +6782,7 @@
       </c>
       <c r="AQ18" s="25" cm="1">
         <f t="array" ref="AQ18">_xlfn.IFS(AP18="D",MAX(AM18-AN18,0),AP18="C",MAX(AL18-AN18,0),AP18="B",MAX(AK18-AN18,0),AP18="A",MAX(AJ18-AN18,0),AP18="OBJETIVO ALCANÇADO",0)</f>
-        <v>89205.540000000008</v>
+        <v>89205.620000000024</v>
       </c>
     </row>
     <row r="19" spans="1:43" x14ac:dyDescent="0.25">
@@ -6852,15 +6813,15 @@
       </c>
       <c r="I19" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>18810</v>
+        <v>18340</v>
       </c>
       <c r="J19" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>13425.569999999992</v>
+        <v>13425.409999999993</v>
       </c>
       <c r="K19" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>5384.4300000000076</v>
+        <v>4914.5900000000074</v>
       </c>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
@@ -6939,7 +6900,7 @@
       </c>
       <c r="AN19" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI19,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>3489.02</v>
+        <v>5238.87</v>
       </c>
       <c r="AO19" s="26" t="str" cm="1">
         <f t="array" ref="AO19">_xlfn.IFS(AN19&gt;=AJ19,"A",AN19&gt;=AK19,"B",AN19&gt;=AL19,"C",AN19&gt;=AM19,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -6951,7 +6912,7 @@
       </c>
       <c r="AQ19" s="25" cm="1">
         <f t="array" ref="AQ19">_xlfn.IFS(AP19="D",MAX(AM19-AN19,0),AP19="C",MAX(AL19-AN19,0),AP19="B",MAX(AK19-AN19,0),AP19="A",MAX(AJ19-AN19,0),AP19="OBJETIVO ALCANÇADO",0)</f>
-        <v>39485.980000000003</v>
+        <v>37736.129999999997</v>
       </c>
     </row>
     <row r="20" spans="1:43" x14ac:dyDescent="0.25">
@@ -6982,15 +6943,15 @@
       </c>
       <c r="I20" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>25860</v>
+        <v>17000</v>
       </c>
       <c r="J20" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>18447.749999999985</v>
+        <v>19596.890000000007</v>
       </c>
       <c r="K20" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>7412.2500000000146</v>
+        <v>-2596.8900000000067</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
@@ -7081,7 +7042,7 @@
       </c>
       <c r="AN20" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI20,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>12662.729999999998</v>
+        <v>14652.809999999996</v>
       </c>
       <c r="AO20" s="26" t="str" cm="1">
         <f t="array" ref="AO20">_xlfn.IFS(AN20&gt;=AJ20,"A",AN20&gt;=AK20,"B",AN20&gt;=AL20,"C",AN20&gt;=AM20,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -7093,7 +7054,7 @@
       </c>
       <c r="AQ20" s="25" cm="1">
         <f t="array" ref="AQ20">_xlfn.IFS(AP20="D",MAX(AM20-AN20,0),AP20="C",MAX(AL20-AN20,0),AP20="B",MAX(AK20-AN20,0),AP20="A",MAX(AJ20-AN20,0),AP20="OBJETIVO ALCANÇADO",0)</f>
-        <v>85212.27</v>
+        <v>83222.19</v>
       </c>
     </row>
     <row r="21" spans="1:43" x14ac:dyDescent="0.25">
@@ -7124,15 +7085,15 @@
       </c>
       <c r="I21" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>4890</v>
+        <v>5990</v>
       </c>
       <c r="J21" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>3433.25</v>
+        <v>4585.25</v>
       </c>
       <c r="K21" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>1456.75</v>
+        <v>1404.75</v>
       </c>
       <c r="L21" s="4"/>
       <c r="M21" s="4"/>
@@ -7164,11 +7125,11 @@
       </c>
       <c r="V21" s="17">
         <f ca="1">IFERROR(VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0),0)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W21" s="17">
         <f t="shared" ref="W21:W26" ca="1" si="1">U21-V21</f>
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="Y21" s="36" t="s">
         <v>60</v>
@@ -7191,13 +7152,13 @@
       </c>
       <c r="AD21" s="37">
         <f>SUBTOTAL(109,Planilha1!$AD$3:$AD$20)</f>
-        <v>56</v>
+        <v>33</v>
       </c>
       <c r="AE21" s="37"/>
       <c r="AF21" s="37"/>
       <c r="AG21" s="38">
         <f>SUBTOTAL(109,Planilha1!$AG$3:$AG$20)</f>
-        <v>204</v>
+        <v>227</v>
       </c>
       <c r="AI21" t="s">
         <v>60</v>
@@ -7220,13 +7181,13 @@
       </c>
       <c r="AN21" s="26">
         <f>SUBTOTAL(109,Tabela817[ATINGIDO])</f>
-        <v>362931.64000000007</v>
+        <v>373148.26000000007</v>
       </c>
       <c r="AO21" s="4"/>
       <c r="AP21" s="4"/>
       <c r="AQ21" s="27">
         <f>SUBTOTAL(109,Tabela817[FALTA])</f>
-        <v>975719.36</v>
+        <v>965502.74</v>
       </c>
     </row>
     <row r="22" spans="1:43" x14ac:dyDescent="0.25">
@@ -7257,15 +7218,15 @@
       </c>
       <c r="I22" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>21810</v>
+        <v>9950</v>
       </c>
       <c r="J22" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>14168.78</v>
+        <v>14168.76</v>
       </c>
       <c r="K22" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>7641.2199999999993</v>
+        <v>-4218.76</v>
       </c>
       <c r="L22" s="4"/>
       <c r="M22" s="4"/>
@@ -7278,11 +7239,11 @@
       </c>
       <c r="P22" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>8666.7999999999993</v>
+        <v>59732.449999999968</v>
       </c>
       <c r="Q22" s="7">
         <f>O22-P22</f>
-        <v>717523.67619047617</v>
+        <v>666458.02619047626</v>
       </c>
       <c r="R22" s="4"/>
       <c r="S22" s="17" t="s">
@@ -7317,11 +7278,11 @@
       </c>
       <c r="D23" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>20124.039999999997</v>
+        <v>20123.86</v>
       </c>
       <c r="E23" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>185875.96</v>
+        <v>185876.14</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="18" t="s">
@@ -7332,15 +7293,15 @@
       </c>
       <c r="I23" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>15240</v>
+        <v>6580</v>
       </c>
       <c r="J23" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>8426.4499999999989</v>
+        <v>8426.4</v>
       </c>
       <c r="K23" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>6813.5500000000011</v>
+        <v>-1846.3999999999996</v>
       </c>
       <c r="L23" s="4"/>
       <c r="M23" s="4"/>
@@ -7392,11 +7353,11 @@
       </c>
       <c r="D24" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>24013.129999999997</v>
+        <v>24013.079999999998</v>
       </c>
       <c r="E24" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>142584.87</v>
+        <v>142584.92000000001</v>
       </c>
       <c r="F24" s="4"/>
       <c r="G24" s="18" t="s">
@@ -7407,15 +7368,15 @@
       </c>
       <c r="I24" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>12050</v>
+        <v>5530</v>
       </c>
       <c r="J24" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>7909.1</v>
+        <v>8884.1</v>
       </c>
       <c r="K24" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>4140.8999999999996</v>
+        <v>-3354.1000000000004</v>
       </c>
       <c r="L24" s="4"/>
       <c r="M24" s="4"/>
@@ -7467,11 +7428,11 @@
       </c>
       <c r="D25" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>12662.729999999998</v>
+        <v>14652.809999999996</v>
       </c>
       <c r="E25" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>204837.27</v>
+        <v>202847.19</v>
       </c>
       <c r="F25" s="4"/>
       <c r="G25" s="18" t="s">
@@ -7482,15 +7443,15 @@
       </c>
       <c r="I25" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>15120</v>
+        <v>5850</v>
       </c>
       <c r="J25" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>9210.7599999999984</v>
+        <v>10532.269999999999</v>
       </c>
       <c r="K25" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>5909.2400000000016</v>
+        <v>-4682.2699999999986</v>
       </c>
       <c r="L25" s="4"/>
       <c r="M25" s="4"/>
@@ -7542,11 +7503,11 @@
       </c>
       <c r="D26" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>3489.02</v>
+        <v>5238.87</v>
       </c>
       <c r="E26" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>92010.98</v>
+        <v>90261.13</v>
       </c>
       <c r="F26" s="4"/>
       <c r="G26" s="18" t="s">
@@ -7557,15 +7518,15 @@
       </c>
       <c r="I26" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>8690</v>
+        <v>3770</v>
       </c>
       <c r="J26" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>3624.6000000000004</v>
+        <v>4425.9999999999991</v>
       </c>
       <c r="K26" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>5065.3999999999996</v>
+        <v>-655.99999999999909</v>
       </c>
       <c r="L26" s="4"/>
       <c r="M26" s="4"/>
@@ -7606,11 +7567,11 @@
       </c>
       <c r="D27" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>37419.410000000025</v>
+        <v>37419.070000000022</v>
       </c>
       <c r="E27" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>231759.58999999997</v>
+        <v>231759.93</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="18" t="s">
@@ -7621,15 +7582,15 @@
       </c>
       <c r="I27" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>6810</v>
+        <v>4820</v>
       </c>
       <c r="J27" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>3066.15</v>
+        <v>3066.1000000000004</v>
       </c>
       <c r="K27" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3743.85</v>
+        <v>1753.8999999999996</v>
       </c>
       <c r="L27" s="4"/>
       <c r="M27" s="4"/>
@@ -7652,11 +7613,11 @@
       </c>
       <c r="D28" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>52714.710000000036</v>
+        <v>52714.41</v>
       </c>
       <c r="E28" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>278785.28999999998</v>
+        <v>278785.58999999997</v>
       </c>
       <c r="F28" s="4"/>
       <c r="L28" s="4"/>
@@ -7731,11 +7692,11 @@
       </c>
       <c r="D30" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>15519.85</v>
+        <v>16296.58</v>
       </c>
       <c r="E30" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>126480.15</v>
+        <v>125703.42</v>
       </c>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
@@ -7788,11 +7749,11 @@
       </c>
       <c r="D31" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>20117.779999999992</v>
+        <v>20419.93</v>
       </c>
       <c r="E31" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>154882.22</v>
+        <v>154580.07</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
@@ -7805,11 +7766,11 @@
       </c>
       <c r="J31" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[1]"),0)</f>
-        <v>120365.8799999999</v>
+        <v>120365.51000000001</v>
       </c>
       <c r="K31" s="7">
         <f>I31-J31</f>
-        <v>162946.21523809538</v>
+        <v>162946.58523809526</v>
       </c>
       <c r="L31" s="4"/>
       <c r="M31" s="4"/>
@@ -7828,11 +7789,11 @@
       </c>
       <c r="V31" s="5">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE 2]",'[1]BASE PYTHON'!$P$83,"[Intervalo 3].[SEMANAL]","[Intervalo 3].[SEMANAL].&amp;[2]"),0)</f>
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="W31" s="6">
         <f t="shared" ref="W31:W33" si="2">U31-V31</f>
-        <v>118.33333333333334</v>
+        <v>115.33333333333334</v>
       </c>
     </row>
     <row r="32" spans="1:43" x14ac:dyDescent="0.25">
@@ -7848,11 +7809,11 @@
       </c>
       <c r="D32" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>32294.459999999985</v>
+        <v>32294.379999999983</v>
       </c>
       <c r="E32" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>237705.54</v>
+        <v>237705.62000000002</v>
       </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
@@ -7865,11 +7826,11 @@
       </c>
       <c r="J32" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>176767.39000000004</v>
+        <v>185235.10000000012</v>
       </c>
       <c r="K32" s="7">
         <f t="shared" ref="K32:K34" si="3">I32-J32</f>
-        <v>531512.84809523809</v>
+        <v>523045.13809523801</v>
       </c>
       <c r="L32" s="4"/>
       <c r="M32" s="4"/>
@@ -7908,11 +7869,11 @@
       </c>
       <c r="D33" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>12237.629999999997</v>
+        <v>13559.139999999998</v>
       </c>
       <c r="E33" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>75762.37</v>
+        <v>74440.86</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -7968,11 +7929,11 @@
       </c>
       <c r="D34" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>6469.4299999999976</v>
+        <v>7270.8299999999963</v>
       </c>
       <c r="E34" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>51530.57</v>
+        <v>50729.170000000006</v>
       </c>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
@@ -8028,11 +7989,11 @@
       </c>
       <c r="D35" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>8237.1200000000008</v>
+        <v>9212.1200000000008</v>
       </c>
       <c r="E35" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>70762.880000000005</v>
+        <v>69787.88</v>
       </c>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
@@ -8188,11 +8149,11 @@
       </c>
       <c r="D40" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[1]"),0)</f>
-        <v>164169.93999999957</v>
+        <v>164169.47999999969</v>
       </c>
       <c r="E40" s="7">
         <f>C40-D40</f>
-        <v>409713.58380952419</v>
+        <v>409714.0438095241</v>
       </c>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
@@ -8224,11 +8185,11 @@
       </c>
       <c r="D41" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>280461.68000000069</v>
+        <v>429012.91000000021</v>
       </c>
       <c r="E41" s="7">
         <f t="shared" ref="E41:E43" si="4">C41-D41</f>
-        <v>1154247.1295238088</v>
+        <v>1005695.8995238093</v>
       </c>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
@@ -8522,10 +8483,10 @@
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <conditionalFormatting sqref="A1:A49 A51:A1048576">
-    <cfRule type="duplicateValues" dxfId="2" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B12">
-    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <tableParts count="14">

</xml_diff>

<commit_message>
Dados atualizados em 07/10/2026 09:30
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48D2EF07-B315-48A9-9137-09EAAA0D77E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E260837-8BDD-4390-B52B-2FA54826FBE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -45,9 +45,9 @@
   <metadataStrings count="5">
     <s v="ThisWorkbookDataModel"/>
     <s v="{[Intervalo 2].[DATA].[All]}"/>
-    <s v="{[Intervalo 2].[DATA].&amp;[2026-10-05T00:00:00]}"/>
-    <s v="{[Intervalo 2].[DES_TIPO_OPERACAO].&amp;[VENDA]}"/>
     <s v="{[Intervalo 2].[PRODUTO].&amp;[MIST PAO DA FAZENDA VIAPANE 10KG]}"/>
+    <s v="{[Intervalo 2].[DATA].&amp;[2026-10-06T00:00:00]}"/>
+    <s v="{[Intervalo 2].[DES_TIPO_OPERACAO].&amp;[VENDA],[Intervalo 2].[DES_TIPO_OPERACAO].&amp;[VENDA SAT]}"/>
   </metadataStrings>
   <mdxMetadata count="4">
     <mdx n="0" f="s">
@@ -2527,8 +2527,8 @@
           <cell r="H2" t="str">
             <v>DATA</v>
           </cell>
-          <cell r="I2" t="str" vm="2">
-            <v>05/10/2026</v>
+          <cell r="I2" t="str" vm="3">
+            <v>06/10/2026</v>
           </cell>
           <cell r="K2" t="str">
             <v>DATA</v>
@@ -2541,8 +2541,8 @@
           <cell r="K3" t="str">
             <v>DES_TIPO_OPERACAO</v>
           </cell>
-          <cell r="L3" t="str" vm="3">
-            <v>VENDA</v>
+          <cell r="L3" t="str" vm="4">
+            <v>(Vários itens)</v>
           </cell>
         </row>
         <row r="4">
@@ -2561,7 +2561,7 @@
           <cell r="K4" t="str">
             <v>PRODUTO</v>
           </cell>
-          <cell r="L4" t="str" vm="4">
+          <cell r="L4" t="str" vm="2">
             <v>MIST PAO DA FAZENDA VIAPANE 10KG</v>
           </cell>
           <cell r="P4" t="str">
@@ -2573,13 +2573,13 @@
             <v>CAMPINAS</v>
           </cell>
           <cell r="F5">
-            <v>4765.8499999999995</v>
+            <v>10063.619999999999</v>
           </cell>
           <cell r="H5" t="str">
             <v>CAMPINAS</v>
           </cell>
           <cell r="I5">
-            <v>3066.1000000000004</v>
+            <v>5297.7699999999995</v>
           </cell>
         </row>
         <row r="6">
@@ -2587,13 +2587,13 @@
             <v>CENTRO</v>
           </cell>
           <cell r="F6">
-            <v>59621.690000000039</v>
+            <v>80195.720000000016</v>
           </cell>
           <cell r="H6" t="str">
             <v>CENTRO</v>
           </cell>
           <cell r="I6">
-            <v>33708.730000000003</v>
+            <v>20574.03</v>
           </cell>
           <cell r="K6" t="str">
             <v>Contagem Distinta de COD_CLIENTE</v>
@@ -2604,16 +2604,16 @@
         </row>
         <row r="7">
           <cell r="E7" t="str">
-            <v>INDAIATUBA</v>
+            <v>IATAGAM JUNIOR</v>
           </cell>
           <cell r="F7">
-            <v>10293.539999999999</v>
+            <v>0</v>
           </cell>
           <cell r="H7" t="str">
-            <v>INDAIATUBA</v>
+            <v>IATAGAM JUNIOR</v>
           </cell>
           <cell r="I7">
-            <v>8426.4</v>
+            <v>0</v>
           </cell>
           <cell r="K7" t="str">
             <v>Rótulos de Linha</v>
@@ -2627,383 +2627,413 @@
         </row>
         <row r="8">
           <cell r="E8" t="str">
-            <v>INTERLAGOS</v>
+            <v>INDAIATUBA</v>
           </cell>
           <cell r="F8">
-            <v>32988.290000000023</v>
+            <v>12079.49</v>
           </cell>
           <cell r="H8" t="str">
-            <v>INTERLAGOS</v>
+            <v>INDAIATUBA</v>
           </cell>
           <cell r="I8">
-            <v>19596.890000000007</v>
+            <v>1785.95</v>
           </cell>
           <cell r="K8" t="str">
-            <v>INTERLAGOS</v>
+            <v>CENTRO</v>
           </cell>
           <cell r="L8">
-            <v>7</v>
+            <v>2</v>
           </cell>
           <cell r="M8">
-            <v>7</v>
+            <v>2</v>
           </cell>
         </row>
         <row r="9">
           <cell r="E9" t="str">
-            <v>JUNDIAI</v>
+            <v>INTERLAGOS</v>
           </cell>
           <cell r="F9">
-            <v>12263.809999999998</v>
+            <v>52315.460000000036</v>
           </cell>
           <cell r="H9" t="str">
-            <v>JUNDIAI</v>
+            <v>INTERLAGOS</v>
           </cell>
           <cell r="I9">
-            <v>4585.25</v>
+            <v>19307.170000000002</v>
           </cell>
           <cell r="K9" t="str">
-            <v>JUNDIAI</v>
+            <v>INTERLAGOS</v>
           </cell>
           <cell r="L9">
-            <v>1</v>
+            <v>7</v>
           </cell>
           <cell r="M9">
-            <v>1</v>
+            <v>7</v>
           </cell>
         </row>
         <row r="10">
           <cell r="E10" t="str">
-            <v>KEY ABC</v>
+            <v>JUNDIAI</v>
           </cell>
           <cell r="F10">
-            <v>2016.6</v>
+            <v>18377.800000000003</v>
           </cell>
           <cell r="H10" t="str">
-            <v>KEY ABC</v>
+            <v>JUNDIAI</v>
           </cell>
           <cell r="I10">
-            <v>0</v>
+            <v>6113.9899999999989</v>
           </cell>
           <cell r="K10" t="str">
-            <v>LESTE MOOCA</v>
+            <v>JUNDIAI</v>
           </cell>
           <cell r="L10">
-            <v>4</v>
+            <v>1</v>
           </cell>
           <cell r="M10">
-            <v>4</v>
+            <v>1</v>
           </cell>
         </row>
         <row r="11">
           <cell r="E11" t="str">
-            <v>KEY CASA</v>
+            <v>KEY ABC</v>
           </cell>
           <cell r="F11">
-            <v>63215.649999999965</v>
+            <v>41478.5</v>
           </cell>
           <cell r="H11" t="str">
-            <v>KEY CASA</v>
+            <v>KEY ABC</v>
           </cell>
           <cell r="I11">
-            <v>59732.449999999968</v>
+            <v>39461.899999999994</v>
           </cell>
           <cell r="K11" t="str">
-            <v>OSASCO</v>
+            <v>LESTE MOOCA</v>
           </cell>
           <cell r="L11">
-            <v>11</v>
+            <v>8</v>
           </cell>
           <cell r="M11">
-            <v>11</v>
+            <v>8</v>
           </cell>
         </row>
         <row r="12">
           <cell r="E12" t="str">
-            <v>KEY INTERIOR</v>
+            <v>KEY CASA</v>
           </cell>
           <cell r="F12">
-            <v>94941.200000000012</v>
+            <v>80120.350000000079</v>
           </cell>
           <cell r="H12" t="str">
-            <v>KEY INTERIOR</v>
+            <v>KEY CASA</v>
           </cell>
           <cell r="I12">
-            <v>87269.200000000012</v>
+            <v>17635.600000000006</v>
           </cell>
           <cell r="K12" t="str">
-            <v>PIRITUBA</v>
+            <v>OSASCO</v>
           </cell>
           <cell r="L12">
-            <v>2</v>
+            <v>15</v>
           </cell>
           <cell r="M12">
-            <v>2</v>
+            <v>15</v>
           </cell>
         </row>
         <row r="13">
           <cell r="E13" t="str">
-            <v>KEY SJC</v>
+            <v>KEY INTERIOR</v>
           </cell>
           <cell r="F13">
-            <v>4315.6000000000004</v>
+            <v>212283.80000000005</v>
           </cell>
           <cell r="H13" t="str">
-            <v>KEY SJC</v>
+            <v>KEY INTERIOR</v>
           </cell>
           <cell r="I13">
-            <v>4315.6000000000004</v>
+            <v>117342.60000000003</v>
           </cell>
           <cell r="K13" t="str">
-            <v>SANTO ANDRE</v>
+            <v>PIRITUBA</v>
           </cell>
           <cell r="L13">
-            <v>2</v>
+            <v>4</v>
           </cell>
           <cell r="M13">
-            <v>2</v>
+            <v>4</v>
           </cell>
         </row>
         <row r="14">
           <cell r="E14" t="str">
-            <v>KEY SP</v>
+            <v>KEY SJC</v>
           </cell>
           <cell r="F14">
-            <v>15188.2</v>
+            <v>4315.6000000000004</v>
           </cell>
           <cell r="H14" t="str">
-            <v>KEY SP</v>
+            <v>KEY SJC</v>
           </cell>
           <cell r="I14">
-            <v>13814.5</v>
+            <v>0</v>
           </cell>
           <cell r="K14" t="str">
-            <v>SBC</v>
+            <v>SANTO ANDRE</v>
           </cell>
           <cell r="L14">
-            <v>4</v>
+            <v>3</v>
           </cell>
           <cell r="M14">
-            <v>4</v>
+            <v>3</v>
           </cell>
         </row>
         <row r="15">
           <cell r="E15" t="str">
-            <v>KEY ZL</v>
+            <v>KEY SP</v>
           </cell>
           <cell r="F15">
-            <v>40356.879999999961</v>
+            <v>38918.429999999993</v>
           </cell>
           <cell r="H15" t="str">
-            <v>KEY ZL</v>
+            <v>KEY SP</v>
           </cell>
           <cell r="I15">
-            <v>34294.479999999967</v>
+            <v>23730.23</v>
           </cell>
           <cell r="K15" t="str">
-            <v>SJC</v>
+            <v>SBC</v>
           </cell>
           <cell r="L15">
-            <v>1</v>
+            <v>5</v>
           </cell>
           <cell r="M15">
-            <v>1</v>
+            <v>5</v>
           </cell>
         </row>
         <row r="16">
           <cell r="E16" t="str">
-            <v>LESTE MOOCA</v>
+            <v>KEY ZL</v>
           </cell>
           <cell r="F16">
-            <v>20123.86</v>
+            <v>78869.479999999967</v>
           </cell>
           <cell r="H16" t="str">
-            <v>LESTE MOOCA</v>
+            <v>KEY ZL</v>
           </cell>
           <cell r="I16">
-            <v>13425.409999999993</v>
+            <v>38512.6</v>
           </cell>
           <cell r="K16" t="str">
-            <v>Total Geral</v>
+            <v>SJC</v>
           </cell>
           <cell r="L16">
-            <v>32</v>
+            <v>1</v>
           </cell>
           <cell r="M16">
-            <v>32</v>
+            <v>1</v>
           </cell>
         </row>
         <row r="17">
           <cell r="E17" t="str">
-            <v>LESTE PENHA</v>
+            <v>LESTE MOOCA</v>
           </cell>
           <cell r="F17">
-            <v>24013.079999999998</v>
+            <v>34826.190000000031</v>
           </cell>
           <cell r="H17" t="str">
-            <v>LESTE PENHA</v>
+            <v>LESTE MOOCA</v>
           </cell>
           <cell r="I17">
-            <v>14168.76</v>
+            <v>14702.329999999998</v>
+          </cell>
+          <cell r="K17" t="str">
+            <v>SJC/VALE</v>
+          </cell>
+          <cell r="L17">
+            <v>2</v>
+          </cell>
+          <cell r="M17">
+            <v>2</v>
           </cell>
         </row>
         <row r="18">
           <cell r="E18" t="str">
-            <v>LESTE TATUAPE</v>
+            <v>LESTE PENHA</v>
           </cell>
           <cell r="F18">
-            <v>14652.809999999996</v>
+            <v>29690.979999999996</v>
           </cell>
           <cell r="H18" t="str">
-            <v>LESTE TATUAPE</v>
+            <v>LESTE PENHA</v>
           </cell>
           <cell r="I18">
-            <v>12159.649999999998</v>
+            <v>5677.8999999999987</v>
+          </cell>
+          <cell r="K18" t="str">
+            <v>Total Geral</v>
+          </cell>
+          <cell r="L18">
+            <v>48</v>
+          </cell>
+          <cell r="M18">
+            <v>48</v>
           </cell>
         </row>
         <row r="19">
           <cell r="E19" t="str">
-            <v>MOGI</v>
+            <v>LESTE TATUAPE</v>
           </cell>
           <cell r="F19">
-            <v>5238.87</v>
+            <v>22063.71000000001</v>
           </cell>
           <cell r="H19" t="str">
-            <v>MOGI</v>
+            <v>LESTE TATUAPE</v>
           </cell>
           <cell r="I19">
-            <v>4213.3100000000004</v>
+            <v>7410.8999999999987</v>
           </cell>
         </row>
         <row r="20">
           <cell r="E20" t="str">
-            <v>NORTE</v>
+            <v>MOGI</v>
           </cell>
           <cell r="F20">
-            <v>37419.070000000022</v>
+            <v>6954.27</v>
           </cell>
           <cell r="H20" t="str">
-            <v>NORTE</v>
+            <v>MOGI</v>
           </cell>
           <cell r="I20">
-            <v>23646.760000000002</v>
+            <v>1715.4</v>
           </cell>
         </row>
         <row r="21">
           <cell r="E21" t="str">
-            <v>OSASCO</v>
+            <v>NORTE</v>
           </cell>
           <cell r="F21">
-            <v>52714.41</v>
+            <v>51568.700000000055</v>
           </cell>
           <cell r="H21" t="str">
-            <v>OSASCO</v>
+            <v>NORTE</v>
           </cell>
           <cell r="I21">
-            <v>28873.46000000001</v>
+            <v>14149.629999999996</v>
           </cell>
         </row>
         <row r="22">
           <cell r="E22" t="str">
-            <v>PIRITUBA</v>
+            <v>OSASCO</v>
           </cell>
           <cell r="F22">
-            <v>16296.58</v>
+            <v>68129</v>
           </cell>
           <cell r="H22" t="str">
-            <v>PIRITUBA</v>
+            <v>OSASCO</v>
           </cell>
           <cell r="I22">
-            <v>10320.560000000003</v>
+            <v>15414.589999999998</v>
           </cell>
         </row>
         <row r="23">
           <cell r="E23" t="str">
-            <v>SANTO ANDRE</v>
+            <v>PIRITUBA</v>
           </cell>
           <cell r="F23">
-            <v>20419.93</v>
+            <v>29370.71000000001</v>
           </cell>
           <cell r="H23" t="str">
-            <v>SANTO ANDRE</v>
+            <v>PIRITUBA</v>
           </cell>
           <cell r="I23">
-            <v>16407.95</v>
+            <v>13074.129999999997</v>
           </cell>
         </row>
         <row r="24">
           <cell r="E24" t="str">
-            <v>SBC</v>
+            <v>SANTO ANDRE</v>
           </cell>
           <cell r="F24">
-            <v>32294.379999999983</v>
+            <v>26662.550000000017</v>
           </cell>
           <cell r="H24" t="str">
-            <v>SBC</v>
+            <v>SANTO ANDRE</v>
           </cell>
           <cell r="I24">
-            <v>13145.080000000002</v>
+            <v>6242.6200000000008</v>
           </cell>
         </row>
         <row r="25">
           <cell r="E25" t="str">
-            <v>SJC</v>
+            <v>SBC</v>
           </cell>
           <cell r="F25">
-            <v>13559.139999999998</v>
+            <v>49731.210000000028</v>
           </cell>
           <cell r="H25" t="str">
-            <v>SJC</v>
+            <v>SBC</v>
           </cell>
           <cell r="I25">
-            <v>10532.269999999999</v>
+            <v>17436.830000000009</v>
           </cell>
         </row>
         <row r="26">
           <cell r="E26" t="str">
-            <v>SJC/VALE</v>
+            <v>SJC</v>
           </cell>
           <cell r="F26">
-            <v>7270.8299999999963</v>
+            <v>16084.539999999992</v>
           </cell>
           <cell r="H26" t="str">
-            <v>SJC/VALE</v>
+            <v>SJC</v>
           </cell>
           <cell r="I26">
-            <v>4425.9999999999991</v>
+            <v>2525.3999999999992</v>
           </cell>
         </row>
         <row r="27">
           <cell r="E27" t="str">
-            <v>VENDEDOR INTERNO 1</v>
+            <v>SJC/VALE</v>
           </cell>
           <cell r="F27">
-            <v>9212.1200000000008</v>
+            <v>9566.7999999999956</v>
           </cell>
           <cell r="H27" t="str">
-            <v>VENDEDOR INTERNO 1</v>
+            <v>SJC/VALE</v>
           </cell>
           <cell r="I27">
-            <v>8884.1</v>
+            <v>2261.0300000000002</v>
           </cell>
         </row>
         <row r="28">
           <cell r="E28" t="str">
-            <v>Total Geral</v>
+            <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="F28">
-            <v>593182.38999999885</v>
+            <v>13919.82</v>
           </cell>
           <cell r="H28" t="str">
-            <v>Total Geral</v>
+            <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="I28">
-            <v>429012.9099999998</v>
+            <v>4707.7</v>
           </cell>
           <cell r="K28" t="str">
             <v>POSITIVAÇÃO GERAL</v>
           </cell>
         </row>
         <row r="29">
+          <cell r="E29" t="str">
+            <v>Total Geral</v>
+          </cell>
+          <cell r="F29">
+            <v>987586.73000000091</v>
+          </cell>
+          <cell r="H29" t="str">
+            <v>Total Geral</v>
+          </cell>
+          <cell r="I29">
+            <v>395080.29999999946</v>
+          </cell>
           <cell r="K29" t="str">
             <v>DATA</v>
           </cell>
@@ -3015,8 +3045,8 @@
           <cell r="K30" t="str">
             <v>DES_TIPO_OPERACAO</v>
           </cell>
-          <cell r="L30" t="str" vm="3">
-            <v>VENDA</v>
+          <cell r="L30" t="str" vm="4">
+            <v>(Vários itens)</v>
           </cell>
         </row>
         <row r="32">
@@ -3046,10 +3076,10 @@
             <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="L34">
-            <v>33</v>
+            <v>42</v>
           </cell>
           <cell r="M34">
-            <v>33</v>
+            <v>42</v>
           </cell>
         </row>
         <row r="35">
@@ -3057,10 +3087,10 @@
             <v>Total Geral</v>
           </cell>
           <cell r="L35">
-            <v>33</v>
+            <v>42</v>
           </cell>
           <cell r="M35">
-            <v>33</v>
+            <v>42</v>
           </cell>
         </row>
         <row r="39">
@@ -3068,7 +3098,7 @@
             <v>CAMPINAS</v>
           </cell>
           <cell r="B39">
-            <v>4820</v>
+            <v>5440</v>
           </cell>
         </row>
         <row r="40">
@@ -3076,7 +3106,7 @@
             <v>CENTRO</v>
           </cell>
           <cell r="B40">
-            <v>25020</v>
+            <v>11360</v>
           </cell>
         </row>
         <row r="41">
@@ -3084,7 +3114,7 @@
             <v>INDAIATUBA</v>
           </cell>
           <cell r="B41">
-            <v>6580</v>
+            <v>5070</v>
           </cell>
         </row>
         <row r="42">
@@ -3092,7 +3122,7 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="B42">
-            <v>17000</v>
+            <v>13370</v>
           </cell>
         </row>
         <row r="43">
@@ -3100,7 +3130,7 @@
             <v>JUNDIAI</v>
           </cell>
           <cell r="B43">
-            <v>5990</v>
+            <v>4460</v>
           </cell>
         </row>
         <row r="44">
@@ -3108,7 +3138,7 @@
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="B44">
-            <v>18340</v>
+            <v>10320</v>
           </cell>
         </row>
         <row r="45">
@@ -3116,7 +3146,7 @@
             <v>LESTE PENHA</v>
           </cell>
           <cell r="B45">
-            <v>9950</v>
+            <v>8680</v>
           </cell>
         </row>
         <row r="46">
@@ -3124,7 +3154,7 @@
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="B46">
-            <v>16120</v>
+            <v>11680</v>
           </cell>
         </row>
         <row r="47">
@@ -3132,7 +3162,7 @@
             <v>MOGI</v>
           </cell>
           <cell r="B47">
-            <v>4590</v>
+            <v>7100</v>
           </cell>
           <cell r="P47" t="str">
             <v>Soma de TOTAL</v>
@@ -3143,7 +3173,7 @@
             <v>NORTE</v>
           </cell>
           <cell r="B48">
-            <v>13060</v>
+            <v>16230</v>
           </cell>
         </row>
         <row r="49">
@@ -3151,7 +3181,7 @@
             <v>OSASCO</v>
           </cell>
           <cell r="B49">
-            <v>20980</v>
+            <v>16760</v>
           </cell>
         </row>
         <row r="50">
@@ -3159,7 +3189,7 @@
             <v>PIRITUBA</v>
           </cell>
           <cell r="B50">
-            <v>9390</v>
+            <v>10030</v>
           </cell>
         </row>
         <row r="51">
@@ -3167,7 +3197,7 @@
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="B51">
-            <v>13880</v>
+            <v>13010</v>
           </cell>
         </row>
         <row r="52">
@@ -3175,7 +3205,7 @@
             <v>SBC</v>
           </cell>
           <cell r="B52">
-            <v>19350</v>
+            <v>14910</v>
           </cell>
         </row>
         <row r="53">
@@ -3183,7 +3213,7 @@
             <v>SJC</v>
           </cell>
           <cell r="B53">
-            <v>5850</v>
+            <v>4770</v>
           </cell>
         </row>
         <row r="54">
@@ -3191,7 +3221,7 @@
             <v>SJC/VALE</v>
           </cell>
           <cell r="B54">
-            <v>3770</v>
+            <v>3190</v>
           </cell>
         </row>
         <row r="55">
@@ -3199,7 +3229,7 @@
             <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="B55">
-            <v>5530</v>
+            <v>3720</v>
           </cell>
         </row>
         <row r="63">
@@ -3384,27 +3414,27 @@
             <v>36</v>
           </cell>
           <cell r="F137">
-            <v>33</v>
+            <v>42</v>
           </cell>
           <cell r="H137" t="str">
-            <v>D</v>
+            <v>C</v>
           </cell>
           <cell r="I137">
-            <v>3</v>
+            <v>14</v>
           </cell>
         </row>
         <row r="138">
           <cell r="E138">
             <v>14</v>
           </cell>
-          <cell r="F138" t="e">
-            <v>#N/A</v>
-          </cell>
-          <cell r="H138" t="e">
-            <v>#N/A</v>
-          </cell>
-          <cell r="I138" t="e">
-            <v>#N/A</v>
+          <cell r="F138">
+            <v>2</v>
+          </cell>
+          <cell r="H138" t="str">
+            <v>D</v>
+          </cell>
+          <cell r="I138">
+            <v>12</v>
           </cell>
         </row>
         <row r="139">
@@ -3412,13 +3442,13 @@
             <v>14</v>
           </cell>
           <cell r="F139">
-            <v>11</v>
+            <v>15</v>
           </cell>
           <cell r="H139" t="str">
-            <v>D</v>
+            <v>C</v>
           </cell>
           <cell r="I139">
-            <v>3</v>
+            <v>9.5</v>
           </cell>
         </row>
         <row r="140">
@@ -3440,13 +3470,13 @@
             <v>14</v>
           </cell>
           <cell r="F141">
-            <v>4</v>
+            <v>8</v>
           </cell>
           <cell r="H141" t="str">
             <v>D</v>
           </cell>
           <cell r="I141">
-            <v>10</v>
+            <v>6</v>
           </cell>
         </row>
         <row r="142">
@@ -3454,83 +3484,83 @@
             <v>14</v>
           </cell>
           <cell r="F142">
-            <v>2</v>
+            <v>3</v>
           </cell>
           <cell r="H142" t="str">
             <v>D</v>
           </cell>
           <cell r="I142">
-            <v>12</v>
+            <v>11</v>
           </cell>
         </row>
         <row r="143">
           <cell r="E143">
             <v>14</v>
           </cell>
-          <cell r="F143" t="e">
-            <v>#N/A</v>
-          </cell>
-          <cell r="H143" t="e">
-            <v>#N/A</v>
-          </cell>
-          <cell r="I143" t="e">
-            <v>#N/A</v>
+          <cell r="F143">
+            <v>0</v>
+          </cell>
+          <cell r="H143" t="str">
+            <v>D</v>
+          </cell>
+          <cell r="I143">
+            <v>14</v>
           </cell>
         </row>
         <row r="144">
           <cell r="E144">
             <v>0</v>
           </cell>
-          <cell r="F144" t="e">
-            <v>#N/A</v>
-          </cell>
-          <cell r="H144" t="e">
-            <v>#N/A</v>
-          </cell>
-          <cell r="I144" t="e">
-            <v>#N/A</v>
+          <cell r="F144">
+            <v>0</v>
+          </cell>
+          <cell r="H144" t="str">
+            <v>OBJETIVO ALCANÇADO</v>
+          </cell>
+          <cell r="I144">
+            <v>0</v>
           </cell>
         </row>
         <row r="145">
           <cell r="E145">
             <v>14</v>
           </cell>
-          <cell r="F145" t="e">
-            <v>#N/A</v>
-          </cell>
-          <cell r="H145" t="e">
-            <v>#N/A</v>
-          </cell>
-          <cell r="I145" t="e">
-            <v>#N/A</v>
+          <cell r="F145">
+            <v>2</v>
+          </cell>
+          <cell r="H145" t="str">
+            <v>D</v>
+          </cell>
+          <cell r="I145">
+            <v>12</v>
           </cell>
         </row>
         <row r="146">
           <cell r="E146">
             <v>14</v>
           </cell>
-          <cell r="F146" t="e">
-            <v>#N/A</v>
-          </cell>
-          <cell r="H146" t="e">
-            <v>#N/A</v>
-          </cell>
-          <cell r="I146" t="e">
-            <v>#N/A</v>
+          <cell r="F146">
+            <v>0</v>
+          </cell>
+          <cell r="H146" t="str">
+            <v>D</v>
+          </cell>
+          <cell r="I146">
+            <v>14</v>
           </cell>
         </row>
         <row r="147">
           <cell r="E147">
             <v>14</v>
           </cell>
-          <cell r="F147" t="e">
-            <v>#N/A</v>
-          </cell>
-          <cell r="H147" t="e">
-            <v>#N/A</v>
-          </cell>
-          <cell r="I147" t="e">
-            <v>#N/A</v>
+          <cell r="F147">
+            <v>0</v>
+          </cell>
+          <cell r="H147" t="str">
+            <v>D</v>
+          </cell>
+          <cell r="I147">
+            <v>14</v>
           </cell>
         </row>
         <row r="148">
@@ -3552,27 +3582,27 @@
             <v>14</v>
           </cell>
           <cell r="F149">
-            <v>2</v>
+            <v>4</v>
           </cell>
           <cell r="H149" t="str">
             <v>D</v>
           </cell>
           <cell r="I149">
-            <v>12</v>
+            <v>10</v>
           </cell>
         </row>
         <row r="150">
           <cell r="E150">
             <v>14</v>
           </cell>
-          <cell r="F150" t="e">
-            <v>#N/A</v>
-          </cell>
-          <cell r="H150" t="e">
-            <v>#N/A</v>
-          </cell>
-          <cell r="I150" t="e">
-            <v>#N/A</v>
+          <cell r="F150">
+            <v>0</v>
+          </cell>
+          <cell r="H150" t="str">
+            <v>D</v>
+          </cell>
+          <cell r="I150">
+            <v>14</v>
           </cell>
         </row>
         <row r="151">
@@ -3580,52 +3610,52 @@
             <v>14</v>
           </cell>
           <cell r="F151">
-            <v>4</v>
+            <v>5</v>
           </cell>
           <cell r="H151" t="str">
             <v>D</v>
           </cell>
           <cell r="I151">
-            <v>10</v>
+            <v>9</v>
           </cell>
         </row>
         <row r="152">
           <cell r="E152">
             <v>14</v>
           </cell>
-          <cell r="F152" t="e">
-            <v>#N/A</v>
-          </cell>
-          <cell r="H152" t="e">
-            <v>#N/A</v>
-          </cell>
-          <cell r="I152" t="e">
-            <v>#N/A</v>
+          <cell r="F152">
+            <v>0</v>
+          </cell>
+          <cell r="H152" t="str">
+            <v>D</v>
+          </cell>
+          <cell r="I152">
+            <v>14</v>
           </cell>
         </row>
         <row r="153">
           <cell r="E153">
             <v>14</v>
           </cell>
-          <cell r="F153" t="e">
-            <v>#N/A</v>
-          </cell>
-          <cell r="H153" t="e">
-            <v>#N/A</v>
-          </cell>
-          <cell r="I153" t="e">
-            <v>#N/A</v>
+          <cell r="F153">
+            <v>0</v>
+          </cell>
+          <cell r="H153" t="str">
+            <v>D</v>
+          </cell>
+          <cell r="I153">
+            <v>14</v>
           </cell>
         </row>
         <row r="154">
           <cell r="E154">
             <v>260</v>
           </cell>
-          <cell r="F154" t="e">
-            <v>#N/A</v>
-          </cell>
-          <cell r="I154" t="e">
-            <v>#N/A</v>
+          <cell r="F154">
+            <v>90</v>
+          </cell>
+          <cell r="I154">
+            <v>200.5</v>
           </cell>
         </row>
         <row r="158">
@@ -3647,13 +3677,13 @@
             <v>39600</v>
           </cell>
           <cell r="F159">
-            <v>13559.139999999998</v>
+            <v>16084.539999999992</v>
           </cell>
           <cell r="H159" t="str">
             <v>D</v>
           </cell>
           <cell r="I159">
-            <v>26040.86</v>
+            <v>23515.460000000006</v>
           </cell>
         </row>
         <row r="160">
@@ -3661,13 +3691,13 @@
             <v>35550</v>
           </cell>
           <cell r="F160">
-            <v>9212.1200000000008</v>
+            <v>13919.82</v>
           </cell>
           <cell r="H160" t="str">
             <v>D</v>
           </cell>
           <cell r="I160">
-            <v>26337.879999999997</v>
+            <v>21630.18</v>
           </cell>
         </row>
         <row r="161">
@@ -3675,13 +3705,13 @@
             <v>155250</v>
           </cell>
           <cell r="F161">
-            <v>59621.690000000039</v>
+            <v>80195.720000000016</v>
           </cell>
           <cell r="H161" t="str">
             <v>D</v>
           </cell>
           <cell r="I161">
-            <v>95628.309999999969</v>
+            <v>75054.279999999984</v>
           </cell>
         </row>
         <row r="162">
@@ -3689,13 +3719,13 @@
             <v>149175</v>
           </cell>
           <cell r="F162">
-            <v>52714.41</v>
+            <v>68129</v>
           </cell>
           <cell r="H162" t="str">
             <v>D</v>
           </cell>
           <cell r="I162">
-            <v>96460.59</v>
+            <v>81046</v>
           </cell>
         </row>
         <row r="163">
@@ -3703,13 +3733,13 @@
             <v>126450</v>
           </cell>
           <cell r="F163">
-            <v>32988.290000000023</v>
+            <v>52315.460000000036</v>
           </cell>
           <cell r="H163" t="str">
             <v>D</v>
           </cell>
           <cell r="I163">
-            <v>93461.709999999977</v>
+            <v>74134.539999999964</v>
           </cell>
         </row>
         <row r="164">
@@ -3717,13 +3747,13 @@
             <v>92700</v>
           </cell>
           <cell r="F164">
-            <v>20123.86</v>
+            <v>34826.190000000031</v>
           </cell>
           <cell r="H164" t="str">
             <v>D</v>
           </cell>
           <cell r="I164">
-            <v>72576.14</v>
+            <v>57873.809999999969</v>
           </cell>
         </row>
         <row r="165">
@@ -3731,27 +3761,27 @@
             <v>78750</v>
           </cell>
           <cell r="F165">
-            <v>20419.93</v>
+            <v>26662.550000000017</v>
           </cell>
           <cell r="H165" t="str">
             <v>D</v>
           </cell>
           <cell r="I165">
-            <v>58330.07</v>
+            <v>52087.449999999983</v>
           </cell>
         </row>
         <row r="166">
           <cell r="E166">
-            <v>121131</v>
+            <v>122400</v>
           </cell>
           <cell r="F166">
-            <v>37419.070000000022</v>
+            <v>51568.700000000055</v>
           </cell>
           <cell r="H166" t="str">
             <v>D</v>
           </cell>
           <cell r="I166">
-            <v>83711.929999999978</v>
+            <v>70831.299999999945</v>
           </cell>
         </row>
         <row r="167">
@@ -3773,13 +3803,13 @@
             <v>26100</v>
           </cell>
           <cell r="F168">
-            <v>7270.8299999999963</v>
+            <v>9566.7999999999956</v>
           </cell>
           <cell r="H168" t="str">
             <v>D</v>
           </cell>
           <cell r="I168">
-            <v>18829.170000000006</v>
+            <v>16533.200000000004</v>
           </cell>
         </row>
         <row r="169">
@@ -3787,13 +3817,13 @@
             <v>43200</v>
           </cell>
           <cell r="F169">
-            <v>10293.539999999999</v>
+            <v>12079.49</v>
           </cell>
           <cell r="H169" t="str">
             <v>D</v>
           </cell>
           <cell r="I169">
-            <v>32906.46</v>
+            <v>31120.510000000002</v>
           </cell>
         </row>
         <row r="170">
@@ -3801,13 +3831,13 @@
             <v>31725</v>
           </cell>
           <cell r="F170">
-            <v>4765.8499999999995</v>
+            <v>10063.619999999999</v>
           </cell>
           <cell r="H170" t="str">
             <v>D</v>
           </cell>
           <cell r="I170">
-            <v>26959.15</v>
+            <v>21661.38</v>
           </cell>
         </row>
         <row r="171">
@@ -3815,13 +3845,13 @@
             <v>37800</v>
           </cell>
           <cell r="F171">
-            <v>12263.809999999998</v>
+            <v>18377.800000000003</v>
           </cell>
           <cell r="H171" t="str">
             <v>D</v>
           </cell>
           <cell r="I171">
-            <v>25536.190000000002</v>
+            <v>19422.199999999997</v>
           </cell>
         </row>
         <row r="172">
@@ -3829,27 +3859,27 @@
             <v>63900</v>
           </cell>
           <cell r="F172">
-            <v>16296.58</v>
+            <v>29370.71000000001</v>
           </cell>
           <cell r="H172" t="str">
             <v>D</v>
           </cell>
           <cell r="I172">
-            <v>47603.42</v>
+            <v>34529.289999999994</v>
           </cell>
         </row>
         <row r="173">
           <cell r="E173">
-            <v>74970</v>
+            <v>76050</v>
           </cell>
           <cell r="F173">
-            <v>24013.079999999998</v>
+            <v>29690.979999999996</v>
           </cell>
           <cell r="H173" t="str">
             <v>D</v>
           </cell>
           <cell r="I173">
-            <v>50956.92</v>
+            <v>46359.020000000004</v>
           </cell>
         </row>
         <row r="174">
@@ -3857,13 +3887,13 @@
             <v>121500</v>
           </cell>
           <cell r="F174">
-            <v>32294.379999999983</v>
+            <v>49731.210000000028</v>
           </cell>
           <cell r="H174" t="str">
             <v>D</v>
           </cell>
           <cell r="I174">
-            <v>89205.620000000024</v>
+            <v>71768.789999999979</v>
           </cell>
         </row>
         <row r="175">
@@ -3871,13 +3901,13 @@
             <v>42975</v>
           </cell>
           <cell r="F175">
-            <v>5238.87</v>
+            <v>6954.27</v>
           </cell>
           <cell r="H175" t="str">
             <v>D</v>
           </cell>
           <cell r="I175">
-            <v>37736.129999999997</v>
+            <v>36020.729999999996</v>
           </cell>
         </row>
         <row r="176">
@@ -3885,24 +3915,24 @@
             <v>97875</v>
           </cell>
           <cell r="F176">
-            <v>14652.809999999996</v>
+            <v>22063.71000000001</v>
           </cell>
           <cell r="H176" t="str">
             <v>D</v>
           </cell>
           <cell r="I176">
-            <v>83222.19</v>
+            <v>75811.289999999994</v>
           </cell>
         </row>
         <row r="177">
           <cell r="E177">
-            <v>1338651</v>
+            <v>1341000</v>
           </cell>
           <cell r="F177">
-            <v>373148.26000000007</v>
+            <v>531600.57000000018</v>
           </cell>
           <cell r="I177">
-            <v>965502.74</v>
+            <v>809399.4299999997</v>
           </cell>
         </row>
       </sheetData>
@@ -4782,7 +4812,7 @@
       </c>
       <c r="AN3" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI3,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>13559.139999999998</v>
+        <v>16084.539999999992</v>
       </c>
       <c r="AO3" s="26" t="str" cm="1">
         <f t="array" ref="AO3">_xlfn.IFS(AN3&gt;=AJ3,"A",AN3&gt;=AK3,"B",AN3&gt;=AL3,"C",AN3&gt;=AM3,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -4794,7 +4824,7 @@
       </c>
       <c r="AQ3" s="25" cm="1">
         <f t="array" ref="AQ3">_xlfn.IFS(AP3="D",MAX(AM3-AN3,0),AP3="C",MAX(AL3-AN3,0),AP3="B",MAX(AK3-AN3,0),AP3="A",MAX(AJ3-AN3,0),AP3="OBJETIVO ALCANÇADO",0)</f>
-        <v>26040.86</v>
+        <v>23515.460000000006</v>
       </c>
     </row>
     <row r="4" spans="1:43" x14ac:dyDescent="0.25">
@@ -4804,7 +4834,7 @@
       </c>
       <c r="C4" s="2">
         <f>SUM(C10:C36)</f>
-        <v>6025777</v>
+        <v>6031000</v>
       </c>
       <c r="D4" s="2"/>
       <c r="E4" s="4"/>
@@ -4815,7 +4845,7 @@
       </c>
       <c r="I4" s="7">
         <f>SUM(I10:I27)</f>
-        <v>200220</v>
+        <v>160100</v>
       </c>
       <c r="J4" s="4"/>
       <c r="K4" s="4"/>
@@ -4862,19 +4892,19 @@
       </c>
       <c r="AD4" s="31">
         <f>IFERROR(_xlfn.XLOOKUP(Y4,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$M:$M,0),0)</f>
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="AE4" s="31" t="str" cm="1">
         <f t="array" ref="AE4">_xlfn.IFS(AD4&gt;=Z4,"A",AD4&gt;=AA4,"B",AD4&gt;=AB4,"C",AD4&gt;=AC4,"D",TRUE,"NÃO ATINGIDO")</f>
-        <v>NÃO ATINGIDO</v>
+        <v>D</v>
       </c>
       <c r="AF4" s="31" t="str" cm="1">
         <f t="array" ref="AF4">_xlfn.IFS(AE4="NÃO ATINGIDO","D",AE4="D","C",AE4="C","B",AE4="B","A",AE4="A","OBJETIVO ALCANÇADO")</f>
-        <v>D</v>
+        <v>C</v>
       </c>
       <c r="AG4" s="31" cm="1">
         <f t="array" ref="AG4">_xlfn.IFS(AF4="D",MAX(AC4-AD4,0),AF4="C",MAX(AB4-AD4,0),AF4="B",MAX(AA4-AD4,0),AF4="A",MAX(Z4-AD4,0),AF4="OBJETIVO ALCANÇADO",0)</f>
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="AI4" t="s">
         <v>24</v>
@@ -4897,7 +4927,7 @@
       </c>
       <c r="AN4" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI4,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>9212.1200000000008</v>
+        <v>13919.82</v>
       </c>
       <c r="AO4" s="26" t="str" cm="1">
         <f t="array" ref="AO4">_xlfn.IFS(AN4&gt;=AJ4,"A",AN4&gt;=AK4,"B",AN4&gt;=AL4,"C",AN4&gt;=AM4,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -4909,7 +4939,7 @@
       </c>
       <c r="AQ4" s="25" cm="1">
         <f t="array" ref="AQ4">_xlfn.IFS(AP4="D",MAX(AM4-AN4,0),AP4="C",MAX(AL4-AN4,0),AP4="B",MAX(AK4-AN4,0),AP4="A",MAX(AJ4-AN4,0),AP4="OBJETIVO ALCANÇADO",0)</f>
-        <v>26337.879999999997</v>
+        <v>21630.18</v>
       </c>
     </row>
     <row r="5" spans="1:43" x14ac:dyDescent="0.25">
@@ -4919,7 +4949,7 @@
       </c>
       <c r="C5" s="2">
         <f>SUM(D10:D36)</f>
-        <v>593182.3899999999</v>
+        <v>987586.73000000033</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -4930,7 +4960,7 @@
       </c>
       <c r="I5" s="7">
         <f ca="1">SUM(J10:J27)</f>
-        <v>229586.68000000005</v>
+        <v>158397.37</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -4941,7 +4971,7 @@
       </c>
       <c r="O5" s="7">
         <f>SUM(P11:P17)</f>
-        <v>59732.449999999968</v>
+        <v>76637.150000000081</v>
       </c>
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
@@ -4952,7 +4982,7 @@
       </c>
       <c r="U5" s="4">
         <f ca="1">SUM(V10:V26)</f>
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -5012,7 +5042,7 @@
       </c>
       <c r="AN5" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI5,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>59621.690000000039</v>
+        <v>80195.720000000016</v>
       </c>
       <c r="AO5" s="26" t="str" cm="1">
         <f t="array" ref="AO5">_xlfn.IFS(AN5&gt;=AJ5,"A",AN5&gt;=AK5,"B",AN5&gt;=AL5,"C",AN5&gt;=AM5,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -5024,7 +5054,7 @@
       </c>
       <c r="AQ5" s="25" cm="1">
         <f t="array" ref="AQ5">_xlfn.IFS(AP5="D",MAX(AM5-AN5,0),AP5="C",MAX(AL5-AN5,0),AP5="B",MAX(AK5-AN5,0),AP5="A",MAX(AJ5-AN5,0),AP5="OBJETIVO ALCANÇADO",0)</f>
-        <v>95628.309999999969</v>
+        <v>75054.279999999984</v>
       </c>
     </row>
     <row r="6" spans="1:43" x14ac:dyDescent="0.25">
@@ -5034,7 +5064,7 @@
       </c>
       <c r="C6" s="2">
         <f>C4-C5</f>
-        <v>5432594.6100000003</v>
+        <v>5043413.2699999996</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="4"/>
@@ -5045,7 +5075,7 @@
       </c>
       <c r="I6" s="7">
         <f ca="1">I4-I5</f>
-        <v>-29366.680000000051</v>
+        <v>1702.6300000000047</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -5056,7 +5086,7 @@
       </c>
       <c r="O6" s="7">
         <f>O4-O5</f>
-        <v>-59732.449999999968</v>
+        <v>-76637.150000000081</v>
       </c>
       <c r="P6" s="4"/>
       <c r="Q6" s="4"/>
@@ -5067,7 +5097,7 @@
       </c>
       <c r="U6" s="4">
         <f ca="1">U4-U5</f>
-        <v>528</v>
+        <v>512</v>
       </c>
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
@@ -5127,7 +5157,7 @@
       </c>
       <c r="AN6" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI6,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>52714.41</v>
+        <v>68129</v>
       </c>
       <c r="AO6" s="26" t="str" cm="1">
         <f t="array" ref="AO6">_xlfn.IFS(AN6&gt;=AJ6,"A",AN6&gt;=AK6,"B",AN6&gt;=AL6,"C",AN6&gt;=AM6,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -5139,7 +5169,7 @@
       </c>
       <c r="AQ6" s="25" cm="1">
         <f t="array" ref="AQ6">_xlfn.IFS(AP6="D",MAX(AM6-AN6,0),AP6="C",MAX(AL6-AN6,0),AP6="B",MAX(AK6-AN6,0),AP6="A",MAX(AJ6-AN6,0),AP6="OBJETIVO ALCANÇADO",0)</f>
-        <v>96460.59</v>
+        <v>81046</v>
       </c>
     </row>
     <row r="7" spans="1:43" x14ac:dyDescent="0.25">
@@ -5149,7 +5179,7 @@
       </c>
       <c r="C7" s="3">
         <f>1-(C6/C4)</f>
-        <v>9.8440813524961146E-2</v>
+        <v>0.16375173768860896</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="4"/>
@@ -5160,7 +5190,7 @@
       </c>
       <c r="I7" s="3">
         <f ca="1">1-(I6/I4)</f>
-        <v>1.1466720607331937</v>
+        <v>0.98936520924422233</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -5169,9 +5199,9 @@
       <c r="N7" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="O7" s="3" t="e">
-        <f>1-(O6/O4)</f>
-        <v>#DIV/0!</v>
+      <c r="O7" s="3">
+        <f>IFERROR(1-(O6/O4),0)</f>
+        <v>0</v>
       </c>
       <c r="P7" s="4"/>
       <c r="Q7" s="4"/>
@@ -5182,7 +5212,7 @@
       </c>
       <c r="U7" s="3">
         <f ca="1">1-(U6/U4)</f>
-        <v>5.7142857142857162E-2</v>
+        <v>8.5714285714285743E-2</v>
       </c>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
@@ -5242,7 +5272,7 @@
       </c>
       <c r="AN7" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI7,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>32988.290000000023</v>
+        <v>52315.460000000036</v>
       </c>
       <c r="AO7" s="26" t="str" cm="1">
         <f t="array" ref="AO7">_xlfn.IFS(AN7&gt;=AJ7,"A",AN7&gt;=AK7,"B",AN7&gt;=AL7,"C",AN7&gt;=AM7,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -5254,7 +5284,7 @@
       </c>
       <c r="AQ7" s="25" cm="1">
         <f t="array" ref="AQ7">_xlfn.IFS(AP7="D",MAX(AM7-AN7,0),AP7="C",MAX(AL7-AN7,0),AP7="B",MAX(AK7-AN7,0),AP7="A",MAX(AJ7-AN7,0),AP7="OBJETIVO ALCANÇADO",0)</f>
-        <v>93461.709999999977</v>
+        <v>74134.539999999964</v>
       </c>
     </row>
     <row r="8" spans="1:43" x14ac:dyDescent="0.25">
@@ -5336,7 +5366,7 @@
       </c>
       <c r="AN8" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI8,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>20123.86</v>
+        <v>34826.190000000031</v>
       </c>
       <c r="AO8" s="26" t="str" cm="1">
         <f t="array" ref="AO8">_xlfn.IFS(AN8&gt;=AJ8,"A",AN8&gt;=AK8,"B",AN8&gt;=AL8,"C",AN8&gt;=AM8,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -5348,7 +5378,7 @@
       </c>
       <c r="AQ8" s="25" cm="1">
         <f t="array" ref="AQ8">_xlfn.IFS(AP8="D",MAX(AM8-AN8,0),AP8="C",MAX(AL8-AN8,0),AP8="B",MAX(AK8-AN8,0),AP8="A",MAX(AJ8-AN8,0),AP8="OBJETIVO ALCANÇADO",0)</f>
-        <v>72576.14</v>
+        <v>57873.809999999969</v>
       </c>
     </row>
     <row r="9" spans="1:43" x14ac:dyDescent="0.25">
@@ -5463,7 +5493,7 @@
       </c>
       <c r="AN9" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI9,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>20419.93</v>
+        <v>26662.550000000017</v>
       </c>
       <c r="AO9" s="26" t="str" cm="1">
         <f t="array" ref="AO9">_xlfn.IFS(AN9&gt;=AJ9,"A",AN9&gt;=AK9,"B",AN9&gt;=AL9,"C",AN9&gt;=AM9,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -5475,7 +5505,7 @@
       </c>
       <c r="AQ9" s="25" cm="1">
         <f t="array" ref="AQ9">_xlfn.IFS(AP9="D",MAX(AM9-AN9,0),AP9="C",MAX(AL9-AN9,0),AP9="B",MAX(AK9-AN9,0),AP9="A",MAX(AJ9-AN9,0),AP9="OBJETIVO ALCANÇADO",0)</f>
-        <v>58330.07</v>
+        <v>52087.449999999983</v>
       </c>
     </row>
     <row r="10" spans="1:43" x14ac:dyDescent="0.25">
@@ -5491,11 +5521,11 @@
       </c>
       <c r="D10" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>4765.8499999999995</v>
+        <v>10063.619999999999</v>
       </c>
       <c r="E10" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>65734.149999999994</v>
+        <v>60436.380000000005</v>
       </c>
       <c r="F10" s="4"/>
       <c r="G10" s="18" t="s">
@@ -5506,15 +5536,15 @@
       </c>
       <c r="I10" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>20980</v>
+        <v>16760</v>
       </c>
       <c r="J10" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>28873.46000000001</v>
+        <v>15414.589999999998</v>
       </c>
       <c r="K10" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>-7893.46000000001</v>
+        <v>1345.4100000000017</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4" t="s">
@@ -5591,23 +5621,23 @@
       </c>
       <c r="AJ10" s="24">
         <f>_xlfn.XLOOKUP(Tabela817[[#This Row],[VENDEDOR]],[1]!Tabela8[VENDEDOR],[1]!Tabela8[META A])</f>
-        <v>269179</v>
+        <v>272000</v>
       </c>
       <c r="AK10" s="24">
         <f>_xlfn.XLOOKUP(Tabela817[[#This Row],[VENDEDOR]],[1]!Tabela8[VENDEDOR],[1]!Tabela8[META B])</f>
-        <v>228803</v>
+        <v>231200</v>
       </c>
       <c r="AL10" s="24">
         <f>_xlfn.XLOOKUP(Tabela817[[#This Row],[VENDEDOR]],[1]!Tabela8[VENDEDOR],[1]!Tabela8[META C])</f>
-        <v>160163</v>
+        <v>190400</v>
       </c>
       <c r="AM10" s="24">
         <f>_xlfn.XLOOKUP(Tabela817[[#This Row],[VENDEDOR]],[1]!Tabela8[VENDEDOR],[1]!Tabela8[META D])</f>
-        <v>121131</v>
+        <v>122400</v>
       </c>
       <c r="AN10" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI10,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>37419.070000000022</v>
+        <v>51568.700000000055</v>
       </c>
       <c r="AO10" s="26" t="str" cm="1">
         <f t="array" ref="AO10">_xlfn.IFS(AN10&gt;=AJ10,"A",AN10&gt;=AK10,"B",AN10&gt;=AL10,"C",AN10&gt;=AM10,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -5619,7 +5649,7 @@
       </c>
       <c r="AQ10" s="25" cm="1">
         <f t="array" ref="AQ10">_xlfn.IFS(AP10="D",MAX(AM10-AN10,0),AP10="C",MAX(AL10-AN10,0),AP10="B",MAX(AK10-AN10,0),AP10="A",MAX(AJ10-AN10,0),AP10="OBJETIVO ALCANÇADO",0)</f>
-        <v>83711.929999999978</v>
+        <v>70831.299999999945</v>
       </c>
     </row>
     <row r="11" spans="1:43" x14ac:dyDescent="0.25">
@@ -5635,11 +5665,11 @@
       </c>
       <c r="D11" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>59621.690000000039</v>
+        <v>80195.720000000016</v>
       </c>
       <c r="E11" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>285378.30999999994</v>
+        <v>264804.27999999997</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="18" t="s">
@@ -5650,15 +5680,15 @@
       </c>
       <c r="I11" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>13060</v>
+        <v>16230</v>
       </c>
       <c r="J11" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>23646.760000000002</v>
+        <v>14149.629999999996</v>
       </c>
       <c r="K11" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>-10586.760000000002</v>
+        <v>2080.3700000000044</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4" t="s">
@@ -5691,12 +5721,12 @@
         <v>35</v>
       </c>
       <c r="V11" s="17">
-        <f>IFERROR(VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0),0)</f>
-        <v>0</v>
+        <f ca="1">IFERROR(VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0),0)</f>
+        <v>2</v>
       </c>
       <c r="W11" s="17">
-        <f t="shared" ref="W11:W20" si="0">U11-V11</f>
-        <v>35</v>
+        <f t="shared" ref="W11:W20" ca="1" si="0">U11-V11</f>
+        <v>33</v>
       </c>
       <c r="Y11" s="32" t="s">
         <v>12</v>
@@ -5797,15 +5827,15 @@
       </c>
       <c r="I12" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>9390</v>
+        <v>10030</v>
       </c>
       <c r="J12" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>10320.560000000003</v>
+        <v>13074.129999999997</v>
       </c>
       <c r="K12" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>-930.56000000000313</v>
+        <v>-3044.1299999999974</v>
       </c>
       <c r="L12" s="4"/>
       <c r="M12" s="4" t="s">
@@ -5901,7 +5931,7 @@
       </c>
       <c r="AN12" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI12,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>7270.8299999999963</v>
+        <v>9566.7999999999956</v>
       </c>
       <c r="AO12" s="26" t="str" cm="1">
         <f t="array" ref="AO12">_xlfn.IFS(AN12&gt;=AJ12,"A",AN12&gt;=AK12,"B",AN12&gt;=AL12,"C",AN12&gt;=AM12,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -5913,7 +5943,7 @@
       </c>
       <c r="AQ12" s="25" cm="1">
         <f t="array" ref="AQ12">_xlfn.IFS(AP12="D",MAX(AM12-AN12,0),AP12="C",MAX(AL12-AN12,0),AP12="B",MAX(AK12-AN12,0),AP12="A",MAX(AJ12-AN12,0),AP12="OBJETIVO ALCANÇADO",0)</f>
-        <v>18829.170000000006</v>
+        <v>16533.200000000004</v>
       </c>
     </row>
     <row r="13" spans="1:43" x14ac:dyDescent="0.25">
@@ -5929,11 +5959,11 @@
       </c>
       <c r="D13" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>10293.539999999999</v>
+        <v>12079.49</v>
       </c>
       <c r="E13" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>85706.46</v>
+        <v>83920.51</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="18" t="s">
@@ -5944,15 +5974,15 @@
       </c>
       <c r="I13" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>19350</v>
+        <v>14910</v>
       </c>
       <c r="J13" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>13145.080000000002</v>
+        <v>17436.830000000009</v>
       </c>
       <c r="K13" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>6204.9199999999983</v>
+        <v>-2526.830000000009</v>
       </c>
       <c r="L13" s="4"/>
       <c r="M13" s="4" t="s">
@@ -6048,7 +6078,7 @@
       </c>
       <c r="AN13" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI13,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>10293.539999999999</v>
+        <v>12079.49</v>
       </c>
       <c r="AO13" s="26" t="str" cm="1">
         <f t="array" ref="AO13">_xlfn.IFS(AN13&gt;=AJ13,"A",AN13&gt;=AK13,"B",AN13&gt;=AL13,"C",AN13&gt;=AM13,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -6060,7 +6090,7 @@
       </c>
       <c r="AQ13" s="25" cm="1">
         <f t="array" ref="AQ13">_xlfn.IFS(AP13="D",MAX(AM13-AN13,0),AP13="C",MAX(AL13-AN13,0),AP13="B",MAX(AK13-AN13,0),AP13="A",MAX(AJ13-AN13,0),AP13="OBJETIVO ALCANÇADO",0)</f>
-        <v>32906.46</v>
+        <v>31120.510000000002</v>
       </c>
     </row>
     <row r="14" spans="1:43" x14ac:dyDescent="0.25">
@@ -6076,11 +6106,11 @@
       </c>
       <c r="D14" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>32988.290000000023</v>
+        <v>52315.460000000036</v>
       </c>
       <c r="E14" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>248011.70999999996</v>
+        <v>228684.53999999998</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="18" t="s">
@@ -6091,15 +6121,15 @@
       </c>
       <c r="I14" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>16120</v>
+        <v>11680</v>
       </c>
       <c r="J14" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>12159.649999999998</v>
+        <v>7410.8999999999987</v>
       </c>
       <c r="K14" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3960.3500000000022</v>
+        <v>4269.1000000000013</v>
       </c>
       <c r="L14" s="4"/>
       <c r="M14" s="4" t="s">
@@ -6195,7 +6225,7 @@
       </c>
       <c r="AN14" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI14,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>4765.8499999999995</v>
+        <v>10063.619999999999</v>
       </c>
       <c r="AO14" s="26" t="str" cm="1">
         <f t="array" ref="AO14">_xlfn.IFS(AN14&gt;=AJ14,"A",AN14&gt;=AK14,"B",AN14&gt;=AL14,"C",AN14&gt;=AM14,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -6207,7 +6237,7 @@
       </c>
       <c r="AQ14" s="25" cm="1">
         <f t="array" ref="AQ14">_xlfn.IFS(AP14="D",MAX(AM14-AN14,0),AP14="C",MAX(AL14-AN14,0),AP14="B",MAX(AK14-AN14,0),AP14="A",MAX(AJ14-AN14,0),AP14="OBJETIVO ALCANÇADO",0)</f>
-        <v>26959.15</v>
+        <v>21661.38</v>
       </c>
     </row>
     <row r="15" spans="1:43" x14ac:dyDescent="0.25">
@@ -6223,11 +6253,11 @@
       </c>
       <c r="D15" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>12263.809999999998</v>
+        <v>18377.800000000003</v>
       </c>
       <c r="E15" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>71736.19</v>
+        <v>65622.2</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="18" t="s">
@@ -6238,15 +6268,15 @@
       </c>
       <c r="I15" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>25020</v>
+        <v>11360</v>
       </c>
       <c r="J15" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>33708.730000000003</v>
+        <v>20574.03</v>
       </c>
       <c r="K15" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>-8688.7300000000032</v>
+        <v>-9214.0299999999988</v>
       </c>
       <c r="L15" s="4"/>
       <c r="M15" s="4" t="s">
@@ -6342,7 +6372,7 @@
       </c>
       <c r="AN15" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI15,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>12263.809999999998</v>
+        <v>18377.800000000003</v>
       </c>
       <c r="AO15" s="26" t="str" cm="1">
         <f t="array" ref="AO15">_xlfn.IFS(AN15&gt;=AJ15,"A",AN15&gt;=AK15,"B",AN15&gt;=AL15,"C",AN15&gt;=AM15,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -6354,7 +6384,7 @@
       </c>
       <c r="AQ15" s="25" cm="1">
         <f t="array" ref="AQ15">_xlfn.IFS(AP15="D",MAX(AM15-AN15,0),AP15="C",MAX(AL15-AN15,0),AP15="B",MAX(AK15-AN15,0),AP15="A",MAX(AJ15-AN15,0),AP15="OBJETIVO ALCANÇADO",0)</f>
-        <v>25536.190000000002</v>
+        <v>19422.199999999997</v>
       </c>
     </row>
     <row r="16" spans="1:43" x14ac:dyDescent="0.25">
@@ -6370,11 +6400,11 @@
       </c>
       <c r="D16" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>2016.6</v>
+        <v>41478.5</v>
       </c>
       <c r="E16" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>347983.4</v>
+        <v>308521.5</v>
       </c>
       <c r="F16" s="4"/>
       <c r="G16" s="18" t="s">
@@ -6385,15 +6415,15 @@
       </c>
       <c r="I16" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>13880</v>
+        <v>13010</v>
       </c>
       <c r="J16" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>16407.95</v>
+        <v>6242.6200000000008</v>
       </c>
       <c r="K16" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>-2527.9500000000007</v>
+        <v>6767.3799999999992</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4" t="s">
@@ -6489,7 +6519,7 @@
       </c>
       <c r="AN16" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI16,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>16296.58</v>
+        <v>29370.71000000001</v>
       </c>
       <c r="AO16" s="26" t="str" cm="1">
         <f t="array" ref="AO16">_xlfn.IFS(AN16&gt;=AJ16,"A",AN16&gt;=AK16,"B",AN16&gt;=AL16,"C",AN16&gt;=AM16,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -6501,7 +6531,7 @@
       </c>
       <c r="AQ16" s="25" cm="1">
         <f t="array" ref="AQ16">_xlfn.IFS(AP16="D",MAX(AM16-AN16,0),AP16="C",MAX(AL16-AN16,0),AP16="B",MAX(AK16-AN16,0),AP16="A",MAX(AJ16-AN16,0),AP16="OBJETIVO ALCANÇADO",0)</f>
-        <v>47603.42</v>
+        <v>34529.289999999994</v>
       </c>
     </row>
     <row r="17" spans="1:43" x14ac:dyDescent="0.25">
@@ -6517,11 +6547,11 @@
       </c>
       <c r="D17" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>63215.649999999965</v>
+        <v>80120.350000000079</v>
       </c>
       <c r="E17" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>436784.35000000003</v>
+        <v>419879.64999999991</v>
       </c>
       <c r="F17" s="4"/>
       <c r="G17" s="18" t="s">
@@ -6532,15 +6562,15 @@
       </c>
       <c r="I17" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>4590</v>
+        <v>7100</v>
       </c>
       <c r="J17" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>4213.3100000000004</v>
+        <v>1715.4</v>
       </c>
       <c r="K17" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>376.6899999999996</v>
+        <v>5384.6</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="4" t="s">
@@ -6555,11 +6585,11 @@
       </c>
       <c r="P17" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[REGIAO]","[Intervalo 2].[REGIAO].&amp;["&amp;N17&amp;"]","[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;["&amp;RIGHT($O$9,1)&amp;"]"),0)</f>
-        <v>59732.449999999968</v>
+        <v>76637.150000000081</v>
       </c>
       <c r="Q17" s="2">
         <f>Tabela8[[#This Row],[COMPROMISSO]]-Tabela8[[#This Row],[ATINGIDO]]</f>
-        <v>-59732.449999999968</v>
+        <v>-76637.150000000081</v>
       </c>
       <c r="R17" s="2"/>
       <c r="S17" s="17" t="s">
@@ -6574,11 +6604,11 @@
       </c>
       <c r="V17" s="17">
         <f ca="1">IFERROR(VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0),0)</f>
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="W17" s="17">
         <f t="shared" ca="1" si="0"/>
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="Y17" s="32" t="s">
         <v>14</v>
@@ -6620,23 +6650,23 @@
       </c>
       <c r="AJ17" s="24">
         <f>_xlfn.XLOOKUP(Tabela817[[#This Row],[VENDEDOR]],[1]!Tabela8[VENDEDOR],[1]!Tabela8[META A])</f>
-        <v>166598</v>
+        <v>169000</v>
       </c>
       <c r="AK17" s="24">
         <f>_xlfn.XLOOKUP(Tabela817[[#This Row],[VENDEDOR]],[1]!Tabela8[VENDEDOR],[1]!Tabela8[META B])</f>
-        <v>141609</v>
+        <v>143650</v>
       </c>
       <c r="AL17" s="24">
         <f>_xlfn.XLOOKUP(Tabela817[[#This Row],[VENDEDOR]],[1]!Tabela8[VENDEDOR],[1]!Tabela8[META C])</f>
-        <v>99127</v>
+        <v>118299.99999999999</v>
       </c>
       <c r="AM17" s="24">
         <f>_xlfn.XLOOKUP(Tabela817[[#This Row],[VENDEDOR]],[1]!Tabela8[VENDEDOR],[1]!Tabela8[META D])</f>
-        <v>74970</v>
+        <v>76050</v>
       </c>
       <c r="AN17" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI17,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>24013.079999999998</v>
+        <v>29690.979999999996</v>
       </c>
       <c r="AO17" s="26" t="str" cm="1">
         <f t="array" ref="AO17">_xlfn.IFS(AN17&gt;=AJ17,"A",AN17&gt;=AK17,"B",AN17&gt;=AL17,"C",AN17&gt;=AM17,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -6648,7 +6678,7 @@
       </c>
       <c r="AQ17" s="25" cm="1">
         <f t="array" ref="AQ17">_xlfn.IFS(AP17="D",MAX(AM17-AN17,0),AP17="C",MAX(AL17-AN17,0),AP17="B",MAX(AK17-AN17,0),AP17="A",MAX(AJ17-AN17,0),AP17="OBJETIVO ALCANÇADO",0)</f>
-        <v>50956.92</v>
+        <v>46359.020000000004</v>
       </c>
     </row>
     <row r="18" spans="1:43" x14ac:dyDescent="0.25">
@@ -6664,11 +6694,11 @@
       </c>
       <c r="D18" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>94941.200000000012</v>
+        <v>212283.80000000005</v>
       </c>
       <c r="E18" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>885058.8</v>
+        <v>767716.2</v>
       </c>
       <c r="F18" s="4"/>
       <c r="G18" s="18" t="s">
@@ -6770,7 +6800,7 @@
       </c>
       <c r="AN18" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI18,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>32294.379999999983</v>
+        <v>49731.210000000028</v>
       </c>
       <c r="AO18" s="26" t="str" cm="1">
         <f t="array" ref="AO18">_xlfn.IFS(AN18&gt;=AJ18,"A",AN18&gt;=AK18,"B",AN18&gt;=AL18,"C",AN18&gt;=AM18,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -6782,7 +6812,7 @@
       </c>
       <c r="AQ18" s="25" cm="1">
         <f t="array" ref="AQ18">_xlfn.IFS(AP18="D",MAX(AM18-AN18,0),AP18="C",MAX(AL18-AN18,0),AP18="B",MAX(AK18-AN18,0),AP18="A",MAX(AJ18-AN18,0),AP18="OBJETIVO ALCANÇADO",0)</f>
-        <v>89205.620000000024</v>
+        <v>71768.789999999979</v>
       </c>
     </row>
     <row r="19" spans="1:43" x14ac:dyDescent="0.25">
@@ -6813,15 +6843,15 @@
       </c>
       <c r="I19" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>18340</v>
+        <v>10320</v>
       </c>
       <c r="J19" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>13425.409999999993</v>
+        <v>14702.329999999998</v>
       </c>
       <c r="K19" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>4914.5900000000074</v>
+        <v>-4382.3299999999981</v>
       </c>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
@@ -6838,11 +6868,11 @@
       </c>
       <c r="V19" s="17">
         <f ca="1">IFERROR(VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0),0)</f>
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="W19" s="17">
         <f t="shared" ca="1" si="0"/>
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="Y19" s="32" t="s">
         <v>16</v>
@@ -6900,7 +6930,7 @@
       </c>
       <c r="AN19" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI19,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>5238.87</v>
+        <v>6954.27</v>
       </c>
       <c r="AO19" s="26" t="str" cm="1">
         <f t="array" ref="AO19">_xlfn.IFS(AN19&gt;=AJ19,"A",AN19&gt;=AK19,"B",AN19&gt;=AL19,"C",AN19&gt;=AM19,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -6912,7 +6942,7 @@
       </c>
       <c r="AQ19" s="25" cm="1">
         <f t="array" ref="AQ19">_xlfn.IFS(AP19="D",MAX(AM19-AN19,0),AP19="C",MAX(AL19-AN19,0),AP19="B",MAX(AK19-AN19,0),AP19="A",MAX(AJ19-AN19,0),AP19="OBJETIVO ALCANÇADO",0)</f>
-        <v>37736.129999999997</v>
+        <v>36020.729999999996</v>
       </c>
     </row>
     <row r="20" spans="1:43" x14ac:dyDescent="0.25">
@@ -6928,11 +6958,11 @@
       </c>
       <c r="D20" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>15188.2</v>
+        <v>38918.429999999993</v>
       </c>
       <c r="E20" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>574811.80000000005</v>
+        <v>551081.57000000007</v>
       </c>
       <c r="F20" s="4"/>
       <c r="G20" s="18" t="s">
@@ -6943,15 +6973,15 @@
       </c>
       <c r="I20" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>17000</v>
+        <v>13370</v>
       </c>
       <c r="J20" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>19596.890000000007</v>
+        <v>19307.170000000002</v>
       </c>
       <c r="K20" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>-2596.8900000000067</v>
+        <v>-5937.1700000000019</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
@@ -7042,7 +7072,7 @@
       </c>
       <c r="AN20" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI20,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>14652.809999999996</v>
+        <v>22063.71000000001</v>
       </c>
       <c r="AO20" s="26" t="str" cm="1">
         <f t="array" ref="AO20">_xlfn.IFS(AN20&gt;=AJ20,"A",AN20&gt;=AK20,"B",AN20&gt;=AL20,"C",AN20&gt;=AM20,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -7054,7 +7084,7 @@
       </c>
       <c r="AQ20" s="25" cm="1">
         <f t="array" ref="AQ20">_xlfn.IFS(AP20="D",MAX(AM20-AN20,0),AP20="C",MAX(AL20-AN20,0),AP20="B",MAX(AK20-AN20,0),AP20="A",MAX(AJ20-AN20,0),AP20="OBJETIVO ALCANÇADO",0)</f>
-        <v>83222.19</v>
+        <v>75811.289999999994</v>
       </c>
     </row>
     <row r="21" spans="1:43" x14ac:dyDescent="0.25">
@@ -7070,11 +7100,11 @@
       </c>
       <c r="D21" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>40356.879999999961</v>
+        <v>78869.479999999967</v>
       </c>
       <c r="E21" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>439643.12000000005</v>
+        <v>401130.52</v>
       </c>
       <c r="F21" s="4"/>
       <c r="G21" s="18" t="s">
@@ -7085,15 +7115,15 @@
       </c>
       <c r="I21" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>5990</v>
+        <v>4460</v>
       </c>
       <c r="J21" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>4585.25</v>
+        <v>6113.9899999999989</v>
       </c>
       <c r="K21" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>1404.75</v>
+        <v>-1653.9899999999989</v>
       </c>
       <c r="L21" s="4"/>
       <c r="M21" s="4"/>
@@ -7125,11 +7155,11 @@
       </c>
       <c r="V21" s="17">
         <f ca="1">IFERROR(VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0),0)</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="W21" s="17">
         <f t="shared" ref="W21:W26" ca="1" si="1">U21-V21</f>
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="Y21" s="36" t="s">
         <v>60</v>
@@ -7152,42 +7182,42 @@
       </c>
       <c r="AD21" s="37">
         <f>SUBTOTAL(109,Planilha1!$AD$3:$AD$20)</f>
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="AE21" s="37"/>
       <c r="AF21" s="37"/>
       <c r="AG21" s="38">
         <f>SUBTOTAL(109,Planilha1!$AG$3:$AG$20)</f>
-        <v>227</v>
+        <v>238</v>
       </c>
       <c r="AI21" t="s">
         <v>60</v>
       </c>
       <c r="AJ21" s="26">
         <f>SUBTOTAL(109,Tabela817[META A])</f>
-        <v>2974777</v>
+        <v>2980000</v>
       </c>
       <c r="AK21" s="26">
         <f>SUBTOTAL(109,Tabela817[META B])</f>
-        <v>2528562</v>
+        <v>2533000</v>
       </c>
       <c r="AL21" s="26">
         <f>SUBTOTAL(109,Tabela817[META C])</f>
-        <v>2036590</v>
+        <v>2086000</v>
       </c>
       <c r="AM21" s="26">
         <f>SUBTOTAL(109,Tabela817[META D])</f>
-        <v>1338651</v>
+        <v>1341000</v>
       </c>
       <c r="AN21" s="26">
         <f>SUBTOTAL(109,Tabela817[ATINGIDO])</f>
-        <v>373148.26000000007</v>
+        <v>531600.57000000018</v>
       </c>
       <c r="AO21" s="4"/>
       <c r="AP21" s="4"/>
       <c r="AQ21" s="27">
         <f>SUBTOTAL(109,Tabela817[FALTA])</f>
-        <v>965502.74</v>
+        <v>809399.4299999997</v>
       </c>
     </row>
     <row r="22" spans="1:43" x14ac:dyDescent="0.25">
@@ -7218,15 +7248,15 @@
       </c>
       <c r="I22" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>9950</v>
+        <v>8680</v>
       </c>
       <c r="J22" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>14168.76</v>
+        <v>5677.8999999999987</v>
       </c>
       <c r="K22" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>-4218.76</v>
+        <v>3002.1000000000013</v>
       </c>
       <c r="L22" s="4"/>
       <c r="M22" s="4"/>
@@ -7239,11 +7269,11 @@
       </c>
       <c r="P22" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>59732.449999999968</v>
+        <v>76637.150000000081</v>
       </c>
       <c r="Q22" s="7">
         <f>O22-P22</f>
-        <v>666458.02619047626</v>
+        <v>649553.32619047607</v>
       </c>
       <c r="R22" s="4"/>
       <c r="S22" s="17" t="s">
@@ -7258,11 +7288,11 @@
       </c>
       <c r="V22" s="17">
         <f ca="1">IFERROR(VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0),0)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="W22" s="17">
         <f t="shared" ca="1" si="1"/>
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="23" spans="1:43" x14ac:dyDescent="0.25">
@@ -7278,11 +7308,11 @@
       </c>
       <c r="D23" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>20123.86</v>
+        <v>34826.190000000031</v>
       </c>
       <c r="E23" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>185876.14</v>
+        <v>171173.80999999997</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="18" t="s">
@@ -7293,15 +7323,15 @@
       </c>
       <c r="I23" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>6580</v>
+        <v>5070</v>
       </c>
       <c r="J23" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>8426.4</v>
+        <v>1785.95</v>
       </c>
       <c r="K23" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>-1846.3999999999996</v>
+        <v>3284.05</v>
       </c>
       <c r="L23" s="4"/>
       <c r="M23" s="4"/>
@@ -7333,11 +7363,11 @@
       </c>
       <c r="V23" s="17">
         <f ca="1">IFERROR(VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0),0)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="W23" s="17">
         <f t="shared" ca="1" si="1"/>
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="24" spans="1:43" x14ac:dyDescent="0.25">
@@ -7349,15 +7379,15 @@
       </c>
       <c r="C24" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],[1]!Tabela2[VENDEDOR],[1]!Tabela2[META A],0)</f>
-        <v>166598</v>
+        <v>169000</v>
       </c>
       <c r="D24" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>24013.079999999998</v>
+        <v>29690.979999999996</v>
       </c>
       <c r="E24" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>142584.92000000001</v>
+        <v>139309.02000000002</v>
       </c>
       <c r="F24" s="4"/>
       <c r="G24" s="18" t="s">
@@ -7368,15 +7398,15 @@
       </c>
       <c r="I24" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>5530</v>
+        <v>3720</v>
       </c>
       <c r="J24" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>8884.1</v>
+        <v>4707.7</v>
       </c>
       <c r="K24" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>-3354.1000000000004</v>
+        <v>-987.69999999999982</v>
       </c>
       <c r="L24" s="4"/>
       <c r="M24" s="4"/>
@@ -7428,11 +7458,11 @@
       </c>
       <c r="D25" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>14652.809999999996</v>
+        <v>22063.71000000001</v>
       </c>
       <c r="E25" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>202847.19</v>
+        <v>195436.28999999998</v>
       </c>
       <c r="F25" s="4"/>
       <c r="G25" s="18" t="s">
@@ -7443,15 +7473,15 @@
       </c>
       <c r="I25" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>5850</v>
+        <v>4770</v>
       </c>
       <c r="J25" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>10532.269999999999</v>
+        <v>2525.3999999999992</v>
       </c>
       <c r="K25" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>-4682.2699999999986</v>
+        <v>2244.6000000000008</v>
       </c>
       <c r="L25" s="4"/>
       <c r="M25" s="4"/>
@@ -7503,11 +7533,11 @@
       </c>
       <c r="D26" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>5238.87</v>
+        <v>6954.27</v>
       </c>
       <c r="E26" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>90261.13</v>
+        <v>88545.73</v>
       </c>
       <c r="F26" s="4"/>
       <c r="G26" s="18" t="s">
@@ -7518,15 +7548,15 @@
       </c>
       <c r="I26" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>3770</v>
+        <v>3190</v>
       </c>
       <c r="J26" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>4425.9999999999991</v>
+        <v>2261.0300000000002</v>
       </c>
       <c r="K26" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>-655.99999999999909</v>
+        <v>928.9699999999998</v>
       </c>
       <c r="L26" s="4"/>
       <c r="M26" s="4"/>
@@ -7546,12 +7576,12 @@
         <v>35</v>
       </c>
       <c r="V26" s="17">
-        <f>IFERROR(VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0),0)</f>
-        <v>0</v>
+        <f ca="1">IFERROR(VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0),0)</f>
+        <v>2</v>
       </c>
       <c r="W26" s="17">
-        <f t="shared" si="1"/>
-        <v>35</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>33</v>
       </c>
     </row>
     <row r="27" spans="1:43" x14ac:dyDescent="0.25">
@@ -7563,15 +7593,15 @@
       </c>
       <c r="C27" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],[1]!Tabela2[VENDEDOR],[1]!Tabela2[META A],0)</f>
-        <v>269179</v>
+        <v>272000</v>
       </c>
       <c r="D27" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>37419.070000000022</v>
+        <v>51568.700000000055</v>
       </c>
       <c r="E27" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>231759.93</v>
+        <v>220431.29999999993</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="18" t="s">
@@ -7582,15 +7612,15 @@
       </c>
       <c r="I27" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>4820</v>
+        <v>5440</v>
       </c>
       <c r="J27" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>3066.1000000000004</v>
+        <v>5297.7699999999995</v>
       </c>
       <c r="K27" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>1753.8999999999996</v>
+        <v>142.23000000000047</v>
       </c>
       <c r="L27" s="4"/>
       <c r="M27" s="4"/>
@@ -7613,11 +7643,11 @@
       </c>
       <c r="D28" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>52714.41</v>
+        <v>68129</v>
       </c>
       <c r="E28" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>278785.58999999997</v>
+        <v>263371</v>
       </c>
       <c r="F28" s="4"/>
       <c r="L28" s="4"/>
@@ -7692,11 +7722,11 @@
       </c>
       <c r="D30" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>16296.58</v>
+        <v>29370.71000000001</v>
       </c>
       <c r="E30" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>125703.42</v>
+        <v>112629.29</v>
       </c>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
@@ -7729,11 +7759,11 @@
       </c>
       <c r="V30" s="5">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE 2]",'[1]BASE PYTHON'!$P$83,"[Intervalo 3].[SEMANAL]","[Intervalo 3].[SEMANAL].&amp;[1]"),0)</f>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="W30" s="6">
         <f>U30-V30</f>
-        <v>39.333333333333336</v>
+        <v>38.333333333333336</v>
       </c>
     </row>
     <row r="31" spans="1:43" x14ac:dyDescent="0.25">
@@ -7749,11 +7779,11 @@
       </c>
       <c r="D31" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>20419.93</v>
+        <v>26662.550000000017</v>
       </c>
       <c r="E31" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>154580.07</v>
+        <v>148337.44999999998</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
@@ -7762,15 +7792,15 @@
       </c>
       <c r="I31" s="2" cm="1">
         <f t="array" ref="I31">_xlfn.XLOOKUP(Tabela6[[#This Row],[SEMANAL]],[1]!Tabela9[[#All],[Coluna1]],[1]!Tabela9[[#All],[Coluna2]])</f>
-        <v>283312.09523809527</v>
+        <v>283809.52380952379</v>
       </c>
       <c r="J31" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[1]"),0)</f>
-        <v>120365.51000000001</v>
+        <v>120365.50999999998</v>
       </c>
       <c r="K31" s="7">
         <f>I31-J31</f>
-        <v>162946.58523809526</v>
+        <v>163444.01380952381</v>
       </c>
       <c r="L31" s="4"/>
       <c r="M31" s="4"/>
@@ -7789,11 +7819,11 @@
       </c>
       <c r="V31" s="5">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE 2]",'[1]BASE PYTHON'!$P$83,"[Intervalo 3].[SEMANAL]","[Intervalo 3].[SEMANAL].&amp;[2]"),0)</f>
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="W31" s="6">
         <f t="shared" ref="W31:W33" si="2">U31-V31</f>
-        <v>115.33333333333334</v>
+        <v>100.33333333333334</v>
       </c>
     </row>
     <row r="32" spans="1:43" x14ac:dyDescent="0.25">
@@ -7809,11 +7839,11 @@
       </c>
       <c r="D32" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>32294.379999999983</v>
+        <v>49731.210000000028</v>
       </c>
       <c r="E32" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>237705.62000000002</v>
+        <v>220268.78999999998</v>
       </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
@@ -7822,15 +7852,15 @@
       </c>
       <c r="I32" s="2" cm="1">
         <f t="array" ref="I32">_xlfn.XLOOKUP(Tabela6[[#This Row],[SEMANAL]],[1]!Tabela9[[#All],[Coluna1]],[1]!Tabela9[[#All],[Coluna2]])</f>
-        <v>708280.23809523811</v>
+        <v>709523.80952380947</v>
       </c>
       <c r="J32" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>185235.10000000012</v>
+        <v>307822.27999999991</v>
       </c>
       <c r="K32" s="7">
         <f t="shared" ref="K32:K34" si="3">I32-J32</f>
-        <v>523045.13809523801</v>
+        <v>401701.52952380956</v>
       </c>
       <c r="L32" s="4"/>
       <c r="M32" s="4"/>
@@ -7869,11 +7899,11 @@
       </c>
       <c r="D33" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>13559.139999999998</v>
+        <v>16084.539999999992</v>
       </c>
       <c r="E33" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>74440.86</v>
+        <v>71915.460000000006</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -7882,7 +7912,7 @@
       </c>
       <c r="I33" s="2" cm="1">
         <f t="array" ref="I33">_xlfn.XLOOKUP(Tabela6[[#This Row],[SEMANAL]],[1]!Tabela9[[#All],[Coluna1]],[1]!Tabela9[[#All],[Coluna2]])</f>
-        <v>566624.19047619053</v>
+        <v>567619.04761904757</v>
       </c>
       <c r="J33" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
@@ -7890,7 +7920,7 @@
       </c>
       <c r="K33" s="7">
         <f t="shared" si="3"/>
-        <v>566624.19047619053</v>
+        <v>567619.04761904757</v>
       </c>
       <c r="L33" s="4"/>
       <c r="M33" s="4"/>
@@ -7929,11 +7959,11 @@
       </c>
       <c r="D34" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>7270.8299999999963</v>
+        <v>9566.7999999999956</v>
       </c>
       <c r="E34" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>50729.170000000006</v>
+        <v>48433.200000000004</v>
       </c>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
@@ -7942,7 +7972,7 @@
       </c>
       <c r="I34" s="2" cm="1">
         <f t="array" ref="I34">_xlfn.XLOOKUP(Tabela6[[#This Row],[SEMANAL]],[1]!Tabela9[[#All],[Coluna1]],[1]!Tabela9[[#All],[Coluna2]])</f>
-        <v>708280.23809523811</v>
+        <v>709523.80952380947</v>
       </c>
       <c r="J34" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
@@ -7950,7 +7980,7 @@
       </c>
       <c r="K34" s="7">
         <f t="shared" si="3"/>
-        <v>708280.23809523811</v>
+        <v>709523.80952380947</v>
       </c>
       <c r="L34" s="4"/>
       <c r="M34" s="4"/>
@@ -7989,11 +8019,11 @@
       </c>
       <c r="D35" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>9212.1200000000008</v>
+        <v>13919.82</v>
       </c>
       <c r="E35" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>69787.88</v>
+        <v>65080.18</v>
       </c>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
@@ -8002,7 +8032,7 @@
       </c>
       <c r="I35" s="2" cm="1">
         <f t="array" ref="I35">_xlfn.XLOOKUP(Tabela6[[#This Row],[SEMANAL]],[1]!Tabela9[[#All],[Coluna1]],[1]!Tabela9[[#All],[Coluna2]])</f>
-        <v>708280.23809523811</v>
+        <v>709523.80952380947</v>
       </c>
       <c r="J35" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
@@ -8010,7 +8040,7 @@
       </c>
       <c r="K35" s="7">
         <f>I35-J35</f>
-        <v>708280.23809523811</v>
+        <v>709523.80952380947</v>
       </c>
       <c r="L35" s="4"/>
       <c r="M35" s="4"/>
@@ -8145,7 +8175,7 @@
       </c>
       <c r="C40" s="2" cm="1">
         <f t="array" ref="C40">_xlfn.XLOOKUP(Tabela3[[#This Row],[SEMANAL]],[1]!Tabela7[[#All],[Coluna1]],[1]!Tabela7[[#All],[Coluna2]])</f>
-        <v>573883.52380952379</v>
+        <v>574380.95238095243</v>
       </c>
       <c r="D40" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[1]"),0)</f>
@@ -8153,7 +8183,7 @@
       </c>
       <c r="E40" s="7">
         <f>C40-D40</f>
-        <v>409714.0438095241</v>
+        <v>410211.47238095273</v>
       </c>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
@@ -8181,15 +8211,15 @@
       </c>
       <c r="C41" s="2" cm="1">
         <f t="array" ref="C41">_xlfn.XLOOKUP(Tabela3[[#This Row],[SEMANAL]],[1]!Tabela7[[#All],[Coluna1]],[1]!Tabela7[[#All],[Coluna2]])</f>
-        <v>1434708.8095238095</v>
+        <v>1435952.3809523811</v>
       </c>
       <c r="D41" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>429012.91000000021</v>
+        <v>823417.25000000081</v>
       </c>
       <c r="E41" s="7">
         <f t="shared" ref="E41:E43" si="4">C41-D41</f>
-        <v>1005695.8995238093</v>
+        <v>612535.13095238025</v>
       </c>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
@@ -8217,7 +8247,7 @@
       </c>
       <c r="C42" s="2" cm="1">
         <f t="array" ref="C42">_xlfn.XLOOKUP(Tabela3[[#This Row],[SEMANAL]],[1]!Tabela7[[#All],[Coluna1]],[1]!Tabela7[[#All],[Coluna2]])</f>
-        <v>1147767.0476190476</v>
+        <v>1148761.9047619049</v>
       </c>
       <c r="D42" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[3]"),0)</f>
@@ -8225,7 +8255,7 @@
       </c>
       <c r="E42" s="7">
         <f t="shared" si="4"/>
-        <v>1147767.0476190476</v>
+        <v>1148761.9047619049</v>
       </c>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>
@@ -8253,7 +8283,7 @@
       </c>
       <c r="C43" s="2" cm="1">
         <f t="array" ref="C43">_xlfn.XLOOKUP(Tabela3[[#This Row],[SEMANAL]],[1]!Tabela7[[#All],[Coluna1]],[1]!Tabela7[[#All],[Coluna2]])</f>
-        <v>1434708.8095238095</v>
+        <v>1435952.3809523811</v>
       </c>
       <c r="D43" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[4]"),0)</f>
@@ -8261,7 +8291,7 @@
       </c>
       <c r="E43" s="7">
         <f t="shared" si="4"/>
-        <v>1434708.8095238095</v>
+        <v>1435952.3809523811</v>
       </c>
     </row>
     <row r="44" spans="1:23" x14ac:dyDescent="0.25">
@@ -8271,7 +8301,7 @@
       </c>
       <c r="C44" s="2" cm="1">
         <f t="array" ref="C44">_xlfn.XLOOKUP(Tabela3[[#This Row],[SEMANAL]],[1]!Tabela7[[#All],[Coluna1]],[1]!Tabela7[[#All],[Coluna2]])</f>
-        <v>1434708.8095238095</v>
+        <v>1435952.3809523811</v>
       </c>
       <c r="D44" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[5]"),0)</f>
@@ -8279,7 +8309,7 @@
       </c>
       <c r="E44" s="7">
         <f t="shared" ref="E44" si="5">C44-D44</f>
-        <v>1434708.8095238095</v>
+        <v>1435952.3809523811</v>
       </c>
     </row>
     <row r="45" spans="1:23" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Dados atualizados em 13/10/2026 08:54
</commit_message>
<xml_diff>
--- a/BASE PYTHON.xlsx
+++ b/BASE PYTHON.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\VENDAS\BASE DADOS\IATAGAM\BASES\ACOMPANHAMENTO DIARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E260837-8BDD-4390-B52B-2FA54826FBE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FA9C3B2-2795-4729-A33F-6198F0EE3186}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FAEB2262-BDE3-4F12-A731-117DAEC20A7D}"/>
   </bookViews>
@@ -46,8 +46,8 @@
     <s v="ThisWorkbookDataModel"/>
     <s v="{[Intervalo 2].[DATA].[All]}"/>
     <s v="{[Intervalo 2].[PRODUTO].&amp;[MIST PAO DA FAZENDA VIAPANE 10KG]}"/>
-    <s v="{[Intervalo 2].[DATA].&amp;[2026-10-06T00:00:00]}"/>
     <s v="{[Intervalo 2].[DES_TIPO_OPERACAO].&amp;[VENDA],[Intervalo 2].[DES_TIPO_OPERACAO].&amp;[VENDA SAT]}"/>
+    <s v="{[Intervalo 2].[DATA].&amp;[2026-10-09T00:00:00]}"/>
   </metadataStrings>
   <mdxMetadata count="4">
     <mdx n="0" f="s">
@@ -2527,8 +2527,8 @@
           <cell r="H2" t="str">
             <v>DATA</v>
           </cell>
-          <cell r="I2" t="str" vm="3">
-            <v>06/10/2026</v>
+          <cell r="I2" t="str" vm="4">
+            <v>09/10/2026</v>
           </cell>
           <cell r="K2" t="str">
             <v>DATA</v>
@@ -2541,7 +2541,7 @@
           <cell r="K3" t="str">
             <v>DES_TIPO_OPERACAO</v>
           </cell>
-          <cell r="L3" t="str" vm="4">
+          <cell r="L3" t="str" vm="3">
             <v>(Vários itens)</v>
           </cell>
         </row>
@@ -2570,30 +2570,30 @@
         </row>
         <row r="5">
           <cell r="E5" t="str">
-            <v>CAMPINAS</v>
+            <v>(vazio)</v>
           </cell>
           <cell r="F5">
-            <v>10063.619999999999</v>
+            <v>175.08999999999997</v>
           </cell>
           <cell r="H5" t="str">
-            <v>CAMPINAS</v>
+            <v>(vazio)</v>
           </cell>
           <cell r="I5">
-            <v>5297.7699999999995</v>
+            <v>175.08999999999997</v>
           </cell>
         </row>
         <row r="6">
           <cell r="E6" t="str">
-            <v>CENTRO</v>
+            <v>CAMPINAS</v>
           </cell>
           <cell r="F6">
-            <v>80195.720000000016</v>
+            <v>19043.580000000002</v>
           </cell>
           <cell r="H6" t="str">
-            <v>CENTRO</v>
+            <v>CAMPINAS</v>
           </cell>
           <cell r="I6">
-            <v>20574.03</v>
+            <v>1270.82</v>
           </cell>
           <cell r="K6" t="str">
             <v>Contagem Distinta de COD_CLIENTE</v>
@@ -2604,16 +2604,16 @@
         </row>
         <row r="7">
           <cell r="E7" t="str">
-            <v>IATAGAM JUNIOR</v>
+            <v>CENTRO</v>
           </cell>
           <cell r="F7">
-            <v>0</v>
+            <v>117001.94999999997</v>
           </cell>
           <cell r="H7" t="str">
-            <v>IATAGAM JUNIOR</v>
+            <v>CENTRO</v>
           </cell>
           <cell r="I7">
-            <v>0</v>
+            <v>11533.52</v>
           </cell>
           <cell r="K7" t="str">
             <v>Rótulos de Linha</v>
@@ -2627,157 +2627,157 @@
         </row>
         <row r="8">
           <cell r="E8" t="str">
-            <v>INDAIATUBA</v>
+            <v>ECOMMERCE</v>
           </cell>
           <cell r="F8">
-            <v>12079.49</v>
+            <v>75.12</v>
           </cell>
           <cell r="H8" t="str">
             <v>INDAIATUBA</v>
           </cell>
           <cell r="I8">
-            <v>1785.95</v>
+            <v>4577.72</v>
           </cell>
           <cell r="K8" t="str">
             <v>CENTRO</v>
           </cell>
           <cell r="L8">
-            <v>2</v>
+            <v>5</v>
           </cell>
           <cell r="M8">
-            <v>2</v>
+            <v>5</v>
           </cell>
         </row>
         <row r="9">
           <cell r="E9" t="str">
-            <v>INTERLAGOS</v>
+            <v>IATAGAM JUNIOR</v>
           </cell>
           <cell r="F9">
-            <v>52315.460000000036</v>
+            <v>324.10000000000002</v>
           </cell>
           <cell r="H9" t="str">
             <v>INTERLAGOS</v>
           </cell>
           <cell r="I9">
-            <v>19307.170000000002</v>
+            <v>10562.029999999999</v>
           </cell>
           <cell r="K9" t="str">
-            <v>INTERLAGOS</v>
+            <v>INDAIATUBA</v>
           </cell>
           <cell r="L9">
-            <v>7</v>
+            <v>4</v>
           </cell>
           <cell r="M9">
-            <v>7</v>
+            <v>4</v>
           </cell>
         </row>
         <row r="10">
           <cell r="E10" t="str">
-            <v>JUNDIAI</v>
+            <v>INDAIATUBA</v>
           </cell>
           <cell r="F10">
-            <v>18377.800000000003</v>
+            <v>25865.750000000011</v>
           </cell>
           <cell r="H10" t="str">
             <v>JUNDIAI</v>
           </cell>
           <cell r="I10">
-            <v>6113.9899999999989</v>
+            <v>2244.54</v>
           </cell>
           <cell r="K10" t="str">
-            <v>JUNDIAI</v>
+            <v>INTERLAGOS</v>
           </cell>
           <cell r="L10">
-            <v>1</v>
+            <v>14</v>
           </cell>
           <cell r="M10">
-            <v>1</v>
+            <v>14</v>
           </cell>
         </row>
         <row r="11">
           <cell r="E11" t="str">
-            <v>KEY ABC</v>
+            <v>INTERLAGOS</v>
           </cell>
           <cell r="F11">
-            <v>41478.5</v>
+            <v>87405.690000000031</v>
           </cell>
           <cell r="H11" t="str">
             <v>KEY ABC</v>
           </cell>
           <cell r="I11">
-            <v>39461.899999999994</v>
+            <v>5041.5</v>
           </cell>
           <cell r="K11" t="str">
-            <v>LESTE MOOCA</v>
+            <v>JUNDIAI</v>
           </cell>
           <cell r="L11">
-            <v>8</v>
+            <v>3</v>
           </cell>
           <cell r="M11">
-            <v>8</v>
+            <v>3</v>
           </cell>
         </row>
         <row r="12">
           <cell r="E12" t="str">
-            <v>KEY CASA</v>
+            <v>JUNDIAI</v>
           </cell>
           <cell r="F12">
-            <v>80120.350000000079</v>
+            <v>28099.500000000029</v>
           </cell>
           <cell r="H12" t="str">
             <v>KEY CASA</v>
           </cell>
           <cell r="I12">
-            <v>17635.600000000006</v>
+            <v>7043</v>
           </cell>
           <cell r="K12" t="str">
-            <v>OSASCO</v>
+            <v>LESTE MOOCA</v>
           </cell>
           <cell r="L12">
-            <v>15</v>
+            <v>12</v>
           </cell>
           <cell r="M12">
-            <v>15</v>
+            <v>12</v>
           </cell>
         </row>
         <row r="13">
           <cell r="E13" t="str">
-            <v>KEY INTERIOR</v>
+            <v>KEY ABC</v>
           </cell>
           <cell r="F13">
-            <v>212283.80000000005</v>
+            <v>90046.700000000012</v>
           </cell>
           <cell r="H13" t="str">
             <v>KEY INTERIOR</v>
           </cell>
           <cell r="I13">
-            <v>117342.60000000003</v>
+            <v>66439.199999999997</v>
           </cell>
           <cell r="K13" t="str">
-            <v>PIRITUBA</v>
+            <v>LESTE PENHA</v>
           </cell>
           <cell r="L13">
-            <v>4</v>
+            <v>9</v>
           </cell>
           <cell r="M13">
-            <v>4</v>
+            <v>9</v>
           </cell>
         </row>
         <row r="14">
           <cell r="E14" t="str">
-            <v>KEY SJC</v>
+            <v>KEY CASA</v>
           </cell>
           <cell r="F14">
-            <v>4315.6000000000004</v>
+            <v>104355.99000000003</v>
           </cell>
           <cell r="H14" t="str">
             <v>KEY SJC</v>
           </cell>
           <cell r="I14">
-            <v>0</v>
+            <v>3909.2</v>
           </cell>
           <cell r="K14" t="str">
-            <v>SANTO ANDRE</v>
+            <v>LESTE TATUAPE</v>
           </cell>
           <cell r="L14">
             <v>3</v>
@@ -2788,234 +2788,261 @@
         </row>
         <row r="15">
           <cell r="E15" t="str">
-            <v>KEY SP</v>
+            <v>KEY INTERIOR</v>
           </cell>
           <cell r="F15">
-            <v>38918.429999999993</v>
+            <v>284976.00000000006</v>
           </cell>
           <cell r="H15" t="str">
             <v>KEY SP</v>
           </cell>
           <cell r="I15">
-            <v>23730.23</v>
+            <v>11131.059999999998</v>
           </cell>
           <cell r="K15" t="str">
-            <v>SBC</v>
+            <v>OSASCO</v>
           </cell>
           <cell r="L15">
-            <v>5</v>
+            <v>21</v>
           </cell>
           <cell r="M15">
-            <v>5</v>
+            <v>21</v>
           </cell>
         </row>
         <row r="16">
           <cell r="E16" t="str">
-            <v>KEY ZL</v>
+            <v>KEY SJC</v>
           </cell>
           <cell r="F16">
-            <v>78869.479999999967</v>
+            <v>10406.4</v>
           </cell>
           <cell r="H16" t="str">
             <v>KEY ZL</v>
           </cell>
           <cell r="I16">
-            <v>38512.6</v>
+            <v>3757.1</v>
           </cell>
           <cell r="K16" t="str">
-            <v>SJC</v>
+            <v>PIRITUBA</v>
           </cell>
           <cell r="L16">
-            <v>1</v>
+            <v>6</v>
           </cell>
           <cell r="M16">
-            <v>1</v>
+            <v>6</v>
           </cell>
         </row>
         <row r="17">
           <cell r="E17" t="str">
-            <v>LESTE MOOCA</v>
+            <v>KEY SP</v>
           </cell>
           <cell r="F17">
-            <v>34826.190000000031</v>
+            <v>76109.040000000023</v>
           </cell>
           <cell r="H17" t="str">
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="I17">
-            <v>14702.329999999998</v>
+            <v>988.43000000000006</v>
           </cell>
           <cell r="K17" t="str">
-            <v>SJC/VALE</v>
+            <v>SANTO ANDRE</v>
           </cell>
           <cell r="L17">
-            <v>2</v>
+            <v>7</v>
           </cell>
           <cell r="M17">
-            <v>2</v>
+            <v>7</v>
           </cell>
         </row>
         <row r="18">
           <cell r="E18" t="str">
-            <v>LESTE PENHA</v>
+            <v>KEY ZL</v>
           </cell>
           <cell r="F18">
-            <v>29690.979999999996</v>
+            <v>112434.5800000001</v>
           </cell>
           <cell r="H18" t="str">
             <v>LESTE PENHA</v>
           </cell>
           <cell r="I18">
-            <v>5677.8999999999987</v>
+            <v>4973.12</v>
           </cell>
           <cell r="K18" t="str">
-            <v>Total Geral</v>
+            <v>SBC</v>
           </cell>
           <cell r="L18">
-            <v>48</v>
+            <v>10</v>
           </cell>
           <cell r="M18">
-            <v>48</v>
+            <v>10</v>
           </cell>
         </row>
         <row r="19">
           <cell r="E19" t="str">
-            <v>LESTE TATUAPE</v>
+            <v>LESTE MOOCA</v>
           </cell>
           <cell r="F19">
-            <v>22063.71000000001</v>
+            <v>56477.170000000086</v>
           </cell>
           <cell r="H19" t="str">
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="I19">
-            <v>7410.8999999999987</v>
+            <v>1402.54</v>
+          </cell>
+          <cell r="K19" t="str">
+            <v>SJC</v>
+          </cell>
+          <cell r="L19">
+            <v>3</v>
+          </cell>
+          <cell r="M19">
+            <v>3</v>
           </cell>
         </row>
         <row r="20">
           <cell r="E20" t="str">
-            <v>MOGI</v>
+            <v>LESTE PENHA</v>
           </cell>
           <cell r="F20">
-            <v>6954.27</v>
+            <v>48456.710000000006</v>
           </cell>
           <cell r="H20" t="str">
             <v>MOGI</v>
           </cell>
           <cell r="I20">
-            <v>1715.4</v>
+            <v>2549.5500000000002</v>
+          </cell>
+          <cell r="K20" t="str">
+            <v>SJC/VALE</v>
+          </cell>
+          <cell r="L20">
+            <v>3</v>
+          </cell>
+          <cell r="M20">
+            <v>3</v>
           </cell>
         </row>
         <row r="21">
           <cell r="E21" t="str">
-            <v>NORTE</v>
+            <v>LESTE TATUAPE</v>
           </cell>
           <cell r="F21">
-            <v>51568.700000000055</v>
+            <v>32493.730000000003</v>
           </cell>
           <cell r="H21" t="str">
             <v>NORTE</v>
           </cell>
           <cell r="I21">
-            <v>14149.629999999996</v>
+            <v>5135.0499999999984</v>
+          </cell>
+          <cell r="K21" t="str">
+            <v>Total Geral</v>
+          </cell>
+          <cell r="L21">
+            <v>100</v>
+          </cell>
+          <cell r="M21">
+            <v>100</v>
           </cell>
         </row>
         <row r="22">
           <cell r="E22" t="str">
-            <v>OSASCO</v>
+            <v>MOGI</v>
           </cell>
           <cell r="F22">
-            <v>68129</v>
+            <v>18272.769999999997</v>
           </cell>
           <cell r="H22" t="str">
             <v>OSASCO</v>
           </cell>
           <cell r="I22">
-            <v>15414.589999999998</v>
+            <v>13963.489999999998</v>
           </cell>
         </row>
         <row r="23">
           <cell r="E23" t="str">
-            <v>PIRITUBA</v>
+            <v>NORTE</v>
           </cell>
           <cell r="F23">
-            <v>29370.71000000001</v>
+            <v>81243.350000000093</v>
           </cell>
           <cell r="H23" t="str">
             <v>PIRITUBA</v>
           </cell>
           <cell r="I23">
-            <v>13074.129999999997</v>
+            <v>2919.1</v>
           </cell>
         </row>
         <row r="24">
           <cell r="E24" t="str">
-            <v>SANTO ANDRE</v>
+            <v>OSASCO</v>
           </cell>
           <cell r="F24">
-            <v>26662.550000000017</v>
+            <v>114216.91000000018</v>
           </cell>
           <cell r="H24" t="str">
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="I24">
-            <v>6242.6200000000008</v>
+            <v>2159.1999999999998</v>
           </cell>
         </row>
         <row r="25">
           <cell r="E25" t="str">
-            <v>SBC</v>
+            <v>PIRITUBA</v>
           </cell>
           <cell r="F25">
-            <v>49731.210000000028</v>
+            <v>44023.619999999988</v>
           </cell>
           <cell r="H25" t="str">
             <v>SBC</v>
           </cell>
           <cell r="I25">
-            <v>17436.830000000009</v>
+            <v>15594.409999999996</v>
           </cell>
         </row>
         <row r="26">
           <cell r="E26" t="str">
-            <v>SJC</v>
+            <v>SANTO ANDRE</v>
           </cell>
           <cell r="F26">
-            <v>16084.539999999992</v>
+            <v>53099.140000000007</v>
           </cell>
           <cell r="H26" t="str">
             <v>SJC</v>
           </cell>
           <cell r="I26">
-            <v>2525.3999999999992</v>
+            <v>5642.74</v>
           </cell>
         </row>
         <row r="27">
           <cell r="E27" t="str">
-            <v>SJC/VALE</v>
+            <v>SBC</v>
           </cell>
           <cell r="F27">
-            <v>9566.7999999999956</v>
+            <v>89009.680000000051</v>
           </cell>
           <cell r="H27" t="str">
             <v>SJC/VALE</v>
           </cell>
           <cell r="I27">
-            <v>2261.0300000000002</v>
+            <v>1484.7000000000003</v>
           </cell>
         </row>
         <row r="28">
           <cell r="E28" t="str">
-            <v>VENDEDOR INTERNO 1</v>
+            <v>SJC</v>
           </cell>
           <cell r="F28">
-            <v>13919.82</v>
+            <v>27951.950000000019</v>
           </cell>
           <cell r="H28" t="str">
             <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="I28">
-            <v>4707.7</v>
+            <v>2619.7000000000003</v>
           </cell>
           <cell r="K28" t="str">
             <v>POSITIVAÇÃO GERAL</v>
@@ -3023,16 +3050,16 @@
         </row>
         <row r="29">
           <cell r="E29" t="str">
-            <v>Total Geral</v>
+            <v>SJC/VALE</v>
           </cell>
           <cell r="F29">
-            <v>987586.73000000091</v>
+            <v>15939.879999999988</v>
           </cell>
           <cell r="H29" t="str">
             <v>Total Geral</v>
           </cell>
           <cell r="I29">
-            <v>395080.29999999946</v>
+            <v>187116.80999999997</v>
           </cell>
           <cell r="K29" t="str">
             <v>DATA</v>
@@ -3042,11 +3069,25 @@
           </cell>
         </row>
         <row r="30">
+          <cell r="E30" t="str">
+            <v>VENDEDOR INTERNO 1</v>
+          </cell>
+          <cell r="F30">
+            <v>24446.020000000004</v>
+          </cell>
           <cell r="K30" t="str">
             <v>DES_TIPO_OPERACAO</v>
           </cell>
-          <cell r="L30" t="str" vm="4">
+          <cell r="L30" t="str" vm="3">
             <v>(Vários itens)</v>
+          </cell>
+        </row>
+        <row r="31">
+          <cell r="E31" t="str">
+            <v>Total Geral</v>
+          </cell>
+          <cell r="F31">
+            <v>1561950.4200000046</v>
           </cell>
         </row>
         <row r="32">
@@ -3076,10 +3117,10 @@
             <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="L34">
-            <v>42</v>
+            <v>53</v>
           </cell>
           <cell r="M34">
-            <v>42</v>
+            <v>53</v>
           </cell>
         </row>
         <row r="35">
@@ -3087,10 +3128,10 @@
             <v>Total Geral</v>
           </cell>
           <cell r="L35">
-            <v>42</v>
+            <v>53</v>
           </cell>
           <cell r="M35">
-            <v>42</v>
+            <v>53</v>
           </cell>
         </row>
         <row r="39">
@@ -3098,7 +3139,7 @@
             <v>CAMPINAS</v>
           </cell>
           <cell r="B39">
-            <v>5440</v>
+            <v>5750</v>
           </cell>
         </row>
         <row r="40">
@@ -3106,7 +3147,7 @@
             <v>CENTRO</v>
           </cell>
           <cell r="B40">
-            <v>11360</v>
+            <v>31000</v>
           </cell>
         </row>
         <row r="41">
@@ -3114,7 +3155,7 @@
             <v>INDAIATUBA</v>
           </cell>
           <cell r="B41">
-            <v>5070</v>
+            <v>15530</v>
           </cell>
         </row>
         <row r="42">
@@ -3122,7 +3163,7 @@
             <v>INTERLAGOS</v>
           </cell>
           <cell r="B42">
-            <v>13370</v>
+            <v>25000</v>
           </cell>
         </row>
         <row r="43">
@@ -3130,7 +3171,7 @@
             <v>JUNDIAI</v>
           </cell>
           <cell r="B43">
-            <v>4460</v>
+            <v>5700</v>
           </cell>
         </row>
         <row r="44">
@@ -3138,7 +3179,7 @@
             <v>LESTE MOOCA</v>
           </cell>
           <cell r="B44">
-            <v>10320</v>
+            <v>19890</v>
           </cell>
         </row>
         <row r="45">
@@ -3146,7 +3187,7 @@
             <v>LESTE PENHA</v>
           </cell>
           <cell r="B45">
-            <v>8680</v>
+            <v>21000</v>
           </cell>
         </row>
         <row r="46">
@@ -3154,7 +3195,7 @@
             <v>LESTE TATUAPE</v>
           </cell>
           <cell r="B46">
-            <v>11680</v>
+            <v>19770</v>
           </cell>
         </row>
         <row r="47">
@@ -3162,7 +3203,7 @@
             <v>MOGI</v>
           </cell>
           <cell r="B47">
-            <v>7100</v>
+            <v>10110</v>
           </cell>
           <cell r="P47" t="str">
             <v>Soma de TOTAL</v>
@@ -3173,7 +3214,7 @@
             <v>NORTE</v>
           </cell>
           <cell r="B48">
-            <v>16230</v>
+            <v>25000</v>
           </cell>
         </row>
         <row r="49">
@@ -3181,7 +3222,7 @@
             <v>OSASCO</v>
           </cell>
           <cell r="B49">
-            <v>16760</v>
+            <v>28000</v>
           </cell>
         </row>
         <row r="50">
@@ -3189,7 +3230,7 @@
             <v>PIRITUBA</v>
           </cell>
           <cell r="B50">
-            <v>10030</v>
+            <v>14510</v>
           </cell>
         </row>
         <row r="51">
@@ -3197,7 +3238,7 @@
             <v>SANTO ANDRE</v>
           </cell>
           <cell r="B51">
-            <v>13010</v>
+            <v>19620</v>
           </cell>
         </row>
         <row r="52">
@@ -3205,7 +3246,7 @@
             <v>SBC</v>
           </cell>
           <cell r="B52">
-            <v>14910</v>
+            <v>24000</v>
           </cell>
         </row>
         <row r="53">
@@ -3213,7 +3254,7 @@
             <v>SJC</v>
           </cell>
           <cell r="B53">
-            <v>4770</v>
+            <v>15300</v>
           </cell>
         </row>
         <row r="54">
@@ -3221,7 +3262,7 @@
             <v>SJC/VALE</v>
           </cell>
           <cell r="B54">
-            <v>3190</v>
+            <v>8980</v>
           </cell>
         </row>
         <row r="55">
@@ -3229,7 +3270,7 @@
             <v>VENDEDOR INTERNO 1</v>
           </cell>
           <cell r="B55">
-            <v>3720</v>
+            <v>10850</v>
           </cell>
         </row>
         <row r="63">
@@ -3400,13 +3441,13 @@
             <v>14</v>
           </cell>
           <cell r="F136">
-            <v>1</v>
+            <v>3</v>
           </cell>
           <cell r="H136" t="str">
             <v>D</v>
           </cell>
           <cell r="I136">
-            <v>13</v>
+            <v>11</v>
           </cell>
         </row>
         <row r="137">
@@ -3414,13 +3455,13 @@
             <v>36</v>
           </cell>
           <cell r="F137">
-            <v>42</v>
+            <v>53</v>
           </cell>
           <cell r="H137" t="str">
             <v>C</v>
           </cell>
           <cell r="I137">
-            <v>14</v>
+            <v>3</v>
           </cell>
         </row>
         <row r="138">
@@ -3428,13 +3469,13 @@
             <v>14</v>
           </cell>
           <cell r="F138">
-            <v>2</v>
+            <v>5</v>
           </cell>
           <cell r="H138" t="str">
             <v>D</v>
           </cell>
           <cell r="I138">
-            <v>12</v>
+            <v>9</v>
           </cell>
         </row>
         <row r="139">
@@ -3442,13 +3483,13 @@
             <v>14</v>
           </cell>
           <cell r="F139">
-            <v>15</v>
+            <v>21</v>
           </cell>
           <cell r="H139" t="str">
             <v>C</v>
           </cell>
           <cell r="I139">
-            <v>9.5</v>
+            <v>3.5</v>
           </cell>
         </row>
         <row r="140">
@@ -3456,13 +3497,13 @@
             <v>14</v>
           </cell>
           <cell r="F140">
-            <v>7</v>
+            <v>14</v>
           </cell>
           <cell r="H140" t="str">
-            <v>D</v>
+            <v>C</v>
           </cell>
           <cell r="I140">
-            <v>7</v>
+            <v>10.5</v>
           </cell>
         </row>
         <row r="141">
@@ -3470,13 +3511,13 @@
             <v>14</v>
           </cell>
           <cell r="F141">
-            <v>8</v>
+            <v>12</v>
           </cell>
           <cell r="H141" t="str">
             <v>D</v>
           </cell>
           <cell r="I141">
-            <v>6</v>
+            <v>2</v>
           </cell>
         </row>
         <row r="142">
@@ -3484,13 +3525,13 @@
             <v>14</v>
           </cell>
           <cell r="F142">
-            <v>3</v>
+            <v>7</v>
           </cell>
           <cell r="H142" t="str">
             <v>D</v>
           </cell>
           <cell r="I142">
-            <v>11</v>
+            <v>7</v>
           </cell>
         </row>
         <row r="143">
@@ -3526,13 +3567,13 @@
             <v>14</v>
           </cell>
           <cell r="F145">
-            <v>2</v>
+            <v>3</v>
           </cell>
           <cell r="H145" t="str">
             <v>D</v>
           </cell>
           <cell r="I145">
-            <v>12</v>
+            <v>11</v>
           </cell>
         </row>
         <row r="146">
@@ -3540,13 +3581,13 @@
             <v>14</v>
           </cell>
           <cell r="F146">
-            <v>0</v>
+            <v>4</v>
           </cell>
           <cell r="H146" t="str">
             <v>D</v>
           </cell>
           <cell r="I146">
-            <v>14</v>
+            <v>10</v>
           </cell>
         </row>
         <row r="147">
@@ -3568,13 +3609,13 @@
             <v>14</v>
           </cell>
           <cell r="F148">
-            <v>1</v>
+            <v>3</v>
           </cell>
           <cell r="H148" t="str">
             <v>D</v>
           </cell>
           <cell r="I148">
-            <v>13</v>
+            <v>11</v>
           </cell>
         </row>
         <row r="149">
@@ -3582,13 +3623,13 @@
             <v>14</v>
           </cell>
           <cell r="F149">
-            <v>4</v>
+            <v>6</v>
           </cell>
           <cell r="H149" t="str">
             <v>D</v>
           </cell>
           <cell r="I149">
-            <v>10</v>
+            <v>8</v>
           </cell>
         </row>
         <row r="150">
@@ -3596,13 +3637,13 @@
             <v>14</v>
           </cell>
           <cell r="F150">
-            <v>0</v>
+            <v>9</v>
           </cell>
           <cell r="H150" t="str">
             <v>D</v>
           </cell>
           <cell r="I150">
-            <v>14</v>
+            <v>5</v>
           </cell>
         </row>
         <row r="151">
@@ -3610,13 +3651,13 @@
             <v>14</v>
           </cell>
           <cell r="F151">
-            <v>5</v>
+            <v>10</v>
           </cell>
           <cell r="H151" t="str">
             <v>D</v>
           </cell>
           <cell r="I151">
-            <v>9</v>
+            <v>4</v>
           </cell>
         </row>
         <row r="152">
@@ -3638,13 +3679,13 @@
             <v>14</v>
           </cell>
           <cell r="F153">
-            <v>0</v>
+            <v>3</v>
           </cell>
           <cell r="H153" t="str">
             <v>D</v>
           </cell>
           <cell r="I153">
-            <v>14</v>
+            <v>11</v>
           </cell>
         </row>
         <row r="154">
@@ -3652,10 +3693,10 @@
             <v>260</v>
           </cell>
           <cell r="F154">
-            <v>90</v>
+            <v>153</v>
           </cell>
           <cell r="I154">
-            <v>200.5</v>
+            <v>148</v>
           </cell>
         </row>
         <row r="158">
@@ -3677,13 +3718,13 @@
             <v>39600</v>
           </cell>
           <cell r="F159">
-            <v>16084.539999999992</v>
+            <v>27951.950000000019</v>
           </cell>
           <cell r="H159" t="str">
             <v>D</v>
           </cell>
           <cell r="I159">
-            <v>23515.460000000006</v>
+            <v>11648.049999999981</v>
           </cell>
         </row>
         <row r="160">
@@ -3691,13 +3732,13 @@
             <v>35550</v>
           </cell>
           <cell r="F160">
-            <v>13919.82</v>
+            <v>24446.020000000004</v>
           </cell>
           <cell r="H160" t="str">
             <v>D</v>
           </cell>
           <cell r="I160">
-            <v>21630.18</v>
+            <v>11103.979999999996</v>
           </cell>
         </row>
         <row r="161">
@@ -3705,13 +3746,13 @@
             <v>155250</v>
           </cell>
           <cell r="F161">
-            <v>80195.720000000016</v>
+            <v>117001.94999999997</v>
           </cell>
           <cell r="H161" t="str">
             <v>D</v>
           </cell>
           <cell r="I161">
-            <v>75054.279999999984</v>
+            <v>38248.050000000032</v>
           </cell>
         </row>
         <row r="162">
@@ -3719,13 +3760,13 @@
             <v>149175</v>
           </cell>
           <cell r="F162">
-            <v>68129</v>
+            <v>114216.91000000018</v>
           </cell>
           <cell r="H162" t="str">
             <v>D</v>
           </cell>
           <cell r="I162">
-            <v>81046</v>
+            <v>34958.089999999822</v>
           </cell>
         </row>
         <row r="163">
@@ -3733,13 +3774,13 @@
             <v>126450</v>
           </cell>
           <cell r="F163">
-            <v>52315.460000000036</v>
+            <v>87405.690000000031</v>
           </cell>
           <cell r="H163" t="str">
             <v>D</v>
           </cell>
           <cell r="I163">
-            <v>74134.539999999964</v>
+            <v>39044.309999999969</v>
           </cell>
         </row>
         <row r="164">
@@ -3747,13 +3788,13 @@
             <v>92700</v>
           </cell>
           <cell r="F164">
-            <v>34826.190000000031</v>
+            <v>56477.170000000086</v>
           </cell>
           <cell r="H164" t="str">
             <v>D</v>
           </cell>
           <cell r="I164">
-            <v>57873.809999999969</v>
+            <v>36222.829999999914</v>
           </cell>
         </row>
         <row r="165">
@@ -3761,13 +3802,13 @@
             <v>78750</v>
           </cell>
           <cell r="F165">
-            <v>26662.550000000017</v>
+            <v>53099.140000000007</v>
           </cell>
           <cell r="H165" t="str">
             <v>D</v>
           </cell>
           <cell r="I165">
-            <v>52087.449999999983</v>
+            <v>25650.859999999993</v>
           </cell>
         </row>
         <row r="166">
@@ -3775,13 +3816,13 @@
             <v>122400</v>
           </cell>
           <cell r="F166">
-            <v>51568.700000000055</v>
+            <v>81243.350000000093</v>
           </cell>
           <cell r="H166" t="str">
             <v>D</v>
           </cell>
           <cell r="I166">
-            <v>70831.299999999945</v>
+            <v>41156.649999999907</v>
           </cell>
         </row>
         <row r="167">
@@ -3803,13 +3844,13 @@
             <v>26100</v>
           </cell>
           <cell r="F168">
-            <v>9566.7999999999956</v>
+            <v>15939.879999999988</v>
           </cell>
           <cell r="H168" t="str">
             <v>D</v>
           </cell>
           <cell r="I168">
-            <v>16533.200000000004</v>
+            <v>10160.120000000012</v>
           </cell>
         </row>
         <row r="169">
@@ -3817,13 +3858,13 @@
             <v>43200</v>
           </cell>
           <cell r="F169">
-            <v>12079.49</v>
+            <v>25865.750000000011</v>
           </cell>
           <cell r="H169" t="str">
             <v>D</v>
           </cell>
           <cell r="I169">
-            <v>31120.510000000002</v>
+            <v>17334.249999999989</v>
           </cell>
         </row>
         <row r="170">
@@ -3831,13 +3872,13 @@
             <v>31725</v>
           </cell>
           <cell r="F170">
-            <v>10063.619999999999</v>
+            <v>19043.580000000002</v>
           </cell>
           <cell r="H170" t="str">
             <v>D</v>
           </cell>
           <cell r="I170">
-            <v>21661.38</v>
+            <v>12681.419999999998</v>
           </cell>
         </row>
         <row r="171">
@@ -3845,13 +3886,13 @@
             <v>37800</v>
           </cell>
           <cell r="F171">
-            <v>18377.800000000003</v>
+            <v>28099.500000000029</v>
           </cell>
           <cell r="H171" t="str">
             <v>D</v>
           </cell>
           <cell r="I171">
-            <v>19422.199999999997</v>
+            <v>9700.4999999999709</v>
           </cell>
         </row>
         <row r="172">
@@ -3859,13 +3900,13 @@
             <v>63900</v>
           </cell>
           <cell r="F172">
-            <v>29370.71000000001</v>
+            <v>44023.619999999988</v>
           </cell>
           <cell r="H172" t="str">
             <v>D</v>
           </cell>
           <cell r="I172">
-            <v>34529.289999999994</v>
+            <v>19876.380000000012</v>
           </cell>
         </row>
         <row r="173">
@@ -3873,13 +3914,13 @@
             <v>76050</v>
           </cell>
           <cell r="F173">
-            <v>29690.979999999996</v>
+            <v>48456.710000000006</v>
           </cell>
           <cell r="H173" t="str">
             <v>D</v>
           </cell>
           <cell r="I173">
-            <v>46359.020000000004</v>
+            <v>27593.289999999994</v>
           </cell>
         </row>
         <row r="174">
@@ -3887,13 +3928,13 @@
             <v>121500</v>
           </cell>
           <cell r="F174">
-            <v>49731.210000000028</v>
+            <v>89009.680000000051</v>
           </cell>
           <cell r="H174" t="str">
             <v>D</v>
           </cell>
           <cell r="I174">
-            <v>71768.789999999979</v>
+            <v>32490.319999999949</v>
           </cell>
         </row>
         <row r="175">
@@ -3901,13 +3942,13 @@
             <v>42975</v>
           </cell>
           <cell r="F175">
-            <v>6954.27</v>
+            <v>18272.769999999997</v>
           </cell>
           <cell r="H175" t="str">
             <v>D</v>
           </cell>
           <cell r="I175">
-            <v>36020.729999999996</v>
+            <v>24702.230000000003</v>
           </cell>
         </row>
         <row r="176">
@@ -3915,13 +3956,13 @@
             <v>97875</v>
           </cell>
           <cell r="F176">
-            <v>22063.71000000001</v>
+            <v>32493.730000000003</v>
           </cell>
           <cell r="H176" t="str">
             <v>D</v>
           </cell>
           <cell r="I176">
-            <v>75811.289999999994</v>
+            <v>65381.27</v>
           </cell>
         </row>
         <row r="177">
@@ -3929,10 +3970,10 @@
             <v>1341000</v>
           </cell>
           <cell r="F177">
-            <v>531600.57000000018</v>
+            <v>883047.40000000037</v>
           </cell>
           <cell r="I177">
-            <v>809399.4299999997</v>
+            <v>457952.59999999945</v>
           </cell>
         </row>
       </sheetData>
@@ -4812,7 +4853,7 @@
       </c>
       <c r="AN3" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI3,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>16084.539999999992</v>
+        <v>27951.950000000019</v>
       </c>
       <c r="AO3" s="26" t="str" cm="1">
         <f t="array" ref="AO3">_xlfn.IFS(AN3&gt;=AJ3,"A",AN3&gt;=AK3,"B",AN3&gt;=AL3,"C",AN3&gt;=AM3,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -4824,7 +4865,7 @@
       </c>
       <c r="AQ3" s="25" cm="1">
         <f t="array" ref="AQ3">_xlfn.IFS(AP3="D",MAX(AM3-AN3,0),AP3="C",MAX(AL3-AN3,0),AP3="B",MAX(AK3-AN3,0),AP3="A",MAX(AJ3-AN3,0),AP3="OBJETIVO ALCANÇADO",0)</f>
-        <v>23515.460000000006</v>
+        <v>11648.049999999981</v>
       </c>
     </row>
     <row r="4" spans="1:43" x14ac:dyDescent="0.25">
@@ -4845,7 +4886,7 @@
       </c>
       <c r="I4" s="7">
         <f>SUM(I10:I27)</f>
-        <v>160100</v>
+        <v>300010</v>
       </c>
       <c r="J4" s="4"/>
       <c r="K4" s="4"/>
@@ -4892,7 +4933,7 @@
       </c>
       <c r="AD4" s="31">
         <f>IFERROR(_xlfn.XLOOKUP(Y4,'[1]BASE PYTHON'!$K:$K,'[1]BASE PYTHON'!$M:$M,0),0)</f>
-        <v>42</v>
+        <v>53</v>
       </c>
       <c r="AE4" s="31" t="str" cm="1">
         <f t="array" ref="AE4">_xlfn.IFS(AD4&gt;=Z4,"A",AD4&gt;=AA4,"B",AD4&gt;=AB4,"C",AD4&gt;=AC4,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -4904,7 +4945,7 @@
       </c>
       <c r="AG4" s="31" cm="1">
         <f t="array" ref="AG4">_xlfn.IFS(AF4="D",MAX(AC4-AD4,0),AF4="C",MAX(AB4-AD4,0),AF4="B",MAX(AA4-AD4,0),AF4="A",MAX(Z4-AD4,0),AF4="OBJETIVO ALCANÇADO",0)</f>
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="AI4" t="s">
         <v>24</v>
@@ -4927,7 +4968,7 @@
       </c>
       <c r="AN4" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI4,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>13919.82</v>
+        <v>24446.020000000004</v>
       </c>
       <c r="AO4" s="26" t="str" cm="1">
         <f t="array" ref="AO4">_xlfn.IFS(AN4&gt;=AJ4,"A",AN4&gt;=AK4,"B",AN4&gt;=AL4,"C",AN4&gt;=AM4,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -4939,7 +4980,7 @@
       </c>
       <c r="AQ4" s="25" cm="1">
         <f t="array" ref="AQ4">_xlfn.IFS(AP4="D",MAX(AM4-AN4,0),AP4="C",MAX(AL4-AN4,0),AP4="B",MAX(AK4-AN4,0),AP4="A",MAX(AJ4-AN4,0),AP4="OBJETIVO ALCANÇADO",0)</f>
-        <v>21630.18</v>
+        <v>11103.979999999996</v>
       </c>
     </row>
     <row r="5" spans="1:43" x14ac:dyDescent="0.25">
@@ -4949,7 +4990,7 @@
       </c>
       <c r="C5" s="2">
         <f>SUM(D10:D36)</f>
-        <v>987586.73000000033</v>
+        <v>1561775.3300000003</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -4960,7 +5001,7 @@
       </c>
       <c r="I5" s="7">
         <f ca="1">SUM(J10:J27)</f>
-        <v>158397.37</v>
+        <v>89620.659999999974</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -4971,7 +5012,7 @@
       </c>
       <c r="O5" s="7">
         <f>SUM(P11:P17)</f>
-        <v>76637.150000000081</v>
+        <v>0</v>
       </c>
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
@@ -4982,7 +5023,7 @@
       </c>
       <c r="U5" s="4">
         <f ca="1">SUM(V10:V26)</f>
-        <v>48</v>
+        <v>100</v>
       </c>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -5042,7 +5083,7 @@
       </c>
       <c r="AN5" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI5,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>80195.720000000016</v>
+        <v>117001.94999999997</v>
       </c>
       <c r="AO5" s="26" t="str" cm="1">
         <f t="array" ref="AO5">_xlfn.IFS(AN5&gt;=AJ5,"A",AN5&gt;=AK5,"B",AN5&gt;=AL5,"C",AN5&gt;=AM5,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -5054,7 +5095,7 @@
       </c>
       <c r="AQ5" s="25" cm="1">
         <f t="array" ref="AQ5">_xlfn.IFS(AP5="D",MAX(AM5-AN5,0),AP5="C",MAX(AL5-AN5,0),AP5="B",MAX(AK5-AN5,0),AP5="A",MAX(AJ5-AN5,0),AP5="OBJETIVO ALCANÇADO",0)</f>
-        <v>75054.279999999984</v>
+        <v>38248.050000000032</v>
       </c>
     </row>
     <row r="6" spans="1:43" x14ac:dyDescent="0.25">
@@ -5064,7 +5105,7 @@
       </c>
       <c r="C6" s="2">
         <f>C4-C5</f>
-        <v>5043413.2699999996</v>
+        <v>4469224.67</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="4"/>
@@ -5075,7 +5116,7 @@
       </c>
       <c r="I6" s="7">
         <f ca="1">I4-I5</f>
-        <v>1702.6300000000047</v>
+        <v>210389.34000000003</v>
       </c>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -5086,7 +5127,7 @@
       </c>
       <c r="O6" s="7">
         <f>O4-O5</f>
-        <v>-76637.150000000081</v>
+        <v>0</v>
       </c>
       <c r="P6" s="4"/>
       <c r="Q6" s="4"/>
@@ -5097,7 +5138,7 @@
       </c>
       <c r="U6" s="4">
         <f ca="1">U4-U5</f>
-        <v>512</v>
+        <v>460</v>
       </c>
       <c r="V6" s="4"/>
       <c r="W6" s="4"/>
@@ -5157,7 +5198,7 @@
       </c>
       <c r="AN6" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI6,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>68129</v>
+        <v>114216.91000000018</v>
       </c>
       <c r="AO6" s="26" t="str" cm="1">
         <f t="array" ref="AO6">_xlfn.IFS(AN6&gt;=AJ6,"A",AN6&gt;=AK6,"B",AN6&gt;=AL6,"C",AN6&gt;=AM6,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -5169,7 +5210,7 @@
       </c>
       <c r="AQ6" s="25" cm="1">
         <f t="array" ref="AQ6">_xlfn.IFS(AP6="D",MAX(AM6-AN6,0),AP6="C",MAX(AL6-AN6,0),AP6="B",MAX(AK6-AN6,0),AP6="A",MAX(AJ6-AN6,0),AP6="OBJETIVO ALCANÇADO",0)</f>
-        <v>81046</v>
+        <v>34958.089999999822</v>
       </c>
     </row>
     <row r="7" spans="1:43" x14ac:dyDescent="0.25">
@@ -5179,7 +5220,7 @@
       </c>
       <c r="C7" s="3">
         <f>1-(C6/C4)</f>
-        <v>0.16375173768860896</v>
+        <v>0.25895793898192676</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="4"/>
@@ -5190,7 +5231,7 @@
       </c>
       <c r="I7" s="3">
         <f ca="1">1-(I6/I4)</f>
-        <v>0.98936520924422233</v>
+        <v>0.29872557581413939</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -5212,7 +5253,7 @@
       </c>
       <c r="U7" s="3">
         <f ca="1">1-(U6/U4)</f>
-        <v>8.5714285714285743E-2</v>
+        <v>0.1785714285714286</v>
       </c>
       <c r="V7" s="4"/>
       <c r="W7" s="4"/>
@@ -5272,7 +5313,7 @@
       </c>
       <c r="AN7" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI7,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>52315.460000000036</v>
+        <v>87405.690000000031</v>
       </c>
       <c r="AO7" s="26" t="str" cm="1">
         <f t="array" ref="AO7">_xlfn.IFS(AN7&gt;=AJ7,"A",AN7&gt;=AK7,"B",AN7&gt;=AL7,"C",AN7&gt;=AM7,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -5284,7 +5325,7 @@
       </c>
       <c r="AQ7" s="25" cm="1">
         <f t="array" ref="AQ7">_xlfn.IFS(AP7="D",MAX(AM7-AN7,0),AP7="C",MAX(AL7-AN7,0),AP7="B",MAX(AK7-AN7,0),AP7="A",MAX(AJ7-AN7,0),AP7="OBJETIVO ALCANÇADO",0)</f>
-        <v>74134.539999999964</v>
+        <v>39044.309999999969</v>
       </c>
     </row>
     <row r="8" spans="1:43" x14ac:dyDescent="0.25">
@@ -5366,7 +5407,7 @@
       </c>
       <c r="AN8" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI8,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>34826.190000000031</v>
+        <v>56477.170000000086</v>
       </c>
       <c r="AO8" s="26" t="str" cm="1">
         <f t="array" ref="AO8">_xlfn.IFS(AN8&gt;=AJ8,"A",AN8&gt;=AK8,"B",AN8&gt;=AL8,"C",AN8&gt;=AM8,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -5378,7 +5419,7 @@
       </c>
       <c r="AQ8" s="25" cm="1">
         <f t="array" ref="AQ8">_xlfn.IFS(AP8="D",MAX(AM8-AN8,0),AP8="C",MAX(AL8-AN8,0),AP8="B",MAX(AK8-AN8,0),AP8="A",MAX(AJ8-AN8,0),AP8="OBJETIVO ALCANÇADO",0)</f>
-        <v>57873.809999999969</v>
+        <v>36222.829999999914</v>
       </c>
     </row>
     <row r="9" spans="1:43" x14ac:dyDescent="0.25">
@@ -5417,7 +5458,7 @@
       <c r="M9" s="4"/>
       <c r="N9" s="4"/>
       <c r="O9" s="8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="P9" s="4"/>
       <c r="Q9" s="4"/>
@@ -5493,7 +5534,7 @@
       </c>
       <c r="AN9" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI9,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>26662.550000000017</v>
+        <v>53099.140000000007</v>
       </c>
       <c r="AO9" s="26" t="str" cm="1">
         <f t="array" ref="AO9">_xlfn.IFS(AN9&gt;=AJ9,"A",AN9&gt;=AK9,"B",AN9&gt;=AL9,"C",AN9&gt;=AM9,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -5505,7 +5546,7 @@
       </c>
       <c r="AQ9" s="25" cm="1">
         <f t="array" ref="AQ9">_xlfn.IFS(AP9="D",MAX(AM9-AN9,0),AP9="C",MAX(AL9-AN9,0),AP9="B",MAX(AK9-AN9,0),AP9="A",MAX(AJ9-AN9,0),AP9="OBJETIVO ALCANÇADO",0)</f>
-        <v>52087.449999999983</v>
+        <v>25650.859999999993</v>
       </c>
     </row>
     <row r="10" spans="1:43" x14ac:dyDescent="0.25">
@@ -5521,11 +5562,11 @@
       </c>
       <c r="D10" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>10063.619999999999</v>
+        <v>19043.580000000002</v>
       </c>
       <c r="E10" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>60436.380000000005</v>
+        <v>51456.42</v>
       </c>
       <c r="F10" s="4"/>
       <c r="G10" s="18" t="s">
@@ -5536,15 +5577,15 @@
       </c>
       <c r="I10" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>16760</v>
+        <v>28000</v>
       </c>
       <c r="J10" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>15414.589999999998</v>
+        <v>13963.489999999998</v>
       </c>
       <c r="K10" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>1345.4100000000017</v>
+        <v>14036.510000000002</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4" t="s">
@@ -5637,7 +5678,7 @@
       </c>
       <c r="AN10" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI10,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>51568.700000000055</v>
+        <v>81243.350000000093</v>
       </c>
       <c r="AO10" s="26" t="str" cm="1">
         <f t="array" ref="AO10">_xlfn.IFS(AN10&gt;=AJ10,"A",AN10&gt;=AK10,"B",AN10&gt;=AL10,"C",AN10&gt;=AM10,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -5649,7 +5690,7 @@
       </c>
       <c r="AQ10" s="25" cm="1">
         <f t="array" ref="AQ10">_xlfn.IFS(AP10="D",MAX(AM10-AN10,0),AP10="C",MAX(AL10-AN10,0),AP10="B",MAX(AK10-AN10,0),AP10="A",MAX(AJ10-AN10,0),AP10="OBJETIVO ALCANÇADO",0)</f>
-        <v>70831.299999999945</v>
+        <v>41156.649999999907</v>
       </c>
     </row>
     <row r="11" spans="1:43" x14ac:dyDescent="0.25">
@@ -5665,11 +5706,11 @@
       </c>
       <c r="D11" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>80195.720000000016</v>
+        <v>117001.94999999997</v>
       </c>
       <c r="E11" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>264804.27999999997</v>
+        <v>227998.05000000005</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="18" t="s">
@@ -5680,15 +5721,15 @@
       </c>
       <c r="I11" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>16230</v>
+        <v>25000</v>
       </c>
       <c r="J11" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>14149.629999999996</v>
+        <v>5135.0499999999984</v>
       </c>
       <c r="K11" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>2080.3700000000044</v>
+        <v>19864.95</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4" t="s">
@@ -5722,11 +5763,11 @@
       </c>
       <c r="V11" s="17">
         <f ca="1">IFERROR(VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0),0)</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="W11" s="17">
         <f t="shared" ref="W11:W20" ca="1" si="0">U11-V11</f>
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="Y11" s="32" t="s">
         <v>12</v>
@@ -5812,11 +5853,11 @@
       </c>
       <c r="D12" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>0</v>
+        <v>324.10000000000002</v>
       </c>
       <c r="E12" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>0</v>
+        <v>-324.10000000000002</v>
       </c>
       <c r="F12" s="4"/>
       <c r="G12" s="18" t="s">
@@ -5827,15 +5868,15 @@
       </c>
       <c r="I12" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>10030</v>
+        <v>14510</v>
       </c>
       <c r="J12" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>13074.129999999997</v>
+        <v>2919.1</v>
       </c>
       <c r="K12" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>-3044.1299999999974</v>
+        <v>11590.9</v>
       </c>
       <c r="L12" s="4"/>
       <c r="M12" s="4" t="s">
@@ -5868,12 +5909,12 @@
         <v>35</v>
       </c>
       <c r="V12" s="17">
-        <f>IFERROR(VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0),0)</f>
-        <v>0</v>
+        <f ca="1">IFERROR(VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0),0)</f>
+        <v>4</v>
       </c>
       <c r="W12" s="17">
-        <f t="shared" si="0"/>
-        <v>35</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>31</v>
       </c>
       <c r="Y12" s="33" t="s">
         <v>23</v>
@@ -5931,7 +5972,7 @@
       </c>
       <c r="AN12" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI12,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>9566.7999999999956</v>
+        <v>15939.879999999988</v>
       </c>
       <c r="AO12" s="26" t="str" cm="1">
         <f t="array" ref="AO12">_xlfn.IFS(AN12&gt;=AJ12,"A",AN12&gt;=AK12,"B",AN12&gt;=AL12,"C",AN12&gt;=AM12,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -5943,7 +5984,7 @@
       </c>
       <c r="AQ12" s="25" cm="1">
         <f t="array" ref="AQ12">_xlfn.IFS(AP12="D",MAX(AM12-AN12,0),AP12="C",MAX(AL12-AN12,0),AP12="B",MAX(AK12-AN12,0),AP12="A",MAX(AJ12-AN12,0),AP12="OBJETIVO ALCANÇADO",0)</f>
-        <v>16533.200000000004</v>
+        <v>10160.120000000012</v>
       </c>
     </row>
     <row r="13" spans="1:43" x14ac:dyDescent="0.25">
@@ -5959,11 +6000,11 @@
       </c>
       <c r="D13" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>12079.49</v>
+        <v>25865.750000000011</v>
       </c>
       <c r="E13" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>83920.51</v>
+        <v>70134.249999999985</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="18" t="s">
@@ -5974,15 +6015,15 @@
       </c>
       <c r="I13" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>14910</v>
+        <v>24000</v>
       </c>
       <c r="J13" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>17436.830000000009</v>
+        <v>15594.409999999996</v>
       </c>
       <c r="K13" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>-2526.830000000009</v>
+        <v>8405.5900000000038</v>
       </c>
       <c r="L13" s="4"/>
       <c r="M13" s="4" t="s">
@@ -6016,11 +6057,11 @@
       </c>
       <c r="V13" s="17">
         <f ca="1">IFERROR(VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0),0)</f>
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="W13" s="17">
         <f t="shared" ca="1" si="0"/>
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="Y13" s="32" t="s">
         <v>9</v>
@@ -6078,7 +6119,7 @@
       </c>
       <c r="AN13" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI13,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>12079.49</v>
+        <v>25865.750000000011</v>
       </c>
       <c r="AO13" s="26" t="str" cm="1">
         <f t="array" ref="AO13">_xlfn.IFS(AN13&gt;=AJ13,"A",AN13&gt;=AK13,"B",AN13&gt;=AL13,"C",AN13&gt;=AM13,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -6090,7 +6131,7 @@
       </c>
       <c r="AQ13" s="25" cm="1">
         <f t="array" ref="AQ13">_xlfn.IFS(AP13="D",MAX(AM13-AN13,0),AP13="C",MAX(AL13-AN13,0),AP13="B",MAX(AK13-AN13,0),AP13="A",MAX(AJ13-AN13,0),AP13="OBJETIVO ALCANÇADO",0)</f>
-        <v>31120.510000000002</v>
+        <v>17334.249999999989</v>
       </c>
     </row>
     <row r="14" spans="1:43" x14ac:dyDescent="0.25">
@@ -6106,11 +6147,11 @@
       </c>
       <c r="D14" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>52315.460000000036</v>
+        <v>87405.690000000031</v>
       </c>
       <c r="E14" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>228684.53999999998</v>
+        <v>193594.30999999997</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="18" t="s">
@@ -6121,15 +6162,15 @@
       </c>
       <c r="I14" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>11680</v>
+        <v>19770</v>
       </c>
       <c r="J14" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>7410.8999999999987</v>
+        <v>1402.54</v>
       </c>
       <c r="K14" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>4269.1000000000013</v>
+        <v>18367.46</v>
       </c>
       <c r="L14" s="4"/>
       <c r="M14" s="4" t="s">
@@ -6163,11 +6204,11 @@
       </c>
       <c r="V14" s="17">
         <f ca="1">IFERROR(VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0),0)</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="W14" s="17">
         <f t="shared" ca="1" si="0"/>
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="Y14" s="33" t="s">
         <v>7</v>
@@ -6225,7 +6266,7 @@
       </c>
       <c r="AN14" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI14,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>10063.619999999999</v>
+        <v>19043.580000000002</v>
       </c>
       <c r="AO14" s="26" t="str" cm="1">
         <f t="array" ref="AO14">_xlfn.IFS(AN14&gt;=AJ14,"A",AN14&gt;=AK14,"B",AN14&gt;=AL14,"C",AN14&gt;=AM14,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -6237,7 +6278,7 @@
       </c>
       <c r="AQ14" s="25" cm="1">
         <f t="array" ref="AQ14">_xlfn.IFS(AP14="D",MAX(AM14-AN14,0),AP14="C",MAX(AL14-AN14,0),AP14="B",MAX(AK14-AN14,0),AP14="A",MAX(AJ14-AN14,0),AP14="OBJETIVO ALCANÇADO",0)</f>
-        <v>21661.38</v>
+        <v>12681.419999999998</v>
       </c>
     </row>
     <row r="15" spans="1:43" x14ac:dyDescent="0.25">
@@ -6253,11 +6294,11 @@
       </c>
       <c r="D15" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>18377.800000000003</v>
+        <v>28099.500000000029</v>
       </c>
       <c r="E15" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>65622.2</v>
+        <v>55900.499999999971</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="18" t="s">
@@ -6268,15 +6309,15 @@
       </c>
       <c r="I15" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>11360</v>
+        <v>31000</v>
       </c>
       <c r="J15" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>20574.03</v>
+        <v>11533.52</v>
       </c>
       <c r="K15" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>-9214.0299999999988</v>
+        <v>19466.48</v>
       </c>
       <c r="L15" s="4"/>
       <c r="M15" s="4" t="s">
@@ -6372,7 +6413,7 @@
       </c>
       <c r="AN15" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI15,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>18377.800000000003</v>
+        <v>28099.500000000029</v>
       </c>
       <c r="AO15" s="26" t="str" cm="1">
         <f t="array" ref="AO15">_xlfn.IFS(AN15&gt;=AJ15,"A",AN15&gt;=AK15,"B",AN15&gt;=AL15,"C",AN15&gt;=AM15,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -6384,7 +6425,7 @@
       </c>
       <c r="AQ15" s="25" cm="1">
         <f t="array" ref="AQ15">_xlfn.IFS(AP15="D",MAX(AM15-AN15,0),AP15="C",MAX(AL15-AN15,0),AP15="B",MAX(AK15-AN15,0),AP15="A",MAX(AJ15-AN15,0),AP15="OBJETIVO ALCANÇADO",0)</f>
-        <v>19422.199999999997</v>
+        <v>9700.4999999999709</v>
       </c>
     </row>
     <row r="16" spans="1:43" x14ac:dyDescent="0.25">
@@ -6400,11 +6441,11 @@
       </c>
       <c r="D16" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>41478.5</v>
+        <v>90046.700000000012</v>
       </c>
       <c r="E16" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>308521.5</v>
+        <v>259953.3</v>
       </c>
       <c r="F16" s="4"/>
       <c r="G16" s="18" t="s">
@@ -6415,15 +6456,15 @@
       </c>
       <c r="I16" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>13010</v>
+        <v>19620</v>
       </c>
       <c r="J16" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>6242.6200000000008</v>
+        <v>2159.1999999999998</v>
       </c>
       <c r="K16" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>6767.3799999999992</v>
+        <v>17460.8</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="4" t="s">
@@ -6519,7 +6560,7 @@
       </c>
       <c r="AN16" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI16,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>29370.71000000001</v>
+        <v>44023.619999999988</v>
       </c>
       <c r="AO16" s="26" t="str" cm="1">
         <f t="array" ref="AO16">_xlfn.IFS(AN16&gt;=AJ16,"A",AN16&gt;=AK16,"B",AN16&gt;=AL16,"C",AN16&gt;=AM16,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -6531,7 +6572,7 @@
       </c>
       <c r="AQ16" s="25" cm="1">
         <f t="array" ref="AQ16">_xlfn.IFS(AP16="D",MAX(AM16-AN16,0),AP16="C",MAX(AL16-AN16,0),AP16="B",MAX(AK16-AN16,0),AP16="A",MAX(AJ16-AN16,0),AP16="OBJETIVO ALCANÇADO",0)</f>
-        <v>34529.289999999994</v>
+        <v>19876.380000000012</v>
       </c>
     </row>
     <row r="17" spans="1:43" x14ac:dyDescent="0.25">
@@ -6547,11 +6588,11 @@
       </c>
       <c r="D17" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>80120.350000000079</v>
+        <v>104355.99000000003</v>
       </c>
       <c r="E17" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>419879.64999999991</v>
+        <v>395644.00999999995</v>
       </c>
       <c r="F17" s="4"/>
       <c r="G17" s="18" t="s">
@@ -6562,15 +6603,15 @@
       </c>
       <c r="I17" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>7100</v>
+        <v>10110</v>
       </c>
       <c r="J17" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1715.4</v>
+        <v>2549.5500000000002</v>
       </c>
       <c r="K17" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>5384.6</v>
+        <v>7560.45</v>
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="4" t="s">
@@ -6585,11 +6626,11 @@
       </c>
       <c r="P17" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[REGIAO]","[Intervalo 2].[REGIAO].&amp;["&amp;N17&amp;"]","[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;["&amp;RIGHT($O$9,1)&amp;"]"),0)</f>
-        <v>76637.150000000081</v>
+        <v>0</v>
       </c>
       <c r="Q17" s="2">
         <f>Tabela8[[#This Row],[COMPROMISSO]]-Tabela8[[#This Row],[ATINGIDO]]</f>
-        <v>-76637.150000000081</v>
+        <v>0</v>
       </c>
       <c r="R17" s="2"/>
       <c r="S17" s="17" t="s">
@@ -6604,11 +6645,11 @@
       </c>
       <c r="V17" s="17">
         <f ca="1">IFERROR(VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0),0)</f>
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="W17" s="17">
         <f t="shared" ca="1" si="0"/>
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="Y17" s="32" t="s">
         <v>14</v>
@@ -6666,7 +6707,7 @@
       </c>
       <c r="AN17" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI17,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>29690.979999999996</v>
+        <v>48456.710000000006</v>
       </c>
       <c r="AO17" s="26" t="str" cm="1">
         <f t="array" ref="AO17">_xlfn.IFS(AN17&gt;=AJ17,"A",AN17&gt;=AK17,"B",AN17&gt;=AL17,"C",AN17&gt;=AM17,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -6678,7 +6719,7 @@
       </c>
       <c r="AQ17" s="25" cm="1">
         <f t="array" ref="AQ17">_xlfn.IFS(AP17="D",MAX(AM17-AN17,0),AP17="C",MAX(AL17-AN17,0),AP17="B",MAX(AK17-AN17,0),AP17="A",MAX(AJ17-AN17,0),AP17="OBJETIVO ALCANÇADO",0)</f>
-        <v>46359.020000000004</v>
+        <v>27593.289999999994</v>
       </c>
     </row>
     <row r="18" spans="1:43" x14ac:dyDescent="0.25">
@@ -6694,11 +6735,11 @@
       </c>
       <c r="D18" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>212283.80000000005</v>
+        <v>284976.00000000006</v>
       </c>
       <c r="E18" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>767716.2</v>
+        <v>695024</v>
       </c>
       <c r="F18" s="4"/>
       <c r="G18" s="18" t="s">
@@ -6800,7 +6841,7 @@
       </c>
       <c r="AN18" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI18,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>49731.210000000028</v>
+        <v>89009.680000000051</v>
       </c>
       <c r="AO18" s="26" t="str" cm="1">
         <f t="array" ref="AO18">_xlfn.IFS(AN18&gt;=AJ18,"A",AN18&gt;=AK18,"B",AN18&gt;=AL18,"C",AN18&gt;=AM18,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -6812,7 +6853,7 @@
       </c>
       <c r="AQ18" s="25" cm="1">
         <f t="array" ref="AQ18">_xlfn.IFS(AP18="D",MAX(AM18-AN18,0),AP18="C",MAX(AL18-AN18,0),AP18="B",MAX(AK18-AN18,0),AP18="A",MAX(AJ18-AN18,0),AP18="OBJETIVO ALCANÇADO",0)</f>
-        <v>71768.789999999979</v>
+        <v>32490.319999999949</v>
       </c>
     </row>
     <row r="19" spans="1:43" x14ac:dyDescent="0.25">
@@ -6828,11 +6869,11 @@
       </c>
       <c r="D19" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>4315.6000000000004</v>
+        <v>10406.4</v>
       </c>
       <c r="E19" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>145684.4</v>
+        <v>139593.60000000001</v>
       </c>
       <c r="F19" s="4"/>
       <c r="G19" s="18" t="s">
@@ -6843,15 +6884,15 @@
       </c>
       <c r="I19" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>10320</v>
+        <v>19890</v>
       </c>
       <c r="J19" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>14702.329999999998</v>
+        <v>988.43000000000006</v>
       </c>
       <c r="K19" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>-4382.3299999999981</v>
+        <v>18901.57</v>
       </c>
       <c r="L19" s="4"/>
       <c r="M19" s="4"/>
@@ -6868,11 +6909,11 @@
       </c>
       <c r="V19" s="17">
         <f ca="1">IFERROR(VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0),0)</f>
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="W19" s="17">
         <f t="shared" ca="1" si="0"/>
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="Y19" s="32" t="s">
         <v>16</v>
@@ -6930,7 +6971,7 @@
       </c>
       <c r="AN19" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI19,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>6954.27</v>
+        <v>18272.769999999997</v>
       </c>
       <c r="AO19" s="26" t="str" cm="1">
         <f t="array" ref="AO19">_xlfn.IFS(AN19&gt;=AJ19,"A",AN19&gt;=AK19,"B",AN19&gt;=AL19,"C",AN19&gt;=AM19,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -6942,7 +6983,7 @@
       </c>
       <c r="AQ19" s="25" cm="1">
         <f t="array" ref="AQ19">_xlfn.IFS(AP19="D",MAX(AM19-AN19,0),AP19="C",MAX(AL19-AN19,0),AP19="B",MAX(AK19-AN19,0),AP19="A",MAX(AJ19-AN19,0),AP19="OBJETIVO ALCANÇADO",0)</f>
-        <v>36020.729999999996</v>
+        <v>24702.230000000003</v>
       </c>
     </row>
     <row r="20" spans="1:43" x14ac:dyDescent="0.25">
@@ -6958,11 +6999,11 @@
       </c>
       <c r="D20" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>38918.429999999993</v>
+        <v>76109.040000000023</v>
       </c>
       <c r="E20" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>551081.57000000007</v>
+        <v>513890.95999999996</v>
       </c>
       <c r="F20" s="4"/>
       <c r="G20" s="18" t="s">
@@ -6973,15 +7014,15 @@
       </c>
       <c r="I20" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>13370</v>
+        <v>25000</v>
       </c>
       <c r="J20" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>19307.170000000002</v>
+        <v>10562.029999999999</v>
       </c>
       <c r="K20" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>-5937.1700000000019</v>
+        <v>14437.970000000001</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="4"/>
@@ -7009,12 +7050,12 @@
         <v>35</v>
       </c>
       <c r="V20" s="17">
-        <f>IFERROR(VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0),0)</f>
-        <v>0</v>
+        <f ca="1">IFERROR(VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0),0)</f>
+        <v>9</v>
       </c>
       <c r="W20" s="17">
-        <f t="shared" si="0"/>
-        <v>35</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>26</v>
       </c>
       <c r="Y20" s="33" t="s">
         <v>15</v>
@@ -7072,7 +7113,7 @@
       </c>
       <c r="AN20" s="25">
         <f>IFERROR(_xlfn.XLOOKUP(AI20,'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0),0)</f>
-        <v>22063.71000000001</v>
+        <v>32493.730000000003</v>
       </c>
       <c r="AO20" s="26" t="str" cm="1">
         <f t="array" ref="AO20">_xlfn.IFS(AN20&gt;=AJ20,"A",AN20&gt;=AK20,"B",AN20&gt;=AL20,"C",AN20&gt;=AM20,"D",TRUE,"NÃO ATINGIDO")</f>
@@ -7084,7 +7125,7 @@
       </c>
       <c r="AQ20" s="25" cm="1">
         <f t="array" ref="AQ20">_xlfn.IFS(AP20="D",MAX(AM20-AN20,0),AP20="C",MAX(AL20-AN20,0),AP20="B",MAX(AK20-AN20,0),AP20="A",MAX(AJ20-AN20,0),AP20="OBJETIVO ALCANÇADO",0)</f>
-        <v>75811.289999999994</v>
+        <v>65381.27</v>
       </c>
     </row>
     <row r="21" spans="1:43" x14ac:dyDescent="0.25">
@@ -7100,11 +7141,11 @@
       </c>
       <c r="D21" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>78869.479999999967</v>
+        <v>112434.5800000001</v>
       </c>
       <c r="E21" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>401130.52</v>
+        <v>367565.41999999993</v>
       </c>
       <c r="F21" s="4"/>
       <c r="G21" s="18" t="s">
@@ -7115,15 +7156,15 @@
       </c>
       <c r="I21" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>4460</v>
+        <v>5700</v>
       </c>
       <c r="J21" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>6113.9899999999989</v>
+        <v>2244.54</v>
       </c>
       <c r="K21" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>-1653.9899999999989</v>
+        <v>3455.46</v>
       </c>
       <c r="L21" s="4"/>
       <c r="M21" s="4"/>
@@ -7155,11 +7196,11 @@
       </c>
       <c r="V21" s="17">
         <f ca="1">IFERROR(VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0),0)</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="W21" s="17">
         <f t="shared" ref="W21:W26" ca="1" si="1">U21-V21</f>
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="Y21" s="36" t="s">
         <v>60</v>
@@ -7182,13 +7223,13 @@
       </c>
       <c r="AD21" s="37">
         <f>SUBTOTAL(109,Planilha1!$AD$3:$AD$20)</f>
-        <v>42</v>
+        <v>53</v>
       </c>
       <c r="AE21" s="37"/>
       <c r="AF21" s="37"/>
       <c r="AG21" s="38">
         <f>SUBTOTAL(109,Planilha1!$AG$3:$AG$20)</f>
-        <v>238</v>
+        <v>227</v>
       </c>
       <c r="AI21" t="s">
         <v>60</v>
@@ -7211,13 +7252,13 @@
       </c>
       <c r="AN21" s="26">
         <f>SUBTOTAL(109,Tabela817[ATINGIDO])</f>
-        <v>531600.57000000018</v>
+        <v>883047.40000000037</v>
       </c>
       <c r="AO21" s="4"/>
       <c r="AP21" s="4"/>
       <c r="AQ21" s="27">
         <f>SUBTOTAL(109,Tabela817[FALTA])</f>
-        <v>809399.4299999997</v>
+        <v>457952.59999999945</v>
       </c>
     </row>
     <row r="22" spans="1:43" x14ac:dyDescent="0.25">
@@ -7248,15 +7289,15 @@
       </c>
       <c r="I22" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>8680</v>
+        <v>21000</v>
       </c>
       <c r="J22" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>5677.8999999999987</v>
+        <v>4973.12</v>
       </c>
       <c r="K22" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3002.1000000000013</v>
+        <v>16026.880000000001</v>
       </c>
       <c r="L22" s="4"/>
       <c r="M22" s="4"/>
@@ -7269,11 +7310,11 @@
       </c>
       <c r="P22" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$32,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>76637.150000000081</v>
+        <v>100872.79000000004</v>
       </c>
       <c r="Q22" s="7">
         <f>O22-P22</f>
-        <v>649553.32619047607</v>
+        <v>625317.68619047618</v>
       </c>
       <c r="R22" s="4"/>
       <c r="S22" s="17" t="s">
@@ -7288,11 +7329,11 @@
       </c>
       <c r="V22" s="17">
         <f ca="1">IFERROR(VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0),0)</f>
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="W22" s="17">
         <f t="shared" ca="1" si="1"/>
-        <v>32</v>
+        <v>28</v>
       </c>
     </row>
     <row r="23" spans="1:43" x14ac:dyDescent="0.25">
@@ -7308,11 +7349,11 @@
       </c>
       <c r="D23" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>34826.190000000031</v>
+        <v>56477.170000000086</v>
       </c>
       <c r="E23" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>171173.80999999997</v>
+        <v>149522.8299999999</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="18" t="s">
@@ -7323,15 +7364,15 @@
       </c>
       <c r="I23" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>5070</v>
+        <v>15530</v>
       </c>
       <c r="J23" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>1785.95</v>
+        <v>4577.72</v>
       </c>
       <c r="K23" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>3284.05</v>
+        <v>10952.279999999999</v>
       </c>
       <c r="L23" s="4"/>
       <c r="M23" s="4"/>
@@ -7363,11 +7404,11 @@
       </c>
       <c r="V23" s="17">
         <f ca="1">IFERROR(VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0),0)</f>
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="W23" s="17">
         <f t="shared" ca="1" si="1"/>
-        <v>30</v>
+        <v>25</v>
       </c>
     </row>
     <row r="24" spans="1:43" x14ac:dyDescent="0.25">
@@ -7383,11 +7424,11 @@
       </c>
       <c r="D24" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>29690.979999999996</v>
+        <v>48456.710000000006</v>
       </c>
       <c r="E24" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>139309.02000000002</v>
+        <v>120543.29</v>
       </c>
       <c r="F24" s="4"/>
       <c r="G24" s="18" t="s">
@@ -7398,15 +7439,15 @@
       </c>
       <c r="I24" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>3720</v>
+        <v>10850</v>
       </c>
       <c r="J24" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>4707.7</v>
+        <v>2619.7000000000003</v>
       </c>
       <c r="K24" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>-987.69999999999982</v>
+        <v>8230.2999999999993</v>
       </c>
       <c r="L24" s="4"/>
       <c r="M24" s="4"/>
@@ -7438,11 +7479,11 @@
       </c>
       <c r="V24" s="17">
         <f ca="1">IFERROR(VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0),0)</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="W24" s="17">
         <f t="shared" ca="1" si="1"/>
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="25" spans="1:43" x14ac:dyDescent="0.25">
@@ -7458,11 +7499,11 @@
       </c>
       <c r="D25" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>22063.71000000001</v>
+        <v>32493.730000000003</v>
       </c>
       <c r="E25" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>195436.28999999998</v>
+        <v>185006.27</v>
       </c>
       <c r="F25" s="4"/>
       <c r="G25" s="18" t="s">
@@ -7473,15 +7514,15 @@
       </c>
       <c r="I25" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>4770</v>
+        <v>15300</v>
       </c>
       <c r="J25" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2525.3999999999992</v>
+        <v>5642.74</v>
       </c>
       <c r="K25" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>2244.6000000000008</v>
+        <v>9657.26</v>
       </c>
       <c r="L25" s="4"/>
       <c r="M25" s="4"/>
@@ -7512,12 +7553,12 @@
         <v>35</v>
       </c>
       <c r="V25" s="17">
-        <f>IFERROR(VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0),0)</f>
-        <v>0</v>
+        <f ca="1">IFERROR(VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0),0)</f>
+        <v>3</v>
       </c>
       <c r="W25" s="17">
-        <f t="shared" si="1"/>
-        <v>35</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>32</v>
       </c>
     </row>
     <row r="26" spans="1:43" x14ac:dyDescent="0.25">
@@ -7533,11 +7574,11 @@
       </c>
       <c r="D26" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>6954.27</v>
+        <v>18272.769999999997</v>
       </c>
       <c r="E26" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>88545.73</v>
+        <v>77227.23000000001</v>
       </c>
       <c r="F26" s="4"/>
       <c r="G26" s="18" t="s">
@@ -7548,15 +7589,15 @@
       </c>
       <c r="I26" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>3190</v>
+        <v>8980</v>
       </c>
       <c r="J26" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>2261.0300000000002</v>
+        <v>1484.7000000000003</v>
       </c>
       <c r="K26" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>928.9699999999998</v>
+        <v>7495.2999999999993</v>
       </c>
       <c r="L26" s="4"/>
       <c r="M26" s="4"/>
@@ -7577,11 +7618,11 @@
       </c>
       <c r="V26" s="17">
         <f ca="1">IFERROR(VLOOKUP(Tabela2[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$K:$N,'[1]BASE PYTHON'!L$1,0),0)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="W26" s="17">
         <f t="shared" ca="1" si="1"/>
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="27" spans="1:43" x14ac:dyDescent="0.25">
@@ -7597,11 +7638,11 @@
       </c>
       <c r="D27" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>51568.700000000055</v>
+        <v>81243.350000000093</v>
       </c>
       <c r="E27" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>220431.29999999993</v>
+        <v>190756.64999999991</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="18" t="s">
@@ -7612,15 +7653,15 @@
       </c>
       <c r="I27" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$A$39:$A$55,'[1]BASE PYTHON'!$B$39:$B$55,0)</f>
-        <v>5440</v>
+        <v>5750</v>
       </c>
       <c r="J27" s="19">
         <f>_xlfn.XLOOKUP(Tabela5[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$H:$H,'[1]BASE PYTHON'!$I:$I,0)</f>
-        <v>5297.7699999999995</v>
+        <v>1270.82</v>
       </c>
       <c r="K27" s="20">
         <f>Tabela5[[#This Row],[COMPROMISSO]]-Tabela5[[#This Row],[ATINGIDO]]</f>
-        <v>142.23000000000047</v>
+        <v>4479.18</v>
       </c>
       <c r="L27" s="4"/>
       <c r="M27" s="4"/>
@@ -7643,11 +7684,11 @@
       </c>
       <c r="D28" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>68129</v>
+        <v>114216.91000000018</v>
       </c>
       <c r="E28" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>263371</v>
+        <v>217283.08999999982</v>
       </c>
       <c r="F28" s="4"/>
       <c r="L28" s="4"/>
@@ -7722,11 +7763,11 @@
       </c>
       <c r="D30" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>29370.71000000001</v>
+        <v>44023.619999999988</v>
       </c>
       <c r="E30" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>112629.29</v>
+        <v>97976.38</v>
       </c>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
@@ -7759,11 +7800,11 @@
       </c>
       <c r="V30" s="5">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE 2]",'[1]BASE PYTHON'!$P$83,"[Intervalo 3].[SEMANAL]","[Intervalo 3].[SEMANAL].&amp;[1]"),0)</f>
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="W30" s="6">
         <f>U30-V30</f>
-        <v>38.333333333333336</v>
+        <v>32.333333333333336</v>
       </c>
     </row>
     <row r="31" spans="1:43" x14ac:dyDescent="0.25">
@@ -7779,11 +7820,11 @@
       </c>
       <c r="D31" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>26662.550000000017</v>
+        <v>53099.140000000007</v>
       </c>
       <c r="E31" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>148337.44999999998</v>
+        <v>121900.85999999999</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
@@ -7796,11 +7837,11 @@
       </c>
       <c r="J31" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[1]"),0)</f>
-        <v>120365.50999999998</v>
+        <v>120065.70999999995</v>
       </c>
       <c r="K31" s="7">
         <f>I31-J31</f>
-        <v>163444.01380952381</v>
+        <v>163743.81380952382</v>
       </c>
       <c r="L31" s="4"/>
       <c r="M31" s="4"/>
@@ -7819,11 +7860,11 @@
       </c>
       <c r="V31" s="5">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Contagem Distinta de COD_CLIENTE 2]",'[1]BASE PYTHON'!$P$83,"[Intervalo 3].[SEMANAL]","[Intervalo 3].[SEMANAL].&amp;[2]"),0)</f>
-        <v>33</v>
+        <v>79</v>
       </c>
       <c r="W31" s="6">
         <f t="shared" ref="W31:W33" si="2">U31-V31</f>
-        <v>100.33333333333334</v>
+        <v>54.333333333333343</v>
       </c>
     </row>
     <row r="32" spans="1:43" x14ac:dyDescent="0.25">
@@ -7839,11 +7880,11 @@
       </c>
       <c r="D32" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>49731.210000000028</v>
+        <v>89009.680000000051</v>
       </c>
       <c r="E32" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>220268.78999999998</v>
+        <v>180990.31999999995</v>
       </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
@@ -7856,11 +7897,11 @@
       </c>
       <c r="J32" s="7">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$4,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>307822.27999999991</v>
+        <v>587944.82000000135</v>
       </c>
       <c r="K32" s="7">
         <f t="shared" ref="K32:K34" si="3">I32-J32</f>
-        <v>401701.52952380956</v>
+        <v>121578.98952380812</v>
       </c>
       <c r="L32" s="4"/>
       <c r="M32" s="4"/>
@@ -7899,11 +7940,11 @@
       </c>
       <c r="D33" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>16084.539999999992</v>
+        <v>27951.950000000019</v>
       </c>
       <c r="E33" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>71915.460000000006</v>
+        <v>60048.049999999981</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -7959,11 +8000,11 @@
       </c>
       <c r="D34" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>9566.7999999999956</v>
+        <v>15939.879999999988</v>
       </c>
       <c r="E34" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>48433.200000000004</v>
+        <v>42060.12000000001</v>
       </c>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
@@ -8019,11 +8060,11 @@
       </c>
       <c r="D35" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>13919.82</v>
+        <v>24446.020000000004</v>
       </c>
       <c r="E35" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>65080.18</v>
+        <v>54553.979999999996</v>
       </c>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
@@ -8068,11 +8109,11 @@
       </c>
       <c r="D36" s="22">
         <f>_xlfn.XLOOKUP(Tabela13[[#This Row],[REFERENCIA]],'[1]BASE PYTHON'!$E:$E,'[1]BASE PYTHON'!$F:$F,0)</f>
-        <v>0</v>
+        <v>75.12</v>
       </c>
       <c r="E36" s="43">
         <f>Tabela13[[#This Row],[META A]]-Tabela13[[#This Row],[ATINGIDO]]</f>
-        <v>1000</v>
+        <v>924.88</v>
       </c>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
@@ -8179,11 +8220,11 @@
       </c>
       <c r="D40" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[1]"),0)</f>
-        <v>164169.47999999969</v>
+        <v>163093.37999999971</v>
       </c>
       <c r="E40" s="7">
         <f>C40-D40</f>
-        <v>410211.47238095273</v>
+        <v>411287.57238095271</v>
       </c>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
@@ -8215,11 +8256,11 @@
       </c>
       <c r="D41" s="2">
         <f>IFERROR(GETPIVOTDATA("[Measures].[Soma de TOTAL 3]",'[1]BASE PYTHON'!$P$47,"[Intervalo 2].[SEMANA]","[Intervalo 2].[SEMANA].&amp;[2]"),0)</f>
-        <v>823417.25000000081</v>
+        <v>1398857.0399999972</v>
       </c>
       <c r="E41" s="7">
         <f t="shared" ref="E41:E43" si="4">C41-D41</f>
-        <v>612535.13095238025</v>
+        <v>37095.34095238382</v>
       </c>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>

</xml_diff>